<commit_message>
leads: обновление 2026-07-03 08:13 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$123</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$159</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q123"/>
+  <dimension ref="A1:Q159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -634,7 +634,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -719,7 +719,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -804,7 +804,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -889,7 +889,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -974,7 +974,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1059,7 +1059,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1144,7 +1144,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1229,7 +1229,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1314,7 +1314,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1399,7 +1399,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1484,7 +1484,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1569,7 +1569,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1654,7 +1654,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1739,7 +1739,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1824,7 +1824,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1909,7 +1909,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -2079,7 +2079,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -2164,7 +2164,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -2249,7 +2249,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2334,7 +2334,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2419,7 +2419,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2504,7 +2504,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -2589,7 +2589,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2674,7 +2674,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -2759,7 +2759,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -2844,7 +2844,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -3014,7 +3014,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -3071,7 +3071,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -3156,7 +3156,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -3241,7 +3241,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3326,7 +3326,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -3411,7 +3411,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -3496,7 +3496,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -3581,7 +3581,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -3666,7 +3666,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -3751,7 +3751,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -3836,7 +3836,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -3921,7 +3921,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -4092,7 +4092,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -4177,7 +4177,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -4262,7 +4262,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -4347,7 +4347,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -4432,7 +4432,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -4602,7 +4602,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -4687,7 +4687,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -4772,7 +4772,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -4857,7 +4857,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -4942,7 +4942,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -5112,7 +5112,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -5197,7 +5197,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -5282,7 +5282,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -5367,7 +5367,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -5452,7 +5452,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -5622,7 +5622,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -5707,7 +5707,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -5792,7 +5792,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -5877,7 +5877,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -5962,7 +5962,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -6132,7 +6132,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -6217,7 +6217,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -6302,7 +6302,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -6387,7 +6387,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -6472,7 +6472,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -6642,7 +6642,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -6727,7 +6727,7 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -6812,7 +6812,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -6897,7 +6897,7 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -6982,7 +6982,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -7152,7 +7152,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -7237,7 +7237,7 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -7322,7 +7322,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -7407,7 +7407,7 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -7492,7 +7492,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -7662,7 +7662,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -7747,7 +7747,7 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -7832,7 +7832,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -7917,7 +7917,7 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -8002,7 +8002,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -8172,7 +8172,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -8257,7 +8257,7 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -8334,7 +8334,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -8411,7 +8411,7 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -8488,7 +8488,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -8565,7 +8565,7 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -8650,7 +8650,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -8735,7 +8735,7 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -8820,7 +8820,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -8905,7 +8905,7 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -8990,7 +8990,7 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -9075,7 +9075,7 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
@@ -9160,7 +9160,7 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -9245,7 +9245,7 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
@@ -9330,7 +9330,7 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -9415,7 +9415,7 @@
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
@@ -9500,7 +9500,7 @@
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -9585,7 +9585,7 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
@@ -9670,7 +9670,7 @@
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
@@ -9755,7 +9755,7 @@
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
@@ -9840,7 +9840,7 @@
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
@@ -9925,7 +9925,7 @@
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
@@ -10010,7 +10010,7 @@
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
@@ -10095,7 +10095,7 @@
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
@@ -10180,7 +10180,7 @@
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -10265,7 +10265,7 @@
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
@@ -10350,7 +10350,7 @@
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
@@ -10435,7 +10435,7 @@
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
@@ -10520,7 +10520,7 @@
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
@@ -10605,7 +10605,7 @@
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
@@ -10690,7 +10690,7 @@
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
@@ -10775,7 +10775,7 @@
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:48</t>
+          <t>2026-07-03 08:13</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
@@ -10857,8 +10857,2848 @@
         </is>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr"/>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>4510835</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>Реализация. Невостребованные складские остатки (не б/у). Запасные части для ГТО (для автосамосвалов, автобусов, легкового транспорта, бульдозеров, экскаваторов, грейдеров)
+Реализация. Запасные части для автосамосвалов HOWO, БЕЛАЗ, КАМАЗ, SCANIA; бульдозеров Cat 834, D9R, DT10T, KOMATSU WD600, PR754, Т-25; грейдера САТ140М; экскаваторов Bucyrus RH120E, Hyundai R520LC, ЭО, ЭШ, ЭКГ, ЕК-400, Liebherr R984C....  2445 V-ACS 32-R1195-9Дорожныйзнак "Осторожно газопровод" ДПТ-М  ... КАТУШКА электромагнитная 1317540-74030 Керамогранитплита300х600мм Керамогранитплита600х600мм Килоамперметр М42301 1, ... 90/460 У2Плита75570-8608180Плитаднища 1080.52.101Плиталотков ПТ  ...</t>
+        </is>
+      </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>ООО "УК "СИБАНТРАЦИТ"</t>
+        </is>
+      </c>
+      <c r="H124" s="2" t="inlineStr">
+        <is>
+          <t>ООО "УК "СИБАНТРАЦИТ"</t>
+        </is>
+      </c>
+      <c r="I124" s="2" t="inlineStr">
+        <is>
+          <t>9703160290</t>
+        </is>
+      </c>
+      <c r="J124" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K124" s="2" t="inlineStr">
+        <is>
+          <t>Мельников Сергей Владимирович</t>
+        </is>
+      </c>
+      <c r="L124" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M124" s="2" t="inlineStr">
+        <is>
+          <t>70.22</t>
+        </is>
+      </c>
+      <c r="N124" s="2" t="inlineStr"/>
+      <c r="O124" s="2" t="inlineStr">
+        <is>
+          <t>02.07.2026 13:09 — 16.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P124" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Усачёва, д 2 стр 1, помещ 2/1</t>
+        </is>
+      </c>
+      <c r="Q124" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=c2040d938e8d3cf8fc199ed3bc440b5b4a1fe4c3&amp;tsid=4510835003</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr"/>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t>4506366</t>
+        </is>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>Ремонтдорожнойплитки на подъездной и выездной дороге от главного входа гостиницы</t>
+        </is>
+      </c>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЛОТТЕ РУС"</t>
+        </is>
+      </c>
+      <c r="H125" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЛОТТЕ РУС"</t>
+        </is>
+      </c>
+      <c r="I125" s="2" t="inlineStr">
+        <is>
+          <t>7704169180</t>
+        </is>
+      </c>
+      <c r="J125" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K125" s="2" t="inlineStr">
+        <is>
+          <t>Андерсен Мортен Бундгорд</t>
+        </is>
+      </c>
+      <c r="L125" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M125" s="2" t="inlineStr">
+        <is>
+          <t>55.10</t>
+        </is>
+      </c>
+      <c r="N125" s="2" t="inlineStr"/>
+      <c r="O125" s="2" t="inlineStr">
+        <is>
+          <t>29.06.2026 16:30 — 03.07.2026 17:18</t>
+        </is>
+      </c>
+      <c r="P125" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Новинский б-р, д 8 стр 2</t>
+        </is>
+      </c>
+      <c r="Q125" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/remont-dorozhnoi-plitki-na-pod-ezdnoi-i-vyezdnoi-doroge-ot-glavnogo/tender-4506366/#btid=2&amp;sqh=c2040d938e8d3cf8fc199ed3bc440b5b4a1fe4c3&amp;tsid=4506366458</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr"/>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>4505276</t>
+        </is>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>Плита дорожнаяПДН 6000х2000х140мм ГОСТ 56600-2015 - 168 штук С доставкой до месторождения</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>ООО "МАНГАЗЕЯ МАЙНИНГ"</t>
+        </is>
+      </c>
+      <c r="H126" s="2" t="inlineStr">
+        <is>
+          <t>ООО "МАНГАЗЕЯ МАЙНИНГ"</t>
+        </is>
+      </c>
+      <c r="I126" s="2" t="inlineStr">
+        <is>
+          <t>5003095828</t>
+        </is>
+      </c>
+      <c r="J126" s="2" t="inlineStr">
+        <is>
+          <t>Забайкальский край</t>
+        </is>
+      </c>
+      <c r="K126" s="2" t="inlineStr">
+        <is>
+          <t>Гусев Михаил Михайлович</t>
+        </is>
+      </c>
+      <c r="L126" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M126" s="2" t="inlineStr">
+        <is>
+          <t>70.22</t>
+        </is>
+      </c>
+      <c r="N126" s="2" t="inlineStr"/>
+      <c r="O126" s="2" t="inlineStr">
+        <is>
+          <t>29.06.2026 10:39 — 03.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P126" s="2" t="inlineStr">
+        <is>
+          <t>г Чита, ул Костюшко-Григоровича, д 5, помещ 13 офис 405</t>
+        </is>
+      </c>
+      <c r="Q126" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/plita-dorozhnaia-pdn-6000kh2000kh140mm-gost-56600-2015-168-shtuk-s/tender-4505276/#btid=2&amp;sqh=c2040d938e8d3cf8fc199ed3bc440b5b4a1fe4c3&amp;tsid=4505276004</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr"/>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr">
+        <is>
+          <t>4503612</t>
+        </is>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>RUNEV-11652 на выполнение работ по сортировке, разделке и вывозу демонтированных 
+трубопроводов и металлоконструкций на склад хранения. Вывозу строительного мусора на утилизацию с площадки Б-9 АО «Невинномысский Азот»....  площадки 600м² для выполнения работ, издорожных плит(60 шт, поставка заказчика), с выравниванием ...</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H127" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I127" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J127" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K127" s="2" t="inlineStr"/>
+      <c r="L127" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M127" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N127" s="2" t="inlineStr"/>
+      <c r="O127" s="2" t="inlineStr">
+        <is>
+          <t>26.06.2026 10:29 — 08.07.2026 17:00</t>
+        </is>
+      </c>
+      <c r="P127" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q127" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=c2040d938e8d3cf8fc199ed3bc440b5b4a1fe4c3&amp;tsid=4503612458</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr"/>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>4130106</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>Реализация ЖБИ изделий с АО "Мальцовский портландцемент"Бордюрдорожный1000х300х150мм Ясногорский завод строительных материалов Кольца  ...  КС-7-3 ЖБИ 24/7Плитаопорная ОП-1К ПС-334-08 ...Плитаперекрытия колодца 1ПП-20-2 D2200  ...</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЦЕМРОС"</t>
+        </is>
+      </c>
+      <c r="H128" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЦЕМРОС"</t>
+        </is>
+      </c>
+      <c r="I128" s="2" t="inlineStr">
+        <is>
+          <t>7708117908</t>
+        </is>
+      </c>
+      <c r="J128" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K128" s="2" t="inlineStr">
+        <is>
+          <t>Шматов Вячеслав Вячеславович</t>
+        </is>
+      </c>
+      <c r="L128" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M128" s="2" t="inlineStr">
+        <is>
+          <t>23.51</t>
+        </is>
+      </c>
+      <c r="N128" s="2" t="inlineStr"/>
+      <c r="O128" s="2" t="inlineStr">
+        <is>
+          <t>06.08.2025 15:30 — 07.08.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P128" s="2" t="inlineStr">
+        <is>
+          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
+        </is>
+      </c>
+      <c r="Q128" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=c2040d938e8d3cf8fc199ed3bc440b5b4a1fe4c3&amp;tsid=4130106003</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr"/>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E129" s="2" t="inlineStr">
+        <is>
+          <t>4156098</t>
+        </is>
+      </c>
+      <c r="F129" s="2" t="inlineStr">
+        <is>
+          <t>Реализация. Линия погрузки угля Б/У (ЛК-60Т 2022 г.в.). Конвейер ленточный подающий ЛК-60Т, линия погрузки угля, бункер приемный, кровельные металлоконструкции. Год ввода в эксплуатацию 2022. Исправное тех.состояние. Продажа бездорожных плит. Демонтаж и самовывоз силами и за счет покупателя.</t>
+        </is>
+      </c>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>ООО "УК "СИБАНТРАЦИТ"</t>
+        </is>
+      </c>
+      <c r="H129" s="2" t="inlineStr">
+        <is>
+          <t>ООО "УК "СИБАНТРАЦИТ"</t>
+        </is>
+      </c>
+      <c r="I129" s="2" t="inlineStr">
+        <is>
+          <t>9703160290</t>
+        </is>
+      </c>
+      <c r="J129" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K129" s="2" t="inlineStr">
+        <is>
+          <t>Мельников Сергей Владимирович</t>
+        </is>
+      </c>
+      <c r="L129" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M129" s="2" t="inlineStr">
+        <is>
+          <t>70.22</t>
+        </is>
+      </c>
+      <c r="N129" s="2" t="inlineStr"/>
+      <c r="O129" s="2" t="inlineStr">
+        <is>
+          <t>02.09.2025 11:51 — 03.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P129" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Усачёва, д 2 стр 1, помещ 2/1</t>
+        </is>
+      </c>
+      <c r="Q129" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/realizatsiia-liniia-pogruzki-uglia-b-u-lk-60t-2022-g-v/tender-4156098/#btid=2&amp;sqh=c2040d938e8d3cf8fc199ed3bc440b5b4a1fe4c3&amp;tsid=4156098003</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr"/>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>4498936</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>Продажа невостребованных ТМЦ -Плиты аэродромные, Фильтр сетчатый МИГ, Ролик лебедки Материалы с хранения. Перечень ориентировочный, может измениться в меньшую сторону за счет возможной востребованности.</t>
+        </is>
+      </c>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СИБУР"</t>
+        </is>
+      </c>
+      <c r="H130" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СИБУР"</t>
+        </is>
+      </c>
+      <c r="I130" s="2" t="inlineStr">
+        <is>
+          <t>7727576505</t>
+        </is>
+      </c>
+      <c r="J130" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K130" s="2" t="inlineStr">
+        <is>
+          <t>Карисалов Михаил Юрьевич</t>
+        </is>
+      </c>
+      <c r="L130" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M130" s="2" t="inlineStr">
+        <is>
+          <t>70.10</t>
+        </is>
+      </c>
+      <c r="N130" s="2" t="inlineStr"/>
+      <c r="O130" s="2" t="inlineStr">
+        <is>
+          <t>23.06.2026 13:41 — 07.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P130" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Кржижановского, д 16 к 3</t>
+        </is>
+      </c>
+      <c r="Q130" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=dabfb68ea959465f2b0252c6591b51dd88144064&amp;tsid=4498936003</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr"/>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>4497016</t>
+        </is>
+      </c>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>BOX_00514 Выполнение работ по строительству общежития №4 на 80 койко-мест временного вахтового поселка на месторождении «Бараньевское»
+Выполнение работ по строительству общежития №4 на 80 койко-мест временного вахтового поселка АО «Камчатское золото», на месторождении «Бараньевское»ЛОТ №1: Монтаж фундамента (висячиезабивные сваииз стальных труб 219×5 мм)  ...</t>
+        </is>
+      </c>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>ООО «Фокси-Бокс»</t>
+        </is>
+      </c>
+      <c r="H131" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ФОКСИ-БОКС"</t>
+        </is>
+      </c>
+      <c r="I131" s="2" t="inlineStr">
+        <is>
+          <t>7805780074</t>
+        </is>
+      </c>
+      <c r="J131" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="K131" s="2" t="inlineStr">
+        <is>
+          <t>Василенко Иван Михайлович</t>
+        </is>
+      </c>
+      <c r="L131" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M131" s="2" t="inlineStr">
+        <is>
+          <t>46.73</t>
+        </is>
+      </c>
+      <c r="N131" s="2" t="inlineStr"/>
+      <c r="O131" s="2" t="inlineStr">
+        <is>
+          <t>22.06.2026 16:20 — 06.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P131" s="2" t="inlineStr">
+        <is>
+          <t>196006, Г.САНКТ-ПЕТЕРБУРГ, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОСКОВСКАЯ ЗАСТАВА, УЛ ЗАСТАВСКАЯ, Д. 7, ЛИТЕРА А, ПОМЕЩ. 1-Н, ПОМЕЩ. № 157</t>
+        </is>
+      </c>
+      <c r="Q131" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=cfd976124f7713c977a6310491949bff7ed27741&amp;tsid=4497016004</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr"/>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>4475879</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>Электро/пневмо и ручной инструмент/Электроизм. инструмент/Расходные мат-лы
+РТИ, РВД, шланги, ремни
+Сварочное обор-е, запчасти и расходные материалы
+Уплотнительный материал (прокладки, паронит, набивка сальниковая)...  Шина цепной пилы Oregon 752HSFL104Кольцостопор. нар. 210х5 DIN471 Andritz ... клин для бревен Sandvik 1401КольцоAbicor Binzel 757.D007 вихреобразующее ...  Kron ЦПВС-5 RAL7012 КрышкаколодцаП10 ж/б Игла клапана ... Kron ПСВС-3 RAL7012 О-кольцо11,3х2,4 NBR70 Ремень ...</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+        </is>
+      </c>
+      <c r="H132" s="2" t="inlineStr">
+        <is>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+        </is>
+      </c>
+      <c r="I132" s="2" t="inlineStr">
+        <is>
+          <t>4704012472</t>
+        </is>
+      </c>
+      <c r="J132" s="2" t="inlineStr">
+        <is>
+          <t>Ленинградская обл</t>
+        </is>
+      </c>
+      <c r="K132" s="2" t="inlineStr">
+        <is>
+          <t>Габидуллин Тимур Махмудович</t>
+        </is>
+      </c>
+      <c r="L132" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M132" s="2" t="inlineStr">
+        <is>
+          <t>17.12</t>
+        </is>
+      </c>
+      <c r="N132" s="2" t="inlineStr"/>
+      <c r="O132" s="2" t="inlineStr">
+        <is>
+          <t>03.06.2026 15:56 — 30.07.2026 20:00</t>
+        </is>
+      </c>
+      <c r="P132" s="2" t="inlineStr">
+        <is>
+          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+        </is>
+      </c>
+      <c r="Q132" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=fd5ef2676c9e0b3e7ca0da300e6a19f6e92e9874&amp;tsid=4475879003</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr"/>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="inlineStr">
+        <is>
+          <t>4508331</t>
+        </is>
+      </c>
+      <c r="F133" s="2" t="inlineStr">
+        <is>
+          <t>Плита ПАГ-14А600ГОСТ 25912-2015 для ООО ГРК Амикан. Требуется жесткая упаковка по ГОСТу КП по форме ТД Полиметалл. В цену включить стоимость доставки до адреса в г. Лесосибирск и обрешетки. При подаче аналогов необходимо приложить тех. документацию</t>
+        </is>
+      </c>
+      <c r="G133" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+        </is>
+      </c>
+      <c r="H133" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+        </is>
+      </c>
+      <c r="I133" s="2" t="inlineStr">
+        <is>
+          <t>7805368914</t>
+        </is>
+      </c>
+      <c r="J133" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="K133" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
+        </is>
+      </c>
+      <c r="L133" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M133" s="2" t="inlineStr">
+        <is>
+          <t>46.90</t>
+        </is>
+      </c>
+      <c r="N133" s="2" t="inlineStr"/>
+      <c r="O133" s="2" t="inlineStr">
+        <is>
+          <t>01.07.2026 05:44 — 08.07.2026 10:00</t>
+        </is>
+      </c>
+      <c r="P133" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
+        </is>
+      </c>
+      <c r="Q133" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=6f11029064c0ad24d84db69e4ec72f186c321785&amp;tsid=4508331004</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr"/>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>4510341</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>ЖБИ(чеч 34\25 7510 \ 17338)</t>
+        </is>
+      </c>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="H134" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="I134" s="2" t="inlineStr">
+        <is>
+          <t>7724498866</t>
+        </is>
+      </c>
+      <c r="J134" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K134" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
+      <c r="L134" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M134" s="2" t="inlineStr">
+        <is>
+          <t>46.73</t>
+        </is>
+      </c>
+      <c r="N134" s="2" t="inlineStr"/>
+      <c r="O134" s="2" t="inlineStr">
+        <is>
+          <t>02.07.2026 09:54 — 03.07.2026 15:00</t>
+        </is>
+      </c>
+      <c r="P134" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+        </is>
+      </c>
+      <c r="Q134" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=c883c80d526059f0f905d92600ab245159b9380e&amp;tsid=4510341459</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr"/>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr">
+        <is>
+          <t>4510662</t>
+        </is>
+      </c>
+      <c r="F135" s="2" t="inlineStr">
+        <is>
+          <t>(ЖБИизделия/кольца колодезные, плиты ПК15)</t>
+        </is>
+      </c>
+      <c r="G135" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="H135" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="I135" s="2" t="inlineStr">
+        <is>
+          <t>7724498866</t>
+        </is>
+      </c>
+      <c r="J135" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K135" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
+      <c r="L135" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M135" s="2" t="inlineStr">
+        <is>
+          <t>46.73</t>
+        </is>
+      </c>
+      <c r="N135" s="2" t="inlineStr"/>
+      <c r="O135" s="2" t="inlineStr">
+        <is>
+          <t>02.07.2026 12:00 — 03.07.2026 15:00</t>
+        </is>
+      </c>
+      <c r="P135" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+        </is>
+      </c>
+      <c r="Q135" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-izdeliia-koltsa-kolodeznye-plity-pk15/tender-4510662/#btid=2&amp;sqh=c883c80d526059f0f905d92600ab245159b9380e&amp;tsid=4510662459</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr"/>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>4510073</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>ЗакупкаЖБИ- лотки, плиты, бруски, блоки</t>
+        </is>
+      </c>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H136" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I136" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J136" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K136" s="2" t="inlineStr"/>
+      <c r="L136" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M136" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N136" s="2" t="inlineStr"/>
+      <c r="O136" s="2" t="inlineStr">
+        <is>
+          <t>02.07.2026 07:55 — 05.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P136" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q136" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-lotki-plity-bruski-bloki/tender-4510073/#btid=2&amp;sqh=c883c80d526059f0f905d92600ab245159b9380e&amp;tsid=4510073458</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr"/>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>4510504</t>
+        </is>
+      </c>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>(Заявка № ДОР-17560) Лестницы/ЖБИ</t>
+        </is>
+      </c>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="H137" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="I137" s="2" t="inlineStr">
+        <is>
+          <t>7724498866</t>
+        </is>
+      </c>
+      <c r="J137" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K137" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
+      <c r="L137" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M137" s="2" t="inlineStr">
+        <is>
+          <t>46.73</t>
+        </is>
+      </c>
+      <c r="N137" s="2" t="inlineStr"/>
+      <c r="O137" s="2" t="inlineStr">
+        <is>
+          <t>02.07.2026 10:55 — 03.07.2026 15:00</t>
+        </is>
+      </c>
+      <c r="P137" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+        </is>
+      </c>
+      <c r="Q137" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zaiavka-dor-17560-lestnitsy-zhbi/tender-4510504/#btid=2&amp;sqh=c883c80d526059f0f905d92600ab245159b9380e&amp;tsid=4510504459</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr"/>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>4510823</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>(ДОР-17553)ЖБИ/Лестницы ВЛ-2/Скоба</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="H138" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="I138" s="2" t="inlineStr">
+        <is>
+          <t>7724498866</t>
+        </is>
+      </c>
+      <c r="J138" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K138" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
+      <c r="L138" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M138" s="2" t="inlineStr">
+        <is>
+          <t>46.73</t>
+        </is>
+      </c>
+      <c r="N138" s="2" t="inlineStr"/>
+      <c r="O138" s="2" t="inlineStr">
+        <is>
+          <t>02.07.2026 12:55 — 03.07.2026 15:00</t>
+        </is>
+      </c>
+      <c r="P138" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+        </is>
+      </c>
+      <c r="Q138" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/dor-17553-zhbi-lestnitsy-vl-2-skoba/tender-4510823/#btid=2&amp;sqh=c883c80d526059f0f905d92600ab245159b9380e&amp;tsid=4510823459</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr"/>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
+          <t>4508347</t>
+        </is>
+      </c>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>ЖБИКЕМГРЭС</t>
+        </is>
+      </c>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H139" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I139" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J139" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K139" s="2" t="inlineStr"/>
+      <c r="L139" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M139" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N139" s="2" t="inlineStr"/>
+      <c r="O139" s="2" t="inlineStr">
+        <is>
+          <t>01.07.2026 05:45 — 10.07.2026 00:00</t>
+        </is>
+      </c>
+      <c r="P139" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q139" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=c883c80d526059f0f905d92600ab245159b9380e&amp;tsid=4508347458</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr"/>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>4508689</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>Железобетонные плиты Б/У 
+Необходимы плиты, это те которые выдерживают нагрузку т.к. на эту плиту будет заезжать техника весом до 70тонн. Приоритетно с целью минимизации затрат рассмотрим плиты Б/У  размер произвольный но ближе 2х4; 3х3; 2х6. Количество плит необходимо +/- 50 шт. (данные плиты предназначаются для размещения на них запчастей и хоз. деятельности Горного цеха)Б/УЖБИплиты</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЦЕМРОС"</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЦЕМРОС"</t>
+        </is>
+      </c>
+      <c r="I140" s="2" t="inlineStr">
+        <is>
+          <t>7708117908</t>
+        </is>
+      </c>
+      <c r="J140" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K140" s="2" t="inlineStr">
+        <is>
+          <t>Шматов Вячеслав Вячеславович</t>
+        </is>
+      </c>
+      <c r="L140" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M140" s="2" t="inlineStr">
+        <is>
+          <t>23.51</t>
+        </is>
+      </c>
+      <c r="N140" s="2" t="inlineStr"/>
+      <c r="O140" s="2" t="inlineStr">
+        <is>
+          <t>01.07.2026 09:45 — 06.07.2026 09:00</t>
+        </is>
+      </c>
+      <c r="P140" s="2" t="inlineStr">
+        <is>
+          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
+        </is>
+      </c>
+      <c r="Q140" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zhelezobetonnye-plity-b-u-neobkhodimy-plity-eto-te-kotorye/tender-4508689/#btid=2&amp;sqh=c883c80d526059f0f905d92600ab245159b9380e&amp;tsid=4508689458</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr"/>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>4489772</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы 1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
+        </is>
+      </c>
+      <c r="H141" s="2" t="inlineStr">
+        <is>
+          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
+        </is>
+      </c>
+      <c r="I141" s="2" t="inlineStr">
+        <is>
+          <t>7736583259</t>
+        </is>
+      </c>
+      <c r="J141" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K141" s="2" t="inlineStr">
+        <is>
+          <t>Масько Александр Вадимович</t>
+        </is>
+      </c>
+      <c r="L141" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M141" s="2" t="inlineStr">
+        <is>
+          <t>70.10</t>
+        </is>
+      </c>
+      <c r="N141" s="2" t="inlineStr"/>
+      <c r="O141" s="2" t="inlineStr">
+        <is>
+          <t>16.06.2026 11:00 — 16.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P141" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Старая Басманная, д 12 стр 1</t>
+        </is>
+      </c>
+      <c r="Q141" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=c883c80d526059f0f905d92600ab245159b9380e&amp;tsid=4489772003</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr"/>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>4474790</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+        </is>
+      </c>
+      <c r="I142" s="2" t="inlineStr">
+        <is>
+          <t>4704012472</t>
+        </is>
+      </c>
+      <c r="J142" s="2" t="inlineStr">
+        <is>
+          <t>Ленинградская обл</t>
+        </is>
+      </c>
+      <c r="K142" s="2" t="inlineStr">
+        <is>
+          <t>Габидуллин Тимур Махмудович</t>
+        </is>
+      </c>
+      <c r="L142" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M142" s="2" t="inlineStr">
+        <is>
+          <t>17.12</t>
+        </is>
+      </c>
+      <c r="N142" s="2" t="inlineStr"/>
+      <c r="O142" s="2" t="inlineStr">
+        <is>
+          <t>03.06.2026 09:59 — 30.07.2026 20:00</t>
+        </is>
+      </c>
+      <c r="P142" s="2" t="inlineStr">
+        <is>
+          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+        </is>
+      </c>
+      <c r="Q142" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=c883c80d526059f0f905d92600ab245159b9380e&amp;tsid=4474790003</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr"/>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>4180328</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, г.Диксон). ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, ПГТ Диксон).</t>
+        </is>
+      </c>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
+        </is>
+      </c>
+      <c r="H143" s="2" t="inlineStr">
+        <is>
+          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
+        </is>
+      </c>
+      <c r="I143" s="2" t="inlineStr">
+        <is>
+          <t>7714456916</t>
+        </is>
+      </c>
+      <c r="J143" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K143" s="2" t="inlineStr">
+        <is>
+          <t>Наумов Андрей Александрович</t>
+        </is>
+      </c>
+      <c r="L143" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M143" s="2" t="inlineStr">
+        <is>
+          <t>70.22</t>
+        </is>
+      </c>
+      <c r="N143" s="2" t="inlineStr"/>
+      <c r="O143" s="2" t="inlineStr">
+        <is>
+          <t>24.09.2025 15:32 — 23.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P143" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Денежный пер, д 9/6</t>
+        </is>
+      </c>
+      <c r="Q143" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=c883c80d526059f0f905d92600ab245159b9380e&amp;tsid=4180328003</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr"/>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>3973258</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="inlineStr">
+        <is>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+        </is>
+      </c>
+      <c r="I144" s="2" t="inlineStr">
+        <is>
+          <t>4704012472</t>
+        </is>
+      </c>
+      <c r="J144" s="2" t="inlineStr">
+        <is>
+          <t>Ленинградская обл</t>
+        </is>
+      </c>
+      <c r="K144" s="2" t="inlineStr">
+        <is>
+          <t>Габидуллин Тимур Махмудович</t>
+        </is>
+      </c>
+      <c r="L144" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M144" s="2" t="inlineStr">
+        <is>
+          <t>17.12</t>
+        </is>
+      </c>
+      <c r="N144" s="2" t="inlineStr"/>
+      <c r="O144" s="2" t="inlineStr">
+        <is>
+          <t>10.03.2025 00:48 — 30.07.2026 23:00</t>
+        </is>
+      </c>
+      <c r="P144" s="2" t="inlineStr">
+        <is>
+          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+        </is>
+      </c>
+      <c r="Q144" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=c883c80d526059f0f905d92600ab245159b9380e&amp;tsid=3973258003</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr"/>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="inlineStr">
+        <is>
+          <t>4509622</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>Производство вторичного щебня из ломажелезобетонных изделий</t>
+        </is>
+      </c>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H145" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I145" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J145" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K145" s="2" t="inlineStr"/>
+      <c r="L145" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M145" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N145" s="2" t="inlineStr"/>
+      <c r="O145" s="2" t="inlineStr">
+        <is>
+          <t>01.07.2026 16:05 — 10.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P145" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q145" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/proizvodstvo-vtorichnogo-shchebnia-iz-loma-zhelezobetonnykh-izdelii/tender-4509622/#btid=2&amp;sqh=8c1a00b72158ca0d4a44fffc89559572d54c0750&amp;tsid=4509622458</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr"/>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>4508845</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>Панель ограждения 3ПБ40.20 2550х4000х160мм 3.017-3.1-7 серия 3.017-3 – 24 шт (чертеж на стр. 11 типового альбомажелезобетонных изделий)</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЦЕМРОС"</t>
+        </is>
+      </c>
+      <c r="H146" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЦЕМРОС"</t>
+        </is>
+      </c>
+      <c r="I146" s="2" t="inlineStr">
+        <is>
+          <t>7708117908</t>
+        </is>
+      </c>
+      <c r="J146" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K146" s="2" t="inlineStr">
+        <is>
+          <t>Шматов Вячеслав Вячеславович</t>
+        </is>
+      </c>
+      <c r="L146" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M146" s="2" t="inlineStr">
+        <is>
+          <t>23.51</t>
+        </is>
+      </c>
+      <c r="N146" s="2" t="inlineStr"/>
+      <c r="O146" s="2" t="inlineStr">
+        <is>
+          <t>01.07.2026 10:44 — 03.07.2026 13:00</t>
+        </is>
+      </c>
+      <c r="P146" s="2" t="inlineStr">
+        <is>
+          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
+        </is>
+      </c>
+      <c r="Q146" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/panel-ograzhdeniia-3pb40-20-2550kh4000kh160mm-3-017-3-1-7-seriia-3-017-3/tender-4508845/#btid=2&amp;sqh=8c1a00b72158ca0d4a44fffc89559572d54c0750&amp;tsid=4508845458</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr"/>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E147" s="2" t="inlineStr">
+        <is>
+          <t>4474238</t>
+        </is>
+      </c>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>Железобетонные изделияПлита перекрытия лотков П22-15И Плитка 2400*1500*160 б/у Плита перекрытия ПК 60-12 б/у</t>
+        </is>
+      </c>
+      <c r="G147" s="2" t="inlineStr">
+        <is>
+          <t>ПАО "Коршуновский ГОК"</t>
+        </is>
+      </c>
+      <c r="H147" s="2" t="inlineStr">
+        <is>
+          <t>ПАО "КОРШУНОВСКИЙ ГОК"</t>
+        </is>
+      </c>
+      <c r="I147" s="2" t="inlineStr">
+        <is>
+          <t>3834002314</t>
+        </is>
+      </c>
+      <c r="J147" s="2" t="inlineStr">
+        <is>
+          <t>Иркутская обл</t>
+        </is>
+      </c>
+      <c r="K147" s="2" t="inlineStr">
+        <is>
+          <t>Иванов Алексей Васильевич</t>
+        </is>
+      </c>
+      <c r="L147" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M147" s="2" t="inlineStr">
+        <is>
+          <t>07.10.2</t>
+        </is>
+      </c>
+      <c r="N147" s="2" t="inlineStr"/>
+      <c r="O147" s="2" t="inlineStr">
+        <is>
+          <t>11.06.2026 09:23 — 06.07.2026 09:00</t>
+        </is>
+      </c>
+      <c r="P147" s="2" t="inlineStr">
+        <is>
+          <t>Иркутская обл, г Железногорск-Илимский, ул Иващенко, д 9А/1</t>
+        </is>
+      </c>
+      <c r="Q147" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/zhelezobetonnye-izdeliia/tender-4474238/#btid=2&amp;sqh=8c1a00b72158ca0d4a44fffc89559572d54c0750&amp;tsid=4474238003</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr"/>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>4511621</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>Закупка аккумуляторных батарей (залитых) для нужд АО "Павловск Неруд" с поставкой в Августе 2026г.
+Обязательная расценка стоимости доставки, возможен забор груза на условиях самовывоза.
+В ТКП просьба отразить локацию склада отгрузки.
+ТКП БЕЗ указания стоимости доставки рассматриваться НЕ БУДУТ.
+Заказчик АО "Павловск Неруд" предприятие АО "Национальная нерудная компания"Аккумулятор ТН-550Перемычкам/ц для АКБ 115,5мм ТН-550Перемычкам/ц для АКБ 212,0мм ТН-550 Транспортная услуга</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="inlineStr">
+        <is>
+          <t>АО "ННК"</t>
+        </is>
+      </c>
+      <c r="H148" s="2" t="inlineStr">
+        <is>
+          <t>АО "ННК-ОЙЛ"</t>
+        </is>
+      </c>
+      <c r="I148" s="2" t="inlineStr">
+        <is>
+          <t>5032049030</t>
+        </is>
+      </c>
+      <c r="J148" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K148" s="2" t="inlineStr">
+        <is>
+          <t>Худайнатов Эдуард Юрьевич</t>
+        </is>
+      </c>
+      <c r="L148" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M148" s="2" t="inlineStr">
+        <is>
+          <t>70.22</t>
+        </is>
+      </c>
+      <c r="N148" s="2" t="inlineStr"/>
+      <c r="O148" s="2" t="inlineStr">
+        <is>
+          <t>03.07.2026 06:22 — 07.07.2026 11:00</t>
+        </is>
+      </c>
+      <c r="P148" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул 1-я Тверская-Ямская, д 5, помещ 1012</t>
+        </is>
+      </c>
+      <c r="Q148" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=f69b60b4476caa237bb19c1c7ba2c7eb638a4ba2&amp;tsid=4511621004</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr"/>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E149" s="2" t="inlineStr">
+        <is>
+          <t>4511787</t>
+        </is>
+      </c>
+      <c r="F149" s="2" t="inlineStr">
+        <is>
+          <t>ЗЧ к автотранспорту... /66 ТЕРМОСТАТ ТС-107-1306100-06ПЕРЕМЫЧКААКБ КЛЕММА-КЛЕММА ПП 500-50 ...</t>
+        </is>
+      </c>
+      <c r="G149" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H149" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I149" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J149" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K149" s="2" t="inlineStr"/>
+      <c r="L149" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M149" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N149" s="2" t="inlineStr"/>
+      <c r="O149" s="2" t="inlineStr">
+        <is>
+          <t>03.07.2026 08:32 — 08.07.2026 00:00</t>
+        </is>
+      </c>
+      <c r="P149" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q149" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=f69b60b4476caa237bb19c1c7ba2c7eb638a4ba2&amp;tsid=4511787458</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr"/>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>4508230</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>Сборный (Изделия электроустановочные и монтажные, Ящики, щиты, шкафы, пункты и комплектующие к ним, Приборы электроизмерительные, реле)
+МГ-019742, МГ-019713, МГ-019696, МГ-019665, МГ-019621, МГ-019620, МГ-019619, МГ-017109... -HESI-EX (5X20), Phoenix Contact 1277638ПеремычкаFBS 10-5, Phoenix Contact 3030213 ...ПеремычкаFBS 10-5 BU, Phoenix Contact  ...</t>
+        </is>
+      </c>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>АО "ИК "АРЛАН"</t>
+        </is>
+      </c>
+      <c r="H150" s="2" t="inlineStr">
+        <is>
+          <t>АО "ИК "АРЛАН"</t>
+        </is>
+      </c>
+      <c r="I150" s="2" t="inlineStr">
+        <is>
+          <t>7722220390</t>
+        </is>
+      </c>
+      <c r="J150" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K150" s="2" t="inlineStr">
+        <is>
+          <t>Барилов Евгений Александрович</t>
+        </is>
+      </c>
+      <c r="L150" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M150" s="2" t="inlineStr">
+        <is>
+          <t>82.99</t>
+        </is>
+      </c>
+      <c r="N150" s="2" t="inlineStr"/>
+      <c r="O150" s="2" t="inlineStr">
+        <is>
+          <t>30.06.2026 17:59 — 09.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P150" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Романов пер, д 4</t>
+        </is>
+      </c>
+      <c r="Q150" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=f69b60b4476caa237bb19c1c7ba2c7eb638a4ba2&amp;tsid=4508230004</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr"/>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E151" s="2" t="inlineStr">
+        <is>
+          <t>4504775</t>
+        </is>
+      </c>
+      <c r="F151" s="2" t="inlineStr">
+        <is>
+          <t>Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники
+Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники...  Трубка пробная № 37-542-000 Соединитель-перемычка04182454 Кольцо стальное №CP48001-0305 Фильтр ...</t>
+        </is>
+      </c>
+      <c r="G151" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+        </is>
+      </c>
+      <c r="H151" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+        </is>
+      </c>
+      <c r="I151" s="2" t="inlineStr">
+        <is>
+          <t>7805368914</t>
+        </is>
+      </c>
+      <c r="J151" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="K151" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
+        </is>
+      </c>
+      <c r="L151" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M151" s="2" t="inlineStr">
+        <is>
+          <t>46.90</t>
+        </is>
+      </c>
+      <c r="N151" s="2" t="inlineStr"/>
+      <c r="O151" s="2" t="inlineStr">
+        <is>
+          <t>27.06.2026 01:36 — 15.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P151" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
+        </is>
+      </c>
+      <c r="Q151" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=f69b60b4476caa237bb19c1c7ba2c7eb638a4ba2&amp;tsid=4504775003</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr"/>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="inlineStr">
+        <is>
+          <t>4501157</t>
+        </is>
+      </c>
+      <c r="F152" s="2" t="inlineStr">
+        <is>
+          <t>Источники электропитания (ИБП, аккумуляторные батареи, блоки питания)...  х 1248 А·ч, включая соединительныеперемычки. Вид положительного электрода - трубчатая пластина ...  с коммутирующей арматурой, межэлементными и межряднымиперемычками, крепежами, комплектом для обслуживания АБ. Тип ...</t>
+        </is>
+      </c>
+      <c r="G152" s="2" t="inlineStr">
+        <is>
+          <t>АО "Мосинжпроект"</t>
+        </is>
+      </c>
+      <c r="H152" s="2" t="inlineStr">
+        <is>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
+        </is>
+      </c>
+      <c r="I152" s="2" t="inlineStr">
+        <is>
+          <t>7701885820</t>
+        </is>
+      </c>
+      <c r="J152" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K152" s="2" t="inlineStr">
+        <is>
+          <t>Сорокин Антон Павлович</t>
+        </is>
+      </c>
+      <c r="L152" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M152" s="2" t="inlineStr">
+        <is>
+          <t>71.12.2</t>
+        </is>
+      </c>
+      <c r="N152" s="2" t="inlineStr"/>
+      <c r="O152" s="2" t="inlineStr">
+        <is>
+          <t>24.06.2026 15:40 — 22.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P152" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+        </is>
+      </c>
+      <c r="Q152" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=f69b60b4476caa237bb19c1c7ba2c7eb638a4ba2&amp;tsid=4501157003</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr"/>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E153" s="2" t="inlineStr">
+        <is>
+          <t>4499964</t>
+        </is>
+      </c>
+      <c r="F153" s="2" t="inlineStr">
+        <is>
+          <t>Автоматика и телемеханика движения поездов... , 13552-00-00В Дроссель-трансформатор (безперемычек) ДТМ-0,17-1000М ЮКЛЯ.672 ...</t>
+        </is>
+      </c>
+      <c r="G153" s="2" t="inlineStr">
+        <is>
+          <t>АО "Мосинжпроект"</t>
+        </is>
+      </c>
+      <c r="H153" s="2" t="inlineStr">
+        <is>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
+        </is>
+      </c>
+      <c r="I153" s="2" t="inlineStr">
+        <is>
+          <t>7701885820</t>
+        </is>
+      </c>
+      <c r="J153" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K153" s="2" t="inlineStr">
+        <is>
+          <t>Сорокин Антон Павлович</t>
+        </is>
+      </c>
+      <c r="L153" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M153" s="2" t="inlineStr">
+        <is>
+          <t>71.12.2</t>
+        </is>
+      </c>
+      <c r="N153" s="2" t="inlineStr"/>
+      <c r="O153" s="2" t="inlineStr">
+        <is>
+          <t>24.06.2026 08:46 — 15.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P153" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+        </is>
+      </c>
+      <c r="Q153" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=f69b60b4476caa237bb19c1c7ba2c7eb638a4ba2&amp;tsid=4499964003</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr"/>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>4501483</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ
+Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ...  d 50x2", внутренняя резьба RTPБлокуправления наружной установки ICEFREE TR-16 ...  Оповещатель звуковой МАЯК-12-ЗМБлокуправления наружной установки ICEFREE TS- ... проводов КС-3 007004 Велос Переходвентиляционный150х100 - D150, из тонколистовой оцинкованной ...</t>
+        </is>
+      </c>
+      <c r="G154" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+        </is>
+      </c>
+      <c r="H154" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+        </is>
+      </c>
+      <c r="I154" s="2" t="inlineStr">
+        <is>
+          <t>7805368914</t>
+        </is>
+      </c>
+      <c r="J154" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="K154" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
+        </is>
+      </c>
+      <c r="L154" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M154" s="2" t="inlineStr">
+        <is>
+          <t>46.90</t>
+        </is>
+      </c>
+      <c r="N154" s="2" t="inlineStr"/>
+      <c r="O154" s="2" t="inlineStr">
+        <is>
+          <t>25.06.2026 05:03 — 09.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P154" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
+        </is>
+      </c>
+      <c r="Q154" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=cda8ddd07c7eea5b97f8375cab564bf926b67092&amp;tsid=4501483003</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr"/>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E155" s="2" t="inlineStr">
+        <is>
+          <t>4501181</t>
+        </is>
+      </c>
+      <c r="F155" s="2" t="inlineStr">
+        <is>
+          <t>Вентиляторы промышленные и оборудование общеобменной вентиляции...  5Ф РешёткавентиляционнаяАМР 600х300М РешёткавентиляционнаяАМР 150х150М РешёткавентиляционнаяАМР 300х200М  ... мм.; масса 0,65 кгБлокконтроля сопротивления БСК-3.1 Канальный ...  533Па, габаритные размеры 700х467х2230 мм,блоков/моноблоков 5/1, в составе: - ...</t>
+        </is>
+      </c>
+      <c r="G155" s="2" t="inlineStr">
+        <is>
+          <t>АО "Мосинжпроект"</t>
+        </is>
+      </c>
+      <c r="H155" s="2" t="inlineStr">
+        <is>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
+        </is>
+      </c>
+      <c r="I155" s="2" t="inlineStr">
+        <is>
+          <t>7701885820</t>
+        </is>
+      </c>
+      <c r="J155" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K155" s="2" t="inlineStr">
+        <is>
+          <t>Сорокин Антон Павлович</t>
+        </is>
+      </c>
+      <c r="L155" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M155" s="2" t="inlineStr">
+        <is>
+          <t>71.12.2</t>
+        </is>
+      </c>
+      <c r="N155" s="2" t="inlineStr"/>
+      <c r="O155" s="2" t="inlineStr">
+        <is>
+          <t>24.06.2026 15:45 — 22.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P155" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+        </is>
+      </c>
+      <c r="Q155" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=cda8ddd07c7eea5b97f8375cab564bf926b67092&amp;tsid=4501181003</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr"/>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>4500120</t>
+        </is>
+      </c>
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>Коммуникационное оборудование, компьютеры, комплектующие к ним, серверное оборудование и ПО...  и кабелей – 1 компл. Удаленныйблок(репитер) BSF414 , питание 220В,  ... 2х2 Комбайнер специализированный OMU Side (блок1) OMUSC1 Комбайнер специализированный OMU ... контроллер для мониторинга в FlexGain View,вентиляционнаяпанель с фильтрами, комплект кабелей, ...</t>
+        </is>
+      </c>
+      <c r="G156" s="2" t="inlineStr">
+        <is>
+          <t>АО "Мосинжпроект"</t>
+        </is>
+      </c>
+      <c r="H156" s="2" t="inlineStr">
+        <is>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
+        </is>
+      </c>
+      <c r="I156" s="2" t="inlineStr">
+        <is>
+          <t>7701885820</t>
+        </is>
+      </c>
+      <c r="J156" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K156" s="2" t="inlineStr">
+        <is>
+          <t>Сорокин Антон Павлович</t>
+        </is>
+      </c>
+      <c r="L156" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M156" s="2" t="inlineStr">
+        <is>
+          <t>71.12.2</t>
+        </is>
+      </c>
+      <c r="N156" s="2" t="inlineStr"/>
+      <c r="O156" s="2" t="inlineStr">
+        <is>
+          <t>24.06.2026 09:48 — 15.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P156" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+        </is>
+      </c>
+      <c r="Q156" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=cda8ddd07c7eea5b97f8375cab564bf926b67092&amp;tsid=4500120003</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="inlineStr"/>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E157" s="2" t="inlineStr">
+        <is>
+          <t>4496006</t>
+        </is>
+      </c>
+      <c r="F157" s="2" t="inlineStr">
+        <is>
+          <t>Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп
+Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп... -316 ***Петля крепежная стальная ***Платаблокауправления ZC5 CAME ***Средство чистящее " ... /распылитель для чаши Генуя ***РешеткавентиляционнаяРВ-1 225Х225 ***Петля анкерная 0 ... мл ***Папка с зажимом ***РешеткавентиляционнаяРВ-1 325Х125 ***Папка на кольцах ...</t>
+        </is>
+      </c>
+      <c r="G157" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СИБУР"</t>
+        </is>
+      </c>
+      <c r="H157" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СИБУР"</t>
+        </is>
+      </c>
+      <c r="I157" s="2" t="inlineStr">
+        <is>
+          <t>7727576505</t>
+        </is>
+      </c>
+      <c r="J157" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K157" s="2" t="inlineStr">
+        <is>
+          <t>Карисалов Михаил Юрьевич</t>
+        </is>
+      </c>
+      <c r="L157" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M157" s="2" t="inlineStr">
+        <is>
+          <t>70.10</t>
+        </is>
+      </c>
+      <c r="N157" s="2" t="inlineStr"/>
+      <c r="O157" s="2" t="inlineStr">
+        <is>
+          <t>20.06.2026 16:19 — 04.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P157" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Кржижановского, д 16 к 3</t>
+        </is>
+      </c>
+      <c r="Q157" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/prodazha-nelikvidnykh-tmts-tarelki-dlia-filtra-prokladki-dvigatel/tender-4496006/#btid=2&amp;sqh=cda8ddd07c7eea5b97f8375cab564bf926b67092&amp;tsid=4496006003</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr"/>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E158" s="2" t="inlineStr">
+        <is>
+          <t>4483529</t>
+        </is>
+      </c>
+      <c r="F158" s="2" t="inlineStr">
+        <is>
+          <t>Продажа невостребованных ТМЦ - Столбы, модули, керамогранит и т.п.
+Материалы с хранения. Перечень ориентировочный, может измениться в меньшую сторону за счет возможной востребованности....  азотнокислое х.ч. ГОСТ 1277-75БлокТРАНСФОРМАТОРНЫЙ 220В АС 3В DC 500 ...  Омега стыковка панелей между со ***РешеткавентиляционнаяКМУ 200х200 ***ТермСопр_50М_-50/180_5/20мм ...</t>
+        </is>
+      </c>
+      <c r="G158" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СИБУР"</t>
+        </is>
+      </c>
+      <c r="H158" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СИБУР"</t>
+        </is>
+      </c>
+      <c r="I158" s="2" t="inlineStr">
+        <is>
+          <t>7727576505</t>
+        </is>
+      </c>
+      <c r="J158" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K158" s="2" t="inlineStr">
+        <is>
+          <t>Карисалов Михаил Юрьевич</t>
+        </is>
+      </c>
+      <c r="L158" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M158" s="2" t="inlineStr">
+        <is>
+          <t>70.10</t>
+        </is>
+      </c>
+      <c r="N158" s="2" t="inlineStr"/>
+      <c r="O158" s="2" t="inlineStr">
+        <is>
+          <t>09.06.2026 16:07 — 06.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P158" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Кржижановского, д 16 к 3</t>
+        </is>
+      </c>
+      <c r="Q158" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-stolby-moduli-keramogranit-i-t-p/tender-4483529/#btid=2&amp;sqh=cda8ddd07c7eea5b97f8375cab564bf926b67092&amp;tsid=4483529003</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 08:13</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr"/>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E159" s="2" t="inlineStr">
+        <is>
+          <t>4129930</t>
+        </is>
+      </c>
+      <c r="F159" s="2" t="inlineStr">
+        <is>
+          <t>Реализация материалов для ремонта (напольные покрытия, настенные покрытия, окна, двери и т.д.) с АО "Мальцовский портландцемент"Блокдверной балконныйБлокдверной филенчатый ДГ 21х9Блококонный 1500х1000 ммБлококонный 1770х1700 мм Желоб ...  Docke Рама оконная 3000х1200 мм Решеткавентиляционнаянаружная Ручка оконная ГОСТ 5087-80 ...</t>
+        </is>
+      </c>
+      <c r="G159" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЦЕМРОС"</t>
+        </is>
+      </c>
+      <c r="H159" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЦЕМРОС"</t>
+        </is>
+      </c>
+      <c r="I159" s="2" t="inlineStr">
+        <is>
+          <t>7708117908</t>
+        </is>
+      </c>
+      <c r="J159" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K159" s="2" t="inlineStr">
+        <is>
+          <t>Шматов Вячеслав Вячеславович</t>
+        </is>
+      </c>
+      <c r="L159" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M159" s="2" t="inlineStr">
+        <is>
+          <t>23.51</t>
+        </is>
+      </c>
+      <c r="N159" s="2" t="inlineStr"/>
+      <c r="O159" s="2" t="inlineStr">
+        <is>
+          <t>06.08.2025 14:33 — 07.08.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P159" s="2" t="inlineStr">
+        <is>
+          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
+        </is>
+      </c>
+      <c r="Q159" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=cda8ddd07c7eea5b97f8375cab564bf926b67092&amp;tsid=4129930003</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q123"/>
+  <autoFilter ref="A1:Q159"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -10982,6 +13822,42 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q121" r:id="rId120"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q122" r:id="rId121"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q123" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q124" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q125" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q126" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q127" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q128" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q129" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q130" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q131" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q132" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q133" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q134" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q135" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q136" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q137" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q138" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q139" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q140" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q141" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q142" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q143" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q144" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q145" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q146" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q147" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q148" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q149" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q150" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q151" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q152" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q153" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q154" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q155" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q156" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q157" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q158" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q159" r:id="rId158"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-03 10:25 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$159</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$162</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q159"/>
+  <dimension ref="A1:Q162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -634,7 +634,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -719,7 +719,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -804,7 +804,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -889,7 +889,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -974,7 +974,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1059,7 +1059,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1144,7 +1144,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1229,7 +1229,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1314,7 +1314,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1399,7 +1399,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1484,7 +1484,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1569,7 +1569,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1654,7 +1654,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1739,7 +1739,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1824,7 +1824,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1909,7 +1909,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -2079,7 +2079,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -2164,7 +2164,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -2249,7 +2249,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2334,7 +2334,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2419,7 +2419,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2504,7 +2504,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -2589,7 +2589,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2674,7 +2674,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -2759,7 +2759,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -2844,7 +2844,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -3014,7 +3014,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -3071,7 +3071,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -3156,7 +3156,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -3241,7 +3241,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3326,7 +3326,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -3411,7 +3411,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -3496,7 +3496,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -3581,7 +3581,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -3666,7 +3666,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -3751,7 +3751,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -3836,7 +3836,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -3921,7 +3921,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -4092,7 +4092,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -4177,7 +4177,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -4262,7 +4262,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -4347,7 +4347,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -4432,7 +4432,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -4602,7 +4602,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -4687,7 +4687,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -4772,7 +4772,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -4857,7 +4857,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -4942,7 +4942,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -5112,7 +5112,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -5197,7 +5197,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -5282,7 +5282,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -5367,7 +5367,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -5452,7 +5452,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -5622,7 +5622,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -5707,7 +5707,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -5792,7 +5792,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -5877,7 +5877,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -5962,7 +5962,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -6132,7 +6132,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -6217,7 +6217,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -6302,7 +6302,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -6387,7 +6387,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -6472,7 +6472,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -6642,7 +6642,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -6727,7 +6727,7 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -6812,7 +6812,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -6897,7 +6897,7 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -6982,7 +6982,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -7152,7 +7152,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -7237,7 +7237,7 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -7322,7 +7322,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -7407,7 +7407,7 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -7492,7 +7492,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -7662,7 +7662,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -7747,7 +7747,7 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -7832,7 +7832,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -7917,7 +7917,7 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -8002,7 +8002,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -8172,7 +8172,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -8257,7 +8257,7 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -8334,7 +8334,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -8411,7 +8411,7 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -8488,7 +8488,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -8565,7 +8565,7 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -8650,7 +8650,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -8735,7 +8735,7 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -8820,7 +8820,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -8905,7 +8905,7 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -8990,7 +8990,7 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -9075,7 +9075,7 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
@@ -9160,7 +9160,7 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -9245,7 +9245,7 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
@@ -9330,7 +9330,7 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -9415,7 +9415,7 @@
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
@@ -9500,7 +9500,7 @@
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -9585,7 +9585,7 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
@@ -9670,7 +9670,7 @@
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
@@ -9755,7 +9755,7 @@
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
@@ -9840,7 +9840,7 @@
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
@@ -9925,7 +9925,7 @@
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
@@ -10010,7 +10010,7 @@
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
@@ -10095,7 +10095,7 @@
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
@@ -10180,7 +10180,7 @@
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -10265,7 +10265,7 @@
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
@@ -10350,7 +10350,7 @@
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
@@ -10435,7 +10435,7 @@
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
@@ -10520,7 +10520,7 @@
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
@@ -10605,7 +10605,7 @@
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
@@ -10690,7 +10690,7 @@
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
@@ -10775,7 +10775,7 @@
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
@@ -10860,7 +10860,7 @@
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
@@ -10933,14 +10933,14 @@
       </c>
       <c r="Q124" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=c2040d938e8d3cf8fc199ed3bc440b5b4a1fe4c3&amp;tsid=4510835003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=a049a4dc83fe81223b334d9bb351553f178aa0b3&amp;tsid=4510835003</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
@@ -11012,14 +11012,14 @@
       </c>
       <c r="Q125" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/remont-dorozhnoi-plitki-na-pod-ezdnoi-i-vyezdnoi-doroge-ot-glavnogo/tender-4506366/#btid=2&amp;sqh=c2040d938e8d3cf8fc199ed3bc440b5b4a1fe4c3&amp;tsid=4506366458</t>
+          <t>https://www.b2b-center.ru/app/market-next/remont-dorozhnoi-plitki-na-pod-ezdnoi-i-vyezdnoi-doroge-ot-glavnogo/tender-4506366/#btid=2&amp;sqh=a049a4dc83fe81223b334d9bb351553f178aa0b3&amp;tsid=4506366458</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
@@ -11030,44 +11030,41 @@
       <c r="C126" s="2" t="inlineStr"/>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Поставка</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>4505276</t>
+          <t>4503612</t>
         </is>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>Плита дорожнаяПДН 6000х2000х140мм ГОСТ 56600-2015 - 168 штук С доставкой до месторождения</t>
+          <t>RUNEV-11652 на выполнение работ по сортировке, разделке и вывозу демонтированных 
+трубопроводов и металлоконструкций на склад хранения. Вывозу строительного мусора на утилизацию с площадки Б-9 АО «Невинномысский Азот»....  площадки 600м² для выполнения работ, издорожных плит(60 шт, поставка заказчика), с выравниванием ...</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>ООО "МАНГАЗЕЯ МАЙНИНГ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
-          <t>ООО "МАНГАЗЕЯ МАЙНИНГ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>5003095828</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
         <is>
-          <t>Забайкальский край</t>
-        </is>
-      </c>
-      <c r="K126" s="2" t="inlineStr">
-        <is>
-          <t>Гусев Михаил Михайлович</t>
-        </is>
-      </c>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K126" s="2" t="inlineStr"/>
       <c r="L126" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -11075,30 +11072,30 @@
       </c>
       <c r="M126" s="2" t="inlineStr">
         <is>
-          <t>70.22</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N126" s="2" t="inlineStr"/>
       <c r="O126" s="2" t="inlineStr">
         <is>
-          <t>29.06.2026 10:39 — 03.07.2026 12:00</t>
+          <t>26.06.2026 10:29 — 08.07.2026 17:00</t>
         </is>
       </c>
       <c r="P126" s="2" t="inlineStr">
         <is>
-          <t>г Чита, ул Костюшко-Григоровича, д 5, помещ 13 офис 405</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q126" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/plita-dorozhnaia-pdn-6000kh2000kh140mm-gost-56600-2015-168-shtuk-s/tender-4505276/#btid=2&amp;sqh=c2040d938e8d3cf8fc199ed3bc440b5b4a1fe4c3&amp;tsid=4505276004</t>
+          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=a049a4dc83fe81223b334d9bb351553f178aa0b3&amp;tsid=4503612458</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
@@ -11109,33 +11106,32 @@
       <c r="C127" s="2" t="inlineStr"/>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>Поставка</t>
+          <t>Прочее</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>4503612</t>
+          <t>4130106</t>
         </is>
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>RUNEV-11652 на выполнение работ по сортировке, разделке и вывозу демонтированных 
-трубопроводов и металлоконструкций на склад хранения. Вывозу строительного мусора на утилизацию с площадки Б-9 АО «Невинномысский Азот»....  площадки 600м² для выполнения работ, издорожных плит(60 шт, поставка заказчика), с выравниванием ...</t>
+          <t>Реализация ЖБИ изделий с АО "Мальцовский портландцемент"Бордюрдорожный1000х300х150мм Ясногорский завод строительных материалов Кольца  ...  КС-7-3 ЖБИ 24/7Плитаопорная ОП-1К ПС-334-08 ...Плитаперекрытия колодца 1ПП-20-2 D2200  ...</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
       <c r="I127" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>7708117908</t>
         </is>
       </c>
       <c r="J127" s="2" t="inlineStr">
@@ -11143,7 +11139,11 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K127" s="2" t="inlineStr"/>
+      <c r="K127" s="2" t="inlineStr">
+        <is>
+          <t>Шматов Вячеслав Вячеславович</t>
+        </is>
+      </c>
       <c r="L127" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -11151,30 +11151,30 @@
       </c>
       <c r="M127" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>23.51</t>
         </is>
       </c>
       <c r="N127" s="2" t="inlineStr"/>
       <c r="O127" s="2" t="inlineStr">
         <is>
-          <t>26.06.2026 10:29 — 08.07.2026 17:00</t>
+          <t>06.08.2025 15:30 — 07.08.2026 12:00</t>
         </is>
       </c>
       <c r="P127" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
         </is>
       </c>
       <c r="Q127" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=c2040d938e8d3cf8fc199ed3bc440b5b4a1fe4c3&amp;tsid=4503612458</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=a049a4dc83fe81223b334d9bb351553f178aa0b3&amp;tsid=4130106003</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
@@ -11190,27 +11190,27 @@
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>4130106</t>
+          <t>4498936</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>Реализация ЖБИ изделий с АО "Мальцовский портландцемент"Бордюрдорожный1000х300х150мм Ясногорский завод строительных материалов Кольца  ...  КС-7-3 ЖБИ 24/7Плитаопорная ОП-1К ПС-334-08 ...Плитаперекрытия колодца 1ПП-20-2 D2200  ...</t>
+          <t>Продажа невостребованных ТМЦ -Плиты аэродромные, Фильтр сетчатый МИГ, Ролик лебедки Материалы с хранения. Перечень ориентировочный, может измениться в меньшую сторону за счет возможной востребованности.</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>АО "ЦЕМРОС"</t>
+          <t>ООО "СИБУР"</t>
         </is>
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t>АО "ЦЕМРОС"</t>
+          <t>ООО "СИБУР"</t>
         </is>
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>7708117908</t>
+          <t>7727576505</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -11220,7 +11220,7 @@
       </c>
       <c r="K128" s="2" t="inlineStr">
         <is>
-          <t>Шматов Вячеслав Вячеславович</t>
+          <t>Карисалов Михаил Юрьевич</t>
         </is>
       </c>
       <c r="L128" s="2" t="inlineStr">
@@ -11230,30 +11230,30 @@
       </c>
       <c r="M128" s="2" t="inlineStr">
         <is>
-          <t>23.51</t>
+          <t>70.10</t>
         </is>
       </c>
       <c r="N128" s="2" t="inlineStr"/>
       <c r="O128" s="2" t="inlineStr">
         <is>
-          <t>06.08.2025 15:30 — 07.08.2026 12:00</t>
+          <t>23.06.2026 13:41 — 07.07.2026 12:00</t>
         </is>
       </c>
       <c r="P128" s="2" t="inlineStr">
         <is>
-          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
+          <t>г Москва, ул Кржижановского, д 16 к 3</t>
         </is>
       </c>
       <c r="Q128" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=c2040d938e8d3cf8fc199ed3bc440b5b4a1fe4c3&amp;tsid=4130106003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=d309f3efe8923eeea3a1874e530b1eda75b90d60&amp;tsid=4498936003</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
@@ -11264,42 +11264,43 @@
       <c r="C129" s="2" t="inlineStr"/>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Работы</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>4156098</t>
+          <t>4497016</t>
         </is>
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>Реализация. Линия погрузки угля Б/У (ЛК-60Т 2022 г.в.). Конвейер ленточный подающий ЛК-60Т, линия погрузки угля, бункер приемный, кровельные металлоконструкции. Год ввода в эксплуатацию 2022. Исправное тех.состояние. Продажа бездорожных плит. Демонтаж и самовывоз силами и за счет покупателя.</t>
+          <t>BOX_00514 Выполнение работ по строительству общежития №4 на 80 койко-мест временного вахтового поселка на месторождении «Бараньевское»
+Выполнение работ по строительству общежития №4 на 80 койко-мест временного вахтового поселка АО «Камчатское золото», на месторождении «Бараньевское»ЛОТ №1: Монтаж фундамента (висячиезабивные сваииз стальных труб 219×5 мм)  ...</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t>ООО "УК "СИБАНТРАЦИТ"</t>
+          <t>ООО «Фокси-Бокс»</t>
         </is>
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
-          <t>ООО "УК "СИБАНТРАЦИТ"</t>
+          <t>ООО "ФОКСИ-БОКС"</t>
         </is>
       </c>
       <c r="I129" s="2" t="inlineStr">
         <is>
-          <t>9703160290</t>
+          <t>7805780074</t>
         </is>
       </c>
       <c r="J129" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
+          <t>г Санкт-Петербург</t>
         </is>
       </c>
       <c r="K129" s="2" t="inlineStr">
         <is>
-          <t>Мельников Сергей Владимирович</t>
+          <t>Василенко Иван Михайлович</t>
         </is>
       </c>
       <c r="L129" s="2" t="inlineStr">
@@ -11309,30 +11310,30 @@
       </c>
       <c r="M129" s="2" t="inlineStr">
         <is>
-          <t>70.22</t>
+          <t>46.73</t>
         </is>
       </c>
       <c r="N129" s="2" t="inlineStr"/>
       <c r="O129" s="2" t="inlineStr">
         <is>
-          <t>02.09.2025 11:51 — 03.07.2026 12:00</t>
+          <t>22.06.2026 16:20 — 06.07.2026 12:00</t>
         </is>
       </c>
       <c r="P129" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Усачёва, д 2 стр 1, помещ 2/1</t>
+          <t>196006, Г.САНКТ-ПЕТЕРБУРГ, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОСКОВСКАЯ ЗАСТАВА, УЛ ЗАСТАВСКАЯ, Д. 7, ЛИТЕРА А, ПОМЕЩ. 1-Н, ПОМЕЩ. № 157</t>
         </is>
       </c>
       <c r="Q129" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-liniia-pogruzki-uglia-b-u-lk-60t-2022-g-v/tender-4156098/#btid=2&amp;sqh=c2040d938e8d3cf8fc199ed3bc440b5b4a1fe4c3&amp;tsid=4156098003</t>
+          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=8d26ca1c28cea5b9297671249ca2c4f061289a6c&amp;tsid=4497016004</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
@@ -11348,27 +11349,27 @@
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>4498936</t>
+          <t>4512196</t>
         </is>
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>Продажа невостребованных ТМЦ -Плиты аэродромные, Фильтр сетчатый МИГ, Ролик лебедки Материалы с хранения. Перечень ориентировочный, может измениться в меньшую сторону за счет возможной востребованности.</t>
+          <t>ОПОРА ЛЭПЛИСТВ НЕПРОПИТАН 22-28СМ L11</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>ООО "СИБУР"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
-          <t>ООО "СИБУР"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>7727576505</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr">
@@ -11376,11 +11377,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K130" s="2" t="inlineStr">
-        <is>
-          <t>Карисалов Михаил Юрьевич</t>
-        </is>
-      </c>
+      <c r="K130" s="2" t="inlineStr"/>
       <c r="L130" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -11388,30 +11385,30 @@
       </c>
       <c r="M130" s="2" t="inlineStr">
         <is>
-          <t>70.10</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N130" s="2" t="inlineStr"/>
       <c r="O130" s="2" t="inlineStr">
         <is>
-          <t>23.06.2026 13:41 — 07.07.2026 12:00</t>
+          <t>03.07.2026 11:30 — 09.07.2026 00:00</t>
         </is>
       </c>
       <c r="P130" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Кржижановского, д 16 к 3</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q130" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=dabfb68ea959465f2b0252c6591b51dd88144064&amp;tsid=4498936003</t>
+          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=3c9f542d50a01fbace7be4204e65d4b3d93ebcfd&amp;tsid=4512196458</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
@@ -11427,38 +11424,37 @@
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>4497016</t>
+          <t>4512292</t>
         </is>
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>BOX_00514 Выполнение работ по строительству общежития №4 на 80 койко-мест временного вахтового поселка на месторождении «Бараньевское»
-Выполнение работ по строительству общежития №4 на 80 койко-мест временного вахтового поселка АО «Камчатское золото», на месторождении «Бараньевское»ЛОТ №1: Монтаж фундамента (висячиезабивные сваииз стальных труб 219×5 мм)  ...</t>
+          <t>ТЕХНИЧЕСКОЕ ЗАДАНИЕ на строительствоЛЭП-6кВдля электроснабжения электрогидравлического экскаватора Liebherr 9200Е Работы по строительствуЛЭП-6кВдля электроснабжения электрогидравлического экскаватора Liebherr 9200Е.</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>ООО «Фокси-Бокс»</t>
+          <t>ООО "СЕРВИС ПЛЮС"</t>
         </is>
       </c>
       <c r="H131" s="2" t="inlineStr">
         <is>
-          <t>ООО "ФОКСИ-БОКС"</t>
+          <t>ООО "СЕРВИС ПЛЮС"</t>
         </is>
       </c>
       <c r="I131" s="2" t="inlineStr">
         <is>
-          <t>7805780074</t>
+          <t>7704643931</t>
         </is>
       </c>
       <c r="J131" s="2" t="inlineStr">
         <is>
-          <t>г Санкт-Петербург</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K131" s="2" t="inlineStr">
         <is>
-          <t>Василенко Иван Михайлович</t>
+          <t>Иванов Владимир Ильич</t>
         </is>
       </c>
       <c r="L131" s="2" t="inlineStr">
@@ -11468,30 +11464,30 @@
       </c>
       <c r="M131" s="2" t="inlineStr">
         <is>
-          <t>46.73</t>
+          <t>68.32</t>
         </is>
       </c>
       <c r="N131" s="2" t="inlineStr"/>
       <c r="O131" s="2" t="inlineStr">
         <is>
-          <t>22.06.2026 16:20 — 06.07.2026 12:00</t>
+          <t>03.07.2026 12:19 — 09.07.2026 12:00</t>
         </is>
       </c>
       <c r="P131" s="2" t="inlineStr">
         <is>
-          <t>196006, Г.САНКТ-ПЕТЕРБУРГ, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОСКОВСКАЯ ЗАСТАВА, УЛ ЗАСТАВСКАЯ, Д. 7, ЛИТЕРА А, ПОМЕЩ. 1-Н, ПОМЕЩ. № 157</t>
+          <t>г Москва, ул Пречистенка, д 40/2 стр 4, помещ I, ком 2А</t>
         </is>
       </c>
       <c r="Q131" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=cfd976124f7713c977a6310491949bff7ed27741&amp;tsid=4497016004</t>
+          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=3c9f542d50a01fbace7be4204e65d4b3d93ebcfd&amp;tsid=4512292004</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
@@ -11566,14 +11562,14 @@
       </c>
       <c r="Q132" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=fd5ef2676c9e0b3e7ca0da300e6a19f6e92e9874&amp;tsid=4475879003</t>
+          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=ee00f109009fbc61e0a1888099b1bf7c19201bcd&amp;tsid=4475879003</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
@@ -11645,14 +11641,14 @@
       </c>
       <c r="Q133" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=6f11029064c0ad24d84db69e4ec72f186c321785&amp;tsid=4508331004</t>
+          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=ea290c8cc0087a22c92a3c6e2e10b9db9f1e9e92&amp;tsid=4508331004</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
@@ -11668,27 +11664,27 @@
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>4510341</t>
+          <t>4512253</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>ЖБИ(чеч 34\25 7510 \ 17338)</t>
+          <t>ЗакупкаЖБИ(кольца)</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t>7724498866</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J134" s="2" t="inlineStr">
@@ -11696,11 +11692,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K134" s="2" t="inlineStr">
-        <is>
-          <t>Городний Анатолий Валерьевич</t>
-        </is>
-      </c>
+      <c r="K134" s="2" t="inlineStr"/>
       <c r="L134" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -11708,30 +11700,30 @@
       </c>
       <c r="M134" s="2" t="inlineStr">
         <is>
-          <t>46.73</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N134" s="2" t="inlineStr"/>
       <c r="O134" s="2" t="inlineStr">
         <is>
-          <t>02.07.2026 09:54 — 03.07.2026 15:00</t>
+          <t>03.07.2026 11:45 — 06.07.2026 12:00</t>
         </is>
       </c>
       <c r="P134" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q134" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=c883c80d526059f0f905d92600ab245159b9380e&amp;tsid=4510341459</t>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-koltsa/tender-4512253/#btid=2&amp;sqh=9d9a56475611a52b0a8d64b319596e56acc70739&amp;tsid=4512253458</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
@@ -11747,12 +11739,12 @@
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>4510662</t>
+          <t>4510341</t>
         </is>
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>(ЖБИизделия/кольца колодезные, плиты ПК15)</t>
+          <t>ЖБИ(чеч 34\25 7510 \ 17338)</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -11793,7 +11785,7 @@
       <c r="N135" s="2" t="inlineStr"/>
       <c r="O135" s="2" t="inlineStr">
         <is>
-          <t>02.07.2026 12:00 — 03.07.2026 15:00</t>
+          <t>02.07.2026 09:54 — 03.07.2026 15:00</t>
         </is>
       </c>
       <c r="P135" s="2" t="inlineStr">
@@ -11803,14 +11795,14 @@
       </c>
       <c r="Q135" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-izdeliia-koltsa-kolodeznye-plity-pk15/tender-4510662/#btid=2&amp;sqh=c883c80d526059f0f905d92600ab245159b9380e&amp;tsid=4510662459</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=9d9a56475611a52b0a8d64b319596e56acc70739&amp;tsid=4510341459</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
@@ -11826,27 +11818,27 @@
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>4510073</t>
+          <t>4510662</t>
         </is>
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>ЗакупкаЖБИ- лотки, плиты, бруски, блоки</t>
+          <t>(ЖБИизделия/кольца колодезные, плиты ПК15)</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>7724498866</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -11854,7 +11846,11 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K136" s="2" t="inlineStr"/>
+      <c r="K136" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
       <c r="L136" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -11862,30 +11858,30 @@
       </c>
       <c r="M136" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>46.73</t>
         </is>
       </c>
       <c r="N136" s="2" t="inlineStr"/>
       <c r="O136" s="2" t="inlineStr">
         <is>
-          <t>02.07.2026 07:55 — 05.07.2026 12:00</t>
+          <t>02.07.2026 12:00 — 03.07.2026 15:00</t>
         </is>
       </c>
       <c r="P136" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
         </is>
       </c>
       <c r="Q136" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-lotki-plity-bruski-bloki/tender-4510073/#btid=2&amp;sqh=c883c80d526059f0f905d92600ab245159b9380e&amp;tsid=4510073458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-izdeliia-koltsa-kolodeznye-plity-pk15/tender-4510662/#btid=2&amp;sqh=9d9a56475611a52b0a8d64b319596e56acc70739&amp;tsid=4510662459</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
@@ -11901,27 +11897,27 @@
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>4510504</t>
+          <t>4510073</t>
         </is>
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>(Заявка № ДОР-17560) Лестницы/ЖБИ</t>
+          <t>ЗакупкаЖБИ- лотки, плиты, бруски, блоки</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I137" s="2" t="inlineStr">
         <is>
-          <t>7724498866</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J137" s="2" t="inlineStr">
@@ -11929,11 +11925,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K137" s="2" t="inlineStr">
-        <is>
-          <t>Городний Анатолий Валерьевич</t>
-        </is>
-      </c>
+      <c r="K137" s="2" t="inlineStr"/>
       <c r="L137" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -11941,30 +11933,30 @@
       </c>
       <c r="M137" s="2" t="inlineStr">
         <is>
-          <t>46.73</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N137" s="2" t="inlineStr"/>
       <c r="O137" s="2" t="inlineStr">
         <is>
-          <t>02.07.2026 10:55 — 03.07.2026 15:00</t>
+          <t>02.07.2026 07:55 — 05.07.2026 12:00</t>
         </is>
       </c>
       <c r="P137" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q137" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zaiavka-dor-17560-lestnitsy-zhbi/tender-4510504/#btid=2&amp;sqh=c883c80d526059f0f905d92600ab245159b9380e&amp;tsid=4510504459</t>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-lotki-plity-bruski-bloki/tender-4510073/#btid=2&amp;sqh=9d9a56475611a52b0a8d64b319596e56acc70739&amp;tsid=4510073458</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
@@ -11980,12 +11972,12 @@
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>4510823</t>
+          <t>4510504</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>(ДОР-17553)ЖБИ/Лестницы ВЛ-2/Скоба</t>
+          <t>(Заявка № ДОР-17560) Лестницы/ЖБИ</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -12026,7 +12018,7 @@
       <c r="N138" s="2" t="inlineStr"/>
       <c r="O138" s="2" t="inlineStr">
         <is>
-          <t>02.07.2026 12:55 — 03.07.2026 15:00</t>
+          <t>02.07.2026 10:55 — 03.07.2026 15:00</t>
         </is>
       </c>
       <c r="P138" s="2" t="inlineStr">
@@ -12036,14 +12028,14 @@
       </c>
       <c r="Q138" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/dor-17553-zhbi-lestnitsy-vl-2-skoba/tender-4510823/#btid=2&amp;sqh=c883c80d526059f0f905d92600ab245159b9380e&amp;tsid=4510823459</t>
+          <t>https://www.b2b-center.ru/app/market-next/zaiavka-dor-17560-lestnitsy-zhbi/tender-4510504/#btid=2&amp;sqh=9d9a56475611a52b0a8d64b319596e56acc70739&amp;tsid=4510504459</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
@@ -12059,27 +12051,27 @@
       </c>
       <c r="E139" s="2" t="inlineStr">
         <is>
-          <t>4508347</t>
+          <t>4510823</t>
         </is>
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>ЖБИКЕМГРЭС</t>
+          <t>(ДОР-17553)ЖБИ/Лестницы ВЛ-2/Скоба</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="H139" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="I139" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>7724498866</t>
         </is>
       </c>
       <c r="J139" s="2" t="inlineStr">
@@ -12087,7 +12079,11 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K139" s="2" t="inlineStr"/>
+      <c r="K139" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
       <c r="L139" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -12095,30 +12091,30 @@
       </c>
       <c r="M139" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>46.73</t>
         </is>
       </c>
       <c r="N139" s="2" t="inlineStr"/>
       <c r="O139" s="2" t="inlineStr">
         <is>
-          <t>01.07.2026 05:45 — 10.07.2026 00:00</t>
+          <t>02.07.2026 12:55 — 03.07.2026 15:00</t>
         </is>
       </c>
       <c r="P139" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
         </is>
       </c>
       <c r="Q139" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=c883c80d526059f0f905d92600ab245159b9380e&amp;tsid=4508347458</t>
+          <t>https://www.b2b-center.ru/app/market-next/dor-17553-zhbi-lestnitsy-vl-2-skoba/tender-4510823/#btid=2&amp;sqh=9d9a56475611a52b0a8d64b319596e56acc70739&amp;tsid=4510823459</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
@@ -12134,150 +12130,146 @@
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
+          <t>4508347</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>ЖБИКЕМГРЭС</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I140" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J140" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K140" s="2" t="inlineStr"/>
+      <c r="L140" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M140" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N140" s="2" t="inlineStr"/>
+      <c r="O140" s="2" t="inlineStr">
+        <is>
+          <t>01.07.2026 05:45 — 10.07.2026 00:00</t>
+        </is>
+      </c>
+      <c r="P140" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q140" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=9d9a56475611a52b0a8d64b319596e56acc70739&amp;tsid=4508347458</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 10:25</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr"/>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
           <t>4508689</t>
         </is>
       </c>
-      <c r="F140" s="2" t="inlineStr">
+      <c r="F141" s="2" t="inlineStr">
         <is>
           <t>Железобетонные плиты Б/У 
 Необходимы плиты, это те которые выдерживают нагрузку т.к. на эту плиту будет заезжать техника весом до 70тонн. Приоритетно с целью минимизации затрат рассмотрим плиты Б/У  размер произвольный но ближе 2х4; 3х3; 2х6. Количество плит необходимо +/- 50 шт. (данные плиты предназначаются для размещения на них запчастей и хоз. деятельности Горного цеха)Б/УЖБИплиты</t>
         </is>
       </c>
-      <c r="G140" s="2" t="inlineStr">
+      <c r="G141" s="2" t="inlineStr">
         <is>
           <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
-      <c r="H140" s="2" t="inlineStr">
+      <c r="H141" s="2" t="inlineStr">
         <is>
           <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
-      <c r="I140" s="2" t="inlineStr">
+      <c r="I141" s="2" t="inlineStr">
         <is>
           <t>7708117908</t>
         </is>
       </c>
-      <c r="J140" s="2" t="inlineStr">
+      <c r="J141" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K140" s="2" t="inlineStr">
+      <c r="K141" s="2" t="inlineStr">
         <is>
           <t>Шматов Вячеслав Вячеславович</t>
         </is>
       </c>
-      <c r="L140" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M140" s="2" t="inlineStr">
+      <c r="L141" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M141" s="2" t="inlineStr">
         <is>
           <t>23.51</t>
-        </is>
-      </c>
-      <c r="N140" s="2" t="inlineStr"/>
-      <c r="O140" s="2" t="inlineStr">
-        <is>
-          <t>01.07.2026 09:45 — 06.07.2026 09:00</t>
-        </is>
-      </c>
-      <c r="P140" s="2" t="inlineStr">
-        <is>
-          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
-        </is>
-      </c>
-      <c r="Q140" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhelezobetonnye-plity-b-u-neobkhodimy-plity-eto-te-kotorye/tender-4508689/#btid=2&amp;sqh=c883c80d526059f0f905d92600ab245159b9380e&amp;tsid=4508689458</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-03 08:13</t>
-        </is>
-      </c>
-      <c r="B141" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C141" s="2" t="inlineStr"/>
-      <c r="D141" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E141" s="2" t="inlineStr">
-        <is>
-          <t>4489772</t>
-        </is>
-      </c>
-      <c r="F141" s="2" t="inlineStr">
-        <is>
-          <t>1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы 1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы</t>
-        </is>
-      </c>
-      <c r="G141" s="2" t="inlineStr">
-        <is>
-          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
-        </is>
-      </c>
-      <c r="H141" s="2" t="inlineStr">
-        <is>
-          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
-        </is>
-      </c>
-      <c r="I141" s="2" t="inlineStr">
-        <is>
-          <t>7736583259</t>
-        </is>
-      </c>
-      <c r="J141" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K141" s="2" t="inlineStr">
-        <is>
-          <t>Масько Александр Вадимович</t>
-        </is>
-      </c>
-      <c r="L141" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M141" s="2" t="inlineStr">
-        <is>
-          <t>70.10</t>
         </is>
       </c>
       <c r="N141" s="2" t="inlineStr"/>
       <c r="O141" s="2" t="inlineStr">
         <is>
-          <t>16.06.2026 11:00 — 16.07.2026 12:00</t>
+          <t>01.07.2026 09:45 — 06.07.2026 09:00</t>
         </is>
       </c>
       <c r="P141" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Старая Басманная, д 12 стр 1</t>
+          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
         </is>
       </c>
       <c r="Q141" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=c883c80d526059f0f905d92600ab245159b9380e&amp;tsid=4489772003</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhelezobetonnye-plity-b-u-neobkhodimy-plity-eto-te-kotorye/tender-4508689/#btid=2&amp;sqh=9d9a56475611a52b0a8d64b319596e56acc70739&amp;tsid=4508689458</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
@@ -12293,37 +12285,37 @@
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
-          <t>4474790</t>
+          <t>4489772</t>
         </is>
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
+          <t>1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы 1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
         </is>
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
         </is>
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>4704012472</t>
+          <t>7736583259</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr">
         <is>
-          <t>Габидуллин Тимур Махмудович</t>
+          <t>Масько Александр Вадимович</t>
         </is>
       </c>
       <c r="L142" s="2" t="inlineStr">
@@ -12333,30 +12325,30 @@
       </c>
       <c r="M142" s="2" t="inlineStr">
         <is>
-          <t>17.12</t>
+          <t>70.10</t>
         </is>
       </c>
       <c r="N142" s="2" t="inlineStr"/>
       <c r="O142" s="2" t="inlineStr">
         <is>
-          <t>03.06.2026 09:59 — 30.07.2026 20:00</t>
+          <t>16.06.2026 11:00 — 16.07.2026 12:00</t>
         </is>
       </c>
       <c r="P142" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+          <t>г Москва, ул Старая Басманная, д 12 стр 1</t>
         </is>
       </c>
       <c r="Q142" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=c883c80d526059f0f905d92600ab245159b9380e&amp;tsid=4474790003</t>
+          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=9d9a56475611a52b0a8d64b319596e56acc70739&amp;tsid=4489772003</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B143" s="2" t="inlineStr">
@@ -12372,37 +12364,37 @@
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>4180328</t>
+          <t>4474790</t>
         </is>
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, г.Диксон). ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, ПГТ Диксон).</t>
+          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
-          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="H143" s="2" t="inlineStr">
         <is>
-          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="I143" s="2" t="inlineStr">
         <is>
-          <t>7714456916</t>
+          <t>4704012472</t>
         </is>
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
+          <t>Ленинградская обл</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>Наумов Андрей Александрович</t>
+          <t>Габидуллин Тимур Махмудович</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr">
@@ -12412,30 +12404,30 @@
       </c>
       <c r="M143" s="2" t="inlineStr">
         <is>
-          <t>70.22</t>
+          <t>17.12</t>
         </is>
       </c>
       <c r="N143" s="2" t="inlineStr"/>
       <c r="O143" s="2" t="inlineStr">
         <is>
-          <t>24.09.2025 15:32 — 23.07.2026 12:00</t>
+          <t>03.06.2026 09:59 — 30.07.2026 20:00</t>
         </is>
       </c>
       <c r="P143" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Денежный пер, д 9/6</t>
+          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
         </is>
       </c>
       <c r="Q143" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=c883c80d526059f0f905d92600ab245159b9380e&amp;tsid=4180328003</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=9d9a56475611a52b0a8d64b319596e56acc70739&amp;tsid=4474790003</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
@@ -12451,37 +12443,37 @@
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>3973258</t>
+          <t>4180328</t>
         </is>
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
+          <t>ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, г.Диксон). ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, ПГТ Диксон).</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
         </is>
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
         </is>
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>4704012472</t>
+          <t>7714456916</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>Габидуллин Тимур Махмудович</t>
+          <t>Наумов Андрей Александрович</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr">
@@ -12491,30 +12483,30 @@
       </c>
       <c r="M144" s="2" t="inlineStr">
         <is>
-          <t>17.12</t>
+          <t>70.22</t>
         </is>
       </c>
       <c r="N144" s="2" t="inlineStr"/>
       <c r="O144" s="2" t="inlineStr">
         <is>
-          <t>10.03.2025 00:48 — 30.07.2026 23:00</t>
+          <t>24.09.2025 15:32 — 23.07.2026 12:00</t>
         </is>
       </c>
       <c r="P144" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+          <t>г Москва, Денежный пер, д 9/6</t>
         </is>
       </c>
       <c r="Q144" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=c883c80d526059f0f905d92600ab245159b9380e&amp;tsid=3973258003</t>
+          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=9d9a56475611a52b0a8d64b319596e56acc70739&amp;tsid=4180328003</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B145" s="2" t="inlineStr">
@@ -12530,35 +12522,39 @@
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>4509622</t>
+          <t>3973258</t>
         </is>
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>Производство вторичного щебня из ломажелезобетонных изделий</t>
+          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="H145" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>4704012472</t>
         </is>
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K145" s="2" t="inlineStr"/>
+          <t>Ленинградская обл</t>
+        </is>
+      </c>
+      <c r="K145" s="2" t="inlineStr">
+        <is>
+          <t>Габидуллин Тимур Махмудович</t>
+        </is>
+      </c>
       <c r="L145" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -12566,30 +12562,30 @@
       </c>
       <c r="M145" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>17.12</t>
         </is>
       </c>
       <c r="N145" s="2" t="inlineStr"/>
       <c r="O145" s="2" t="inlineStr">
         <is>
-          <t>01.07.2026 16:05 — 10.07.2026 12:00</t>
+          <t>10.03.2025 00:48 — 30.07.2026 23:00</t>
         </is>
       </c>
       <c r="P145" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
         </is>
       </c>
       <c r="Q145" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/proizvodstvo-vtorichnogo-shchebnia-iz-loma-zhelezobetonnykh-izdelii/tender-4509622/#btid=2&amp;sqh=8c1a00b72158ca0d4a44fffc89559572d54c0750&amp;tsid=4509622458</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=9d9a56475611a52b0a8d64b319596e56acc70739&amp;tsid=3973258003</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
@@ -12600,32 +12596,32 @@
       <c r="C146" s="2" t="inlineStr"/>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Поставка</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>4508845</t>
+          <t>4512260</t>
         </is>
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>Панель ограждения 3ПБ40.20 2550х4000х160мм 3.017-3.1-7 серия 3.017-3 – 24 шт (чертеж на стр. 11 типового альбомажелезобетонных изделий)</t>
+          <t>ТМЦ. Срочный отбор предложений на право заключения договора поставкижелезобетонных изделийдля нужд филиала «Канская теплосеть» АО «Енисейская ТГК (ТГК-13)».</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
         <is>
-          <t>АО "ЦЕМРОС"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
-          <t>АО "ЦЕМРОС"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>7708117908</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr">
@@ -12633,11 +12629,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K146" s="2" t="inlineStr">
-        <is>
-          <t>Шматов Вячеслав Вячеславович</t>
-        </is>
-      </c>
+      <c r="K146" s="2" t="inlineStr"/>
       <c r="L146" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -12645,30 +12637,30 @@
       </c>
       <c r="M146" s="2" t="inlineStr">
         <is>
-          <t>23.51</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N146" s="2" t="inlineStr"/>
       <c r="O146" s="2" t="inlineStr">
         <is>
-          <t>01.07.2026 10:44 — 03.07.2026 13:00</t>
+          <t>03.07.2026 11:52 — 08.07.2026 12:00</t>
         </is>
       </c>
       <c r="P146" s="2" t="inlineStr">
         <is>
-          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q146" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/panel-ograzhdeniia-3pb40-20-2550kh4000kh160mm-3-017-3-1-7-seriia-3-017-3/tender-4508845/#btid=2&amp;sqh=8c1a00b72158ca0d4a44fffc89559572d54c0750&amp;tsid=4508845458</t>
+          <t>https://www.b2b-center.ru/app/market-next/tmts-srochnyi-otbor-predlozhenii-na-pravo-zakliucheniia-dogovora-postavki/tender-4512260/#btid=2&amp;sqh=bb9b4c632662fafd66df93a242cb376ac0767e77&amp;tsid=4512260458</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B147" s="2" t="inlineStr">
@@ -12684,39 +12676,35 @@
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>4474238</t>
+          <t>4509622</t>
         </is>
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>Железобетонные изделияПлита перекрытия лотков П22-15И Плитка 2400*1500*160 б/у Плита перекрытия ПК 60-12 б/у</t>
+          <t>Производство вторичного щебня из ломажелезобетонных изделий</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
         <is>
-          <t>ПАО "Коршуновский ГОК"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H147" s="2" t="inlineStr">
         <is>
-          <t>ПАО "КОРШУНОВСКИЙ ГОК"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I147" s="2" t="inlineStr">
         <is>
-          <t>3834002314</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J147" s="2" t="inlineStr">
         <is>
-          <t>Иркутская обл</t>
-        </is>
-      </c>
-      <c r="K147" s="2" t="inlineStr">
-        <is>
-          <t>Иванов Алексей Васильевич</t>
-        </is>
-      </c>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K147" s="2" t="inlineStr"/>
       <c r="L147" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -12724,30 +12712,30 @@
       </c>
       <c r="M147" s="2" t="inlineStr">
         <is>
-          <t>07.10.2</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N147" s="2" t="inlineStr"/>
       <c r="O147" s="2" t="inlineStr">
         <is>
-          <t>11.06.2026 09:23 — 06.07.2026 09:00</t>
+          <t>01.07.2026 16:05 — 10.07.2026 12:00</t>
         </is>
       </c>
       <c r="P147" s="2" t="inlineStr">
         <is>
-          <t>Иркутская обл, г Железногорск-Илимский, ул Иващенко, д 9А/1</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q147" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zhelezobetonnye-izdeliia/tender-4474238/#btid=2&amp;sqh=8c1a00b72158ca0d4a44fffc89559572d54c0750&amp;tsid=4474238003</t>
+          <t>https://www.b2b-center.ru/app/market-next/proizvodstvo-vtorichnogo-shchebnia-iz-loma-zhelezobetonnykh-izdelii/tender-4509622/#btid=2&amp;sqh=bb9b4c632662fafd66df93a242cb376ac0767e77&amp;tsid=4509622458</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
@@ -12758,15 +12746,94 @@
       <c r="C148" s="2" t="inlineStr"/>
       <c r="D148" s="2" t="inlineStr">
         <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>4474238</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>Железобетонные изделияПлита перекрытия лотков П22-15И Плитка 2400*1500*160 б/у Плита перекрытия ПК 60-12 б/у</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="inlineStr">
+        <is>
+          <t>ПАО "Коршуновский ГОК"</t>
+        </is>
+      </c>
+      <c r="H148" s="2" t="inlineStr">
+        <is>
+          <t>ПАО "КОРШУНОВСКИЙ ГОК"</t>
+        </is>
+      </c>
+      <c r="I148" s="2" t="inlineStr">
+        <is>
+          <t>3834002314</t>
+        </is>
+      </c>
+      <c r="J148" s="2" t="inlineStr">
+        <is>
+          <t>Иркутская обл</t>
+        </is>
+      </c>
+      <c r="K148" s="2" t="inlineStr">
+        <is>
+          <t>Иванов Алексей Васильевич</t>
+        </is>
+      </c>
+      <c r="L148" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M148" s="2" t="inlineStr">
+        <is>
+          <t>07.10.2</t>
+        </is>
+      </c>
+      <c r="N148" s="2" t="inlineStr"/>
+      <c r="O148" s="2" t="inlineStr">
+        <is>
+          <t>11.06.2026 09:23 — 06.07.2026 09:00</t>
+        </is>
+      </c>
+      <c r="P148" s="2" t="inlineStr">
+        <is>
+          <t>Иркутская обл, г Железногорск-Илимский, ул Иващенко, д 9А/1</t>
+        </is>
+      </c>
+      <c r="Q148" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/zhelezobetonnye-izdeliia/tender-4474238/#btid=2&amp;sqh=bb9b4c632662fafd66df93a242cb376ac0767e77&amp;tsid=4474238003</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 10:25</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr"/>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
           <t>Поставка</t>
         </is>
       </c>
-      <c r="E148" s="2" t="inlineStr">
+      <c r="E149" s="2" t="inlineStr">
         <is>
           <t>4511621</t>
         </is>
       </c>
-      <c r="F148" s="2" t="inlineStr">
+      <c r="F149" s="2" t="inlineStr">
         <is>
           <t>Закупка аккумуляторных батарей (залитых) для нужд АО "Павловск Неруд" с поставкой в Августе 2026г.
 Обязательная расценка стоимости доставки, возможен забор груза на условиях самовывоза.
@@ -12775,137 +12842,62 @@
 Заказчик АО "Павловск Неруд" предприятие АО "Национальная нерудная компания"Аккумулятор ТН-550Перемычкам/ц для АКБ 115,5мм ТН-550Перемычкам/ц для АКБ 212,0мм ТН-550 Транспортная услуга</t>
         </is>
       </c>
-      <c r="G148" s="2" t="inlineStr">
+      <c r="G149" s="2" t="inlineStr">
         <is>
           <t>АО "ННК"</t>
         </is>
       </c>
-      <c r="H148" s="2" t="inlineStr">
+      <c r="H149" s="2" t="inlineStr">
         <is>
           <t>АО "ННК-ОЙЛ"</t>
         </is>
       </c>
-      <c r="I148" s="2" t="inlineStr">
+      <c r="I149" s="2" t="inlineStr">
         <is>
           <t>5032049030</t>
         </is>
       </c>
-      <c r="J148" s="2" t="inlineStr">
+      <c r="J149" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K148" s="2" t="inlineStr">
+      <c r="K149" s="2" t="inlineStr">
         <is>
           <t>Худайнатов Эдуард Юрьевич</t>
         </is>
       </c>
-      <c r="L148" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M148" s="2" t="inlineStr">
+      <c r="L149" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M149" s="2" t="inlineStr">
         <is>
           <t>70.22</t>
-        </is>
-      </c>
-      <c r="N148" s="2" t="inlineStr"/>
-      <c r="O148" s="2" t="inlineStr">
-        <is>
-          <t>03.07.2026 06:22 — 07.07.2026 11:00</t>
-        </is>
-      </c>
-      <c r="P148" s="2" t="inlineStr">
-        <is>
-          <t>г Москва, ул 1-я Тверская-Ямская, д 5, помещ 1012</t>
-        </is>
-      </c>
-      <c r="Q148" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=f69b60b4476caa237bb19c1c7ba2c7eb638a4ba2&amp;tsid=4511621004</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-03 08:13</t>
-        </is>
-      </c>
-      <c r="B149" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C149" s="2" t="inlineStr"/>
-      <c r="D149" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E149" s="2" t="inlineStr">
-        <is>
-          <t>4511787</t>
-        </is>
-      </c>
-      <c r="F149" s="2" t="inlineStr">
-        <is>
-          <t>ЗЧ к автотранспорту... /66 ТЕРМОСТАТ ТС-107-1306100-06ПЕРЕМЫЧКААКБ КЛЕММА-КЛЕММА ПП 500-50 ...</t>
-        </is>
-      </c>
-      <c r="G149" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="H149" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="I149" s="2" t="inlineStr">
-        <is>
-          <t>9725042029</t>
-        </is>
-      </c>
-      <c r="J149" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K149" s="2" t="inlineStr"/>
-      <c r="L149" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M149" s="2" t="inlineStr">
-        <is>
-          <t>64.20</t>
         </is>
       </c>
       <c r="N149" s="2" t="inlineStr"/>
       <c r="O149" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 08:32 — 08.07.2026 00:00</t>
+          <t>03.07.2026 06:22 — 07.07.2026 11:00</t>
         </is>
       </c>
       <c r="P149" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Москва, ул 1-я Тверская-Ямская, д 5, помещ 1012</t>
         </is>
       </c>
       <c r="Q149" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=f69b60b4476caa237bb19c1c7ba2c7eb638a4ba2&amp;tsid=4511787458</t>
+          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=0ca549e468445c11519f78660f42d04b3782a4f3&amp;tsid=4511621004</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
@@ -12921,230 +12913,226 @@
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
+          <t>4511787</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>ЗЧ к автотранспорту... /66 ТЕРМОСТАТ ТС-107-1306100-06ПЕРЕМЫЧКААКБ КЛЕММА-КЛЕММА ПП 500-50 ...</t>
+        </is>
+      </c>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H150" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I150" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J150" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K150" s="2" t="inlineStr"/>
+      <c r="L150" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M150" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N150" s="2" t="inlineStr"/>
+      <c r="O150" s="2" t="inlineStr">
+        <is>
+          <t>03.07.2026 08:32 — 08.07.2026 00:00</t>
+        </is>
+      </c>
+      <c r="P150" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q150" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=0ca549e468445c11519f78660f42d04b3782a4f3&amp;tsid=4511787458</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 10:25</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr"/>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E151" s="2" t="inlineStr">
+        <is>
           <t>4508230</t>
         </is>
       </c>
-      <c r="F150" s="2" t="inlineStr">
+      <c r="F151" s="2" t="inlineStr">
         <is>
           <t>Сборный (Изделия электроустановочные и монтажные, Ящики, щиты, шкафы, пункты и комплектующие к ним, Приборы электроизмерительные, реле)
 МГ-019742, МГ-019713, МГ-019696, МГ-019665, МГ-019621, МГ-019620, МГ-019619, МГ-017109... -HESI-EX (5X20), Phoenix Contact 1277638ПеремычкаFBS 10-5, Phoenix Contact 3030213 ...ПеремычкаFBS 10-5 BU, Phoenix Contact  ...</t>
         </is>
       </c>
-      <c r="G150" s="2" t="inlineStr">
+      <c r="G151" s="2" t="inlineStr">
         <is>
           <t>АО "ИК "АРЛАН"</t>
         </is>
       </c>
-      <c r="H150" s="2" t="inlineStr">
+      <c r="H151" s="2" t="inlineStr">
         <is>
           <t>АО "ИК "АРЛАН"</t>
         </is>
       </c>
-      <c r="I150" s="2" t="inlineStr">
+      <c r="I151" s="2" t="inlineStr">
         <is>
           <t>7722220390</t>
         </is>
       </c>
-      <c r="J150" s="2" t="inlineStr">
+      <c r="J151" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K150" s="2" t="inlineStr">
+      <c r="K151" s="2" t="inlineStr">
         <is>
           <t>Барилов Евгений Александрович</t>
         </is>
       </c>
-      <c r="L150" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M150" s="2" t="inlineStr">
+      <c r="L151" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M151" s="2" t="inlineStr">
         <is>
           <t>82.99</t>
         </is>
       </c>
-      <c r="N150" s="2" t="inlineStr"/>
-      <c r="O150" s="2" t="inlineStr">
+      <c r="N151" s="2" t="inlineStr"/>
+      <c r="O151" s="2" t="inlineStr">
         <is>
           <t>30.06.2026 17:59 — 09.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P150" s="2" t="inlineStr">
+      <c r="P151" s="2" t="inlineStr">
         <is>
           <t>г Москва, Романов пер, д 4</t>
         </is>
       </c>
-      <c r="Q150" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=f69b60b4476caa237bb19c1c7ba2c7eb638a4ba2&amp;tsid=4508230004</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-03 08:13</t>
-        </is>
-      </c>
-      <c r="B151" s="2" t="inlineStr">
+      <c r="Q151" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=0ca549e468445c11519f78660f42d04b3782a4f3&amp;tsid=4508230004</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 10:25</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
         <is>
           <t>b2b-center</t>
         </is>
       </c>
-      <c r="C151" s="2" t="inlineStr"/>
-      <c r="D151" s="2" t="inlineStr">
+      <c r="C152" s="2" t="inlineStr"/>
+      <c r="D152" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E151" s="2" t="inlineStr">
+      <c r="E152" s="2" t="inlineStr">
         <is>
           <t>4504775</t>
         </is>
       </c>
-      <c r="F151" s="2" t="inlineStr">
+      <c r="F152" s="2" t="inlineStr">
         <is>
           <t>Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники
 Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники...  Трубка пробная № 37-542-000 Соединитель-перемычка04182454 Кольцо стальное №CP48001-0305 Фильтр ...</t>
         </is>
       </c>
-      <c r="G151" s="2" t="inlineStr">
+      <c r="G152" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="H151" s="2" t="inlineStr">
+      <c r="H152" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="I151" s="2" t="inlineStr">
+      <c r="I152" s="2" t="inlineStr">
         <is>
           <t>7805368914</t>
         </is>
       </c>
-      <c r="J151" s="2" t="inlineStr">
+      <c r="J152" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург</t>
         </is>
       </c>
-      <c r="K151" s="2" t="inlineStr">
+      <c r="K152" s="2" t="inlineStr">
         <is>
           <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
-      <c r="L151" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M151" s="2" t="inlineStr">
+      <c r="L152" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M152" s="2" t="inlineStr">
         <is>
           <t>46.90</t>
-        </is>
-      </c>
-      <c r="N151" s="2" t="inlineStr"/>
-      <c r="O151" s="2" t="inlineStr">
-        <is>
-          <t>27.06.2026 01:36 — 15.07.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P151" s="2" t="inlineStr">
-        <is>
-          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
-        </is>
-      </c>
-      <c r="Q151" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=f69b60b4476caa237bb19c1c7ba2c7eb638a4ba2&amp;tsid=4504775003</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-03 08:13</t>
-        </is>
-      </c>
-      <c r="B152" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C152" s="2" t="inlineStr"/>
-      <c r="D152" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E152" s="2" t="inlineStr">
-        <is>
-          <t>4501157</t>
-        </is>
-      </c>
-      <c r="F152" s="2" t="inlineStr">
-        <is>
-          <t>Источники электропитания (ИБП, аккумуляторные батареи, блоки питания)...  х 1248 А·ч, включая соединительныеперемычки. Вид положительного электрода - трубчатая пластина ...  с коммутирующей арматурой, межэлементными и межряднымиперемычками, крепежами, комплектом для обслуживания АБ. Тип ...</t>
-        </is>
-      </c>
-      <c r="G152" s="2" t="inlineStr">
-        <is>
-          <t>АО "Мосинжпроект"</t>
-        </is>
-      </c>
-      <c r="H152" s="2" t="inlineStr">
-        <is>
-          <t>АО "МОСИНЖПРОЕКТ"</t>
-        </is>
-      </c>
-      <c r="I152" s="2" t="inlineStr">
-        <is>
-          <t>7701885820</t>
-        </is>
-      </c>
-      <c r="J152" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K152" s="2" t="inlineStr">
-        <is>
-          <t>Сорокин Антон Павлович</t>
-        </is>
-      </c>
-      <c r="L152" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M152" s="2" t="inlineStr">
-        <is>
-          <t>71.12.2</t>
         </is>
       </c>
       <c r="N152" s="2" t="inlineStr"/>
       <c r="O152" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 15:40 — 22.07.2026 12:00</t>
+          <t>27.06.2026 01:36 — 15.07.2026 12:00</t>
         </is>
       </c>
       <c r="P152" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
       <c r="Q152" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=f69b60b4476caa237bb19c1c7ba2c7eb638a4ba2&amp;tsid=4501157003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=0ca549e468445c11519f78660f42d04b3782a4f3&amp;tsid=4504775003</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
@@ -13160,12 +13148,12 @@
       </c>
       <c r="E153" s="2" t="inlineStr">
         <is>
-          <t>4499964</t>
+          <t>4501157</t>
         </is>
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>Автоматика и телемеханика движения поездов... , 13552-00-00В Дроссель-трансформатор (безперемычек) ДТМ-0,17-1000М ЮКЛЯ.672 ...</t>
+          <t>Источники электропитания (ИБП, аккумуляторные батареи, блоки питания)...  х 1248 А·ч, включая соединительныеперемычки. Вид положительного электрода - трубчатая пластина ...  с коммутирующей арматурой, межэлементными и межряднымиперемычками, крепежами, комплектом для обслуживания АБ. Тип ...</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -13206,7 +13194,7 @@
       <c r="N153" s="2" t="inlineStr"/>
       <c r="O153" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 08:46 — 15.07.2026 12:00</t>
+          <t>24.06.2026 15:40 — 22.07.2026 12:00</t>
         </is>
       </c>
       <c r="P153" s="2" t="inlineStr">
@@ -13216,14 +13204,14 @@
       </c>
       <c r="Q153" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=f69b60b4476caa237bb19c1c7ba2c7eb638a4ba2&amp;tsid=4499964003</t>
+          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=0ca549e468445c11519f78660f42d04b3782a4f3&amp;tsid=4501157003</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 08:13</t>
+          <t>2026-07-03 10:25</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
@@ -13239,466 +13227,704 @@
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
+          <t>4499964</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>Автоматика и телемеханика движения поездов... , 13552-00-00В Дроссель-трансформатор (безперемычек) ДТМ-0,17-1000М ЮКЛЯ.672 ...</t>
+        </is>
+      </c>
+      <c r="G154" s="2" t="inlineStr">
+        <is>
+          <t>АО "Мосинжпроект"</t>
+        </is>
+      </c>
+      <c r="H154" s="2" t="inlineStr">
+        <is>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
+        </is>
+      </c>
+      <c r="I154" s="2" t="inlineStr">
+        <is>
+          <t>7701885820</t>
+        </is>
+      </c>
+      <c r="J154" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K154" s="2" t="inlineStr">
+        <is>
+          <t>Сорокин Антон Павлович</t>
+        </is>
+      </c>
+      <c r="L154" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M154" s="2" t="inlineStr">
+        <is>
+          <t>71.12.2</t>
+        </is>
+      </c>
+      <c r="N154" s="2" t="inlineStr"/>
+      <c r="O154" s="2" t="inlineStr">
+        <is>
+          <t>24.06.2026 08:46 — 15.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P154" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+        </is>
+      </c>
+      <c r="Q154" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=0ca549e468445c11519f78660f42d04b3782a4f3&amp;tsid=4499964003</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 10:25</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr"/>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E155" s="2" t="inlineStr">
+        <is>
+          <t>4480614</t>
+        </is>
+      </c>
+      <c r="F155" s="2" t="inlineStr">
+        <is>
+          <t>Плановое и аварийное техническое обслуживание зданий и сооружений (годовое обслуживание август 2026 - август 2027) ГК Логика молока, производственная площадка в г. Ялуторовске
+Обслуживание зданий и сооружений завода в г. Ялуторовске....  стен из газобетонных блоков Устройство металлическихперемычекс устройством штраб Усиление кирпичных стен ...</t>
+        </is>
+      </c>
+      <c r="G155" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЭЙЧ ЭНД ЭН"</t>
+        </is>
+      </c>
+      <c r="H155" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЭЙЧ ЭНД ЭН"</t>
+        </is>
+      </c>
+      <c r="I155" s="2" t="inlineStr">
+        <is>
+          <t>7714626332</t>
+        </is>
+      </c>
+      <c r="J155" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K155" s="2" t="inlineStr">
+        <is>
+          <t>Закриев Якуб Салманович</t>
+        </is>
+      </c>
+      <c r="L155" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M155" s="2" t="inlineStr">
+        <is>
+          <t>10.51.9</t>
+        </is>
+      </c>
+      <c r="N155" s="2" t="inlineStr"/>
+      <c r="O155" s="2" t="inlineStr">
+        <is>
+          <t>08.06.2026 14:44 — 03.07.2026 23:00</t>
+        </is>
+      </c>
+      <c r="P155" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Вятская, д 27 стр 13</t>
+        </is>
+      </c>
+      <c r="Q155" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/planovoe-i-avariinoe-tekhnicheskoe-obsluzhivanie-zdanii-i-sooruzhenii/tender-4480614/#btid=2&amp;sqh=0ca549e468445c11519f78660f42d04b3782a4f3&amp;tsid=4480614004</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 10:25</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr"/>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>4512370</t>
+        </is>
+      </c>
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>ТО Сплит систем Лабинск Эйч энд Эн... кондиционирования Техническое обслуживание внутреннегоблокакассетного типа мультизональной  ...блокакондиционера. Мойка теплообменника внутреннегоблокакондиционера Чистка фильтров внутреннегоблокакондиционера Чистка фильтров приточнойвентиляционной...</t>
+        </is>
+      </c>
+      <c r="G156" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЭЙЧ ЭНД ЭН"</t>
+        </is>
+      </c>
+      <c r="H156" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЭЙЧ ЭНД ЭН"</t>
+        </is>
+      </c>
+      <c r="I156" s="2" t="inlineStr">
+        <is>
+          <t>7714626332</t>
+        </is>
+      </c>
+      <c r="J156" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K156" s="2" t="inlineStr">
+        <is>
+          <t>Закриев Якуб Салманович</t>
+        </is>
+      </c>
+      <c r="L156" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M156" s="2" t="inlineStr">
+        <is>
+          <t>10.51.9</t>
+        </is>
+      </c>
+      <c r="N156" s="2" t="inlineStr"/>
+      <c r="O156" s="2" t="inlineStr">
+        <is>
+          <t>03.07.2026 12:40 — 14.07.2026 18:30</t>
+        </is>
+      </c>
+      <c r="P156" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Вятская, д 27 стр 13</t>
+        </is>
+      </c>
+      <c r="Q156" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=cdef101190208a85fa93ffe6d33a72032c24383b&amp;tsid=4512370458</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 10:25</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="inlineStr"/>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E157" s="2" t="inlineStr">
+        <is>
           <t>4501483</t>
         </is>
       </c>
-      <c r="F154" s="2" t="inlineStr">
+      <c r="F157" s="2" t="inlineStr">
         <is>
           <t>Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ
 Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ...  d 50x2", внутренняя резьба RTPБлокуправления наружной установки ICEFREE TR-16 ...  Оповещатель звуковой МАЯК-12-ЗМБлокуправления наружной установки ICEFREE TS- ... проводов КС-3 007004 Велос Переходвентиляционный150х100 - D150, из тонколистовой оцинкованной ...</t>
         </is>
       </c>
-      <c r="G154" s="2" t="inlineStr">
+      <c r="G157" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="H154" s="2" t="inlineStr">
+      <c r="H157" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="I154" s="2" t="inlineStr">
+      <c r="I157" s="2" t="inlineStr">
         <is>
           <t>7805368914</t>
         </is>
       </c>
-      <c r="J154" s="2" t="inlineStr">
+      <c r="J157" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург</t>
         </is>
       </c>
-      <c r="K154" s="2" t="inlineStr">
+      <c r="K157" s="2" t="inlineStr">
         <is>
           <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
-      <c r="L154" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M154" s="2" t="inlineStr">
+      <c r="L157" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M157" s="2" t="inlineStr">
         <is>
           <t>46.90</t>
         </is>
       </c>
-      <c r="N154" s="2" t="inlineStr"/>
-      <c r="O154" s="2" t="inlineStr">
+      <c r="N157" s="2" t="inlineStr"/>
+      <c r="O157" s="2" t="inlineStr">
         <is>
           <t>25.06.2026 05:03 — 09.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P154" s="2" t="inlineStr">
+      <c r="P157" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
-      <c r="Q154" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=cda8ddd07c7eea5b97f8375cab564bf926b67092&amp;tsid=4501483003</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-03 08:13</t>
-        </is>
-      </c>
-      <c r="B155" s="2" t="inlineStr">
+      <c r="Q157" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=cdef101190208a85fa93ffe6d33a72032c24383b&amp;tsid=4501483003</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 10:25</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
         <is>
           <t>b2b-center</t>
         </is>
       </c>
-      <c r="C155" s="2" t="inlineStr"/>
-      <c r="D155" s="2" t="inlineStr">
+      <c r="C158" s="2" t="inlineStr"/>
+      <c r="D158" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E155" s="2" t="inlineStr">
+      <c r="E158" s="2" t="inlineStr">
         <is>
           <t>4501181</t>
         </is>
       </c>
-      <c r="F155" s="2" t="inlineStr">
+      <c r="F158" s="2" t="inlineStr">
         <is>
           <t>Вентиляторы промышленные и оборудование общеобменной вентиляции...  5Ф РешёткавентиляционнаяАМР 600х300М РешёткавентиляционнаяАМР 150х150М РешёткавентиляционнаяАМР 300х200М  ... мм.; масса 0,65 кгБлокконтроля сопротивления БСК-3.1 Канальный ...  533Па, габаритные размеры 700х467х2230 мм,блоков/моноблоков 5/1, в составе: - ...</t>
         </is>
       </c>
-      <c r="G155" s="2" t="inlineStr">
+      <c r="G158" s="2" t="inlineStr">
         <is>
           <t>АО "Мосинжпроект"</t>
         </is>
       </c>
-      <c r="H155" s="2" t="inlineStr">
+      <c r="H158" s="2" t="inlineStr">
         <is>
           <t>АО "МОСИНЖПРОЕКТ"</t>
         </is>
       </c>
-      <c r="I155" s="2" t="inlineStr">
+      <c r="I158" s="2" t="inlineStr">
         <is>
           <t>7701885820</t>
         </is>
       </c>
-      <c r="J155" s="2" t="inlineStr">
+      <c r="J158" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K155" s="2" t="inlineStr">
+      <c r="K158" s="2" t="inlineStr">
         <is>
           <t>Сорокин Антон Павлович</t>
         </is>
       </c>
-      <c r="L155" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M155" s="2" t="inlineStr">
+      <c r="L158" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M158" s="2" t="inlineStr">
         <is>
           <t>71.12.2</t>
         </is>
       </c>
-      <c r="N155" s="2" t="inlineStr"/>
-      <c r="O155" s="2" t="inlineStr">
+      <c r="N158" s="2" t="inlineStr"/>
+      <c r="O158" s="2" t="inlineStr">
         <is>
           <t>24.06.2026 15:45 — 22.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P155" s="2" t="inlineStr">
+      <c r="P158" s="2" t="inlineStr">
         <is>
           <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
         </is>
       </c>
-      <c r="Q155" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=cda8ddd07c7eea5b97f8375cab564bf926b67092&amp;tsid=4501181003</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-03 08:13</t>
-        </is>
-      </c>
-      <c r="B156" s="2" t="inlineStr">
+      <c r="Q158" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=cdef101190208a85fa93ffe6d33a72032c24383b&amp;tsid=4501181003</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 10:25</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
         <is>
           <t>b2b-center</t>
         </is>
       </c>
-      <c r="C156" s="2" t="inlineStr"/>
-      <c r="D156" s="2" t="inlineStr">
+      <c r="C159" s="2" t="inlineStr"/>
+      <c r="D159" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E156" s="2" t="inlineStr">
+      <c r="E159" s="2" t="inlineStr">
         <is>
           <t>4500120</t>
         </is>
       </c>
-      <c r="F156" s="2" t="inlineStr">
+      <c r="F159" s="2" t="inlineStr">
         <is>
           <t>Коммуникационное оборудование, компьютеры, комплектующие к ним, серверное оборудование и ПО...  и кабелей – 1 компл. Удаленныйблок(репитер) BSF414 , питание 220В,  ... 2х2 Комбайнер специализированный OMU Side (блок1) OMUSC1 Комбайнер специализированный OMU ... контроллер для мониторинга в FlexGain View,вентиляционнаяпанель с фильтрами, комплект кабелей, ...</t>
         </is>
       </c>
-      <c r="G156" s="2" t="inlineStr">
+      <c r="G159" s="2" t="inlineStr">
         <is>
           <t>АО "Мосинжпроект"</t>
         </is>
       </c>
-      <c r="H156" s="2" t="inlineStr">
+      <c r="H159" s="2" t="inlineStr">
         <is>
           <t>АО "МОСИНЖПРОЕКТ"</t>
         </is>
       </c>
-      <c r="I156" s="2" t="inlineStr">
+      <c r="I159" s="2" t="inlineStr">
         <is>
           <t>7701885820</t>
         </is>
       </c>
-      <c r="J156" s="2" t="inlineStr">
+      <c r="J159" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K156" s="2" t="inlineStr">
+      <c r="K159" s="2" t="inlineStr">
         <is>
           <t>Сорокин Антон Павлович</t>
         </is>
       </c>
-      <c r="L156" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M156" s="2" t="inlineStr">
+      <c r="L159" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M159" s="2" t="inlineStr">
         <is>
           <t>71.12.2</t>
         </is>
       </c>
-      <c r="N156" s="2" t="inlineStr"/>
-      <c r="O156" s="2" t="inlineStr">
+      <c r="N159" s="2" t="inlineStr"/>
+      <c r="O159" s="2" t="inlineStr">
         <is>
           <t>24.06.2026 09:48 — 15.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P156" s="2" t="inlineStr">
+      <c r="P159" s="2" t="inlineStr">
         <is>
           <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
         </is>
       </c>
-      <c r="Q156" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=cda8ddd07c7eea5b97f8375cab564bf926b67092&amp;tsid=4500120003</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-03 08:13</t>
-        </is>
-      </c>
-      <c r="B157" s="2" t="inlineStr">
+      <c r="Q159" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=cdef101190208a85fa93ffe6d33a72032c24383b&amp;tsid=4500120003</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 10:25</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
         <is>
           <t>b2b-center</t>
         </is>
       </c>
-      <c r="C157" s="2" t="inlineStr"/>
-      <c r="D157" s="2" t="inlineStr">
+      <c r="C160" s="2" t="inlineStr"/>
+      <c r="D160" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E157" s="2" t="inlineStr">
+      <c r="E160" s="2" t="inlineStr">
         <is>
           <t>4496006</t>
         </is>
       </c>
-      <c r="F157" s="2" t="inlineStr">
+      <c r="F160" s="2" t="inlineStr">
         <is>
           <t>Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп
 Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп... -316 ***Петля крепежная стальная ***Платаблокауправления ZC5 CAME ***Средство чистящее " ... /распылитель для чаши Генуя ***РешеткавентиляционнаяРВ-1 225Х225 ***Петля анкерная 0 ... мл ***Папка с зажимом ***РешеткавентиляционнаяРВ-1 325Х125 ***Папка на кольцах ...</t>
         </is>
       </c>
-      <c r="G157" s="2" t="inlineStr">
+      <c r="G160" s="2" t="inlineStr">
         <is>
           <t>ООО "СИБУР"</t>
         </is>
       </c>
-      <c r="H157" s="2" t="inlineStr">
+      <c r="H160" s="2" t="inlineStr">
         <is>
           <t>ООО "СИБУР"</t>
         </is>
       </c>
-      <c r="I157" s="2" t="inlineStr">
+      <c r="I160" s="2" t="inlineStr">
         <is>
           <t>7727576505</t>
         </is>
       </c>
-      <c r="J157" s="2" t="inlineStr">
+      <c r="J160" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K157" s="2" t="inlineStr">
+      <c r="K160" s="2" t="inlineStr">
         <is>
           <t>Карисалов Михаил Юрьевич</t>
         </is>
       </c>
-      <c r="L157" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M157" s="2" t="inlineStr">
+      <c r="L160" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M160" s="2" t="inlineStr">
         <is>
           <t>70.10</t>
         </is>
       </c>
-      <c r="N157" s="2" t="inlineStr"/>
-      <c r="O157" s="2" t="inlineStr">
+      <c r="N160" s="2" t="inlineStr"/>
+      <c r="O160" s="2" t="inlineStr">
         <is>
           <t>20.06.2026 16:19 — 04.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P157" s="2" t="inlineStr">
+      <c r="P160" s="2" t="inlineStr">
         <is>
           <t>г Москва, ул Кржижановского, д 16 к 3</t>
         </is>
       </c>
-      <c r="Q157" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nelikvidnykh-tmts-tarelki-dlia-filtra-prokladki-dvigatel/tender-4496006/#btid=2&amp;sqh=cda8ddd07c7eea5b97f8375cab564bf926b67092&amp;tsid=4496006003</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-03 08:13</t>
-        </is>
-      </c>
-      <c r="B158" s="2" t="inlineStr">
+      <c r="Q160" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/prodazha-nelikvidnykh-tmts-tarelki-dlia-filtra-prokladki-dvigatel/tender-4496006/#btid=2&amp;sqh=cdef101190208a85fa93ffe6d33a72032c24383b&amp;tsid=4496006003</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 10:25</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
         <is>
           <t>b2b-center</t>
         </is>
       </c>
-      <c r="C158" s="2" t="inlineStr"/>
-      <c r="D158" s="2" t="inlineStr">
+      <c r="C161" s="2" t="inlineStr"/>
+      <c r="D161" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E158" s="2" t="inlineStr">
+      <c r="E161" s="2" t="inlineStr">
         <is>
           <t>4483529</t>
         </is>
       </c>
-      <c r="F158" s="2" t="inlineStr">
+      <c r="F161" s="2" t="inlineStr">
         <is>
           <t>Продажа невостребованных ТМЦ - Столбы, модули, керамогранит и т.п.
 Материалы с хранения. Перечень ориентировочный, может измениться в меньшую сторону за счет возможной востребованности....  азотнокислое х.ч. ГОСТ 1277-75БлокТРАНСФОРМАТОРНЫЙ 220В АС 3В DC 500 ...  Омега стыковка панелей между со ***РешеткавентиляционнаяКМУ 200х200 ***ТермСопр_50М_-50/180_5/20мм ...</t>
         </is>
       </c>
-      <c r="G158" s="2" t="inlineStr">
+      <c r="G161" s="2" t="inlineStr">
         <is>
           <t>ООО "СИБУР"</t>
         </is>
       </c>
-      <c r="H158" s="2" t="inlineStr">
+      <c r="H161" s="2" t="inlineStr">
         <is>
           <t>ООО "СИБУР"</t>
         </is>
       </c>
-      <c r="I158" s="2" t="inlineStr">
+      <c r="I161" s="2" t="inlineStr">
         <is>
           <t>7727576505</t>
         </is>
       </c>
-      <c r="J158" s="2" t="inlineStr">
+      <c r="J161" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K158" s="2" t="inlineStr">
+      <c r="K161" s="2" t="inlineStr">
         <is>
           <t>Карисалов Михаил Юрьевич</t>
         </is>
       </c>
-      <c r="L158" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M158" s="2" t="inlineStr">
+      <c r="L161" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M161" s="2" t="inlineStr">
         <is>
           <t>70.10</t>
         </is>
       </c>
-      <c r="N158" s="2" t="inlineStr"/>
-      <c r="O158" s="2" t="inlineStr">
+      <c r="N161" s="2" t="inlineStr"/>
+      <c r="O161" s="2" t="inlineStr">
         <is>
           <t>09.06.2026 16:07 — 06.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P158" s="2" t="inlineStr">
+      <c r="P161" s="2" t="inlineStr">
         <is>
           <t>г Москва, ул Кржижановского, д 16 к 3</t>
         </is>
       </c>
-      <c r="Q158" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-stolby-moduli-keramogranit-i-t-p/tender-4483529/#btid=2&amp;sqh=cda8ddd07c7eea5b97f8375cab564bf926b67092&amp;tsid=4483529003</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-03 08:13</t>
-        </is>
-      </c>
-      <c r="B159" s="2" t="inlineStr">
+      <c r="Q161" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-stolby-moduli-keramogranit-i-t-p/tender-4483529/#btid=2&amp;sqh=cdef101190208a85fa93ffe6d33a72032c24383b&amp;tsid=4483529003</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 10:25</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
         <is>
           <t>b2b-center</t>
         </is>
       </c>
-      <c r="C159" s="2" t="inlineStr"/>
-      <c r="D159" s="2" t="inlineStr">
+      <c r="C162" s="2" t="inlineStr"/>
+      <c r="D162" s="2" t="inlineStr">
         <is>
           <t>Работы</t>
         </is>
       </c>
-      <c r="E159" s="2" t="inlineStr">
+      <c r="E162" s="2" t="inlineStr">
         <is>
           <t>4129930</t>
         </is>
       </c>
-      <c r="F159" s="2" t="inlineStr">
+      <c r="F162" s="2" t="inlineStr">
         <is>
           <t>Реализация материалов для ремонта (напольные покрытия, настенные покрытия, окна, двери и т.д.) с АО "Мальцовский портландцемент"Блокдверной балконныйБлокдверной филенчатый ДГ 21х9Блококонный 1500х1000 ммБлококонный 1770х1700 мм Желоб ...  Docke Рама оконная 3000х1200 мм Решеткавентиляционнаянаружная Ручка оконная ГОСТ 5087-80 ...</t>
         </is>
       </c>
-      <c r="G159" s="2" t="inlineStr">
+      <c r="G162" s="2" t="inlineStr">
         <is>
           <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
-      <c r="H159" s="2" t="inlineStr">
+      <c r="H162" s="2" t="inlineStr">
         <is>
           <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
-      <c r="I159" s="2" t="inlineStr">
+      <c r="I162" s="2" t="inlineStr">
         <is>
           <t>7708117908</t>
         </is>
       </c>
-      <c r="J159" s="2" t="inlineStr">
+      <c r="J162" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K159" s="2" t="inlineStr">
+      <c r="K162" s="2" t="inlineStr">
         <is>
           <t>Шматов Вячеслав Вячеславович</t>
         </is>
       </c>
-      <c r="L159" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M159" s="2" t="inlineStr">
+      <c r="L162" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M162" s="2" t="inlineStr">
         <is>
           <t>23.51</t>
         </is>
       </c>
-      <c r="N159" s="2" t="inlineStr"/>
-      <c r="O159" s="2" t="inlineStr">
+      <c r="N162" s="2" t="inlineStr"/>
+      <c r="O162" s="2" t="inlineStr">
         <is>
           <t>06.08.2025 14:33 — 07.08.2026 12:00</t>
         </is>
       </c>
-      <c r="P159" s="2" t="inlineStr">
+      <c r="P162" s="2" t="inlineStr">
         <is>
           <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
         </is>
       </c>
-      <c r="Q159" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=cda8ddd07c7eea5b97f8375cab564bf926b67092&amp;tsid=4129930003</t>
+      <c r="Q162" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=cdef101190208a85fa93ffe6d33a72032c24383b&amp;tsid=4129930003</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q159"/>
+  <autoFilter ref="A1:Q162"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -13858,6 +14084,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q157" r:id="rId156"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q158" r:id="rId157"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q159" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q160" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q161" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q162" r:id="rId161"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-04 09:12 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q36"/>
+  <dimension ref="A1:Q35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -622,14 +622,14 @@
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=a04c8aa6498d6ded68b79f93cfca66f83c25eb14&amp;tsid=4510835003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=ca7152d7443b6c09eab4b82410bb0b1ce22dd659&amp;tsid=4510835003</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -698,14 +698,14 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=a04c8aa6498d6ded68b79f93cfca66f83c25eb14&amp;tsid=4503612458</t>
+          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=ca7152d7443b6c09eab4b82410bb0b1ce22dd659&amp;tsid=4503612458</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -777,14 +777,14 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=a04c8aa6498d6ded68b79f93cfca66f83c25eb14&amp;tsid=4130106003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=ca7152d7443b6c09eab4b82410bb0b1ce22dd659&amp;tsid=4130106003</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -856,14 +856,14 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=4869d6df5023f5004ba24a6678b6c986444abaaf&amp;tsid=4498936003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=e0fe664a9b26ee99de3aad44e34c9efb73628f59&amp;tsid=4498936003</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -936,14 +936,14 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=d87f5d95d84fb7db4a4b761c01857d4518d0f6cc&amp;tsid=4497016004</t>
+          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=6dfdf02a2e0623fbca2d3ae971b18ba8e8505ec0&amp;tsid=4497016004</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1011,14 +1011,14 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=ea460cd06daffa78b6f6185dc7dcc8e3d0e7000f&amp;tsid=4512196458</t>
+          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=4d0de3927a3de1206bbd480c71d12e6c166c66b5&amp;tsid=4512196458</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1090,14 +1090,14 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=ea460cd06daffa78b6f6185dc7dcc8e3d0e7000f&amp;tsid=4512292004</t>
+          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=4d0de3927a3de1206bbd480c71d12e6c166c66b5&amp;tsid=4512292004</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1172,14 +1172,14 @@
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=b2e9d8f2a7bf35077eaff64d4d6ec061f4239c02&amp;tsid=4475879003</t>
+          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=e3d0e0a1fac35dee5f474fdaad63a817fafe5b45&amp;tsid=4475879003</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1251,14 +1251,14 @@
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=a02f205d4192d6656e3abc74b8307203d1596ce1&amp;tsid=4508331004</t>
+          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=46d2e0f9de921c6e3bf553aaba050c4e3dc8a4ca&amp;tsid=4508331004</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1326,14 +1326,14 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-koltsa/tender-4512253/#btid=2&amp;sqh=8bc2d2528235b965078f3c9c249c1b19489e7f9b&amp;tsid=4512253458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-koltsa/tender-4512253/#btid=2&amp;sqh=8fa7c6b8a6ab41b32abeaaadb029866c3f7b68d8&amp;tsid=4512253458</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1405,14 +1405,14 @@
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=8bc2d2528235b965078f3c9c249c1b19489e7f9b&amp;tsid=4510341459</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=8fa7c6b8a6ab41b32abeaaadb029866c3f7b68d8&amp;tsid=4510341459</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1480,14 +1480,14 @@
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-lotki-plity-bruski-bloki/tender-4510073/#btid=2&amp;sqh=8bc2d2528235b965078f3c9c249c1b19489e7f9b&amp;tsid=4510073458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-lotki-plity-bruski-bloki/tender-4510073/#btid=2&amp;sqh=8fa7c6b8a6ab41b32abeaaadb029866c3f7b68d8&amp;tsid=4510073458</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1555,14 +1555,14 @@
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=8bc2d2528235b965078f3c9c249c1b19489e7f9b&amp;tsid=4508347458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=8fa7c6b8a6ab41b32abeaaadb029866c3f7b68d8&amp;tsid=4508347458</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1635,14 +1635,14 @@
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhelezobetonnye-plity-b-u-neobkhodimy-plity-eto-te-kotorye/tender-4508689/#btid=2&amp;sqh=8bc2d2528235b965078f3c9c249c1b19489e7f9b&amp;tsid=4508689458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhelezobetonnye-plity-b-u-neobkhodimy-plity-eto-te-kotorye/tender-4508689/#btid=2&amp;sqh=8fa7c6b8a6ab41b32abeaaadb029866c3f7b68d8&amp;tsid=4508689458</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1714,14 +1714,14 @@
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=8bc2d2528235b965078f3c9c249c1b19489e7f9b&amp;tsid=4489772003</t>
+          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=8fa7c6b8a6ab41b32abeaaadb029866c3f7b68d8&amp;tsid=4489772003</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1793,14 +1793,14 @@
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=8bc2d2528235b965078f3c9c249c1b19489e7f9b&amp;tsid=4474790003</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=8fa7c6b8a6ab41b32abeaaadb029866c3f7b68d8&amp;tsid=4474790003</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1872,14 +1872,14 @@
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=8bc2d2528235b965078f3c9c249c1b19489e7f9b&amp;tsid=4180328003</t>
+          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=8fa7c6b8a6ab41b32abeaaadb029866c3f7b68d8&amp;tsid=4180328003</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1951,14 +1951,14 @@
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=8bc2d2528235b965078f3c9c249c1b19489e7f9b&amp;tsid=3973258003</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=8fa7c6b8a6ab41b32abeaaadb029866c3f7b68d8&amp;tsid=3973258003</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -2026,14 +2026,14 @@
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/tmts-srochnyi-otbor-predlozhenii-na-pravo-zakliucheniia-dogovora-postavki/tender-4512260/#btid=2&amp;sqh=8b267722c64204efe448e99352761f0aebbd9844&amp;tsid=4512260458</t>
+          <t>https://www.b2b-center.ru/app/market-next/tmts-srochnyi-otbor-predlozhenii-na-pravo-zakliucheniia-dogovora-postavki/tender-4512260/#btid=2&amp;sqh=3cedf1d27a28cd07cf1325a91217b5baa6e1e85d&amp;tsid=4512260458</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -2101,14 +2101,14 @@
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/proizvodstvo-vtorichnogo-shchebnia-iz-loma-zhelezobetonnykh-izdelii/tender-4509622/#btid=2&amp;sqh=8b267722c64204efe448e99352761f0aebbd9844&amp;tsid=4509622458</t>
+          <t>https://www.b2b-center.ru/app/market-next/proizvodstvo-vtorichnogo-shchebnia-iz-loma-zhelezobetonnykh-izdelii/tender-4509622/#btid=2&amp;sqh=3cedf1d27a28cd07cf1325a91217b5baa6e1e85d&amp;tsid=4509622458</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2180,14 +2180,14 @@
       </c>
       <c r="Q22" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zhelezobetonnye-izdeliia/tender-4474238/#btid=2&amp;sqh=8b267722c64204efe448e99352761f0aebbd9844&amp;tsid=4474238003</t>
+          <t>https://www.b2b-center.ru/market/zhelezobetonnye-izdeliia/tender-4474238/#btid=2&amp;sqh=3cedf1d27a28cd07cf1325a91217b5baa6e1e85d&amp;tsid=4474238003</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2263,14 +2263,14 @@
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=d07e585279e8a4e0a3fa7cd7e94e651e8b318b0c&amp;tsid=4511621004</t>
+          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=cd059b5c09ff075170b66ce17cc52fef9dac41d7&amp;tsid=4511621004</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2338,14 +2338,14 @@
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=d07e585279e8a4e0a3fa7cd7e94e651e8b318b0c&amp;tsid=4511787458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=cd059b5c09ff075170b66ce17cc52fef9dac41d7&amp;tsid=4511787458</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -2417,14 +2417,14 @@
       </c>
       <c r="Q25" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=d07e585279e8a4e0a3fa7cd7e94e651e8b318b0c&amp;tsid=4512541003</t>
+          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=cd059b5c09ff075170b66ce17cc52fef9dac41d7&amp;tsid=4512541003</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2497,14 +2497,14 @@
       </c>
       <c r="Q26" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=d07e585279e8a4e0a3fa7cd7e94e651e8b318b0c&amp;tsid=4508230004</t>
+          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=cd059b5c09ff075170b66ce17cc52fef9dac41d7&amp;tsid=4508230004</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -2577,14 +2577,14 @@
       </c>
       <c r="Q27" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=d07e585279e8a4e0a3fa7cd7e94e651e8b318b0c&amp;tsid=4504775003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=cd059b5c09ff075170b66ce17cc52fef9dac41d7&amp;tsid=4504775003</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -2656,14 +2656,14 @@
       </c>
       <c r="Q28" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=d07e585279e8a4e0a3fa7cd7e94e651e8b318b0c&amp;tsid=4501157003</t>
+          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=cd059b5c09ff075170b66ce17cc52fef9dac41d7&amp;tsid=4501157003</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -2735,14 +2735,14 @@
       </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=d07e585279e8a4e0a3fa7cd7e94e651e8b318b0c&amp;tsid=4499964003</t>
+          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=cd059b5c09ff075170b66ce17cc52fef9dac41d7&amp;tsid=4499964003</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -2814,14 +2814,14 @@
       </c>
       <c r="Q30" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=d90d6bffb80a9fc19a580a410f26dce799f08af8&amp;tsid=4512370458</t>
+          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=d0a502b801ef2c72807b6d154b15babd124b893d&amp;tsid=4512370458</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -2893,14 +2893,14 @@
       </c>
       <c r="Q31" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=d90d6bffb80a9fc19a580a410f26dce799f08af8&amp;tsid=4500120003</t>
+          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=d0a502b801ef2c72807b6d154b15babd124b893d&amp;tsid=4500120003</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -2972,14 +2972,14 @@
       </c>
       <c r="Q32" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=d90d6bffb80a9fc19a580a410f26dce799f08af8&amp;tsid=4501181003</t>
+          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=d0a502b801ef2c72807b6d154b15babd124b893d&amp;tsid=4501181003</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -3052,14 +3052,14 @@
       </c>
       <c r="Q33" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=d90d6bffb80a9fc19a580a410f26dce799f08af8&amp;tsid=4501483003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=d0a502b801ef2c72807b6d154b15babd124b893d&amp;tsid=4501483003</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3075,13 +3075,13 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>4496006</t>
+          <t>4483529</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп
-Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп... -316 ***Петля крепежная стальная ***Платаблокауправления ZC5 CAME ***Средство чистящее " ... /распылитель для чаши Генуя ***РешеткавентиляционнаяРВ-1 225Х225 ***Петля анкерная 0 ... мл ***Папка с зажимом ***РешеткавентиляционнаяРВ-1 325Х125 ***Папка на кольцах ...</t>
+          <t>Продажа невостребованных ТМЦ - Столбы, модули, керамогранит и т.п.
+Материалы с хранения. Перечень ориентировочный, может измениться в меньшую сторону за счет возможной востребованности....  азотнокислое х.ч. ГОСТ 1277-75БлокТРАНСФОРМАТОРНЫЙ 220В АС 3В DC 500 ...  Омега стыковка панелей между со ***РешеткавентиляционнаяКМУ 200х200 ***ТермСопр_50М_-50/180_5/20мм ...</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3122,7 +3122,7 @@
       <c r="N34" s="2" t="inlineStr"/>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>20.06.2026 16:19 — 04.07.2026 12:00</t>
+          <t>09.06.2026 16:07 — 06.07.2026 12:00</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr">
@@ -3132,14 +3132,14 @@
       </c>
       <c r="Q34" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nelikvidnykh-tmts-tarelki-dlia-filtra-prokladki-dvigatel/tender-4496006/#btid=2&amp;sqh=d90d6bffb80a9fc19a580a410f26dce799f08af8&amp;tsid=4496006003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-stolby-moduli-keramogranit-i-t-p/tender-4483529/#btid=2&amp;sqh=d0a502b801ef2c72807b6d154b15babd124b893d&amp;tsid=4483529003</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03 21:48</t>
+          <t>2026-07-04 09:12</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -3150,33 +3150,32 @@
       <c r="C35" s="2" t="inlineStr"/>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Работы</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>4483529</t>
+          <t>4129930</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Продажа невостребованных ТМЦ - Столбы, модули, керамогранит и т.п.
-Материалы с хранения. Перечень ориентировочный, может измениться в меньшую сторону за счет возможной востребованности....  азотнокислое х.ч. ГОСТ 1277-75БлокТРАНСФОРМАТОРНЫЙ 220В АС 3В DC 500 ...  Омега стыковка панелей между со ***РешеткавентиляционнаяКМУ 200х200 ***ТермСопр_50М_-50/180_5/20мм ...</t>
+          <t>Реализация материалов для ремонта (напольные покрытия, настенные покрытия, окна, двери и т.д.) с АО "Мальцовский портландцемент"Блокдверной балконныйБлокдверной филенчатый ДГ 21х9Блококонный 1500х1000 ммБлококонный 1770х1700 мм Желоб ...  Docke Рама оконная 3000х1200 мм Решеткавентиляционнаянаружная Ручка оконная ГОСТ 5087-80 ...</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>ООО "СИБУР"</t>
+          <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>ООО "СИБУР"</t>
+          <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>7727576505</t>
+          <t>7708117908</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -3186,7 +3185,7 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>Карисалов Михаил Юрьевич</t>
+          <t>Шматов Вячеслав Вячеславович</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
@@ -3196,107 +3195,28 @@
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>70.10</t>
+          <t>23.51</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr"/>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>09.06.2026 16:07 — 06.07.2026 12:00</t>
+          <t>06.08.2025 14:33 — 07.08.2026 12:00</t>
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Кржижановского, д 16 к 3</t>
+          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
         </is>
       </c>
       <c r="Q35" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-stolby-moduli-keramogranit-i-t-p/tender-4483529/#btid=2&amp;sqh=d90d6bffb80a9fc19a580a410f26dce799f08af8&amp;tsid=4483529003</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-03 21:48</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>Работы</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>4129930</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>Реализация материалов для ремонта (напольные покрытия, настенные покрытия, окна, двери и т.д.) с АО "Мальцовский портландцемент"Блокдверной балконныйБлокдверной филенчатый ДГ 21х9Блококонный 1500х1000 ммБлококонный 1770х1700 мм Желоб ...  Docke Рама оконная 3000х1200 мм Решеткавентиляционнаянаружная Ручка оконная ГОСТ 5087-80 ...</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>АО "ЦЕМРОС"</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>АО "ЦЕМРОС"</t>
-        </is>
-      </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>7708117908</t>
-        </is>
-      </c>
-      <c r="J36" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K36" s="2" t="inlineStr">
-        <is>
-          <t>Шматов Вячеслав Вячеславович</t>
-        </is>
-      </c>
-      <c r="L36" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M36" s="2" t="inlineStr">
-        <is>
-          <t>23.51</t>
-        </is>
-      </c>
-      <c r="N36" s="2" t="inlineStr"/>
-      <c r="O36" s="2" t="inlineStr">
-        <is>
-          <t>06.08.2025 14:33 — 07.08.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P36" s="2" t="inlineStr">
-        <is>
-          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
-        </is>
-      </c>
-      <c r="Q36" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=d90d6bffb80a9fc19a580a410f26dce799f08af8&amp;tsid=4129930003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=d0a502b801ef2c72807b6d154b15babd124b893d&amp;tsid=4129930003</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q36"/>
+  <autoFilter ref="A1:Q35"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -3332,7 +3252,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId35"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-04 15:49 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -622,14 +622,14 @@
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=ca7152d7443b6c09eab4b82410bb0b1ce22dd659&amp;tsid=4510835003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=3f73214a0d8d273d960c27f43517fa2df31c9b66&amp;tsid=4510835003</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -698,14 +698,14 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=ca7152d7443b6c09eab4b82410bb0b1ce22dd659&amp;tsid=4503612458</t>
+          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=3f73214a0d8d273d960c27f43517fa2df31c9b66&amp;tsid=4503612458</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -777,14 +777,14 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=ca7152d7443b6c09eab4b82410bb0b1ce22dd659&amp;tsid=4130106003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=3f73214a0d8d273d960c27f43517fa2df31c9b66&amp;tsid=4130106003</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -856,14 +856,14 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=e0fe664a9b26ee99de3aad44e34c9efb73628f59&amp;tsid=4498936003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=7b31880c49dc0b788847fd82e6bbc6d6fb229d25&amp;tsid=4498936003</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -936,14 +936,14 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=6dfdf02a2e0623fbca2d3ae971b18ba8e8505ec0&amp;tsid=4497016004</t>
+          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=529ed0bbab0db5c96d2e97248c731119697f7502&amp;tsid=4497016004</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1011,14 +1011,14 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=4d0de3927a3de1206bbd480c71d12e6c166c66b5&amp;tsid=4512196458</t>
+          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=64852083d17ef46820e79a6a1147b463051fae27&amp;tsid=4512196458</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1090,14 +1090,14 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=4d0de3927a3de1206bbd480c71d12e6c166c66b5&amp;tsid=4512292004</t>
+          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=64852083d17ef46820e79a6a1147b463051fae27&amp;tsid=4512292004</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1172,14 +1172,14 @@
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=e3d0e0a1fac35dee5f474fdaad63a817fafe5b45&amp;tsid=4475879003</t>
+          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=ac64738f1ecac381702c5f007684e4f527ee7313&amp;tsid=4475879003</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1251,14 +1251,14 @@
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=46d2e0f9de921c6e3bf553aaba050c4e3dc8a4ca&amp;tsid=4508331004</t>
+          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=8a3e7264c166892aa6231e29dc192b6ec923f1c0&amp;tsid=4508331004</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1326,14 +1326,14 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-koltsa/tender-4512253/#btid=2&amp;sqh=8fa7c6b8a6ab41b32abeaaadb029866c3f7b68d8&amp;tsid=4512253458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-koltsa/tender-4512253/#btid=2&amp;sqh=50aed0e7e88a0af51c99f1014a74ea344da5b75f&amp;tsid=4512253458</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1405,14 +1405,14 @@
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=8fa7c6b8a6ab41b32abeaaadb029866c3f7b68d8&amp;tsid=4510341459</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=50aed0e7e88a0af51c99f1014a74ea344da5b75f&amp;tsid=4510341459</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1480,14 +1480,14 @@
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-lotki-plity-bruski-bloki/tender-4510073/#btid=2&amp;sqh=8fa7c6b8a6ab41b32abeaaadb029866c3f7b68d8&amp;tsid=4510073458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-lotki-plity-bruski-bloki/tender-4510073/#btid=2&amp;sqh=50aed0e7e88a0af51c99f1014a74ea344da5b75f&amp;tsid=4510073458</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1555,14 +1555,14 @@
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=8fa7c6b8a6ab41b32abeaaadb029866c3f7b68d8&amp;tsid=4508347458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=50aed0e7e88a0af51c99f1014a74ea344da5b75f&amp;tsid=4508347458</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1635,14 +1635,14 @@
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhelezobetonnye-plity-b-u-neobkhodimy-plity-eto-te-kotorye/tender-4508689/#btid=2&amp;sqh=8fa7c6b8a6ab41b32abeaaadb029866c3f7b68d8&amp;tsid=4508689458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhelezobetonnye-plity-b-u-neobkhodimy-plity-eto-te-kotorye/tender-4508689/#btid=2&amp;sqh=50aed0e7e88a0af51c99f1014a74ea344da5b75f&amp;tsid=4508689458</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1714,14 +1714,14 @@
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=8fa7c6b8a6ab41b32abeaaadb029866c3f7b68d8&amp;tsid=4489772003</t>
+          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=50aed0e7e88a0af51c99f1014a74ea344da5b75f&amp;tsid=4489772003</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1793,14 +1793,14 @@
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=8fa7c6b8a6ab41b32abeaaadb029866c3f7b68d8&amp;tsid=4474790003</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=50aed0e7e88a0af51c99f1014a74ea344da5b75f&amp;tsid=4474790003</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1872,14 +1872,14 @@
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=8fa7c6b8a6ab41b32abeaaadb029866c3f7b68d8&amp;tsid=4180328003</t>
+          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=50aed0e7e88a0af51c99f1014a74ea344da5b75f&amp;tsid=4180328003</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1951,14 +1951,14 @@
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=8fa7c6b8a6ab41b32abeaaadb029866c3f7b68d8&amp;tsid=3973258003</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=50aed0e7e88a0af51c99f1014a74ea344da5b75f&amp;tsid=3973258003</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -2026,14 +2026,14 @@
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/tmts-srochnyi-otbor-predlozhenii-na-pravo-zakliucheniia-dogovora-postavki/tender-4512260/#btid=2&amp;sqh=3cedf1d27a28cd07cf1325a91217b5baa6e1e85d&amp;tsid=4512260458</t>
+          <t>https://www.b2b-center.ru/app/market-next/tmts-srochnyi-otbor-predlozhenii-na-pravo-zakliucheniia-dogovora-postavki/tender-4512260/#btid=2&amp;sqh=abf3a923922bac17f427316782728da1176b6bb1&amp;tsid=4512260458</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -2101,14 +2101,14 @@
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/proizvodstvo-vtorichnogo-shchebnia-iz-loma-zhelezobetonnykh-izdelii/tender-4509622/#btid=2&amp;sqh=3cedf1d27a28cd07cf1325a91217b5baa6e1e85d&amp;tsid=4509622458</t>
+          <t>https://www.b2b-center.ru/app/market-next/proizvodstvo-vtorichnogo-shchebnia-iz-loma-zhelezobetonnykh-izdelii/tender-4509622/#btid=2&amp;sqh=abf3a923922bac17f427316782728da1176b6bb1&amp;tsid=4509622458</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2180,14 +2180,14 @@
       </c>
       <c r="Q22" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zhelezobetonnye-izdeliia/tender-4474238/#btid=2&amp;sqh=3cedf1d27a28cd07cf1325a91217b5baa6e1e85d&amp;tsid=4474238003</t>
+          <t>https://www.b2b-center.ru/market/zhelezobetonnye-izdeliia/tender-4474238/#btid=2&amp;sqh=abf3a923922bac17f427316782728da1176b6bb1&amp;tsid=4474238003</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2263,14 +2263,14 @@
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=cd059b5c09ff075170b66ce17cc52fef9dac41d7&amp;tsid=4511621004</t>
+          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=c8c7a7905f31e96914e7b7f393d12c875cf5175d&amp;tsid=4511621004</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2338,14 +2338,14 @@
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=cd059b5c09ff075170b66ce17cc52fef9dac41d7&amp;tsid=4511787458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=c8c7a7905f31e96914e7b7f393d12c875cf5175d&amp;tsid=4511787458</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -2417,14 +2417,14 @@
       </c>
       <c r="Q25" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=cd059b5c09ff075170b66ce17cc52fef9dac41d7&amp;tsid=4512541003</t>
+          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=c8c7a7905f31e96914e7b7f393d12c875cf5175d&amp;tsid=4512541003</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2497,14 +2497,14 @@
       </c>
       <c r="Q26" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=cd059b5c09ff075170b66ce17cc52fef9dac41d7&amp;tsid=4508230004</t>
+          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=c8c7a7905f31e96914e7b7f393d12c875cf5175d&amp;tsid=4508230004</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -2577,14 +2577,14 @@
       </c>
       <c r="Q27" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=cd059b5c09ff075170b66ce17cc52fef9dac41d7&amp;tsid=4504775003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=c8c7a7905f31e96914e7b7f393d12c875cf5175d&amp;tsid=4504775003</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -2656,14 +2656,14 @@
       </c>
       <c r="Q28" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=cd059b5c09ff075170b66ce17cc52fef9dac41d7&amp;tsid=4501157003</t>
+          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=c8c7a7905f31e96914e7b7f393d12c875cf5175d&amp;tsid=4501157003</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -2735,14 +2735,14 @@
       </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=cd059b5c09ff075170b66ce17cc52fef9dac41d7&amp;tsid=4499964003</t>
+          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=c8c7a7905f31e96914e7b7f393d12c875cf5175d&amp;tsid=4499964003</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -2814,14 +2814,14 @@
       </c>
       <c r="Q30" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=d0a502b801ef2c72807b6d154b15babd124b893d&amp;tsid=4512370458</t>
+          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=1d858c29d8c276cacafc5e738c9ecc2cfd7a44fe&amp;tsid=4512370458</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -2893,14 +2893,14 @@
       </c>
       <c r="Q31" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=d0a502b801ef2c72807b6d154b15babd124b893d&amp;tsid=4500120003</t>
+          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=1d858c29d8c276cacafc5e738c9ecc2cfd7a44fe&amp;tsid=4500120003</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -2972,14 +2972,14 @@
       </c>
       <c r="Q32" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=d0a502b801ef2c72807b6d154b15babd124b893d&amp;tsid=4501181003</t>
+          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=1d858c29d8c276cacafc5e738c9ecc2cfd7a44fe&amp;tsid=4501181003</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -3052,14 +3052,14 @@
       </c>
       <c r="Q33" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=d0a502b801ef2c72807b6d154b15babd124b893d&amp;tsid=4501483003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=1d858c29d8c276cacafc5e738c9ecc2cfd7a44fe&amp;tsid=4501483003</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3132,14 +3132,14 @@
       </c>
       <c r="Q34" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-stolby-moduli-keramogranit-i-t-p/tender-4483529/#btid=2&amp;sqh=d0a502b801ef2c72807b6d154b15babd124b893d&amp;tsid=4483529003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-stolby-moduli-keramogranit-i-t-p/tender-4483529/#btid=2&amp;sqh=1d858c29d8c276cacafc5e738c9ecc2cfd7a44fe&amp;tsid=4483529003</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 09:12</t>
+          <t>2026-07-04 15:49</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -3211,7 +3211,7 @@
       </c>
       <c r="Q35" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=d0a502b801ef2c72807b6d154b15babd124b893d&amp;tsid=4129930003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=1d858c29d8c276cacafc5e738c9ecc2cfd7a44fe&amp;tsid=4129930003</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
leads: обновление 2026-07-04 21:19 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -622,14 +622,14 @@
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=3f73214a0d8d273d960c27f43517fa2df31c9b66&amp;tsid=4510835003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=17908fe97b42c52a7e7096e5a2a963adf7700f02&amp;tsid=4510835003</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -698,14 +698,14 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=3f73214a0d8d273d960c27f43517fa2df31c9b66&amp;tsid=4503612458</t>
+          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=17908fe97b42c52a7e7096e5a2a963adf7700f02&amp;tsid=4503612458</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -777,14 +777,14 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=3f73214a0d8d273d960c27f43517fa2df31c9b66&amp;tsid=4130106003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=17908fe97b42c52a7e7096e5a2a963adf7700f02&amp;tsid=4130106003</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -856,14 +856,14 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=7b31880c49dc0b788847fd82e6bbc6d6fb229d25&amp;tsid=4498936003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=2edbe8ed662baefa059299d04be518c9ca90b9da&amp;tsid=4498936003</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -936,14 +936,14 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=529ed0bbab0db5c96d2e97248c731119697f7502&amp;tsid=4497016004</t>
+          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=ba24d8710ffc1412e561709405761a58bb867813&amp;tsid=4497016004</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1011,14 +1011,14 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=64852083d17ef46820e79a6a1147b463051fae27&amp;tsid=4512196458</t>
+          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=e07385dee9fadb56a805470bc85ea2cd60cae164&amp;tsid=4512196458</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1090,14 +1090,14 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=64852083d17ef46820e79a6a1147b463051fae27&amp;tsid=4512292004</t>
+          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=e07385dee9fadb56a805470bc85ea2cd60cae164&amp;tsid=4512292004</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1172,14 +1172,14 @@
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=ac64738f1ecac381702c5f007684e4f527ee7313&amp;tsid=4475879003</t>
+          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=c6cf5189b31c0778879d9520c85ef3251f06bccc&amp;tsid=4475879003</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1251,14 +1251,14 @@
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=8a3e7264c166892aa6231e29dc192b6ec923f1c0&amp;tsid=4508331004</t>
+          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=6dbeb5c15f041e06076aa0ddf4a36a7687211fbf&amp;tsid=4508331004</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1326,14 +1326,14 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-koltsa/tender-4512253/#btid=2&amp;sqh=50aed0e7e88a0af51c99f1014a74ea344da5b75f&amp;tsid=4512253458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-koltsa/tender-4512253/#btid=2&amp;sqh=ccabd4b308d62c6e194d525fd4d127a64484e00d&amp;tsid=4512253458</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1405,14 +1405,14 @@
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=50aed0e7e88a0af51c99f1014a74ea344da5b75f&amp;tsid=4510341459</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=ccabd4b308d62c6e194d525fd4d127a64484e00d&amp;tsid=4510341459</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1480,14 +1480,14 @@
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-lotki-plity-bruski-bloki/tender-4510073/#btid=2&amp;sqh=50aed0e7e88a0af51c99f1014a74ea344da5b75f&amp;tsid=4510073458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-lotki-plity-bruski-bloki/tender-4510073/#btid=2&amp;sqh=ccabd4b308d62c6e194d525fd4d127a64484e00d&amp;tsid=4510073458</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1555,14 +1555,14 @@
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=50aed0e7e88a0af51c99f1014a74ea344da5b75f&amp;tsid=4508347458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=ccabd4b308d62c6e194d525fd4d127a64484e00d&amp;tsid=4508347458</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1635,14 +1635,14 @@
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhelezobetonnye-plity-b-u-neobkhodimy-plity-eto-te-kotorye/tender-4508689/#btid=2&amp;sqh=50aed0e7e88a0af51c99f1014a74ea344da5b75f&amp;tsid=4508689458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhelezobetonnye-plity-b-u-neobkhodimy-plity-eto-te-kotorye/tender-4508689/#btid=2&amp;sqh=ccabd4b308d62c6e194d525fd4d127a64484e00d&amp;tsid=4508689458</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1714,14 +1714,14 @@
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=50aed0e7e88a0af51c99f1014a74ea344da5b75f&amp;tsid=4489772003</t>
+          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=ccabd4b308d62c6e194d525fd4d127a64484e00d&amp;tsid=4489772003</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1793,14 +1793,14 @@
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=50aed0e7e88a0af51c99f1014a74ea344da5b75f&amp;tsid=4474790003</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=ccabd4b308d62c6e194d525fd4d127a64484e00d&amp;tsid=4474790003</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1872,14 +1872,14 @@
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=50aed0e7e88a0af51c99f1014a74ea344da5b75f&amp;tsid=4180328003</t>
+          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=ccabd4b308d62c6e194d525fd4d127a64484e00d&amp;tsid=4180328003</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1951,14 +1951,14 @@
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=50aed0e7e88a0af51c99f1014a74ea344da5b75f&amp;tsid=3973258003</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=ccabd4b308d62c6e194d525fd4d127a64484e00d&amp;tsid=3973258003</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -2026,14 +2026,14 @@
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/tmts-srochnyi-otbor-predlozhenii-na-pravo-zakliucheniia-dogovora-postavki/tender-4512260/#btid=2&amp;sqh=abf3a923922bac17f427316782728da1176b6bb1&amp;tsid=4512260458</t>
+          <t>https://www.b2b-center.ru/app/market-next/tmts-srochnyi-otbor-predlozhenii-na-pravo-zakliucheniia-dogovora-postavki/tender-4512260/#btid=2&amp;sqh=2b17cbcd92015c0353fd604c6e0cd9988e7a99f9&amp;tsid=4512260458</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -2101,14 +2101,14 @@
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/proizvodstvo-vtorichnogo-shchebnia-iz-loma-zhelezobetonnykh-izdelii/tender-4509622/#btid=2&amp;sqh=abf3a923922bac17f427316782728da1176b6bb1&amp;tsid=4509622458</t>
+          <t>https://www.b2b-center.ru/app/market-next/proizvodstvo-vtorichnogo-shchebnia-iz-loma-zhelezobetonnykh-izdelii/tender-4509622/#btid=2&amp;sqh=2b17cbcd92015c0353fd604c6e0cd9988e7a99f9&amp;tsid=4509622458</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2180,14 +2180,14 @@
       </c>
       <c r="Q22" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zhelezobetonnye-izdeliia/tender-4474238/#btid=2&amp;sqh=abf3a923922bac17f427316782728da1176b6bb1&amp;tsid=4474238003</t>
+          <t>https://www.b2b-center.ru/market/zhelezobetonnye-izdeliia/tender-4474238/#btid=2&amp;sqh=2b17cbcd92015c0353fd604c6e0cd9988e7a99f9&amp;tsid=4474238003</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2263,14 +2263,14 @@
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=c8c7a7905f31e96914e7b7f393d12c875cf5175d&amp;tsid=4511621004</t>
+          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=764f7b975590c25aafb2e56a0b40e89ad2f94f05&amp;tsid=4511621004</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2338,14 +2338,14 @@
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=c8c7a7905f31e96914e7b7f393d12c875cf5175d&amp;tsid=4511787458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=764f7b975590c25aafb2e56a0b40e89ad2f94f05&amp;tsid=4511787458</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -2417,14 +2417,14 @@
       </c>
       <c r="Q25" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=c8c7a7905f31e96914e7b7f393d12c875cf5175d&amp;tsid=4512541003</t>
+          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=764f7b975590c25aafb2e56a0b40e89ad2f94f05&amp;tsid=4512541003</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2497,14 +2497,14 @@
       </c>
       <c r="Q26" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=c8c7a7905f31e96914e7b7f393d12c875cf5175d&amp;tsid=4508230004</t>
+          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=764f7b975590c25aafb2e56a0b40e89ad2f94f05&amp;tsid=4508230004</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -2577,14 +2577,14 @@
       </c>
       <c r="Q27" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=c8c7a7905f31e96914e7b7f393d12c875cf5175d&amp;tsid=4504775003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=764f7b975590c25aafb2e56a0b40e89ad2f94f05&amp;tsid=4504775003</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -2656,14 +2656,14 @@
       </c>
       <c r="Q28" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=c8c7a7905f31e96914e7b7f393d12c875cf5175d&amp;tsid=4501157003</t>
+          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=764f7b975590c25aafb2e56a0b40e89ad2f94f05&amp;tsid=4501157003</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -2735,14 +2735,14 @@
       </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=c8c7a7905f31e96914e7b7f393d12c875cf5175d&amp;tsid=4499964003</t>
+          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=764f7b975590c25aafb2e56a0b40e89ad2f94f05&amp;tsid=4499964003</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -2814,14 +2814,14 @@
       </c>
       <c r="Q30" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=1d858c29d8c276cacafc5e738c9ecc2cfd7a44fe&amp;tsid=4512370458</t>
+          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=752f8f4e12298f98d03356292e8c3559e0a07e8c&amp;tsid=4512370458</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -2893,14 +2893,14 @@
       </c>
       <c r="Q31" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=1d858c29d8c276cacafc5e738c9ecc2cfd7a44fe&amp;tsid=4500120003</t>
+          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=752f8f4e12298f98d03356292e8c3559e0a07e8c&amp;tsid=4500120003</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -2972,14 +2972,14 @@
       </c>
       <c r="Q32" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=1d858c29d8c276cacafc5e738c9ecc2cfd7a44fe&amp;tsid=4501181003</t>
+          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=752f8f4e12298f98d03356292e8c3559e0a07e8c&amp;tsid=4501181003</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -3052,14 +3052,14 @@
       </c>
       <c r="Q33" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=1d858c29d8c276cacafc5e738c9ecc2cfd7a44fe&amp;tsid=4501483003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=752f8f4e12298f98d03356292e8c3559e0a07e8c&amp;tsid=4501483003</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3132,14 +3132,14 @@
       </c>
       <c r="Q34" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-stolby-moduli-keramogranit-i-t-p/tender-4483529/#btid=2&amp;sqh=1d858c29d8c276cacafc5e738c9ecc2cfd7a44fe&amp;tsid=4483529003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-stolby-moduli-keramogranit-i-t-p/tender-4483529/#btid=2&amp;sqh=752f8f4e12298f98d03356292e8c3559e0a07e8c&amp;tsid=4483529003</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 15:49</t>
+          <t>2026-07-04 21:19</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -3211,7 +3211,7 @@
       </c>
       <c r="Q35" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=1d858c29d8c276cacafc5e738c9ecc2cfd7a44fe&amp;tsid=4129930003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=752f8f4e12298f98d03356292e8c3559e0a07e8c&amp;tsid=4129930003</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
leads: обновление 2026-07-05 09:50 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q35"/>
+  <dimension ref="A1:Q34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -622,14 +622,14 @@
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=17908fe97b42c52a7e7096e5a2a963adf7700f02&amp;tsid=4510835003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=f431bf5deed92d26699fb82489597fd930a712df&amp;tsid=4510835003</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -698,14 +698,14 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=17908fe97b42c52a7e7096e5a2a963adf7700f02&amp;tsid=4503612458</t>
+          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=f431bf5deed92d26699fb82489597fd930a712df&amp;tsid=4503612458</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -777,14 +777,14 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=17908fe97b42c52a7e7096e5a2a963adf7700f02&amp;tsid=4130106003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=f431bf5deed92d26699fb82489597fd930a712df&amp;tsid=4130106003</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -856,14 +856,14 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=2edbe8ed662baefa059299d04be518c9ca90b9da&amp;tsid=4498936003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=1313bdf2ad60affdb7864a770e2630ca3204ec6c&amp;tsid=4498936003</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -936,14 +936,14 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=ba24d8710ffc1412e561709405761a58bb867813&amp;tsid=4497016004</t>
+          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=5edeed2377775e26a0d70dd800e24630c9cd631b&amp;tsid=4497016004</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1011,14 +1011,14 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=e07385dee9fadb56a805470bc85ea2cd60cae164&amp;tsid=4512196458</t>
+          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=17ae0a61972805788379fe67f041a59836181c00&amp;tsid=4512196458</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1090,14 +1090,14 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=e07385dee9fadb56a805470bc85ea2cd60cae164&amp;tsid=4512292004</t>
+          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=17ae0a61972805788379fe67f041a59836181c00&amp;tsid=4512292004</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1172,14 +1172,14 @@
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=c6cf5189b31c0778879d9520c85ef3251f06bccc&amp;tsid=4475879003</t>
+          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=d0c30dacff00a2297a86912863f764752acf0c66&amp;tsid=4475879003</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1251,14 +1251,14 @@
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=6dbeb5c15f041e06076aa0ddf4a36a7687211fbf&amp;tsid=4508331004</t>
+          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=29a3f2cd8d9309a332ee43a080a5faf8df2cc1e5&amp;tsid=4508331004</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1326,14 +1326,14 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-koltsa/tender-4512253/#btid=2&amp;sqh=ccabd4b308d62c6e194d525fd4d127a64484e00d&amp;tsid=4512253458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-koltsa/tender-4512253/#btid=2&amp;sqh=b35b145472817391c6cebc99d86f69411520e5d6&amp;tsid=4512253458</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1405,14 +1405,14 @@
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=ccabd4b308d62c6e194d525fd4d127a64484e00d&amp;tsid=4510341459</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=b35b145472817391c6cebc99d86f69411520e5d6&amp;tsid=4510341459</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1428,12 +1428,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>4510073</t>
+          <t>4508347</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>ЗакупкаЖБИ- лотки, плиты, бруски, блоки</t>
+          <t>ЖБИКЕМГРЭС</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1470,7 +1470,7 @@
       <c r="N13" s="2" t="inlineStr"/>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>02.07.2026 07:55 — 05.07.2026 12:00</t>
+          <t>01.07.2026 05:45 — 10.07.2026 00:00</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -1480,14 +1480,14 @@
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-lotki-plity-bruski-bloki/tender-4510073/#btid=2&amp;sqh=ccabd4b308d62c6e194d525fd4d127a64484e00d&amp;tsid=4510073458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=b35b145472817391c6cebc99d86f69411520e5d6&amp;tsid=4508347458</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1503,27 +1503,28 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>4508347</t>
+          <t>4508689</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>ЖБИКЕМГРЭС</t>
+          <t>Железобетонные плиты Б/У 
+Необходимы плиты, это те которые выдерживают нагрузку т.к. на эту плиту будет заезжать техника весом до 70тонн. Приоритетно с целью минимизации затрат рассмотрим плиты Б/У  размер произвольный но ближе 2х4; 3х3; 2х6. Количество плит необходимо +/- 50 шт. (данные плиты предназначаются для размещения на них запчастей и хоз. деятельности Горного цеха)Б/УЖБИплиты</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>7708117908</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1531,7 +1532,11 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Шматов Вячеслав Вячеславович</t>
+        </is>
+      </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1539,30 +1544,30 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>23.51</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr"/>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>01.07.2026 05:45 — 10.07.2026 00:00</t>
+          <t>01.07.2026 09:45 — 06.07.2026 09:00</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
         </is>
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=ccabd4b308d62c6e194d525fd4d127a64484e00d&amp;tsid=4508347458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhelezobetonnye-plity-b-u-neobkhodimy-plity-eto-te-kotorye/tender-4508689/#btid=2&amp;sqh=b35b145472817391c6cebc99d86f69411520e5d6&amp;tsid=4508689458</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1578,28 +1583,27 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>4508689</t>
+          <t>4489772</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Железобетонные плиты Б/У 
-Необходимы плиты, это те которые выдерживают нагрузку т.к. на эту плиту будет заезжать техника весом до 70тонн. Приоритетно с целью минимизации затрат рассмотрим плиты Б/У  размер произвольный но ближе 2х4; 3х3; 2х6. Количество плит необходимо +/- 50 шт. (данные плиты предназначаются для размещения на них запчастей и хоз. деятельности Горного цеха)Б/УЖБИплиты</t>
+          <t>1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы 1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>АО "ЦЕМРОС"</t>
+          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>АО "ЦЕМРОС"</t>
+          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>7708117908</t>
+          <t>7736583259</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -1609,7 +1613,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Шматов Вячеслав Вячеславович</t>
+          <t>Масько Александр Вадимович</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1619,30 +1623,30 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>23.51</t>
+          <t>70.10</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr"/>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>01.07.2026 09:45 — 06.07.2026 09:00</t>
+          <t>16.06.2026 11:00 — 16.07.2026 12:00</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
+          <t>г Москва, ул Старая Басманная, д 12 стр 1</t>
         </is>
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhelezobetonnye-plity-b-u-neobkhodimy-plity-eto-te-kotorye/tender-4508689/#btid=2&amp;sqh=ccabd4b308d62c6e194d525fd4d127a64484e00d&amp;tsid=4508689458</t>
+          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=b35b145472817391c6cebc99d86f69411520e5d6&amp;tsid=4489772003</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1658,37 +1662,37 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>4489772</t>
+          <t>4474790</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы 1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы</t>
+          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>7736583259</t>
+          <t>4704012472</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
+          <t>Ленинградская обл</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Масько Александр Вадимович</t>
+          <t>Габидуллин Тимур Махмудович</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -1698,30 +1702,30 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>70.10</t>
+          <t>17.12</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr"/>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>16.06.2026 11:00 — 16.07.2026 12:00</t>
+          <t>03.06.2026 09:59 — 30.07.2026 20:00</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Старая Басманная, д 12 стр 1</t>
+          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
         </is>
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=ccabd4b308d62c6e194d525fd4d127a64484e00d&amp;tsid=4489772003</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=b35b145472817391c6cebc99d86f69411520e5d6&amp;tsid=4474790003</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1737,37 +1741,37 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>4474790</t>
+          <t>4180328</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
+          <t>ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, г.Диксон). ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, ПГТ Диксон).</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>4704012472</t>
+          <t>7714456916</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Габидуллин Тимур Махмудович</t>
+          <t>Наумов Андрей Александрович</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -1777,30 +1781,30 @@
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>17.12</t>
+          <t>70.22</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr"/>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>03.06.2026 09:59 — 30.07.2026 20:00</t>
+          <t>24.09.2025 15:32 — 23.07.2026 12:00</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+          <t>г Москва, Денежный пер, д 9/6</t>
         </is>
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=ccabd4b308d62c6e194d525fd4d127a64484e00d&amp;tsid=4474790003</t>
+          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=b35b145472817391c6cebc99d86f69411520e5d6&amp;tsid=4180328003</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1816,37 +1820,37 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>4180328</t>
+          <t>3973258</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, г.Диксон). ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, ПГТ Диксон).</t>
+          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>7714456916</t>
+          <t>4704012472</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
+          <t>Ленинградская обл</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Наумов Андрей Александрович</t>
+          <t>Габидуллин Тимур Махмудович</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -1856,30 +1860,30 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>70.22</t>
+          <t>17.12</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr"/>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>24.09.2025 15:32 — 23.07.2026 12:00</t>
+          <t>10.03.2025 00:48 — 30.07.2026 23:00</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Денежный пер, д 9/6</t>
+          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
         </is>
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=ccabd4b308d62c6e194d525fd4d127a64484e00d&amp;tsid=4180328003</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=b35b145472817391c6cebc99d86f69411520e5d6&amp;tsid=3973258003</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1890,44 +1894,40 @@
       <c r="C19" s="2" t="inlineStr"/>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Поставка</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>3973258</t>
+          <t>4512260</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
+          <t>ТМЦ. Срочный отбор предложений на право заключения договора поставкижелезобетонных изделийдля нужд филиала «Канская теплосеть» АО «Енисейская ТГК (ТГК-13)».</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>4704012472</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>Габидуллин Тимур Махмудович</t>
-        </is>
-      </c>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1935,30 +1935,30 @@
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>17.12</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr"/>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>10.03.2025 00:48 — 30.07.2026 23:00</t>
+          <t>03.07.2026 11:52 — 08.07.2026 12:00</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=ccabd4b308d62c6e194d525fd4d127a64484e00d&amp;tsid=3973258003</t>
+          <t>https://www.b2b-center.ru/app/market-next/tmts-srochnyi-otbor-predlozhenii-na-pravo-zakliucheniia-dogovora-postavki/tender-4512260/#btid=2&amp;sqh=88398bcbfde16c074acc7710ac4b34ebd6c6079d&amp;tsid=4512260458</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1969,17 +1969,17 @@
       <c r="C20" s="2" t="inlineStr"/>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Поставка</t>
+          <t>Прочее</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>4512260</t>
+          <t>4509622</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>ТМЦ. Срочный отбор предложений на право заключения договора поставкижелезобетонных изделийдля нужд филиала «Канская теплосеть» АО «Енисейская ТГК (ТГК-13)».</t>
+          <t>Производство вторичного щебня из ломажелезобетонных изделий</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2016,7 +2016,7 @@
       <c r="N20" s="2" t="inlineStr"/>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 11:52 — 08.07.2026 12:00</t>
+          <t>01.07.2026 16:05 — 10.07.2026 12:00</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2026,14 +2026,14 @@
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/tmts-srochnyi-otbor-predlozhenii-na-pravo-zakliucheniia-dogovora-postavki/tender-4512260/#btid=2&amp;sqh=2b17cbcd92015c0353fd604c6e0cd9988e7a99f9&amp;tsid=4512260458</t>
+          <t>https://www.b2b-center.ru/app/market-next/proizvodstvo-vtorichnogo-shchebnia-iz-loma-zhelezobetonnykh-izdelii/tender-4509622/#btid=2&amp;sqh=88398bcbfde16c074acc7710ac4b34ebd6c6079d&amp;tsid=4509622458</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -2049,35 +2049,39 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>4509622</t>
+          <t>4474238</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Производство вторичного щебня из ломажелезобетонных изделий</t>
+          <t>Железобетонные изделияПлита перекрытия лотков П22-15И Плитка 2400*1500*160 б/у Плита перекрытия ПК 60-12 б/у</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ПАО "Коршуновский ГОК"</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ПАО "КОРШУНОВСКИЙ ГОК"</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>3834002314</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr"/>
+          <t>Иркутская обл</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Иванов Алексей Васильевич</t>
+        </is>
+      </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -2085,30 +2089,30 @@
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>07.10.2</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr"/>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>01.07.2026 16:05 — 10.07.2026 12:00</t>
+          <t>11.06.2026 09:23 — 06.07.2026 09:00</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>Иркутская обл, г Железногорск-Илимский, ул Иващенко, д 9А/1</t>
         </is>
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/proizvodstvo-vtorichnogo-shchebnia-iz-loma-zhelezobetonnykh-izdelii/tender-4509622/#btid=2&amp;sqh=2b17cbcd92015c0353fd604c6e0cd9988e7a99f9&amp;tsid=4509622458</t>
+          <t>https://www.b2b-center.ru/market/zhelezobetonnye-izdeliia/tender-4474238/#btid=2&amp;sqh=88398bcbfde16c074acc7710ac4b34ebd6c6079d&amp;tsid=4474238003</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2119,94 +2123,15 @@
       <c r="C22" s="2" t="inlineStr"/>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Поставка</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>4474238</t>
+          <t>4511621</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>Железобетонные изделияПлита перекрытия лотков П22-15И Плитка 2400*1500*160 б/у Плита перекрытия ПК 60-12 б/у</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>ПАО "Коршуновский ГОК"</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>ПАО "КОРШУНОВСКИЙ ГОК"</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>3834002314</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>Иркутская обл</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>Иванов Алексей Васильевич</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="inlineStr">
-        <is>
-          <t>07.10.2</t>
-        </is>
-      </c>
-      <c r="N22" s="2" t="inlineStr"/>
-      <c r="O22" s="2" t="inlineStr">
-        <is>
-          <t>11.06.2026 09:23 — 06.07.2026 09:00</t>
-        </is>
-      </c>
-      <c r="P22" s="2" t="inlineStr">
-        <is>
-          <t>Иркутская обл, г Железногорск-Илимский, ул Иващенко, д 9А/1</t>
-        </is>
-      </c>
-      <c r="Q22" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/zhelezobetonnye-izdeliia/tender-4474238/#btid=2&amp;sqh=2b17cbcd92015c0353fd604c6e0cd9988e7a99f9&amp;tsid=4474238003</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-04 21:19</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr"/>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>Поставка</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>4511621</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>Закупка аккумуляторных батарей (залитых) для нужд АО "Павловск Неруд" с поставкой в Августе 2026г.
 Обязательная расценка стоимости доставки, возможен забор груза на условиях самовывоза.
@@ -2215,19 +2140,98 @@
 Заказчик АО "Павловск Неруд" предприятие АО "Национальная нерудная компания"Аккумулятор ТН-550Перемычкам/ц для АКБ 115,5мм ТН-550Перемычкам/ц для АКБ 212,0мм ТН-550 Транспортная услуга</t>
         </is>
       </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>АО "ННК"</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>АО "ННК-ОЙЛ"</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>5032049030</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Худайнатов Эдуард Юрьевич</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>70.22</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>03.07.2026 06:22 — 07.07.2026 11:00</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул 1-я Тверская-Ямская, д 5, помещ 1012</t>
+        </is>
+      </c>
+      <c r="Q22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=a93904ea4932a9261d49865202ba9c5a2bb6bbe5&amp;tsid=4511621004</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05 09:50</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr"/>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>4511787</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>ЗЧ к автотранспорту... /66 ТЕРМОСТАТ ТС-107-1306100-06ПЕРЕМЫЧКААКБ КЛЕММА-КЛЕММА ПП 500-50 ...</t>
+        </is>
+      </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>АО "ННК"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>АО "ННК-ОЙЛ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>5032049030</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
@@ -2235,11 +2239,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>Худайнатов Эдуард Юрьевич</t>
-        </is>
-      </c>
+      <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -2247,30 +2247,30 @@
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>70.22</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr"/>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 06:22 — 07.07.2026 11:00</t>
+          <t>03.07.2026 08:32 — 08.07.2026 00:00</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул 1-я Тверская-Ямская, д 5, помещ 1012</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=764f7b975590c25aafb2e56a0b40e89ad2f94f05&amp;tsid=4511621004</t>
+          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=a93904ea4932a9261d49865202ba9c5a2bb6bbe5&amp;tsid=4511787458</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2286,35 +2286,39 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>4511787</t>
+          <t>4512541</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>ЗЧ к автотранспорту... /66 ТЕРМОСТАТ ТС-107-1306100-06ПЕРЕМЫЧКААКБ КЛЕММА-КЛЕММА ПП 500-50 ...</t>
+          <t>Запасные части CAT.... -3748 Cat Опора 348-9537 CatПеремычка140-0860 Cat Скоба 8X-3130 ...</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>1004001744</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr"/>
+          <t>Респ Карелия</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "СЕВЕРСТАЛЬ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -2322,30 +2326,30 @@
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>07.10.2</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr"/>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 08:32 — 08.07.2026 00:00</t>
+          <t>03.07.2026 14:07 — 10.07.2026 11:00</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>Респ Карелия, г Костомукша, шоссе Горняков, стр 284</t>
         </is>
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=764f7b975590c25aafb2e56a0b40e89ad2f94f05&amp;tsid=4511787458</t>
+          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=a93904ea4932a9261d49865202ba9c5a2bb6bbe5&amp;tsid=4512541003</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -2361,37 +2365,38 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>4512541</t>
+          <t>4508230</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Запасные части CAT.... -3748 Cat Опора 348-9537 CatПеремычка140-0860 Cat Скоба 8X-3130 ...</t>
+          <t>Сборный (Изделия электроустановочные и монтажные, Ящики, щиты, шкафы, пункты и комплектующие к ним, Приборы электроизмерительные, реле)
+МГ-019742, МГ-019713, МГ-019696, МГ-019665, МГ-019621, МГ-019620, МГ-019619, МГ-017109... -HESI-EX (5X20), Phoenix Contact 1277638ПеремычкаFBS 10-5, Phoenix Contact 3030213 ...ПеремычкаFBS 10-5 BU, Phoenix Contact  ...</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
+          <t>АО "ИК "АРЛАН"</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
+          <t>АО "ИК "АРЛАН"</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>1004001744</t>
+          <t>7722220390</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Респ Карелия</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "СЕВЕРСТАЛЬ МЕНЕДЖМЕНТ"</t>
+          <t>Барилов Евгений Александрович</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
@@ -2401,30 +2406,30 @@
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>07.10.2</t>
+          <t>82.99</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr"/>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 14:07 — 10.07.2026 11:00</t>
+          <t>30.06.2026 17:59 — 09.07.2026 12:00</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>Респ Карелия, г Костомукша, шоссе Горняков, стр 284</t>
+          <t>г Москва, Романов пер, д 4</t>
         </is>
       </c>
       <c r="Q25" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=764f7b975590c25aafb2e56a0b40e89ad2f94f05&amp;tsid=4512541003</t>
+          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=a93904ea4932a9261d49865202ba9c5a2bb6bbe5&amp;tsid=4508230004</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2440,38 +2445,38 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>4508230</t>
+          <t>4504775</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Сборный (Изделия электроустановочные и монтажные, Ящики, щиты, шкафы, пункты и комплектующие к ним, Приборы электроизмерительные, реле)
-МГ-019742, МГ-019713, МГ-019696, МГ-019665, МГ-019621, МГ-019620, МГ-019619, МГ-017109... -HESI-EX (5X20), Phoenix Contact 1277638ПеремычкаFBS 10-5, Phoenix Contact 3030213 ...ПеремычкаFBS 10-5 BU, Phoenix Contact  ...</t>
+          <t>Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники
+Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники...  Трубка пробная № 37-542-000 Соединитель-перемычка04182454 Кольцо стальное №CP48001-0305 Фильтр ...</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>АО "ИК "АРЛАН"</t>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>АО "ИК "АРЛАН"</t>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>7722220390</t>
+          <t>7805368914</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
+          <t>г Санкт-Петербург</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>Барилов Евгений Александрович</t>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
@@ -2481,30 +2486,30 @@
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>82.99</t>
+          <t>46.90</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr"/>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>30.06.2026 17:59 — 09.07.2026 12:00</t>
+          <t>27.06.2026 01:36 — 15.07.2026 12:00</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Романов пер, д 4</t>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
       <c r="Q26" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=764f7b975590c25aafb2e56a0b40e89ad2f94f05&amp;tsid=4508230004</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=a93904ea4932a9261d49865202ba9c5a2bb6bbe5&amp;tsid=4504775003</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -2520,38 +2525,37 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>4504775</t>
+          <t>4501157</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники
-Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники...  Трубка пробная № 37-542-000 Соединитель-перемычка04182454 Кольцо стальное №CP48001-0305 Фильтр ...</t>
+          <t>Источники электропитания (ИБП, аккумуляторные батареи, блоки питания)...  х 1248 А·ч, включая соединительныеперемычки. Вид положительного электрода - трубчатая пластина ...  с коммутирующей арматурой, межэлементными и межряднымиперемычками, крепежами, комплектом для обслуживания АБ. Тип ...</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+          <t>АО "Мосинжпроект"</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>7805368914</t>
+          <t>7701885820</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>г Санкт-Петербург</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
+          <t>Сорокин Антон Павлович</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
@@ -2561,30 +2565,30 @@
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>46.90</t>
+          <t>71.12.2</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr"/>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>27.06.2026 01:36 — 15.07.2026 12:00</t>
+          <t>24.06.2026 15:40 — 22.07.2026 12:00</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
         </is>
       </c>
       <c r="Q27" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=764f7b975590c25aafb2e56a0b40e89ad2f94f05&amp;tsid=4504775003</t>
+          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=a93904ea4932a9261d49865202ba9c5a2bb6bbe5&amp;tsid=4501157003</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -2600,12 +2604,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>4501157</t>
+          <t>4499964</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Источники электропитания (ИБП, аккумуляторные батареи, блоки питания)...  х 1248 А·ч, включая соединительныеперемычки. Вид положительного электрода - трубчатая пластина ...  с коммутирующей арматурой, межэлементными и межряднымиперемычками, крепежами, комплектом для обслуживания АБ. Тип ...</t>
+          <t>Автоматика и телемеханика движения поездов... , 13552-00-00В Дроссель-трансформатор (безперемычек) ДТМ-0,17-1000М ЮКЛЯ.672 ...</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -2646,7 +2650,7 @@
       <c r="N28" s="2" t="inlineStr"/>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 15:40 — 22.07.2026 12:00</t>
+          <t>24.06.2026 08:46 — 15.07.2026 12:00</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
@@ -2656,14 +2660,14 @@
       </c>
       <c r="Q28" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=764f7b975590c25aafb2e56a0b40e89ad2f94f05&amp;tsid=4501157003</t>
+          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=a93904ea4932a9261d49865202ba9c5a2bb6bbe5&amp;tsid=4499964003</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -2679,27 +2683,27 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>4499964</t>
+          <t>4512370</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Автоматика и телемеханика движения поездов... , 13552-00-00В Дроссель-трансформатор (безперемычек) ДТМ-0,17-1000М ЮКЛЯ.672 ...</t>
+          <t>ТО Сплит систем Лабинск Эйч энд Эн... кондиционирования Техническое обслуживание внутреннегоблокакассетного типа мультизональной  ...блокакондиционера. Мойка теплообменника внутреннегоблокакондиционера Чистка фильтров внутреннегоблокакондиционера Чистка фильтров приточнойвентиляционной...</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>АО "Мосинжпроект"</t>
+          <t>АО "ЭЙЧ ЭНД ЭН"</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>АО "МОСИНЖПРОЕКТ"</t>
+          <t>АО "ЭЙЧ ЭНД ЭН"</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>7701885820</t>
+          <t>7714626332</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
@@ -2709,7 +2713,7 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>Сорокин Антон Павлович</t>
+          <t>Закриев Якуб Салманович</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
@@ -2719,30 +2723,30 @@
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>71.12.2</t>
+          <t>10.51.9</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr"/>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 08:46 — 15.07.2026 12:00</t>
+          <t>03.07.2026 12:40 — 14.07.2026 18:30</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+          <t>г Москва, ул Вятская, д 27 стр 13</t>
         </is>
       </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=764f7b975590c25aafb2e56a0b40e89ad2f94f05&amp;tsid=4499964003</t>
+          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=4b6f954faf9ad4fe1ac5d29e7cead3e1ed296a01&amp;tsid=4512370458</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -2758,27 +2762,27 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>4512370</t>
+          <t>4500120</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>ТО Сплит систем Лабинск Эйч энд Эн... кондиционирования Техническое обслуживание внутреннегоблокакассетного типа мультизональной  ...блокакондиционера. Мойка теплообменника внутреннегоблокакондиционера Чистка фильтров внутреннегоблокакондиционера Чистка фильтров приточнойвентиляционной...</t>
+          <t>Коммуникационное оборудование, компьютеры, комплектующие к ним, серверное оборудование и ПО...  и кабелей – 1 компл. Удаленныйблок(репитер) BSF414 , питание 220В,  ... 2х2 Комбайнер специализированный OMU Side (блок1) OMUSC1 Комбайнер специализированный OMU ... контроллер для мониторинга в FlexGain View,вентиляционнаяпанель с фильтрами, комплект кабелей, ...</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>АО "ЭЙЧ ЭНД ЭН"</t>
+          <t>АО "Мосинжпроект"</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>АО "ЭЙЧ ЭНД ЭН"</t>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>7714626332</t>
+          <t>7701885820</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -2788,7 +2792,7 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>Закриев Якуб Салманович</t>
+          <t>Сорокин Антон Павлович</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
@@ -2798,30 +2802,30 @@
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>10.51.9</t>
+          <t>71.12.2</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr"/>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 12:40 — 14.07.2026 18:30</t>
+          <t>24.06.2026 09:48 — 15.07.2026 12:00</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Вятская, д 27 стр 13</t>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
         </is>
       </c>
       <c r="Q30" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=752f8f4e12298f98d03356292e8c3559e0a07e8c&amp;tsid=4512370458</t>
+          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=4b6f954faf9ad4fe1ac5d29e7cead3e1ed296a01&amp;tsid=4500120003</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -2837,12 +2841,12 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>4500120</t>
+          <t>4501181</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Коммуникационное оборудование, компьютеры, комплектующие к ним, серверное оборудование и ПО...  и кабелей – 1 компл. Удаленныйблок(репитер) BSF414 , питание 220В,  ... 2х2 Комбайнер специализированный OMU Side (блок1) OMUSC1 Комбайнер специализированный OMU ... контроллер для мониторинга в FlexGain View,вентиляционнаяпанель с фильтрами, комплект кабелей, ...</t>
+          <t>Вентиляторы промышленные и оборудование общеобменной вентиляции...  5Ф РешёткавентиляционнаяАМР 600х300М РешёткавентиляционнаяАМР 150х150М РешёткавентиляционнаяАМР 300х200М  ... мм.; масса 0,65 кгБлокконтроля сопротивления БСК-3.1 Канальный ...  533Па, габаритные размеры 700х467х2230 мм,блоков/моноблоков 5/1, в составе: - ...</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -2883,7 +2887,7 @@
       <c r="N31" s="2" t="inlineStr"/>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 09:48 — 15.07.2026 12:00</t>
+          <t>24.06.2026 15:45 — 22.07.2026 12:00</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
@@ -2893,14 +2897,14 @@
       </c>
       <c r="Q31" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=752f8f4e12298f98d03356292e8c3559e0a07e8c&amp;tsid=4500120003</t>
+          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=4b6f954faf9ad4fe1ac5d29e7cead3e1ed296a01&amp;tsid=4501181003</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -2916,37 +2920,38 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>4501181</t>
+          <t>4501483</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Вентиляторы промышленные и оборудование общеобменной вентиляции...  5Ф РешёткавентиляционнаяАМР 600х300М РешёткавентиляционнаяАМР 150х150М РешёткавентиляционнаяАМР 300х200М  ... мм.; масса 0,65 кгБлокконтроля сопротивления БСК-3.1 Канальный ...  533Па, габаритные размеры 700х467х2230 мм,блоков/моноблоков 5/1, в составе: - ...</t>
+          <t>Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ
+Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ...  d 50x2", внутренняя резьба RTPБлокуправления наружной установки ICEFREE TR-16 ...  Оповещатель звуковой МАЯК-12-ЗМБлокуправления наружной установки ICEFREE TS- ... проводов КС-3 007004 Велос Переходвентиляционный150х100 - D150, из тонколистовой оцинкованной ...</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>АО "Мосинжпроект"</t>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>АО "МОСИНЖПРОЕКТ"</t>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>7701885820</t>
+          <t>7805368914</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
+          <t>г Санкт-Петербург</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>Сорокин Антон Павлович</t>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
@@ -2956,30 +2961,30 @@
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>71.12.2</t>
+          <t>46.90</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr"/>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 15:45 — 22.07.2026 12:00</t>
+          <t>25.06.2026 05:03 — 09.07.2026 12:00</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
       <c r="Q32" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=752f8f4e12298f98d03356292e8c3559e0a07e8c&amp;tsid=4501181003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=4b6f954faf9ad4fe1ac5d29e7cead3e1ed296a01&amp;tsid=4501483003</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -2995,38 +3000,38 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>4501483</t>
+          <t>4483529</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ
-Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ...  d 50x2", внутренняя резьба RTPБлокуправления наружной установки ICEFREE TR-16 ...  Оповещатель звуковой МАЯК-12-ЗМБлокуправления наружной установки ICEFREE TS- ... проводов КС-3 007004 Велос Переходвентиляционный150х100 - D150, из тонколистовой оцинкованной ...</t>
+          <t>Продажа невостребованных ТМЦ - Столбы, модули, керамогранит и т.п.
+Материалы с хранения. Перечень ориентировочный, может измениться в меньшую сторону за счет возможной востребованности....  азотнокислое х.ч. ГОСТ 1277-75БлокТРАНСФОРМАТОРНЫЙ 220В АС 3В DC 500 ...  Омега стыковка панелей между со ***РешеткавентиляционнаяКМУ 200х200 ***ТермСопр_50М_-50/180_5/20мм ...</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+          <t>ООО "СИБУР"</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+          <t>ООО "СИБУР"</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>7805368914</t>
+          <t>7727576505</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>г Санкт-Петербург</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
+          <t>Карисалов Михаил Юрьевич</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
@@ -3036,30 +3041,30 @@
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>46.90</t>
+          <t>70.10</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr"/>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>25.06.2026 05:03 — 09.07.2026 12:00</t>
+          <t>09.06.2026 16:07 — 06.07.2026 12:00</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
+          <t>г Москва, ул Кржижановского, д 16 к 3</t>
         </is>
       </c>
       <c r="Q33" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=752f8f4e12298f98d03356292e8c3559e0a07e8c&amp;tsid=4501483003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-stolby-moduli-keramogranit-i-t-p/tender-4483529/#btid=2&amp;sqh=4b6f954faf9ad4fe1ac5d29e7cead3e1ed296a01&amp;tsid=4483529003</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04 21:19</t>
+          <t>2026-07-05 09:50</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3070,33 +3075,32 @@
       <c r="C34" s="2" t="inlineStr"/>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Работы</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>4483529</t>
+          <t>4129930</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Продажа невостребованных ТМЦ - Столбы, модули, керамогранит и т.п.
-Материалы с хранения. Перечень ориентировочный, может измениться в меньшую сторону за счет возможной востребованности....  азотнокислое х.ч. ГОСТ 1277-75БлокТРАНСФОРМАТОРНЫЙ 220В АС 3В DC 500 ...  Омега стыковка панелей между со ***РешеткавентиляционнаяКМУ 200х200 ***ТермСопр_50М_-50/180_5/20мм ...</t>
+          <t>Реализация материалов для ремонта (напольные покрытия, настенные покрытия, окна, двери и т.д.) с АО "Мальцовский портландцемент"Блокдверной балконныйБлокдверной филенчатый ДГ 21х9Блококонный 1500х1000 ммБлококонный 1770х1700 мм Желоб ...  Docke Рама оконная 3000х1200 мм Решеткавентиляционнаянаружная Ручка оконная ГОСТ 5087-80 ...</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>ООО "СИБУР"</t>
+          <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>ООО "СИБУР"</t>
+          <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>7727576505</t>
+          <t>7708117908</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -3106,7 +3110,7 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>Карисалов Михаил Юрьевич</t>
+          <t>Шматов Вячеслав Вячеславович</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
@@ -3116,107 +3120,28 @@
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>70.10</t>
+          <t>23.51</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr"/>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>09.06.2026 16:07 — 06.07.2026 12:00</t>
+          <t>06.08.2025 14:33 — 07.08.2026 12:00</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Кржижановского, д 16 к 3</t>
+          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
         </is>
       </c>
       <c r="Q34" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-stolby-moduli-keramogranit-i-t-p/tender-4483529/#btid=2&amp;sqh=752f8f4e12298f98d03356292e8c3559e0a07e8c&amp;tsid=4483529003</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-04 21:19</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr"/>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>Работы</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>4129930</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>Реализация материалов для ремонта (напольные покрытия, настенные покрытия, окна, двери и т.д.) с АО "Мальцовский портландцемент"Блокдверной балконныйБлокдверной филенчатый ДГ 21х9Блококонный 1500х1000 ммБлококонный 1770х1700 мм Желоб ...  Docke Рама оконная 3000х1200 мм Решеткавентиляционнаянаружная Ручка оконная ГОСТ 5087-80 ...</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>АО "ЦЕМРОС"</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>АО "ЦЕМРОС"</t>
-        </is>
-      </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>7708117908</t>
-        </is>
-      </c>
-      <c r="J35" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="inlineStr">
-        <is>
-          <t>Шматов Вячеслав Вячеславович</t>
-        </is>
-      </c>
-      <c r="L35" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M35" s="2" t="inlineStr">
-        <is>
-          <t>23.51</t>
-        </is>
-      </c>
-      <c r="N35" s="2" t="inlineStr"/>
-      <c r="O35" s="2" t="inlineStr">
-        <is>
-          <t>06.08.2025 14:33 — 07.08.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P35" s="2" t="inlineStr">
-        <is>
-          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
-        </is>
-      </c>
-      <c r="Q35" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=752f8f4e12298f98d03356292e8c3559e0a07e8c&amp;tsid=4129930003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=4b6f954faf9ad4fe1ac5d29e7cead3e1ed296a01&amp;tsid=4129930003</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q35"/>
+  <autoFilter ref="A1:Q34"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -3251,7 +3176,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId34"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-05 15:59 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -622,14 +622,14 @@
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=f431bf5deed92d26699fb82489597fd930a712df&amp;tsid=4510835003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=d871b994def30167b8d0ed304a7962a2f858f8c2&amp;tsid=4510835003</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -698,14 +698,14 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=f431bf5deed92d26699fb82489597fd930a712df&amp;tsid=4503612458</t>
+          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=d871b994def30167b8d0ed304a7962a2f858f8c2&amp;tsid=4503612458</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -777,14 +777,14 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=f431bf5deed92d26699fb82489597fd930a712df&amp;tsid=4130106003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=d871b994def30167b8d0ed304a7962a2f858f8c2&amp;tsid=4130106003</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -856,14 +856,14 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=1313bdf2ad60affdb7864a770e2630ca3204ec6c&amp;tsid=4498936003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=62e5d82083a718ac040e48421b5a98f7c969d01e&amp;tsid=4498936003</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -936,14 +936,14 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=5edeed2377775e26a0d70dd800e24630c9cd631b&amp;tsid=4497016004</t>
+          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=db6362917c6252f15d22f17073bd0b42a46c79e5&amp;tsid=4497016004</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1011,14 +1011,14 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=17ae0a61972805788379fe67f041a59836181c00&amp;tsid=4512196458</t>
+          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=f48d6bd925efebc90519daf85d6ce79820cb0cf8&amp;tsid=4512196458</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1090,14 +1090,14 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=17ae0a61972805788379fe67f041a59836181c00&amp;tsid=4512292004</t>
+          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=f48d6bd925efebc90519daf85d6ce79820cb0cf8&amp;tsid=4512292004</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1172,14 +1172,14 @@
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=d0c30dacff00a2297a86912863f764752acf0c66&amp;tsid=4475879003</t>
+          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=0baa18f70b788793a2662a2bb2f9ae00523b6ac9&amp;tsid=4475879003</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1251,14 +1251,14 @@
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=29a3f2cd8d9309a332ee43a080a5faf8df2cc1e5&amp;tsid=4508331004</t>
+          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=5b150ad76700f789f7aba2d3172dda4aecad53d0&amp;tsid=4508331004</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1326,14 +1326,14 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-koltsa/tender-4512253/#btid=2&amp;sqh=b35b145472817391c6cebc99d86f69411520e5d6&amp;tsid=4512253458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-koltsa/tender-4512253/#btid=2&amp;sqh=0975b466b9fdfd14a7ca0be008b95e8f7f4aadfa&amp;tsid=4512253458</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1405,14 +1405,14 @@
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=b35b145472817391c6cebc99d86f69411520e5d6&amp;tsid=4510341459</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=0975b466b9fdfd14a7ca0be008b95e8f7f4aadfa&amp;tsid=4510341459</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1480,14 +1480,14 @@
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=b35b145472817391c6cebc99d86f69411520e5d6&amp;tsid=4508347458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=0975b466b9fdfd14a7ca0be008b95e8f7f4aadfa&amp;tsid=4508347458</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1560,14 +1560,14 @@
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhelezobetonnye-plity-b-u-neobkhodimy-plity-eto-te-kotorye/tender-4508689/#btid=2&amp;sqh=b35b145472817391c6cebc99d86f69411520e5d6&amp;tsid=4508689458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhelezobetonnye-plity-b-u-neobkhodimy-plity-eto-te-kotorye/tender-4508689/#btid=2&amp;sqh=0975b466b9fdfd14a7ca0be008b95e8f7f4aadfa&amp;tsid=4508689458</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1639,14 +1639,14 @@
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=b35b145472817391c6cebc99d86f69411520e5d6&amp;tsid=4489772003</t>
+          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=0975b466b9fdfd14a7ca0be008b95e8f7f4aadfa&amp;tsid=4489772003</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1718,14 +1718,14 @@
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=b35b145472817391c6cebc99d86f69411520e5d6&amp;tsid=4474790003</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=0975b466b9fdfd14a7ca0be008b95e8f7f4aadfa&amp;tsid=4474790003</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1797,14 +1797,14 @@
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=b35b145472817391c6cebc99d86f69411520e5d6&amp;tsid=4180328003</t>
+          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=0975b466b9fdfd14a7ca0be008b95e8f7f4aadfa&amp;tsid=4180328003</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1876,14 +1876,14 @@
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=b35b145472817391c6cebc99d86f69411520e5d6&amp;tsid=3973258003</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=0975b466b9fdfd14a7ca0be008b95e8f7f4aadfa&amp;tsid=3973258003</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1951,14 +1951,14 @@
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/tmts-srochnyi-otbor-predlozhenii-na-pravo-zakliucheniia-dogovora-postavki/tender-4512260/#btid=2&amp;sqh=88398bcbfde16c074acc7710ac4b34ebd6c6079d&amp;tsid=4512260458</t>
+          <t>https://www.b2b-center.ru/app/market-next/tmts-srochnyi-otbor-predlozhenii-na-pravo-zakliucheniia-dogovora-postavki/tender-4512260/#btid=2&amp;sqh=1da8395aa189435b0f857148e2c896aef12c5217&amp;tsid=4512260458</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -2026,14 +2026,14 @@
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/proizvodstvo-vtorichnogo-shchebnia-iz-loma-zhelezobetonnykh-izdelii/tender-4509622/#btid=2&amp;sqh=88398bcbfde16c074acc7710ac4b34ebd6c6079d&amp;tsid=4509622458</t>
+          <t>https://www.b2b-center.ru/app/market-next/proizvodstvo-vtorichnogo-shchebnia-iz-loma-zhelezobetonnykh-izdelii/tender-4509622/#btid=2&amp;sqh=1da8395aa189435b0f857148e2c896aef12c5217&amp;tsid=4509622458</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -2105,14 +2105,14 @@
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zhelezobetonnye-izdeliia/tender-4474238/#btid=2&amp;sqh=88398bcbfde16c074acc7710ac4b34ebd6c6079d&amp;tsid=4474238003</t>
+          <t>https://www.b2b-center.ru/market/zhelezobetonnye-izdeliia/tender-4474238/#btid=2&amp;sqh=1da8395aa189435b0f857148e2c896aef12c5217&amp;tsid=4474238003</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2188,14 +2188,14 @@
       </c>
       <c r="Q22" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=a93904ea4932a9261d49865202ba9c5a2bb6bbe5&amp;tsid=4511621004</t>
+          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=eac7df6ef90b308e872ece59df0b7bdde918bfb8&amp;tsid=4511621004</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2263,14 +2263,14 @@
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=a93904ea4932a9261d49865202ba9c5a2bb6bbe5&amp;tsid=4511787458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=eac7df6ef90b308e872ece59df0b7bdde918bfb8&amp;tsid=4511787458</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2342,14 +2342,14 @@
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=a93904ea4932a9261d49865202ba9c5a2bb6bbe5&amp;tsid=4512541003</t>
+          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=eac7df6ef90b308e872ece59df0b7bdde918bfb8&amp;tsid=4512541003</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -2422,14 +2422,14 @@
       </c>
       <c r="Q25" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=a93904ea4932a9261d49865202ba9c5a2bb6bbe5&amp;tsid=4508230004</t>
+          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=eac7df6ef90b308e872ece59df0b7bdde918bfb8&amp;tsid=4508230004</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2502,14 +2502,14 @@
       </c>
       <c r="Q26" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=a93904ea4932a9261d49865202ba9c5a2bb6bbe5&amp;tsid=4504775003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=eac7df6ef90b308e872ece59df0b7bdde918bfb8&amp;tsid=4504775003</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -2581,14 +2581,14 @@
       </c>
       <c r="Q27" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=a93904ea4932a9261d49865202ba9c5a2bb6bbe5&amp;tsid=4501157003</t>
+          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=eac7df6ef90b308e872ece59df0b7bdde918bfb8&amp;tsid=4501157003</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -2660,14 +2660,14 @@
       </c>
       <c r="Q28" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=a93904ea4932a9261d49865202ba9c5a2bb6bbe5&amp;tsid=4499964003</t>
+          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=eac7df6ef90b308e872ece59df0b7bdde918bfb8&amp;tsid=4499964003</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -2739,14 +2739,14 @@
       </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=4b6f954faf9ad4fe1ac5d29e7cead3e1ed296a01&amp;tsid=4512370458</t>
+          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=8b423ef59abcef2fad984e6a6fd545f8548b83c4&amp;tsid=4512370458</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -2762,12 +2762,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>4500120</t>
+          <t>4501181</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Коммуникационное оборудование, компьютеры, комплектующие к ним, серверное оборудование и ПО...  и кабелей – 1 компл. Удаленныйблок(репитер) BSF414 , питание 220В,  ... 2х2 Комбайнер специализированный OMU Side (блок1) OMUSC1 Комбайнер специализированный OMU ... контроллер для мониторинга в FlexGain View,вентиляционнаяпанель с фильтрами, комплект кабелей, ...</t>
+          <t>Вентиляторы промышленные и оборудование общеобменной вентиляции...  5Ф РешёткавентиляционнаяАМР 600х300М РешёткавентиляционнаяАМР 150х150М РешёткавентиляционнаяАМР 300х200М  ... мм.; масса 0,65 кгБлокконтроля сопротивления БСК-3.1 Канальный ...  533Па, габаритные размеры 700х467х2230 мм,блоков/моноблоков 5/1, в составе: - ...</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -2808,7 +2808,7 @@
       <c r="N30" s="2" t="inlineStr"/>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 09:48 — 15.07.2026 12:00</t>
+          <t>24.06.2026 15:45 — 22.07.2026 12:00</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
@@ -2818,14 +2818,14 @@
       </c>
       <c r="Q30" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=4b6f954faf9ad4fe1ac5d29e7cead3e1ed296a01&amp;tsid=4500120003</t>
+          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=8b423ef59abcef2fad984e6a6fd545f8548b83c4&amp;tsid=4501181003</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -2841,37 +2841,38 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>4501181</t>
+          <t>4501483</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Вентиляторы промышленные и оборудование общеобменной вентиляции...  5Ф РешёткавентиляционнаяАМР 600х300М РешёткавентиляционнаяАМР 150х150М РешёткавентиляционнаяАМР 300х200М  ... мм.; масса 0,65 кгБлокконтроля сопротивления БСК-3.1 Канальный ...  533Па, габаритные размеры 700х467х2230 мм,блоков/моноблоков 5/1, в составе: - ...</t>
+          <t>Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ
+Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ...  d 50x2", внутренняя резьба RTPБлокуправления наружной установки ICEFREE TR-16 ...  Оповещатель звуковой МАЯК-12-ЗМБлокуправления наружной установки ICEFREE TS- ... проводов КС-3 007004 Велос Переходвентиляционный150х100 - D150, из тонколистовой оцинкованной ...</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>АО "Мосинжпроект"</t>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>АО "МОСИНЖПРОЕКТ"</t>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>7701885820</t>
+          <t>7805368914</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
+          <t>г Санкт-Петербург</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>Сорокин Антон Павлович</t>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
@@ -2881,30 +2882,30 @@
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>71.12.2</t>
+          <t>46.90</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr"/>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 15:45 — 22.07.2026 12:00</t>
+          <t>25.06.2026 05:03 — 09.07.2026 12:00</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
       <c r="Q31" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=4b6f954faf9ad4fe1ac5d29e7cead3e1ed296a01&amp;tsid=4501181003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=8b423ef59abcef2fad984e6a6fd545f8548b83c4&amp;tsid=4501483003</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -2920,38 +2921,37 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>4501483</t>
+          <t>4500120</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ
-Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ...  d 50x2", внутренняя резьба RTPБлокуправления наружной установки ICEFREE TR-16 ...  Оповещатель звуковой МАЯК-12-ЗМБлокуправления наружной установки ICEFREE TS- ... проводов КС-3 007004 Велос Переходвентиляционный150х100 - D150, из тонколистовой оцинкованной ...</t>
+          <t>Коммуникационное оборудование, компьютеры, комплектующие к ним, серверное оборудование и ПО...  и кабелей – 1 компл. Удаленныйблок(репитер) BSF414 , питание 220В,  ... 2х2 Комбайнер специализированный OMU Side (блок1) OMUSC1 Комбайнер специализированный OMU ... контроллер для мониторинга в FlexGain View,вентиляционнаяпанель с фильтрами, комплект кабелей, ...</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+          <t>АО "Мосинжпроект"</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>7805368914</t>
+          <t>7701885820</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>г Санкт-Петербург</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
+          <t>Сорокин Антон Павлович</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
@@ -2961,30 +2961,30 @@
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>46.90</t>
+          <t>71.12.2</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr"/>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>25.06.2026 05:03 — 09.07.2026 12:00</t>
+          <t>24.06.2026 09:48 — 15.07.2026 12:00</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
         </is>
       </c>
       <c r="Q32" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=4b6f954faf9ad4fe1ac5d29e7cead3e1ed296a01&amp;tsid=4501483003</t>
+          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=8b423ef59abcef2fad984e6a6fd545f8548b83c4&amp;tsid=4500120003</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -3057,14 +3057,14 @@
       </c>
       <c r="Q33" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-stolby-moduli-keramogranit-i-t-p/tender-4483529/#btid=2&amp;sqh=4b6f954faf9ad4fe1ac5d29e7cead3e1ed296a01&amp;tsid=4483529003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-stolby-moduli-keramogranit-i-t-p/tender-4483529/#btid=2&amp;sqh=8b423ef59abcef2fad984e6a6fd545f8548b83c4&amp;tsid=4483529003</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 09:50</t>
+          <t>2026-07-05 15:59</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="Q34" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=4b6f954faf9ad4fe1ac5d29e7cead3e1ed296a01&amp;tsid=4129930003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=8b423ef59abcef2fad984e6a6fd545f8548b83c4&amp;tsid=4129930003</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
leads: обновление 2026-07-05 21:41 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -622,14 +622,14 @@
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=d871b994def30167b8d0ed304a7962a2f858f8c2&amp;tsid=4510835003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=952bdb82196e4ba85d9ece6533c828a3cd57a811&amp;tsid=4510835003</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -698,14 +698,14 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=d871b994def30167b8d0ed304a7962a2f858f8c2&amp;tsid=4503612458</t>
+          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=952bdb82196e4ba85d9ece6533c828a3cd57a811&amp;tsid=4503612458</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -777,14 +777,14 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=d871b994def30167b8d0ed304a7962a2f858f8c2&amp;tsid=4130106003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=952bdb82196e4ba85d9ece6533c828a3cd57a811&amp;tsid=4130106003</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -856,14 +856,14 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=62e5d82083a718ac040e48421b5a98f7c969d01e&amp;tsid=4498936003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=b96f91112694e49278e5673fbb2e250115161abf&amp;tsid=4498936003</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -936,14 +936,14 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=db6362917c6252f15d22f17073bd0b42a46c79e5&amp;tsid=4497016004</t>
+          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=5b6f3ebe26bd49128c4715ce06e8b1aaf1aa5442&amp;tsid=4497016004</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1011,14 +1011,14 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=f48d6bd925efebc90519daf85d6ce79820cb0cf8&amp;tsid=4512196458</t>
+          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=38e4924f76821f63ed51b9e478478279d92864ed&amp;tsid=4512196458</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1090,14 +1090,14 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=f48d6bd925efebc90519daf85d6ce79820cb0cf8&amp;tsid=4512292004</t>
+          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=38e4924f76821f63ed51b9e478478279d92864ed&amp;tsid=4512292004</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1172,14 +1172,14 @@
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=0baa18f70b788793a2662a2bb2f9ae00523b6ac9&amp;tsid=4475879003</t>
+          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=dc7900349aeac044b1025cf79c7f4bbab8cddc17&amp;tsid=4475879003</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1251,14 +1251,14 @@
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=5b150ad76700f789f7aba2d3172dda4aecad53d0&amp;tsid=4508331004</t>
+          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=8ced20eec9268039e2daadb29b2220002af526d4&amp;tsid=4508331004</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1326,14 +1326,14 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-koltsa/tender-4512253/#btid=2&amp;sqh=0975b466b9fdfd14a7ca0be008b95e8f7f4aadfa&amp;tsid=4512253458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-koltsa/tender-4512253/#btid=2&amp;sqh=0fe936678e1d271e4619794d79d89f36d75d67e1&amp;tsid=4512253458</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1405,14 +1405,14 @@
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=0975b466b9fdfd14a7ca0be008b95e8f7f4aadfa&amp;tsid=4510341459</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=0fe936678e1d271e4619794d79d89f36d75d67e1&amp;tsid=4510341459</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1480,14 +1480,14 @@
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=0975b466b9fdfd14a7ca0be008b95e8f7f4aadfa&amp;tsid=4508347458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=0fe936678e1d271e4619794d79d89f36d75d67e1&amp;tsid=4508347458</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1560,14 +1560,14 @@
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhelezobetonnye-plity-b-u-neobkhodimy-plity-eto-te-kotorye/tender-4508689/#btid=2&amp;sqh=0975b466b9fdfd14a7ca0be008b95e8f7f4aadfa&amp;tsid=4508689458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhelezobetonnye-plity-b-u-neobkhodimy-plity-eto-te-kotorye/tender-4508689/#btid=2&amp;sqh=0fe936678e1d271e4619794d79d89f36d75d67e1&amp;tsid=4508689458</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1639,14 +1639,14 @@
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=0975b466b9fdfd14a7ca0be008b95e8f7f4aadfa&amp;tsid=4489772003</t>
+          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=0fe936678e1d271e4619794d79d89f36d75d67e1&amp;tsid=4489772003</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1718,14 +1718,14 @@
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=0975b466b9fdfd14a7ca0be008b95e8f7f4aadfa&amp;tsid=4474790003</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=0fe936678e1d271e4619794d79d89f36d75d67e1&amp;tsid=4474790003</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1797,14 +1797,14 @@
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=0975b466b9fdfd14a7ca0be008b95e8f7f4aadfa&amp;tsid=4180328003</t>
+          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=0fe936678e1d271e4619794d79d89f36d75d67e1&amp;tsid=4180328003</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1876,14 +1876,14 @@
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=0975b466b9fdfd14a7ca0be008b95e8f7f4aadfa&amp;tsid=3973258003</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=0fe936678e1d271e4619794d79d89f36d75d67e1&amp;tsid=3973258003</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1951,14 +1951,14 @@
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/tmts-srochnyi-otbor-predlozhenii-na-pravo-zakliucheniia-dogovora-postavki/tender-4512260/#btid=2&amp;sqh=1da8395aa189435b0f857148e2c896aef12c5217&amp;tsid=4512260458</t>
+          <t>https://www.b2b-center.ru/app/market-next/tmts-srochnyi-otbor-predlozhenii-na-pravo-zakliucheniia-dogovora-postavki/tender-4512260/#btid=2&amp;sqh=394bd67ad41069f98321e77ad41a359826cdb494&amp;tsid=4512260458</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -2026,14 +2026,14 @@
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/proizvodstvo-vtorichnogo-shchebnia-iz-loma-zhelezobetonnykh-izdelii/tender-4509622/#btid=2&amp;sqh=1da8395aa189435b0f857148e2c896aef12c5217&amp;tsid=4509622458</t>
+          <t>https://www.b2b-center.ru/app/market-next/proizvodstvo-vtorichnogo-shchebnia-iz-loma-zhelezobetonnykh-izdelii/tender-4509622/#btid=2&amp;sqh=394bd67ad41069f98321e77ad41a359826cdb494&amp;tsid=4509622458</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -2105,14 +2105,14 @@
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zhelezobetonnye-izdeliia/tender-4474238/#btid=2&amp;sqh=1da8395aa189435b0f857148e2c896aef12c5217&amp;tsid=4474238003</t>
+          <t>https://www.b2b-center.ru/market/zhelezobetonnye-izdeliia/tender-4474238/#btid=2&amp;sqh=394bd67ad41069f98321e77ad41a359826cdb494&amp;tsid=4474238003</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2188,14 +2188,14 @@
       </c>
       <c r="Q22" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=eac7df6ef90b308e872ece59df0b7bdde918bfb8&amp;tsid=4511621004</t>
+          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=43251c5994706ef2f47f7f206cccf7b74e950374&amp;tsid=4511621004</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2263,14 +2263,14 @@
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=eac7df6ef90b308e872ece59df0b7bdde918bfb8&amp;tsid=4511787458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=43251c5994706ef2f47f7f206cccf7b74e950374&amp;tsid=4511787458</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2342,14 +2342,14 @@
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=eac7df6ef90b308e872ece59df0b7bdde918bfb8&amp;tsid=4512541003</t>
+          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=43251c5994706ef2f47f7f206cccf7b74e950374&amp;tsid=4512541003</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -2422,14 +2422,14 @@
       </c>
       <c r="Q25" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=eac7df6ef90b308e872ece59df0b7bdde918bfb8&amp;tsid=4508230004</t>
+          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=43251c5994706ef2f47f7f206cccf7b74e950374&amp;tsid=4508230004</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2502,14 +2502,14 @@
       </c>
       <c r="Q26" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=eac7df6ef90b308e872ece59df0b7bdde918bfb8&amp;tsid=4504775003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=43251c5994706ef2f47f7f206cccf7b74e950374&amp;tsid=4504775003</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -2581,14 +2581,14 @@
       </c>
       <c r="Q27" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=eac7df6ef90b308e872ece59df0b7bdde918bfb8&amp;tsid=4501157003</t>
+          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=43251c5994706ef2f47f7f206cccf7b74e950374&amp;tsid=4501157003</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -2660,14 +2660,14 @@
       </c>
       <c r="Q28" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=eac7df6ef90b308e872ece59df0b7bdde918bfb8&amp;tsid=4499964003</t>
+          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=43251c5994706ef2f47f7f206cccf7b74e950374&amp;tsid=4499964003</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -2739,14 +2739,14 @@
       </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=8b423ef59abcef2fad984e6a6fd545f8548b83c4&amp;tsid=4512370458</t>
+          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=7474cc1ab5d66183b3313194fdc6aeb61602c1ed&amp;tsid=4512370458</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -2818,14 +2818,14 @@
       </c>
       <c r="Q30" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=8b423ef59abcef2fad984e6a6fd545f8548b83c4&amp;tsid=4501181003</t>
+          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=7474cc1ab5d66183b3313194fdc6aeb61602c1ed&amp;tsid=4501181003</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -2898,14 +2898,14 @@
       </c>
       <c r="Q31" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=8b423ef59abcef2fad984e6a6fd545f8548b83c4&amp;tsid=4501483003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=7474cc1ab5d66183b3313194fdc6aeb61602c1ed&amp;tsid=4501483003</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -2977,14 +2977,14 @@
       </c>
       <c r="Q32" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=8b423ef59abcef2fad984e6a6fd545f8548b83c4&amp;tsid=4500120003</t>
+          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=7474cc1ab5d66183b3313194fdc6aeb61602c1ed&amp;tsid=4500120003</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -3057,14 +3057,14 @@
       </c>
       <c r="Q33" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-stolby-moduli-keramogranit-i-t-p/tender-4483529/#btid=2&amp;sqh=8b423ef59abcef2fad984e6a6fd545f8548b83c4&amp;tsid=4483529003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-stolby-moduli-keramogranit-i-t-p/tender-4483529/#btid=2&amp;sqh=7474cc1ab5d66183b3313194fdc6aeb61602c1ed&amp;tsid=4483529003</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 15:59</t>
+          <t>2026-07-05 21:41</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="Q34" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=8b423ef59abcef2fad984e6a6fd545f8548b83c4&amp;tsid=4129930003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=7474cc1ab5d66183b3313194fdc6aeb61602c1ed&amp;tsid=4129930003</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
leads: обновление 2026-07-06 14:11 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q34"/>
+  <dimension ref="A1:Q35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -622,14 +622,14 @@
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=952bdb82196e4ba85d9ece6533c828a3cd57a811&amp;tsid=4510835003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=163f8e2e4073535c88d27b469a95f347fe7e1861&amp;tsid=4510835003</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -698,14 +698,14 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=952bdb82196e4ba85d9ece6533c828a3cd57a811&amp;tsid=4503612458</t>
+          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=163f8e2e4073535c88d27b469a95f347fe7e1861&amp;tsid=4503612458</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -777,14 +777,14 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=952bdb82196e4ba85d9ece6533c828a3cd57a811&amp;tsid=4130106003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=163f8e2e4073535c88d27b469a95f347fe7e1861&amp;tsid=4130106003</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -856,14 +856,14 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=b96f91112694e49278e5673fbb2e250115161abf&amp;tsid=4498936003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=8385288804917d040873ddced03bfd0eeb4f87dc&amp;tsid=4498936003</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -926,7 +926,7 @@
       <c r="N6" s="2" t="inlineStr"/>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>22.06.2026 16:20 — 06.07.2026 12:00</t>
+          <t>22.06.2026 16:20 — 09.07.2026 12:00</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -936,14 +936,14 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=5b6f3ebe26bd49128c4715ce06e8b1aaf1aa5442&amp;tsid=4497016004</t>
+          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=420ff314b316ade50f5d54007d807032f9dc870c&amp;tsid=4497016004</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1011,14 +1011,14 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=38e4924f76821f63ed51b9e478478279d92864ed&amp;tsid=4512196458</t>
+          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=e420765976372a60db8c86bf4e365bab65129250&amp;tsid=4512196458</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1090,14 +1090,14 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=38e4924f76821f63ed51b9e478478279d92864ed&amp;tsid=4512292004</t>
+          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=e420765976372a60db8c86bf4e365bab65129250&amp;tsid=4512292004</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1172,14 +1172,14 @@
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=dc7900349aeac044b1025cf79c7f4bbab8cddc17&amp;tsid=4475879003</t>
+          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=a44b2cde27516c18754a7005c4c8d5029a4da23c&amp;tsid=4475879003</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1251,14 +1251,14 @@
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=8ced20eec9268039e2daadb29b2220002af526d4&amp;tsid=4508331004</t>
+          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=9d5f90707b26c8e10458f99e604d4a7872f3c2f0&amp;tsid=4508331004</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1274,12 +1274,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>4512253</t>
+          <t>4514583</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>ЗакупкаЖБИ(кольца)</t>
+          <t>Закупка ЖБИ (плитыПДН3*1,5)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1316,7 +1316,7 @@
       <c r="N11" s="2" t="inlineStr"/>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 11:45 — 06.07.2026 12:00</t>
+          <t>06.07.2026 15:00 — 09.07.2026 12:00</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1326,14 +1326,14 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-koltsa/tender-4512253/#btid=2&amp;sqh=0fe936678e1d271e4619794d79d89f36d75d67e1&amp;tsid=4512253458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-plity-pdn-3-1-5/tender-4514583/#btid=2&amp;sqh=a9fae5a70d5ab8c93ccf2ffc068c750b655b544a&amp;tsid=4514583458</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1349,27 +1349,27 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>4510341</t>
+          <t>4513278</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>ЖБИ(чеч 34\25 7510 \ 17338)</t>
+          <t>ЖБИблоки ФБС</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>7724498866</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1377,11 +1377,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>Городний Анатолий Валерьевич</t>
-        </is>
-      </c>
+      <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1389,30 +1385,30 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>46.73</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr"/>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>02.07.2026 09:54 — 07.07.2026 16:00</t>
+          <t>06.07.2026 04:17 — 09.07.2026 00:00</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=0fe936678e1d271e4619794d79d89f36d75d67e1&amp;tsid=4510341459</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-bloki-fbs/tender-4513278/#btid=2&amp;sqh=f9fe44f277b7f45996a1a6d0bc25f78fee0fe018&amp;tsid=4513278458</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1423,32 +1419,32 @@
       <c r="C13" s="2" t="inlineStr"/>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Поставка</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>4508347</t>
+          <t>4514839</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>ЖБИКЕМГРЭС</t>
+          <t>12-х-1 Заключение договора на поставку материалов для наружных сетей водоснабжения и водоотведения на объект строительства «Дальневосточный детский центр отдыха и оздоровления в Хабаровском крае». (9 лотов) Лот №1 ВодоснабжениеЖБИ</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "ПРОМСТРОЙ"</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "ПРОМСТРОЙ"</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>9723169975</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1456,7 +1452,11 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Султанов Владислав Назипович</t>
+        </is>
+      </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1464,30 +1464,30 @@
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>71.12.2</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr"/>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>01.07.2026 05:45 — 10.07.2026 00:00</t>
+          <t>06.07.2026 16:45 — 10.07.2026 11:00</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Москва, Волгоградский пр-кт, д 42 к 5, ком 9</t>
         </is>
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=0fe936678e1d271e4619794d79d89f36d75d67e1&amp;tsid=4508347458</t>
+          <t>https://www.b2b-center.ru/market/12-kh-1-zakliuchenie-dogovora-na-postavku-materialov-dlia-naruzhnykh-setei/tender-4514839/#btid=2&amp;sqh=f9fe44f277b7f45996a1a6d0bc25f78fee0fe018&amp;tsid=4514839004</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1503,28 +1503,27 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>4508689</t>
+          <t>4510341</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Железобетонные плиты Б/У 
-Необходимы плиты, это те которые выдерживают нагрузку т.к. на эту плиту будет заезжать техника весом до 70тонн. Приоритетно с целью минимизации затрат рассмотрим плиты Б/У  размер произвольный но ближе 2х4; 3х3; 2х6. Количество плит необходимо +/- 50 шт. (данные плиты предназначаются для размещения на них запчастей и хоз. деятельности Горного цеха)Б/УЖБИплиты</t>
+          <t>ЖБИ(чеч 34\25 7510 \ 17338)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>АО "ЦЕМРОС"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>АО "ЦЕМРОС"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>7708117908</t>
+          <t>7724498866</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1534,7 +1533,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Шматов Вячеслав Вячеславович</t>
+          <t>Городний Анатолий Валерьевич</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -1544,30 +1543,30 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>23.51</t>
+          <t>46.73</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr"/>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>01.07.2026 09:45 — 06.07.2026 09:00</t>
+          <t>02.07.2026 09:54 — 07.07.2026 16:00</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
         </is>
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhelezobetonnye-plity-b-u-neobkhodimy-plity-eto-te-kotorye/tender-4508689/#btid=2&amp;sqh=0fe936678e1d271e4619794d79d89f36d75d67e1&amp;tsid=4508689458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=f9fe44f277b7f45996a1a6d0bc25f78fee0fe018&amp;tsid=4510341459</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1583,27 +1582,27 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>4489772</t>
+          <t>4508347</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы 1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы</t>
+          <t>ЖБИКЕМГРЭС</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>7736583259</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -1611,11 +1610,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>Масько Александр Вадимович</t>
-        </is>
-      </c>
+      <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1623,30 +1618,30 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>70.10</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr"/>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>16.06.2026 11:00 — 16.07.2026 12:00</t>
+          <t>01.07.2026 05:45 — 10.07.2026 00:00</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Старая Басманная, д 12 стр 1</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=0fe936678e1d271e4619794d79d89f36d75d67e1&amp;tsid=4489772003</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=f9fe44f277b7f45996a1a6d0bc25f78fee0fe018&amp;tsid=4508347458</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1662,37 +1657,37 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>4474790</t>
+          <t>4489772</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
+          <t>1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы 1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>4704012472</t>
+          <t>7736583259</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Габидуллин Тимур Махмудович</t>
+          <t>Масько Александр Вадимович</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -1702,30 +1697,30 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>17.12</t>
+          <t>70.10</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr"/>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>03.06.2026 09:59 — 30.07.2026 20:00</t>
+          <t>16.06.2026 11:00 — 16.07.2026 12:00</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+          <t>г Москва, ул Старая Басманная, д 12 стр 1</t>
         </is>
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=0fe936678e1d271e4619794d79d89f36d75d67e1&amp;tsid=4474790003</t>
+          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=f9fe44f277b7f45996a1a6d0bc25f78fee0fe018&amp;tsid=4489772003</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1741,37 +1736,37 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>4180328</t>
+          <t>4474790</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, г.Диксон). ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, ПГТ Диксон).</t>
+          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>7714456916</t>
+          <t>4704012472</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
+          <t>Ленинградская обл</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Наумов Андрей Александрович</t>
+          <t>Габидуллин Тимур Махмудович</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -1781,30 +1776,30 @@
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>70.22</t>
+          <t>17.12</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr"/>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>24.09.2025 15:32 — 23.07.2026 12:00</t>
+          <t>03.06.2026 09:59 — 30.07.2026 20:00</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Денежный пер, д 9/6</t>
+          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
         </is>
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=0fe936678e1d271e4619794d79d89f36d75d67e1&amp;tsid=4180328003</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=f9fe44f277b7f45996a1a6d0bc25f78fee0fe018&amp;tsid=4474790003</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1820,37 +1815,37 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>3973258</t>
+          <t>4180328</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
+          <t>ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, г.Диксон). ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, ПГТ Диксон).</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>4704012472</t>
+          <t>7714456916</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Габидуллин Тимур Махмудович</t>
+          <t>Наумов Андрей Александрович</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -1860,30 +1855,30 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>17.12</t>
+          <t>70.22</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr"/>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>10.03.2025 00:48 — 30.07.2026 23:00</t>
+          <t>24.09.2025 15:32 — 23.07.2026 12:00</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+          <t>г Москва, Денежный пер, д 9/6</t>
         </is>
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=0fe936678e1d271e4619794d79d89f36d75d67e1&amp;tsid=3973258003</t>
+          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=f9fe44f277b7f45996a1a6d0bc25f78fee0fe018&amp;tsid=4180328003</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1894,40 +1889,44 @@
       <c r="C19" s="2" t="inlineStr"/>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Поставка</t>
+          <t>Прочее</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>4512260</t>
+          <t>3973258</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>ТМЦ. Срочный отбор предложений на право заключения договора поставкижелезобетонных изделийдля нужд филиала «Канская теплосеть» АО «Енисейская ТГК (ТГК-13)».</t>
+          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>4704012472</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr"/>
+          <t>Ленинградская обл</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Габидуллин Тимур Махмудович</t>
+        </is>
+      </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1935,30 +1934,30 @@
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>17.12</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr"/>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 11:52 — 08.07.2026 12:00</t>
+          <t>10.03.2025 00:48 — 30.07.2026 23:00</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
         </is>
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/tmts-srochnyi-otbor-predlozhenii-na-pravo-zakliucheniia-dogovora-postavki/tender-4512260/#btid=2&amp;sqh=394bd67ad41069f98321e77ad41a359826cdb494&amp;tsid=4512260458</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=f9fe44f277b7f45996a1a6d0bc25f78fee0fe018&amp;tsid=3973258003</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1969,17 +1968,17 @@
       <c r="C20" s="2" t="inlineStr"/>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Поставка</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>4509622</t>
+          <t>4512260</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Производство вторичного щебня из ломажелезобетонных изделий</t>
+          <t>ТМЦ. Срочный отбор предложений на право заключения договора поставкижелезобетонных изделийдля нужд филиала «Канская теплосеть» АО «Енисейская ТГК (ТГК-13)».</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2016,7 +2015,7 @@
       <c r="N20" s="2" t="inlineStr"/>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>01.07.2026 16:05 — 10.07.2026 12:00</t>
+          <t>03.07.2026 11:52 — 08.07.2026 12:00</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2026,14 +2025,14 @@
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/proizvodstvo-vtorichnogo-shchebnia-iz-loma-zhelezobetonnykh-izdelii/tender-4509622/#btid=2&amp;sqh=394bd67ad41069f98321e77ad41a359826cdb494&amp;tsid=4509622458</t>
+          <t>https://www.b2b-center.ru/app/market-next/tmts-srochnyi-otbor-predlozhenii-na-pravo-zakliucheniia-dogovora-postavki/tender-4512260/#btid=2&amp;sqh=033ee602578d21ec9b4af0bff23cd79861d9d3fc&amp;tsid=4512260458</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -2049,39 +2048,35 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>4474238</t>
+          <t>4509622</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Железобетонные изделияПлита перекрытия лотков П22-15И Плитка 2400*1500*160 б/у Плита перекрытия ПК 60-12 б/у</t>
+          <t>Производство вторичного щебня из ломажелезобетонных изделий</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>ПАО "Коршуновский ГОК"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>ПАО "КОРШУНОВСКИЙ ГОК"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>3834002314</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Иркутская обл</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>Иванов Алексей Васильевич</t>
-        </is>
-      </c>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -2089,30 +2084,30 @@
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>07.10.2</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr"/>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>11.06.2026 09:23 — 06.07.2026 09:00</t>
+          <t>01.07.2026 16:05 — 10.07.2026 12:00</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>Иркутская обл, г Железногорск-Илимский, ул Иващенко, д 9А/1</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zhelezobetonnye-izdeliia/tender-4474238/#btid=2&amp;sqh=394bd67ad41069f98321e77ad41a359826cdb494&amp;tsid=4474238003</t>
+          <t>https://www.b2b-center.ru/app/market-next/proizvodstvo-vtorichnogo-shchebnia-iz-loma-zhelezobetonnykh-izdelii/tender-4509622/#btid=2&amp;sqh=033ee602578d21ec9b4af0bff23cd79861d9d3fc&amp;tsid=4509622458</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2188,14 +2183,14 @@
       </c>
       <c r="Q22" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=43251c5994706ef2f47f7f206cccf7b74e950374&amp;tsid=4511621004</t>
+          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=45dbd0fd67b523c4ca37137dd4b00bb065e06d78&amp;tsid=4511621004</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2263,14 +2258,14 @@
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=43251c5994706ef2f47f7f206cccf7b74e950374&amp;tsid=4511787458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=45dbd0fd67b523c4ca37137dd4b00bb065e06d78&amp;tsid=4511787458</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2342,14 +2337,14 @@
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=43251c5994706ef2f47f7f206cccf7b74e950374&amp;tsid=4512541003</t>
+          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=45dbd0fd67b523c4ca37137dd4b00bb065e06d78&amp;tsid=4512541003</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -2422,14 +2417,14 @@
       </c>
       <c r="Q25" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=43251c5994706ef2f47f7f206cccf7b74e950374&amp;tsid=4508230004</t>
+          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=45dbd0fd67b523c4ca37137dd4b00bb065e06d78&amp;tsid=4508230004</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2502,14 +2497,14 @@
       </c>
       <c r="Q26" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=43251c5994706ef2f47f7f206cccf7b74e950374&amp;tsid=4504775003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=45dbd0fd67b523c4ca37137dd4b00bb065e06d78&amp;tsid=4504775003</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -2581,14 +2576,14 @@
       </c>
       <c r="Q27" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=43251c5994706ef2f47f7f206cccf7b74e950374&amp;tsid=4501157003</t>
+          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=45dbd0fd67b523c4ca37137dd4b00bb065e06d78&amp;tsid=4501157003</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -2660,14 +2655,14 @@
       </c>
       <c r="Q28" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=43251c5994706ef2f47f7f206cccf7b74e950374&amp;tsid=4499964003</t>
+          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=45dbd0fd67b523c4ca37137dd4b00bb065e06d78&amp;tsid=4499964003</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -2683,12 +2678,13 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>4512370</t>
+          <t>4480614</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>ТО Сплит систем Лабинск Эйч энд Эн... кондиционирования Техническое обслуживание внутреннегоблокакассетного типа мультизональной  ...блокакондиционера. Мойка теплообменника внутреннегоблокакондиционера Чистка фильтров внутреннегоблокакондиционера Чистка фильтров приточнойвентиляционной...</t>
+          <t>Плановое и аварийное техническое обслуживание зданий и сооружений (годовое обслуживание август 2026 - август 2027) ГК Логика молока, производственная площадка в г. Ялуторовске
+Обслуживание зданий и сооружений завода в г. Ялуторовске....  стен из газобетонных блоков Устройство металлическихперемычекс устройством штраб Усиление кирпичных стен ...</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -2729,7 +2725,7 @@
       <c r="N29" s="2" t="inlineStr"/>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 12:40 — 14.07.2026 18:30</t>
+          <t>08.06.2026 14:44 — 08.07.2026 23:00</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
@@ -2739,14 +2735,14 @@
       </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=7474cc1ab5d66183b3313194fdc6aeb61602c1ed&amp;tsid=4512370458</t>
+          <t>https://www.b2b-center.ru/market/planovoe-i-avariinoe-tekhnicheskoe-obsluzhivanie-zdanii-i-sooruzhenii/tender-4480614/#btid=2&amp;sqh=45dbd0fd67b523c4ca37137dd4b00bb065e06d78&amp;tsid=4480614004</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -2762,27 +2758,27 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>4501181</t>
+          <t>4512370</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Вентиляторы промышленные и оборудование общеобменной вентиляции...  5Ф РешёткавентиляционнаяАМР 600х300М РешёткавентиляционнаяАМР 150х150М РешёткавентиляционнаяАМР 300х200М  ... мм.; масса 0,65 кгБлокконтроля сопротивления БСК-3.1 Канальный ...  533Па, габаритные размеры 700х467х2230 мм,блоков/моноблоков 5/1, в составе: - ...</t>
+          <t>ТО Сплит систем Лабинск Эйч энд Эн... кондиционирования Техническое обслуживание внутреннегоблокакассетного типа мультизональной  ...блокакондиционера. Мойка теплообменника внутреннегоблокакондиционера Чистка фильтров внутреннегоблокакондиционера Чистка фильтров приточнойвентиляционной...</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>АО "Мосинжпроект"</t>
+          <t>АО "ЭЙЧ ЭНД ЭН"</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>АО "МОСИНЖПРОЕКТ"</t>
+          <t>АО "ЭЙЧ ЭНД ЭН"</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>7701885820</t>
+          <t>7714626332</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -2792,7 +2788,7 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>Сорокин Антон Павлович</t>
+          <t>Закриев Якуб Салманович</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
@@ -2802,30 +2798,30 @@
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>71.12.2</t>
+          <t>10.51.9</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr"/>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 15:45 — 22.07.2026 12:00</t>
+          <t>03.07.2026 12:40 — 14.07.2026 18:30</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+          <t>г Москва, ул Вятская, д 27 стр 13</t>
         </is>
       </c>
       <c r="Q30" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=7474cc1ab5d66183b3313194fdc6aeb61602c1ed&amp;tsid=4501181003</t>
+          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=0a65cd04d994a200988cac92f51cd6de345d7a6e&amp;tsid=4512370458</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -2841,150 +2837,150 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
+          <t>4501181</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Вентиляторы промышленные и оборудование общеобменной вентиляции...  5Ф РешёткавентиляционнаяАМР 600х300М РешёткавентиляционнаяАМР 150х150М РешёткавентиляционнаяАМР 300х200М  ... мм.; масса 0,65 кгБлокконтроля сопротивления БСК-3.1 Канальный ...  533Па, габаритные размеры 700х467х2230 мм,блоков/моноблоков 5/1, в составе: - ...</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>АО "Мосинжпроект"</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>7701885820</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Сорокин Антон Павлович</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>71.12.2</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr"/>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>24.06.2026 15:45 — 22.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+        </is>
+      </c>
+      <c r="Q31" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=0a65cd04d994a200988cac92f51cd6de345d7a6e&amp;tsid=4501181003</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06 14:11</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
           <t>4501483</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ
 Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ...  d 50x2", внутренняя резьба RTPБлокуправления наружной установки ICEFREE TR-16 ...  Оповещатель звуковой МАЯК-12-ЗМБлокуправления наружной установки ICEFREE TS- ... проводов КС-3 007004 Велос Переходвентиляционный150х100 - D150, из тонколистовой оцинкованной ...</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>7805368914</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr">
+      <c r="J32" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург</t>
         </is>
       </c>
-      <c r="K31" s="2" t="inlineStr">
+      <c r="K32" s="2" t="inlineStr">
         <is>
           <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
-      <c r="L31" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M31" s="2" t="inlineStr">
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
         <is>
           <t>46.90</t>
-        </is>
-      </c>
-      <c r="N31" s="2" t="inlineStr"/>
-      <c r="O31" s="2" t="inlineStr">
-        <is>
-          <t>25.06.2026 05:03 — 09.07.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P31" s="2" t="inlineStr">
-        <is>
-          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
-        </is>
-      </c>
-      <c r="Q31" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=7474cc1ab5d66183b3313194fdc6aeb61602c1ed&amp;tsid=4501483003</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-05 21:41</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>4500120</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Коммуникационное оборудование, компьютеры, комплектующие к ним, серверное оборудование и ПО...  и кабелей – 1 компл. Удаленныйблок(репитер) BSF414 , питание 220В,  ... 2х2 Комбайнер специализированный OMU Side (блок1) OMUSC1 Комбайнер специализированный OMU ... контроллер для мониторинга в FlexGain View,вентиляционнаяпанель с фильтрами, комплект кабелей, ...</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>АО "Мосинжпроект"</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>АО "МОСИНЖПРОЕКТ"</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>7701885820</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr">
-        <is>
-          <t>Сорокин Антон Павлович</t>
-        </is>
-      </c>
-      <c r="L32" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M32" s="2" t="inlineStr">
-        <is>
-          <t>71.12.2</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr"/>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 09:48 — 15.07.2026 12:00</t>
+          <t>25.06.2026 05:03 — 09.07.2026 12:00</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
       <c r="Q32" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=7474cc1ab5d66183b3313194fdc6aeb61602c1ed&amp;tsid=4500120003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=0a65cd04d994a200988cac92f51cd6de345d7a6e&amp;tsid=4501483003</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -3000,28 +2996,27 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>4483529</t>
+          <t>4500120</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Продажа невостребованных ТМЦ - Столбы, модули, керамогранит и т.п.
-Материалы с хранения. Перечень ориентировочный, может измениться в меньшую сторону за счет возможной востребованности....  азотнокислое х.ч. ГОСТ 1277-75БлокТРАНСФОРМАТОРНЫЙ 220В АС 3В DC 500 ...  Омега стыковка панелей между со ***РешеткавентиляционнаяКМУ 200х200 ***ТермСопр_50М_-50/180_5/20мм ...</t>
+          <t>Коммуникационное оборудование, компьютеры, комплектующие к ним, серверное оборудование и ПО...  и кабелей – 1 компл. Удаленныйблок(репитер) BSF414 , питание 220В,  ... 2х2 Комбайнер специализированный OMU Side (блок1) OMUSC1 Комбайнер специализированный OMU ... контроллер для мониторинга в FlexGain View,вентиляционнаяпанель с фильтрами, комплект кабелей, ...</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>ООО "СИБУР"</t>
+          <t>АО "Мосинжпроект"</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>ООО "СИБУР"</t>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>7727576505</t>
+          <t>7701885820</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -3031,7 +3026,7 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Карисалов Михаил Юрьевич</t>
+          <t>Сорокин Антон Павлович</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
@@ -3041,30 +3036,30 @@
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>70.10</t>
+          <t>71.12.2</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr"/>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>09.06.2026 16:07 — 06.07.2026 12:00</t>
+          <t>24.06.2026 09:48 — 15.07.2026 12:00</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Кржижановского, д 16 к 3</t>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
         </is>
       </c>
       <c r="Q33" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-stolby-moduli-keramogranit-i-t-p/tender-4483529/#btid=2&amp;sqh=7474cc1ab5d66183b3313194fdc6aeb61602c1ed&amp;tsid=4483529003</t>
+          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=0a65cd04d994a200988cac92f51cd6de345d7a6e&amp;tsid=4500120003</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05 21:41</t>
+          <t>2026-07-06 14:11</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3075,32 +3070,33 @@
       <c r="C34" s="2" t="inlineStr"/>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Работы</t>
+          <t>Прочее</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>4129930</t>
+          <t>4496006</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Реализация материалов для ремонта (напольные покрытия, настенные покрытия, окна, двери и т.д.) с АО "Мальцовский портландцемент"Блокдверной балконныйБлокдверной филенчатый ДГ 21х9Блококонный 1500х1000 ммБлококонный 1770х1700 мм Желоб ...  Docke Рама оконная 3000х1200 мм Решеткавентиляционнаянаружная Ручка оконная ГОСТ 5087-80 ...</t>
+          <t>Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп
+Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп... -316 ***Петля крепежная стальная ***Платаблокауправления ZC5 CAME ***Средство чистящее " ... /распылитель для чаши Генуя ***РешеткавентиляционнаяРВ-1 225Х225 ***Петля анкерная 0 ... мл ***Папка с зажимом ***РешеткавентиляционнаяРВ-1 325Х125 ***Папка на кольцах ...</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>АО "ЦЕМРОС"</t>
+          <t>ООО "СИБУР"</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>АО "ЦЕМРОС"</t>
+          <t>ООО "СИБУР"</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>7708117908</t>
+          <t>7727576505</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -3110,7 +3106,7 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>Шматов Вячеслав Вячеславович</t>
+          <t>Карисалов Михаил Юрьевич</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
@@ -3120,28 +3116,107 @@
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>23.51</t>
+          <t>70.10</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr"/>
       <c r="O34" s="2" t="inlineStr">
         <is>
+          <t>20.06.2026 16:19 — 11.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Кржижановского, д 16 к 3</t>
+        </is>
+      </c>
+      <c r="Q34" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/prodazha-nelikvidnykh-tmts-tarelki-dlia-filtra-prokladki-dvigatel/tender-4496006/#btid=2&amp;sqh=0a65cd04d994a200988cac92f51cd6de345d7a6e&amp;tsid=4496006003</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06 14:11</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr"/>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>4129930</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Реализация материалов для ремонта (напольные покрытия, настенные покрытия, окна, двери и т.д.) с АО "Мальцовский портландцемент"Блокдверной балконныйБлокдверной филенчатый ДГ 21х9Блококонный 1500х1000 ммБлококонный 1770х1700 мм Желоб ...  Docke Рама оконная 3000х1200 мм Решеткавентиляционнаянаружная Ручка оконная ГОСТ 5087-80 ...</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЦЕМРОС"</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЦЕМРОС"</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>7708117908</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Шматов Вячеслав Вячеславович</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>23.51</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr"/>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
           <t>06.08.2025 14:33 — 07.08.2026 12:00</t>
         </is>
       </c>
-      <c r="P34" s="2" t="inlineStr">
+      <c r="P35" s="2" t="inlineStr">
         <is>
           <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
         </is>
       </c>
-      <c r="Q34" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=7474cc1ab5d66183b3313194fdc6aeb61602c1ed&amp;tsid=4129930003</t>
+      <c r="Q35" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=0a65cd04d994a200988cac92f51cd6de345d7a6e&amp;tsid=4129930003</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q34"/>
+  <autoFilter ref="A1:Q35"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -3176,6 +3251,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId34"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-06 22:48 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q35"/>
+  <dimension ref="A1:Q37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -622,14 +622,14 @@
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=163f8e2e4073535c88d27b469a95f347fe7e1861&amp;tsid=4510835003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=3972e93777eef3c496200683293d516c6b95b872&amp;tsid=4510835003</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -698,14 +698,14 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=163f8e2e4073535c88d27b469a95f347fe7e1861&amp;tsid=4503612458</t>
+          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=3972e93777eef3c496200683293d516c6b95b872&amp;tsid=4503612458</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -777,14 +777,14 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=163f8e2e4073535c88d27b469a95f347fe7e1861&amp;tsid=4130106003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=3972e93777eef3c496200683293d516c6b95b872&amp;tsid=4130106003</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -856,14 +856,14 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=8385288804917d040873ddced03bfd0eeb4f87dc&amp;tsid=4498936003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=a3f17bdc1b84dc77e6d415f5a4dae78e2e6e3295&amp;tsid=4498936003</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -936,14 +936,14 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=420ff314b316ade50f5d54007d807032f9dc870c&amp;tsid=4497016004</t>
+          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=a8cd893161e0f9a84fd68238c104b56d73861858&amp;tsid=4497016004</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1011,14 +1011,14 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=e420765976372a60db8c86bf4e365bab65129250&amp;tsid=4512196458</t>
+          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=2c2dc9a5c7e2769edb077c6980aaf039341552d8&amp;tsid=4512196458</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1090,14 +1090,14 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=e420765976372a60db8c86bf4e365bab65129250&amp;tsid=4512292004</t>
+          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=2c2dc9a5c7e2769edb077c6980aaf039341552d8&amp;tsid=4512292004</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1172,14 +1172,14 @@
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=a44b2cde27516c18754a7005c4c8d5029a4da23c&amp;tsid=4475879003</t>
+          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=84b3fc74822d1b6423791ca20f93740cc324eacf&amp;tsid=4475879003</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1251,14 +1251,14 @@
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=9d5f90707b26c8e10458f99e604d4a7872f3c2f0&amp;tsid=4508331004</t>
+          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=cf639e1efd36c817f2b51c49ee96bb146f873e48&amp;tsid=4508331004</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1326,14 +1326,14 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-plity-pdn-3-1-5/tender-4514583/#btid=2&amp;sqh=a9fae5a70d5ab8c93ccf2ffc068c750b655b544a&amp;tsid=4514583458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-plity-pdn-3-1-5/tender-4514583/#btid=2&amp;sqh=3b472204201f001370372e672ecb96d2c0e73c78&amp;tsid=4514583458</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1401,14 +1401,14 @@
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-bloki-fbs/tender-4513278/#btid=2&amp;sqh=f9fe44f277b7f45996a1a6d0bc25f78fee0fe018&amp;tsid=4513278458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-bloki-fbs/tender-4513278/#btid=2&amp;sqh=151673791dd86b46cd73cea65ff7694df2446a4f&amp;tsid=4513278458</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1480,14 +1480,14 @@
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/12-kh-1-zakliuchenie-dogovora-na-postavku-materialov-dlia-naruzhnykh-setei/tender-4514839/#btid=2&amp;sqh=f9fe44f277b7f45996a1a6d0bc25f78fee0fe018&amp;tsid=4514839004</t>
+          <t>https://www.b2b-center.ru/market/12-kh-1-zakliuchenie-dogovora-na-postavku-materialov-dlia-naruzhnykh-setei/tender-4514839/#btid=2&amp;sqh=151673791dd86b46cd73cea65ff7694df2446a4f&amp;tsid=4514839004</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1559,14 +1559,14 @@
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=f9fe44f277b7f45996a1a6d0bc25f78fee0fe018&amp;tsid=4510341459</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=151673791dd86b46cd73cea65ff7694df2446a4f&amp;tsid=4510341459</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1634,14 +1634,14 @@
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=f9fe44f277b7f45996a1a6d0bc25f78fee0fe018&amp;tsid=4508347458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=151673791dd86b46cd73cea65ff7694df2446a4f&amp;tsid=4508347458</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1713,14 +1713,14 @@
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=f9fe44f277b7f45996a1a6d0bc25f78fee0fe018&amp;tsid=4489772003</t>
+          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=151673791dd86b46cd73cea65ff7694df2446a4f&amp;tsid=4489772003</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1792,14 +1792,14 @@
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=f9fe44f277b7f45996a1a6d0bc25f78fee0fe018&amp;tsid=4474790003</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=151673791dd86b46cd73cea65ff7694df2446a4f&amp;tsid=4474790003</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1871,14 +1871,14 @@
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=f9fe44f277b7f45996a1a6d0bc25f78fee0fe018&amp;tsid=4180328003</t>
+          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=151673791dd86b46cd73cea65ff7694df2446a4f&amp;tsid=4180328003</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1950,14 +1950,14 @@
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=f9fe44f277b7f45996a1a6d0bc25f78fee0fe018&amp;tsid=3973258003</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=151673791dd86b46cd73cea65ff7694df2446a4f&amp;tsid=3973258003</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1973,12 +1973,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>4512260</t>
+          <t>4513525</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>ТМЦ. Срочный отбор предложений на право заключения договора поставкижелезобетонных изделийдля нужд филиала «Канская теплосеть» АО «Енисейская ТГК (ТГК-13)».</t>
+          <t>Поставка модульных защитных сооруженийЗДАНИЕ ЗАЩИТНОЕ ДЛЯ УКРЫТИЯ 4,4*2,4*2,2МЖЕЛЕЗОБЕТОННОЕСБОРНОЕ</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2015,7 +2015,7 @@
       <c r="N20" s="2" t="inlineStr"/>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 11:52 — 08.07.2026 12:00</t>
+          <t>06.07.2026 08:36 — 10.07.2026 14:00</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2025,14 +2025,14 @@
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/tmts-srochnyi-otbor-predlozhenii-na-pravo-zakliucheniia-dogovora-postavki/tender-4512260/#btid=2&amp;sqh=033ee602578d21ec9b4af0bff23cd79861d9d3fc&amp;tsid=4512260458</t>
+          <t>https://www.b2b-center.ru/app/market-next/postavka-modulnykh-zashchitnykh-sooruzhenii/tender-4513525/#btid=2&amp;sqh=4ef150eb83696b854ab192649a455db804155e2c&amp;tsid=4513525458</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -2048,35 +2048,43 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>4509622</t>
+          <t>4513563</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Производство вторичного щебня из ломажелезобетонных изделий</t>
+          <t>Блок ФБС 12.4.6-Т-и
+Кольцо стеновое КС 20.9 ГОСТ 8020-2016
+на К-ПМ
+Блок ФБС 12.4.6-Т-и типовой проект 709-9-126.93 альбом 3 кжи-14.00
+Кольцо стеновое КС 20.9 ГОСТ 8020-20164513563 ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "ТОРГОВЫЙ ДОМ ПОЛИМЕТАЛЛ"Железобетонные изделия</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>7805368914</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr"/>
+          <t>г Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
+        </is>
+      </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -2084,30 +2092,30 @@
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>46.90</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr"/>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>01.07.2026 16:05 — 10.07.2026 12:00</t>
+          <t>06.07.2026 08:49 — 10.07.2026 12:00</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/proizvodstvo-vtorichnogo-shchebnia-iz-loma-zhelezobetonnykh-izdelii/tender-4509622/#btid=2&amp;sqh=033ee602578d21ec9b4af0bff23cd79861d9d3fc&amp;tsid=4509622458</t>
+          <t>https://www.b2b-center.ru/market/blok-fbs-12-4-6-t-i-koltso-stenovoe-ks-20-9-gost-8020-2016-na-k-pm/tender-4513563/#btid=2&amp;sqh=4ef150eb83696b854ab192649a455db804155e2c&amp;tsid=4513563004</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2123,10 +2131,165 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
+          <t>4512260</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>ТМЦ. Срочный отбор предложений на право заключения договора поставкижелезобетонных изделийдля нужд филиала «Канская теплосеть» АО «Енисейская ТГК (ТГК-13)».</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>03.07.2026 11:52 — 08.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/tmts-srochnyi-otbor-predlozhenii-na-pravo-zakliucheniia-dogovora-postavki/tender-4512260/#btid=2&amp;sqh=4ef150eb83696b854ab192649a455db804155e2c&amp;tsid=4512260458</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06 22:48</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr"/>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>4512082</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Оголовок с платформенным опиранием 4ОСП 32-3 серия 1.111.1-4 в. 2 для ООО "Сахавольфрам"
+Оголовок с платформенным опиранием 4ОСП 32-3 серия 1.111.1-4 в. 2 для ООО "Сахавольфрам"4512082 ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "ТОРГОВЫЙ ДОМ ПОЛИМЕТАЛЛ"Железобетонные изделия</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>7805368914</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>46.90</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr"/>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>03.07.2026 11:05 — 08.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
+        </is>
+      </c>
+      <c r="Q23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/ogolovok-s-platformennym-opiraniem-4osp-32-3-seriia-1-111-1-4-v-2-dlia/tender-4512082/#btid=2&amp;sqh=4ef150eb83696b854ab192649a455db804155e2c&amp;tsid=4512082004</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06 22:48</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
           <t>4511621</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Закупка аккумуляторных батарей (залитых) для нужд АО "Павловск Неруд" с поставкой в Августе 2026г.
 Обязательная расценка стоимости доставки, возможен забор груза на условиях самовывоза.
@@ -2135,216 +2298,62 @@
 Заказчик АО "Павловск Неруд" предприятие АО "Национальная нерудная компания"Аккумулятор ТН-550Перемычкам/ц для АКБ 115,5мм ТН-550Перемычкам/ц для АКБ 212,0мм ТН-550 Транспортная услуга</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>АО "ННК"</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>АО "ННК-ОЙЛ"</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>5032049030</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr">
+      <c r="K24" s="2" t="inlineStr">
         <is>
           <t>Худайнатов Эдуард Юрьевич</t>
         </is>
       </c>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="inlineStr">
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>70.22</t>
-        </is>
-      </c>
-      <c r="N22" s="2" t="inlineStr"/>
-      <c r="O22" s="2" t="inlineStr">
-        <is>
-          <t>03.07.2026 06:22 — 07.07.2026 11:00</t>
-        </is>
-      </c>
-      <c r="P22" s="2" t="inlineStr">
-        <is>
-          <t>г Москва, ул 1-я Тверская-Ямская, д 5, помещ 1012</t>
-        </is>
-      </c>
-      <c r="Q22" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=45dbd0fd67b523c4ca37137dd4b00bb065e06d78&amp;tsid=4511621004</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 14:11</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr"/>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>4511787</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>ЗЧ к автотранспорту... /66 ТЕРМОСТАТ ТС-107-1306100-06ПЕРЕМЫЧКААКБ КЛЕММА-КЛЕММА ПП 500-50 ...</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>9725042029</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr"/>
-      <c r="L23" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M23" s="2" t="inlineStr">
-        <is>
-          <t>64.20</t>
-        </is>
-      </c>
-      <c r="N23" s="2" t="inlineStr"/>
-      <c r="O23" s="2" t="inlineStr">
-        <is>
-          <t>03.07.2026 08:32 — 08.07.2026 00:00</t>
-        </is>
-      </c>
-      <c r="P23" s="2" t="inlineStr">
-        <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
-        </is>
-      </c>
-      <c r="Q23" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=45dbd0fd67b523c4ca37137dd4b00bb065e06d78&amp;tsid=4511787458</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 14:11</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>4512541</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>Запасные части CAT.... -3748 Cat Опора 348-9537 CatПеремычка140-0860 Cat Скоба 8X-3130 ...</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>1004001744</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>Респ Карелия</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "СЕВЕРСТАЛЬ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="inlineStr">
-        <is>
-          <t>07.10.2</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr"/>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 14:07 — 10.07.2026 11:00</t>
+          <t>03.07.2026 06:22 — 07.07.2026 11:00</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>Респ Карелия, г Костомукша, шоссе Горняков, стр 284</t>
+          <t>г Москва, ул 1-я Тверская-Ямская, д 5, помещ 1012</t>
         </is>
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=45dbd0fd67b523c4ca37137dd4b00bb065e06d78&amp;tsid=4512541003</t>
+          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=8f2b34eb3bfa17574b43f4dfd1edd9879569d029&amp;tsid=4511621004</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -2360,309 +2369,305 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
+          <t>4511787</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>ЗЧ к автотранспорту... /66 ТЕРМОСТАТ ТС-107-1306100-06ПЕРЕМЫЧКААКБ КЛЕММА-КЛЕММА ПП 500-50 ...</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr"/>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>03.07.2026 08:32 — 08.07.2026 00:00</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q25" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=8f2b34eb3bfa17574b43f4dfd1edd9879569d029&amp;tsid=4511787458</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06 22:48</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>4512541</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Запасные части CAT.... -3748 Cat Опора 348-9537 CatПеремычка140-0860 Cat Скоба 8X-3130 ...</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>1004001744</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Респ Карелия</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "СЕВЕРСТАЛЬ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>07.10.2</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>03.07.2026 14:07 — 10.07.2026 11:00</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>Респ Карелия, г Костомукша, шоссе Горняков, стр 284</t>
+        </is>
+      </c>
+      <c r="Q26" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=8f2b34eb3bfa17574b43f4dfd1edd9879569d029&amp;tsid=4512541003</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06 22:48</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr"/>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
           <t>4508230</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>Сборный (Изделия электроустановочные и монтажные, Ящики, щиты, шкафы, пункты и комплектующие к ним, Приборы электроизмерительные, реле)
 МГ-019742, МГ-019713, МГ-019696, МГ-019665, МГ-019621, МГ-019620, МГ-019619, МГ-017109... -HESI-EX (5X20), Phoenix Contact 1277638ПеремычкаFBS 10-5, Phoenix Contact 3030213 ...ПеремычкаFBS 10-5 BU, Phoenix Contact  ...</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>АО "ИК "АРЛАН"</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>АО "ИК "АРЛАН"</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>7722220390</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
+      <c r="J27" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K25" s="2" t="inlineStr">
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>Барилов Евгений Александрович</t>
         </is>
       </c>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M25" s="2" t="inlineStr">
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
         <is>
           <t>82.99</t>
         </is>
       </c>
-      <c r="N25" s="2" t="inlineStr"/>
-      <c r="O25" s="2" t="inlineStr">
+      <c r="N27" s="2" t="inlineStr"/>
+      <c r="O27" s="2" t="inlineStr">
         <is>
           <t>30.06.2026 17:59 — 09.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P25" s="2" t="inlineStr">
+      <c r="P27" s="2" t="inlineStr">
         <is>
           <t>г Москва, Романов пер, д 4</t>
         </is>
       </c>
-      <c r="Q25" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=45dbd0fd67b523c4ca37137dd4b00bb065e06d78&amp;tsid=4508230004</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 14:11</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="Q27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=8f2b34eb3bfa17574b43f4dfd1edd9879569d029&amp;tsid=4508230004</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06 22:48</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>4504775</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники
 Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники...  Трубка пробная № 37-542-000 Соединитель-перемычка04182454 Кольцо стальное №CP48001-0305 Фильтр ...</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>7805368914</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="J28" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr">
+      <c r="K28" s="2" t="inlineStr">
         <is>
           <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="inlineStr">
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
         <is>
           <t>46.90</t>
-        </is>
-      </c>
-      <c r="N26" s="2" t="inlineStr"/>
-      <c r="O26" s="2" t="inlineStr">
-        <is>
-          <t>27.06.2026 01:36 — 15.07.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P26" s="2" t="inlineStr">
-        <is>
-          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
-        </is>
-      </c>
-      <c r="Q26" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=45dbd0fd67b523c4ca37137dd4b00bb065e06d78&amp;tsid=4504775003</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 14:11</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr"/>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>4501157</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>Источники электропитания (ИБП, аккумуляторные батареи, блоки питания)...  х 1248 А·ч, включая соединительныеперемычки. Вид положительного электрода - трубчатая пластина ...  с коммутирующей арматурой, межэлементными и межряднымиперемычками, крепежами, комплектом для обслуживания АБ. Тип ...</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>АО "Мосинжпроект"</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>АО "МОСИНЖПРОЕКТ"</t>
-        </is>
-      </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>7701885820</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>Сорокин Антон Павлович</t>
-        </is>
-      </c>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M27" s="2" t="inlineStr">
-        <is>
-          <t>71.12.2</t>
-        </is>
-      </c>
-      <c r="N27" s="2" t="inlineStr"/>
-      <c r="O27" s="2" t="inlineStr">
-        <is>
-          <t>24.06.2026 15:40 — 22.07.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P27" s="2" t="inlineStr">
-        <is>
-          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
-        </is>
-      </c>
-      <c r="Q27" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=45dbd0fd67b523c4ca37137dd4b00bb065e06d78&amp;tsid=4501157003</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 14:11</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>4499964</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>Автоматика и телемеханика движения поездов... , 13552-00-00В Дроссель-трансформатор (безперемычек) ДТМ-0,17-1000М ЮКЛЯ.672 ...</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>АО "Мосинжпроект"</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>АО "МОСИНЖПРОЕКТ"</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>7701885820</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>Сорокин Антон Павлович</t>
-        </is>
-      </c>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M28" s="2" t="inlineStr">
-        <is>
-          <t>71.12.2</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr"/>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 08:46 — 15.07.2026 12:00</t>
+          <t>27.06.2026 01:36 — 15.07.2026 12:00</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
       <c r="Q28" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=45dbd0fd67b523c4ca37137dd4b00bb065e06d78&amp;tsid=4499964003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=8f2b34eb3bfa17574b43f4dfd1edd9879569d029&amp;tsid=4504775003</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -2678,229 +2683,229 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
+          <t>4501157</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Источники электропитания (ИБП, аккумуляторные батареи, блоки питания)...  х 1248 А·ч, включая соединительныеперемычки. Вид положительного электрода - трубчатая пластина ...  с коммутирующей арматурой, межэлементными и межряднымиперемычками, крепежами, комплектом для обслуживания АБ. Тип ...</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>АО "Мосинжпроект"</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>7701885820</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Сорокин Антон Павлович</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>71.12.2</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr"/>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>24.06.2026 15:40 — 22.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+        </is>
+      </c>
+      <c r="Q29" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=8f2b34eb3bfa17574b43f4dfd1edd9879569d029&amp;tsid=4501157003</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06 22:48</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>4499964</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Автоматика и телемеханика движения поездов... , 13552-00-00В Дроссель-трансформатор (безперемычек) ДТМ-0,17-1000М ЮКЛЯ.672 ...</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>АО "Мосинжпроект"</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>7701885820</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Сорокин Антон Павлович</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>71.12.2</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr"/>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>24.06.2026 08:46 — 15.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+        </is>
+      </c>
+      <c r="Q30" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=8f2b34eb3bfa17574b43f4dfd1edd9879569d029&amp;tsid=4499964003</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06 22:48</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr"/>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
           <t>4480614</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>Плановое и аварийное техническое обслуживание зданий и сооружений (годовое обслуживание август 2026 - август 2027) ГК Логика молока, производственная площадка в г. Ялуторовске
 Обслуживание зданий и сооружений завода в г. Ялуторовске....  стен из газобетонных блоков Устройство металлическихперемычекс устройством штраб Усиление кирпичных стен ...</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>АО "ЭЙЧ ЭНД ЭН"</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>АО "ЭЙЧ ЭНД ЭН"</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>7714626332</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr">
+      <c r="J31" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K29" s="2" t="inlineStr">
+      <c r="K31" s="2" t="inlineStr">
         <is>
           <t>Закриев Якуб Салманович</t>
         </is>
       </c>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M29" s="2" t="inlineStr">
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
         <is>
           <t>10.51.9</t>
-        </is>
-      </c>
-      <c r="N29" s="2" t="inlineStr"/>
-      <c r="O29" s="2" t="inlineStr">
-        <is>
-          <t>08.06.2026 14:44 — 08.07.2026 23:00</t>
-        </is>
-      </c>
-      <c r="P29" s="2" t="inlineStr">
-        <is>
-          <t>г Москва, ул Вятская, д 27 стр 13</t>
-        </is>
-      </c>
-      <c r="Q29" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/planovoe-i-avariinoe-tekhnicheskoe-obsluzhivanie-zdanii-i-sooruzhenii/tender-4480614/#btid=2&amp;sqh=45dbd0fd67b523c4ca37137dd4b00bb065e06d78&amp;tsid=4480614004</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 14:11</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>4512370</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>ТО Сплит систем Лабинск Эйч энд Эн... кондиционирования Техническое обслуживание внутреннегоблокакассетного типа мультизональной  ...блокакондиционера. Мойка теплообменника внутреннегоблокакондиционера Чистка фильтров внутреннегоблокакондиционера Чистка фильтров приточнойвентиляционной...</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>АО "ЭЙЧ ЭНД ЭН"</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>АО "ЭЙЧ ЭНД ЭН"</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>7714626332</t>
-        </is>
-      </c>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>Закриев Якуб Салманович</t>
-        </is>
-      </c>
-      <c r="L30" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M30" s="2" t="inlineStr">
-        <is>
-          <t>10.51.9</t>
-        </is>
-      </c>
-      <c r="N30" s="2" t="inlineStr"/>
-      <c r="O30" s="2" t="inlineStr">
-        <is>
-          <t>03.07.2026 12:40 — 14.07.2026 18:30</t>
-        </is>
-      </c>
-      <c r="P30" s="2" t="inlineStr">
-        <is>
-          <t>г Москва, ул Вятская, д 27 стр 13</t>
-        </is>
-      </c>
-      <c r="Q30" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=0a65cd04d994a200988cac92f51cd6de345d7a6e&amp;tsid=4512370458</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 14:11</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr"/>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>4501181</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>Вентиляторы промышленные и оборудование общеобменной вентиляции...  5Ф РешёткавентиляционнаяАМР 600х300М РешёткавентиляционнаяАМР 150х150М РешёткавентиляционнаяАМР 300х200М  ... мм.; масса 0,65 кгБлокконтроля сопротивления БСК-3.1 Канальный ...  533Па, габаритные размеры 700х467х2230 мм,блоков/моноблоков 5/1, в составе: - ...</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>АО "Мосинжпроект"</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>АО "МОСИНЖПРОЕКТ"</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>7701885820</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>Сорокин Антон Павлович</t>
-        </is>
-      </c>
-      <c r="L31" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M31" s="2" t="inlineStr">
-        <is>
-          <t>71.12.2</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr"/>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 15:45 — 22.07.2026 12:00</t>
+          <t>08.06.2026 14:44 — 08.07.2026 23:00</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+          <t>г Москва, ул Вятская, д 27 стр 13</t>
         </is>
       </c>
       <c r="Q31" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=0a65cd04d994a200988cac92f51cd6de345d7a6e&amp;tsid=4501181003</t>
+          <t>https://www.b2b-center.ru/market/planovoe-i-avariinoe-tekhnicheskoe-obsluzhivanie-zdanii-i-sooruzhenii/tender-4480614/#btid=2&amp;sqh=8f2b34eb3bfa17574b43f4dfd1edd9879569d029&amp;tsid=4480614004</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 14:11</t>
+          <t>2026-07-06 22:48</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -2916,307 +2921,465 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
+          <t>4512370</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>ТО Сплит систем Лабинск Эйч энд Эн... кондиционирования Техническое обслуживание внутреннегоблокакассетного типа мультизональной  ...блокакондиционера. Мойка теплообменника внутреннегоблокакондиционера Чистка фильтров внутреннегоблокакондиционера Чистка фильтров приточнойвентиляционной...</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЭЙЧ ЭНД ЭН"</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЭЙЧ ЭНД ЭН"</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>7714626332</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Закриев Якуб Салманович</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>10.51.9</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr"/>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>03.07.2026 12:40 — 14.07.2026 18:30</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Вятская, д 27 стр 13</t>
+        </is>
+      </c>
+      <c r="Q32" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=48fb12302dd23d97fd728136e7c312e5ed2dcf94&amp;tsid=4512370458</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06 22:48</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr"/>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>4501181</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Вентиляторы промышленные и оборудование общеобменной вентиляции...  5Ф РешёткавентиляционнаяАМР 600х300М РешёткавентиляционнаяАМР 150х150М РешёткавентиляционнаяАМР 300х200М  ... мм.; масса 0,65 кгБлокконтроля сопротивления БСК-3.1 Канальный ...  533Па, габаритные размеры 700х467х2230 мм,блоков/моноблоков 5/1, в составе: - ...</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>АО "Мосинжпроект"</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>7701885820</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Сорокин Антон Павлович</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>71.12.2</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr"/>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>24.06.2026 15:45 — 22.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+        </is>
+      </c>
+      <c r="Q33" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=48fb12302dd23d97fd728136e7c312e5ed2dcf94&amp;tsid=4501181003</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06 22:48</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
           <t>4501483</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ
 Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ...  d 50x2", внутренняя резьба RTPБлокуправления наружной установки ICEFREE TR-16 ...  Оповещатель звуковой МАЯК-12-ЗМБлокуправления наружной установки ICEFREE TS- ... проводов КС-3 007004 Велос Переходвентиляционный150х100 - D150, из тонколистовой оцинкованной ...</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>7805368914</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr">
+      <c r="J34" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург</t>
         </is>
       </c>
-      <c r="K32" s="2" t="inlineStr">
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
-      <c r="L32" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M32" s="2" t="inlineStr">
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
         <is>
           <t>46.90</t>
         </is>
       </c>
-      <c r="N32" s="2" t="inlineStr"/>
-      <c r="O32" s="2" t="inlineStr">
+      <c r="N34" s="2" t="inlineStr"/>
+      <c r="O34" s="2" t="inlineStr">
         <is>
           <t>25.06.2026 05:03 — 09.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P32" s="2" t="inlineStr">
+      <c r="P34" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
-      <c r="Q32" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=0a65cd04d994a200988cac92f51cd6de345d7a6e&amp;tsid=4501483003</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 14:11</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr"/>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="Q34" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=48fb12302dd23d97fd728136e7c312e5ed2dcf94&amp;tsid=4501483003</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06 22:48</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr"/>
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>4500120</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>Коммуникационное оборудование, компьютеры, комплектующие к ним, серверное оборудование и ПО...  и кабелей – 1 компл. Удаленныйблок(репитер) BSF414 , питание 220В,  ... 2х2 Комбайнер специализированный OMU Side (блок1) OMUSC1 Комбайнер специализированный OMU ... контроллер для мониторинга в FlexGain View,вентиляционнаяпанель с фильтрами, комплект кабелей, ...</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>АО "Мосинжпроект"</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>АО "МОСИНЖПРОЕКТ"</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr">
+      <c r="I35" s="2" t="inlineStr">
         <is>
           <t>7701885820</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr">
+      <c r="J35" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K33" s="2" t="inlineStr">
+      <c r="K35" s="2" t="inlineStr">
         <is>
           <t>Сорокин Антон Павлович</t>
         </is>
       </c>
-      <c r="L33" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M33" s="2" t="inlineStr">
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
         <is>
           <t>71.12.2</t>
         </is>
       </c>
-      <c r="N33" s="2" t="inlineStr"/>
-      <c r="O33" s="2" t="inlineStr">
+      <c r="N35" s="2" t="inlineStr"/>
+      <c r="O35" s="2" t="inlineStr">
         <is>
           <t>24.06.2026 09:48 — 15.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P33" s="2" t="inlineStr">
+      <c r="P35" s="2" t="inlineStr">
         <is>
           <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
         </is>
       </c>
-      <c r="Q33" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=0a65cd04d994a200988cac92f51cd6de345d7a6e&amp;tsid=4500120003</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 14:11</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="Q35" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=48fb12302dd23d97fd728136e7c312e5ed2dcf94&amp;tsid=4500120003</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06 22:48</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>4496006</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп
 Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп... -316 ***Петля крепежная стальная ***Платаблокауправления ZC5 CAME ***Средство чистящее " ... /распылитель для чаши Генуя ***РешеткавентиляционнаяРВ-1 225Х225 ***Петля анкерная 0 ... мл ***Папка с зажимом ***РешеткавентиляционнаяРВ-1 325Х125 ***Папка на кольцах ...</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>ООО "СИБУР"</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>ООО "СИБУР"</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr">
+      <c r="I36" s="2" t="inlineStr">
         <is>
           <t>7727576505</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr">
+      <c r="J36" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K34" s="2" t="inlineStr">
+      <c r="K36" s="2" t="inlineStr">
         <is>
           <t>Карисалов Михаил Юрьевич</t>
         </is>
       </c>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M34" s="2" t="inlineStr">
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
         <is>
           <t>70.10</t>
         </is>
       </c>
-      <c r="N34" s="2" t="inlineStr"/>
-      <c r="O34" s="2" t="inlineStr">
+      <c r="N36" s="2" t="inlineStr"/>
+      <c r="O36" s="2" t="inlineStr">
         <is>
           <t>20.06.2026 16:19 — 11.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P34" s="2" t="inlineStr">
+      <c r="P36" s="2" t="inlineStr">
         <is>
           <t>г Москва, ул Кржижановского, д 16 к 3</t>
         </is>
       </c>
-      <c r="Q34" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nelikvidnykh-tmts-tarelki-dlia-filtra-prokladki-dvigatel/tender-4496006/#btid=2&amp;sqh=0a65cd04d994a200988cac92f51cd6de345d7a6e&amp;tsid=4496006003</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 14:11</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr"/>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="Q36" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/prodazha-nelikvidnykh-tmts-tarelki-dlia-filtra-prokladki-dvigatel/tender-4496006/#btid=2&amp;sqh=48fb12302dd23d97fd728136e7c312e5ed2dcf94&amp;tsid=4496006003</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06 22:48</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr"/>
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>Работы</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>4129930</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>Реализация материалов для ремонта (напольные покрытия, настенные покрытия, окна, двери и т.д.) с АО "Мальцовский портландцемент"Блокдверной балконныйБлокдверной филенчатый ДГ 21х9Блококонный 1500х1000 ммБлококонный 1770х1700 мм Желоб ...  Docke Рама оконная 3000х1200 мм Решеткавентиляционнаянаружная Ручка оконная ГОСТ 5087-80 ...</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr">
+      <c r="I37" s="2" t="inlineStr">
         <is>
           <t>7708117908</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr">
+      <c r="J37" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K35" s="2" t="inlineStr">
+      <c r="K37" s="2" t="inlineStr">
         <is>
           <t>Шматов Вячеслав Вячеславович</t>
         </is>
       </c>
-      <c r="L35" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M35" s="2" t="inlineStr">
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
         <is>
           <t>23.51</t>
         </is>
       </c>
-      <c r="N35" s="2" t="inlineStr"/>
-      <c r="O35" s="2" t="inlineStr">
+      <c r="N37" s="2" t="inlineStr"/>
+      <c r="O37" s="2" t="inlineStr">
         <is>
           <t>06.08.2025 14:33 — 07.08.2026 12:00</t>
         </is>
       </c>
-      <c r="P35" s="2" t="inlineStr">
+      <c r="P37" s="2" t="inlineStr">
         <is>
           <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
         </is>
       </c>
-      <c r="Q35" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=0a65cd04d994a200988cac92f51cd6de345d7a6e&amp;tsid=4129930003</t>
+      <c r="Q37" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=48fb12302dd23d97fd728136e7c312e5ed2dcf94&amp;tsid=4129930003</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q35"/>
+  <autoFilter ref="A1:Q37"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -3252,6 +3415,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId36"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-07 11:28 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q37"/>
+  <dimension ref="A1:Q40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 22:48</t>
+          <t>2026-07-07 11:28</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -560,310 +560,311 @@
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>4515159</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Строительные материалы (поставка в Находку/Для ООО Светлое) поставка в срок до 10.09.2026
+Строительные материалы... -021 серый Краска ПФ-115 белаяПлита дорожнаяпостоянная железобетонная 1ПДН-14 6000х2000х140 мм ...</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>7805368914</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>46.90</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>07.07.2026 05:38 — 13.07.2026 10:00</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/stroitelnye-materialy-postavka-v-nakhodku-dlia-ooo-svetloe-postavka/tender-4515159/#btid=2&amp;sqh=4fab989164db7b10ecec829f6897bdac08350c55&amp;tsid=4515159004</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>4510835</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Реализация. Невостребованные складские остатки (не б/у). Запасные части для ГТО (для автосамосвалов, автобусов, легкового транспорта, бульдозеров, экскаваторов, грейдеров)
 Реализация. Запасные части для автосамосвалов HOWO, БЕЛАЗ, КАМАЗ, SCANIA; бульдозеров Cat 834, D9R, DT10T, KOMATSU WD600, PR754, Т-25; грейдера САТ140М; экскаваторов Bucyrus RH120E, Hyundai R520LC, ЭО, ЭШ, ЭКГ, ЕК-400, Liebherr R984C....  2445 V-ACS 32-R1195-9Дорожныйзнак "Осторожно газопровод" ДПТ-М  ... КАТУШКА электромагнитная 1317540-74030 Керамогранитплита300х600мм Керамогранитплита600х600мм Килоамперметр М42301 1, ... 90/460 У2Плита75570-8608180Плитаднища 1080.52.101Плиталотков ПТ  ...</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>ООО "УК "СИБАНТРАЦИТ"</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>ООО "УК "СИБАНТРАЦИТ"</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>9703160290</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Мельников Сергей Владимирович</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>70.22</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>02.07.2026 13:09 — 16.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>г Москва, ул Усачёва, д 2 стр 1, помещ 2/1</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=3972e93777eef3c496200683293d516c6b95b872&amp;tsid=4510835003</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 22:48</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=4fab989164db7b10ecec829f6897bdac08350c55&amp;tsid=4510835003</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>4506366</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Ремонтдорожнойплитки на подъездной и выездной дороге от главного входа гостиницы</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЛОТТЕ РУС"</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЛОТТЕ РУС"</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>7704169180</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Андерсен Мортен Бундгорд</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>55.10</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>29.06.2026 16:30 — 09.07.2026 17:18</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Новинский б-р, д 8 стр 2</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/remont-dorozhnoi-plitki-na-pod-ezdnoi-i-vyezdnoi-doroge-ot-glavnogo/tender-4506366/#btid=2&amp;sqh=4fab989164db7b10ecec829f6897bdac08350c55&amp;tsid=4506366458</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Поставка</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>4503612</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>RUNEV-11652 на выполнение работ по сортировке, разделке и вывозу демонтированных 
 трубопроводов и металлоконструкций на склад хранения. Вывозу строительного мусора на утилизацию с площадки Б-9 АО «Невинномысский Азот»....  площадки 600м² для выполнения работ, издорожных плит(60 шт, поставка заказчика), с выравниванием ...</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>9725042029</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>64.20</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr"/>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>26.06.2026 10:29 — 08.07.2026 17:00</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
-        </is>
-      </c>
-      <c r="Q3" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=3972e93777eef3c496200683293d516c6b95b872&amp;tsid=4503612458</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 22:48</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>4130106</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Реализация ЖБИ изделий с АО "Мальцовский портландцемент"Бордюрдорожный1000х300х150мм Ясногорский завод строительных материалов Кольца  ...  КС-7-3 ЖБИ 24/7Плитаопорная ОП-1К ПС-334-08 ...Плитаперекрытия колодца 1ПП-20-2 D2200  ...</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>АО "ЦЕМРОС"</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>АО "ЦЕМРОС"</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>7708117908</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>Шматов Вячеслав Вячеславович</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>23.51</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr"/>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>06.08.2025 15:30 — 07.08.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P4" s="2" t="inlineStr">
-        <is>
-          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
-        </is>
-      </c>
-      <c r="Q4" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=3972e93777eef3c496200683293d516c6b95b872&amp;tsid=4130106003</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 22:48</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>4498936</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Продажа невостребованных ТМЦ -Плиты аэродромные, Фильтр сетчатый МИГ, Ролик лебедки Материалы с хранения. Перечень ориентировочный, может измениться в меньшую сторону за счет возможной востребованности.</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>ООО "СИБУР"</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>ООО "СИБУР"</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>7727576505</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>Карисалов Михаил Юрьевич</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>70.10</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr"/>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>23.06.2026 13:41 — 07.07.2026 12:00</t>
+          <t>26.06.2026 10:29 — 08.07.2026 17:00</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Кржижановского, д 16 к 3</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=a3f17bdc1b84dc77e6d415f5a4dae78e2e6e3295&amp;tsid=4498936003</t>
+          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=4fab989164db7b10ecec829f6897bdac08350c55&amp;tsid=4503612458</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 22:48</t>
+          <t>2026-07-07 11:28</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -874,230 +875,234 @@
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>4130106</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Реализация ЖБИ изделий с АО "Мальцовский портландцемент"Бордюрдорожный1000х300х150мм Ясногорский завод строительных материалов Кольца  ...  КС-7-3 ЖБИ 24/7Плитаопорная ОП-1К ПС-334-08 ...Плитаперекрытия колодца 1ПП-20-2 D2200  ...</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЦЕМРОС"</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЦЕМРОС"</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>7708117908</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Шматов Вячеслав Вячеславович</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>23.51</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr"/>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>06.08.2025 15:30 — 07.08.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
+        </is>
+      </c>
+      <c r="Q6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=4fab989164db7b10ecec829f6897bdac08350c55&amp;tsid=4130106003</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>4498936</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Продажа невостребованных ТМЦ -Плиты аэродромные, Фильтр сетчатый МИГ, Ролик лебедки Материалы с хранения. Перечень ориентировочный, может измениться в меньшую сторону за счет возможной востребованности.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СИБУР"</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СИБУР"</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>7727576505</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Карисалов Михаил Юрьевич</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>70.10</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr"/>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>23.06.2026 13:41 — 14.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Кржижановского, д 16 к 3</t>
+        </is>
+      </c>
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=10aaad04274a74c975e4784773a70ef40b0bcff6&amp;tsid=4498936003</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
           <t>Работы</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>4497016</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>BOX_00514 Выполнение работ по строительству общежития №4 на 80 койко-мест временного вахтового поселка на месторождении «Бараньевское»
 Выполнение работ по строительству общежития №4 на 80 койко-мест временного вахтового поселка АО «Камчатское золото», на месторождении «Бараньевское»ЛОТ №1: Монтаж фундамента (висячиезабивные сваииз стальных труб 219×5 мм)  ...</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>ООО «Фокси-Бокс»</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>ООО "ФОКСИ-БОКС"</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>7805780074</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Василенко Иван Михайлович</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>46.73</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr"/>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>22.06.2026 16:20 — 09.07.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P6" s="2" t="inlineStr">
-        <is>
-          <t>196006, Г.САНКТ-ПЕТЕРБУРГ, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОСКОВСКАЯ ЗАСТАВА, УЛ ЗАСТАВСКАЯ, Д. 7, ЛИТЕРА А, ПОМЕЩ. 1-Н, ПОМЕЩ. № 157</t>
-        </is>
-      </c>
-      <c r="Q6" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=a8cd893161e0f9a84fd68238c104b56d73861858&amp;tsid=4497016004</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 22:48</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>4512196</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>ОПОРА ЛЭПЛИСТВ НЕПРОПИТАН 22-28СМ L11</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>9725042029</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>64.20</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr"/>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>03.07.2026 11:30 — 09.07.2026 00:00</t>
-        </is>
-      </c>
-      <c r="P7" s="2" t="inlineStr">
-        <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
-        </is>
-      </c>
-      <c r="Q7" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=2c2dc9a5c7e2769edb077c6980aaf039341552d8&amp;tsid=4512196458</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 22:48</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Работы</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>4512292</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>ТЕХНИЧЕСКОЕ ЗАДАНИЕ на строительствоЛЭП-6кВдля электроснабжения электрогидравлического экскаватора Liebherr 9200Е Работы по строительствуЛЭП-6кВдля электроснабжения электрогидравлического экскаватора Liebherr 9200Е.</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>ООО "СЕРВИС ПЛЮС"</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>ООО "СЕРВИС ПЛЮС"</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>7704643931</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>Иванов Владимир Ильич</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>68.32</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr"/>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 12:19 — 09.07.2026 12:00</t>
+          <t>22.06.2026 16:20 — 09.07.2026 12:00</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Пречистенка, д 40/2 стр 4, помещ I, ком 2А</t>
+          <t>196006, Г.САНКТ-ПЕТЕРБУРГ, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОСКОВСКАЯ ЗАСТАВА, УЛ ЗАСТАВСКАЯ, Д. 7, ЛИТЕРА А, ПОМЕЩ. 1-Н, ПОМЕЩ. № 157</t>
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=2c2dc9a5c7e2769edb077c6980aaf039341552d8&amp;tsid=4512292004</t>
+          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=aebe24b8163e25d0928f7986e508a491655fa5fb&amp;tsid=4497016004</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 22:48</t>
+          <t>2026-07-07 11:28</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1113,10 +1118,164 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
+          <t>4512196</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>ОПОРА ЛЭПЛИСТВ НЕПРОПИТАН 22-28СМ L11</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr"/>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>03.07.2026 11:30 — 09.07.2026 00:00</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=daff8080cf9b8da16c0725b58565f69b83594a24&amp;tsid=4512196458</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>4512292</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>ТЕХНИЧЕСКОЕ ЗАДАНИЕ на строительствоЛЭП-6кВдля электроснабжения электрогидравлического экскаватора Liebherr 9200Е Работы по строительствуЛЭП-6кВдля электроснабжения электрогидравлического экскаватора Liebherr 9200Е.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СЕРВИС ПЛЮС"</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СЕРВИС ПЛЮС"</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>7704643931</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Иванов Владимир Ильич</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>68.32</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>03.07.2026 12:19 — 14.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Пречистенка, д 40/2 стр 4, помещ I, ком 2А</t>
+        </is>
+      </c>
+      <c r="Q10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=daff8080cf9b8da16c0725b58565f69b83594a24&amp;tsid=4512292004</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr"/>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
           <t>4475879</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Электро/пневмо и ручной инструмент/Электроизм. инструмент/Расходные мат-лы
 РТИ, РВД, шланги, ремни
@@ -1124,216 +1283,62 @@
 Уплотнительный материал (прокладки, паронит, набивка сальниковая)...  Шина цепной пилы Oregon 752HSFL104Кольцостопор. нар. 210х5 DIN471 Andritz ... клин для бревен Sandvik 1401КольцоAbicor Binzel 757.D007 вихреобразующее ...  Kron ЦПВС-5 RAL7012 КрышкаколодцаП10 ж/б Игла клапана ... Kron ПСВС-3 RAL7012 О-кольцо11,3х2,4 NBR70 Ремень ...</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>4704012472</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>Ленинградская обл</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>Габидуллин Тимур Махмудович</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>17.12</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr"/>
-      <c r="O9" s="2" t="inlineStr">
-        <is>
-          <t>03.06.2026 15:56 — 30.07.2026 20:00</t>
-        </is>
-      </c>
-      <c r="P9" s="2" t="inlineStr">
-        <is>
-          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
-        </is>
-      </c>
-      <c r="Q9" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=84b3fc74822d1b6423791ca20f93740cc324eacf&amp;tsid=4475879003</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 22:48</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>4508331</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Плита ПАГ-14А600ГОСТ 25912-2015 для ООО ГРК Амикан. Требуется жесткая упаковка по ГОСТу КП по форме ТД Полиметалл. В цену включить стоимость доставки до адреса в г. Лесосибирск и обрешетки. При подаче аналогов необходимо приложить тех. документацию</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>7805368914</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>г Санкт-Петербург</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>46.90</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr"/>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>01.07.2026 05:44 — 08.07.2026 10:00</t>
-        </is>
-      </c>
-      <c r="P10" s="2" t="inlineStr">
-        <is>
-          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
-        </is>
-      </c>
-      <c r="Q10" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=cf639e1efd36c817f2b51c49ee96bb146f873e48&amp;tsid=4508331004</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 22:48</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr"/>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>4514583</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Закупка ЖБИ (плитыПДН3*1,5)</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>9725042029</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>64.20</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr"/>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>06.07.2026 15:00 — 09.07.2026 12:00</t>
+          <t>03.06.2026 15:56 — 30.07.2026 20:00</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
         </is>
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-plity-pdn-3-1-5/tender-4514583/#btid=2&amp;sqh=3b472204201f001370372e672ecb96d2c0e73c78&amp;tsid=4514583458</t>
+          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=3dd94215dadaf9910b48b26d09dfaa0e13a663da&amp;tsid=4475879003</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 22:48</t>
+          <t>2026-07-07 11:28</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1349,35 +1354,39 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>4513278</t>
+          <t>4508331</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>ЖБИблоки ФБС</t>
+          <t>Плита ПАГ-14А600ГОСТ 25912-2015 для ООО ГРК Амикан. Требуется жесткая упаковка по ГОСТу КП по форме ТД Полиметалл. В цену включить стоимость доставки до адреса в г. Лесосибирск и обрешетки. При подаче аналогов необходимо приложить тех. документацию</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>7805368914</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr"/>
+          <t>г Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
+        </is>
+      </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1385,30 +1394,30 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>46.90</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr"/>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>06.07.2026 04:17 — 09.07.2026 00:00</t>
+          <t>01.07.2026 05:44 — 08.07.2026 10:00</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-bloki-fbs/tender-4513278/#btid=2&amp;sqh=151673791dd86b46cd73cea65ff7694df2446a4f&amp;tsid=4513278458</t>
+          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=358aa82398996a91e344701708c2c096b691b14a&amp;tsid=4508331004</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 22:48</t>
+          <t>2026-07-07 11:28</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1419,32 +1428,32 @@
       <c r="C13" s="2" t="inlineStr"/>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Поставка</t>
+          <t>Прочее</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>4514839</t>
+          <t>4514583</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>12-х-1 Заключение договора на поставку материалов для наружных сетей водоснабжения и водоотведения на объект строительства «Дальневосточный детский центр отдыха и оздоровления в Хабаровском крае». (9 лотов) Лот №1 ВодоснабжениеЖБИ</t>
+          <t>Закупка ЖБИ (плитыПДН3*1,5)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>ООО "ПРОМСТРОЙ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>ООО "ПРОМСТРОЙ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>9723169975</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1452,11 +1461,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>Султанов Владислав Назипович</t>
-        </is>
-      </c>
+      <c r="K13" s="2" t="inlineStr"/>
       <c r="L13" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1464,30 +1469,30 @@
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>71.12.2</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr"/>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>06.07.2026 16:45 — 10.07.2026 11:00</t>
+          <t>06.07.2026 15:00 — 09.07.2026 12:00</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Волгоградский пр-кт, д 42 к 5, ком 9</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/12-kh-1-zakliuchenie-dogovora-na-postavku-materialov-dlia-naruzhnykh-setei/tender-4514839/#btid=2&amp;sqh=151673791dd86b46cd73cea65ff7694df2446a4f&amp;tsid=4514839004</t>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-plity-pdn-3-1-5/tender-4514583/#btid=2&amp;sqh=9509cf995bcfa53f7089eec3503c1a45f4370746&amp;tsid=4514583458</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 22:48</t>
+          <t>2026-07-07 11:28</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1503,27 +1508,27 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>4510341</t>
+          <t>4513278</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>ЖБИ(чеч 34\25 7510 \ 17338)</t>
+          <t>ЖБИблоки ФБС</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>7724498866</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1531,11 +1536,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>Городний Анатолий Валерьевич</t>
-        </is>
-      </c>
+      <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1543,30 +1544,30 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>46.73</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr"/>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>02.07.2026 09:54 — 07.07.2026 16:00</t>
+          <t>06.07.2026 04:17 — 09.07.2026 00:00</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=151673791dd86b46cd73cea65ff7694df2446a4f&amp;tsid=4510341459</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-bloki-fbs/tender-4513278/#btid=2&amp;sqh=e231a923af9fe898f079520bf0b78e917c1dcd36&amp;tsid=4513278458</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 22:48</t>
+          <t>2026-07-07 11:28</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1577,32 +1578,32 @@
       <c r="C15" s="2" t="inlineStr"/>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Поставка</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>4508347</t>
+          <t>4514839</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>ЖБИКЕМГРЭС</t>
+          <t>12-х-1 Заключение договора на поставку материалов для наружных сетей водоснабжения и водоотведения на объект строительства «Дальневосточный детский центр отдыха и оздоровления в Хабаровском крае». (9 лотов) Лот №1 ВодоснабжениеЖБИ</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "ПРОМСТРОЙ"</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "ПРОМСТРОЙ"</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>9723169975</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -1610,7 +1611,11 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Султанов Владислав Назипович</t>
+        </is>
+      </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1618,30 +1623,30 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>71.12.2</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr"/>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>01.07.2026 05:45 — 10.07.2026 00:00</t>
+          <t>06.07.2026 16:45 — 10.07.2026 11:00</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Москва, Волгоградский пр-кт, д 42 к 5, ком 9</t>
         </is>
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=151673791dd86b46cd73cea65ff7694df2446a4f&amp;tsid=4508347458</t>
+          <t>https://www.b2b-center.ru/market/12-kh-1-zakliuchenie-dogovora-na-postavku-materialov-dlia-naruzhnykh-setei/tender-4514839/#btid=2&amp;sqh=e231a923af9fe898f079520bf0b78e917c1dcd36&amp;tsid=4514839004</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 22:48</t>
+          <t>2026-07-07 11:28</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1657,27 +1662,27 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>4489772</t>
+          <t>4510341</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы 1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы</t>
+          <t>ЖБИ(чеч 34\25 7510 \ 17338)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>7736583259</t>
+          <t>7724498866</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1687,7 +1692,7 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Масько Александр Вадимович</t>
+          <t>Городний Анатолий Валерьевич</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -1697,30 +1702,30 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>70.10</t>
+          <t>46.73</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr"/>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>16.06.2026 11:00 — 16.07.2026 12:00</t>
+          <t>02.07.2026 09:54 — 07.07.2026 16:00</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Старая Басманная, д 12 стр 1</t>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
         </is>
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=151673791dd86b46cd73cea65ff7694df2446a4f&amp;tsid=4489772003</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=e231a923af9fe898f079520bf0b78e917c1dcd36&amp;tsid=4510341459</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 22:48</t>
+          <t>2026-07-07 11:28</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1736,39 +1741,35 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>4474790</t>
+          <t>4508347</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
+          <t>ЖБИКЕМГРЭС</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>4704012472</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>Габидуллин Тимур Махмудович</t>
-        </is>
-      </c>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr"/>
       <c r="L17" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1776,30 +1777,30 @@
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>17.12</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr"/>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>03.06.2026 09:59 — 30.07.2026 20:00</t>
+          <t>01.07.2026 05:45 — 10.07.2026 00:00</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=151673791dd86b46cd73cea65ff7694df2446a4f&amp;tsid=4474790003</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=e231a923af9fe898f079520bf0b78e917c1dcd36&amp;tsid=4508347458</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 22:48</t>
+          <t>2026-07-07 11:28</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1815,27 +1816,27 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>4180328</t>
+          <t>4489772</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, г.Диксон). ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, ПГТ Диксон).</t>
+          <t>1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы 1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
+          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
+          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>7714456916</t>
+          <t>7736583259</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1845,7 +1846,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Наумов Андрей Александрович</t>
+          <t>Масько Александр Вадимович</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -1855,30 +1856,30 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>70.22</t>
+          <t>70.10</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr"/>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>24.09.2025 15:32 — 23.07.2026 12:00</t>
+          <t>16.06.2026 11:00 — 16.07.2026 12:00</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Денежный пер, д 9/6</t>
+          <t>г Москва, ул Старая Басманная, д 12 стр 1</t>
         </is>
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=151673791dd86b46cd73cea65ff7694df2446a4f&amp;tsid=4180328003</t>
+          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=e231a923af9fe898f079520bf0b78e917c1dcd36&amp;tsid=4489772003</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 22:48</t>
+          <t>2026-07-07 11:28</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1894,7 +1895,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>3973258</t>
+          <t>4474790</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1940,7 +1941,7 @@
       <c r="N19" s="2" t="inlineStr"/>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>10.03.2025 00:48 — 30.07.2026 23:00</t>
+          <t>03.06.2026 09:59 — 30.07.2026 20:00</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -1950,14 +1951,14 @@
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=151673791dd86b46cd73cea65ff7694df2446a4f&amp;tsid=3973258003</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=e231a923af9fe898f079520bf0b78e917c1dcd36&amp;tsid=4474790003</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 22:48</t>
+          <t>2026-07-07 11:28</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1968,32 +1969,32 @@
       <c r="C20" s="2" t="inlineStr"/>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Поставка</t>
+          <t>Прочее</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>4513525</t>
+          <t>4180328</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Поставка модульных защитных сооруженийЗДАНИЕ ЗАЩИТНОЕ ДЛЯ УКРЫТИЯ 4,4*2,4*2,2МЖЕЛЕЗОБЕТОННОЕСБОРНОЕ</t>
+          <t>ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, г.Диксон). ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, ПГТ Диксон).</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>7714456916</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -2001,7 +2002,11 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Наумов Андрей Александрович</t>
+        </is>
+      </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -2009,30 +2014,30 @@
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>70.22</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr"/>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>06.07.2026 08:36 — 10.07.2026 14:00</t>
+          <t>24.09.2025 15:32 — 23.07.2026 12:00</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Москва, Денежный пер, д 9/6</t>
         </is>
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/postavka-modulnykh-zashchitnykh-sooruzhenii/tender-4513525/#btid=2&amp;sqh=4ef150eb83696b854ab192649a455db804155e2c&amp;tsid=4513525458</t>
+          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=e231a923af9fe898f079520bf0b78e917c1dcd36&amp;tsid=4180328003</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 22:48</t>
+          <t>2026-07-07 11:28</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -2048,10 +2053,164 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
+          <t>3973258</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>4704012472</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Ленинградская обл</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Габидуллин Тимур Махмудович</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>17.12</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>10.03.2025 00:48 — 30.07.2026 23:00</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+        </is>
+      </c>
+      <c r="Q21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=e231a923af9fe898f079520bf0b78e917c1dcd36&amp;tsid=3973258003</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>4513525</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Поставка модульных защитных сооруженийЗДАНИЕ ЗАЩИТНОЕ ДЛЯ УКРЫТИЯ 4,4*2,4*2,2МЖЕЛЕЗОБЕТОННОЕСБОРНОЕ</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>06.07.2026 08:36 — 10.07.2026 14:00</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/postavka-modulnykh-zashchitnykh-sooruzhenii/tender-4513525/#btid=2&amp;sqh=c1daba5a5e59db9c1d36b293d05151486b52ae02&amp;tsid=4513525458</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr"/>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
           <t>4513563</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>Блок ФБС 12.4.6-Т-и
 Кольцо стеновое КС 20.9 ГОСТ 8020-2016
@@ -2060,236 +2219,315 @@
 Кольцо стеновое КС 20.9 ГОСТ 8020-20164513563 ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "ТОРГОВЫЙ ДОМ ПОЛИМЕТАЛЛ"Железобетонные изделия</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>7805368914</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="J23" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="K23" s="2" t="inlineStr">
         <is>
           <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
         <is>
           <t>46.90</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr"/>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="N23" s="2" t="inlineStr"/>
+      <c r="O23" s="2" t="inlineStr">
         <is>
           <t>06.07.2026 08:49 — 10.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P21" s="2" t="inlineStr">
+      <c r="P23" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
-      <c r="Q21" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/blok-fbs-12-4-6-t-i-koltso-stenovoe-ks-20-9-gost-8020-2016-na-k-pm/tender-4513563/#btid=2&amp;sqh=4ef150eb83696b854ab192649a455db804155e2c&amp;tsid=4513563004</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 22:48</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="Q23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/blok-fbs-12-4-6-t-i-koltso-stenovoe-ks-20-9-gost-8020-2016-na-k-pm/tender-4513563/#btid=2&amp;sqh=c1daba5a5e59db9c1d36b293d05151486b52ae02&amp;tsid=4513563004</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>Поставка</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>4512260</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>ТМЦ. Срочный отбор предложений на право заключения договора поставкижелезобетонных изделийдля нужд филиала «Канская теплосеть» АО «Енисейская ТГК (ТГК-13)».</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>9725042029</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="inlineStr">
+      <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>64.20</t>
         </is>
       </c>
-      <c r="N22" s="2" t="inlineStr"/>
-      <c r="O22" s="2" t="inlineStr">
+      <c r="N24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr">
         <is>
           <t>03.07.2026 11:52 — 08.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P22" s="2" t="inlineStr">
+      <c r="P24" s="2" t="inlineStr">
         <is>
           <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
-      <c r="Q22" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/app/market-next/tmts-srochnyi-otbor-predlozhenii-na-pravo-zakliucheniia-dogovora-postavki/tender-4512260/#btid=2&amp;sqh=4ef150eb83696b854ab192649a455db804155e2c&amp;tsid=4512260458</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 22:48</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr"/>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="Q24" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/tmts-srochnyi-otbor-predlozhenii-na-pravo-zakliucheniia-dogovora-postavki/tender-4512260/#btid=2&amp;sqh=c1daba5a5e59db9c1d36b293d05151486b52ae02&amp;tsid=4512260458</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr"/>
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>4512082</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>Оголовок с платформенным опиранием 4ОСП 32-3 серия 1.111.1-4 в. 2 для ООО "Сахавольфрам"
 Оголовок с платформенным опиранием 4ОСП 32-3 серия 1.111.1-4 в. 2 для ООО "Сахавольфрам"4512082 ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "ТОРГОВЫЙ ДОМ ПОЛИМЕТАЛЛ"Железобетонные изделия</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="I25" s="2" t="inlineStr">
         <is>
           <t>7805368914</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="J25" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr">
+      <c r="K25" s="2" t="inlineStr">
         <is>
           <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
-      <c r="L23" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M23" s="2" t="inlineStr">
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
         <is>
           <t>46.90</t>
         </is>
       </c>
-      <c r="N23" s="2" t="inlineStr"/>
-      <c r="O23" s="2" t="inlineStr">
+      <c r="N25" s="2" t="inlineStr"/>
+      <c r="O25" s="2" t="inlineStr">
         <is>
           <t>03.07.2026 11:05 — 08.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P23" s="2" t="inlineStr">
+      <c r="P25" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
-      <c r="Q23" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/ogolovok-s-platformennym-opiraniem-4osp-32-3-seriia-1-111-1-4-v-2-dlia/tender-4512082/#btid=2&amp;sqh=4ef150eb83696b854ab192649a455db804155e2c&amp;tsid=4512082004</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 22:48</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="Q25" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/ogolovok-s-platformennym-opiraniem-4osp-32-3-seriia-1-111-1-4-v-2-dlia/tender-4512082/#btid=2&amp;sqh=c1daba5a5e59db9c1d36b293d05151486b52ae02&amp;tsid=4512082004</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>4511065</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Защитноежелезобетонноеукрытие 8.0х2.4</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>ООО "Группа Полипластик"</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ГРУППА ПОЛИПЛАСТИК"</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>5021013384</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Коржов Олег Викторович</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>22.21.9</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>02.07.2026 14:23 — 16.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Очаковское шоссе, д 18 стр 3, помещ 014</t>
+        </is>
+      </c>
+      <c r="Q26" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/zashchitnoe-zhelezobetonnoe-ukrytie-8-0kh2-4/tender-4511065/#btid=2&amp;sqh=c1daba5a5e59db9c1d36b293d05151486b52ae02&amp;tsid=4511065004</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr"/>
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>Поставка</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>4511621</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>Закупка аккумуляторных батарей (залитых) для нужд АО "Павловск Неруд" с поставкой в Августе 2026г.
 Обязательная расценка стоимости доставки, возможен забор груза на условиях самовывоза.
@@ -2298,1088 +2536,1088 @@
 Заказчик АО "Павловск Неруд" предприятие АО "Национальная нерудная компания"Аккумулятор ТН-550Перемычкам/ц для АКБ 115,5мм ТН-550Перемычкам/ц для АКБ 212,0мм ТН-550 Транспортная услуга</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>АО "ННК"</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>АО "ННК-ОЙЛ"</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>5032049030</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="J27" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr">
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>Худайнатов Эдуард Юрьевич</t>
         </is>
       </c>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="inlineStr">
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
         <is>
           <t>70.22</t>
         </is>
       </c>
-      <c r="N24" s="2" t="inlineStr"/>
-      <c r="O24" s="2" t="inlineStr">
-        <is>
-          <t>03.07.2026 06:22 — 07.07.2026 11:00</t>
-        </is>
-      </c>
-      <c r="P24" s="2" t="inlineStr">
+      <c r="N27" s="2" t="inlineStr"/>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>03.07.2026 06:22 — 08.07.2026 11:00</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
         <is>
           <t>г Москва, ул 1-я Тверская-Ямская, д 5, помещ 1012</t>
         </is>
       </c>
-      <c r="Q24" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=8f2b34eb3bfa17574b43f4dfd1edd9879569d029&amp;tsid=4511621004</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 22:48</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr"/>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="Q27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=d255ff9d8c195ac53abc2fedf2afd4988a73c57f&amp;tsid=4511621004</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>4511787</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>ЗЧ к автотранспорту... /66 ТЕРМОСТАТ ТС-107-1306100-06ПЕРЕМЫЧКААКБ КЛЕММА-КЛЕММА ПП 500-50 ...</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>9725042029</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
+      <c r="J28" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K25" s="2" t="inlineStr"/>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M25" s="2" t="inlineStr">
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
         <is>
           <t>64.20</t>
         </is>
       </c>
-      <c r="N25" s="2" t="inlineStr"/>
-      <c r="O25" s="2" t="inlineStr">
+      <c r="N28" s="2" t="inlineStr"/>
+      <c r="O28" s="2" t="inlineStr">
         <is>
           <t>03.07.2026 08:32 — 08.07.2026 00:00</t>
         </is>
       </c>
-      <c r="P25" s="2" t="inlineStr">
+      <c r="P28" s="2" t="inlineStr">
         <is>
           <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
-      <c r="Q25" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=8f2b34eb3bfa17574b43f4dfd1edd9879569d029&amp;tsid=4511787458</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 22:48</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="Q28" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=d255ff9d8c195ac53abc2fedf2afd4988a73c57f&amp;tsid=4511787458</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr"/>
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>4512541</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>Запасные части CAT.... -3748 Cat Опора 348-9537 CatПеремычка140-0860 Cat Скоба 8X-3130 ...</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>1004001744</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="J29" s="2" t="inlineStr">
         <is>
           <t>Респ Карелия</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr">
+      <c r="K29" s="2" t="inlineStr">
         <is>
           <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "СЕВЕРСТАЛЬ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="inlineStr">
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
         <is>
           <t>07.10.2</t>
         </is>
       </c>
-      <c r="N26" s="2" t="inlineStr"/>
-      <c r="O26" s="2" t="inlineStr">
+      <c r="N29" s="2" t="inlineStr"/>
+      <c r="O29" s="2" t="inlineStr">
         <is>
           <t>03.07.2026 14:07 — 10.07.2026 11:00</t>
         </is>
       </c>
-      <c r="P26" s="2" t="inlineStr">
+      <c r="P29" s="2" t="inlineStr">
         <is>
           <t>Респ Карелия, г Костомукша, шоссе Горняков, стр 284</t>
         </is>
       </c>
-      <c r="Q26" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=8f2b34eb3bfa17574b43f4dfd1edd9879569d029&amp;tsid=4512541003</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 22:48</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr"/>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="Q29" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=d255ff9d8c195ac53abc2fedf2afd4988a73c57f&amp;tsid=4512541003</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>4508230</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Сборный (Изделия электроустановочные и монтажные, Ящики, щиты, шкафы, пункты и комплектующие к ним, Приборы электроизмерительные, реле)
 МГ-019742, МГ-019713, МГ-019696, МГ-019665, МГ-019621, МГ-019620, МГ-019619, МГ-017109... -HESI-EX (5X20), Phoenix Contact 1277638ПеремычкаFBS 10-5, Phoenix Contact 3030213 ...ПеремычкаFBS 10-5 BU, Phoenix Contact  ...</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>АО "ИК "АРЛАН"</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>АО "ИК "АРЛАН"</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>7722220390</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="J30" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K27" s="2" t="inlineStr">
+      <c r="K30" s="2" t="inlineStr">
         <is>
           <t>Барилов Евгений Александрович</t>
         </is>
       </c>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M27" s="2" t="inlineStr">
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
         <is>
           <t>82.99</t>
         </is>
       </c>
-      <c r="N27" s="2" t="inlineStr"/>
-      <c r="O27" s="2" t="inlineStr">
+      <c r="N30" s="2" t="inlineStr"/>
+      <c r="O30" s="2" t="inlineStr">
         <is>
           <t>30.06.2026 17:59 — 09.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P27" s="2" t="inlineStr">
+      <c r="P30" s="2" t="inlineStr">
         <is>
           <t>г Москва, Романов пер, д 4</t>
         </is>
       </c>
-      <c r="Q27" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=8f2b34eb3bfa17574b43f4dfd1edd9879569d029&amp;tsid=4508230004</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 22:48</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="Q30" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=d255ff9d8c195ac53abc2fedf2afd4988a73c57f&amp;tsid=4508230004</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr"/>
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>4504775</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники
 Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники...  Трубка пробная № 37-542-000 Соединитель-перемычка04182454 Кольцо стальное №CP48001-0305 Фильтр ...</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>7805368914</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="J31" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург</t>
         </is>
       </c>
-      <c r="K28" s="2" t="inlineStr">
+      <c r="K31" s="2" t="inlineStr">
         <is>
           <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M28" s="2" t="inlineStr">
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
         <is>
           <t>46.90</t>
         </is>
       </c>
-      <c r="N28" s="2" t="inlineStr"/>
-      <c r="O28" s="2" t="inlineStr">
+      <c r="N31" s="2" t="inlineStr"/>
+      <c r="O31" s="2" t="inlineStr">
         <is>
           <t>27.06.2026 01:36 — 15.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P28" s="2" t="inlineStr">
+      <c r="P31" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
-      <c r="Q28" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=8f2b34eb3bfa17574b43f4dfd1edd9879569d029&amp;tsid=4504775003</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 22:48</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr"/>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="Q31" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=d255ff9d8c195ac53abc2fedf2afd4988a73c57f&amp;tsid=4504775003</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>4501157</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Источники электропитания (ИБП, аккумуляторные батареи, блоки питания)...  х 1248 А·ч, включая соединительныеперемычки. Вид положительного электрода - трубчатая пластина ...  с коммутирующей арматурой, межэлементными и межряднымиперемычками, крепежами, комплектом для обслуживания АБ. Тип ...</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>АО "Мосинжпроект"</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>АО "МОСИНЖПРОЕКТ"</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>7701885820</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr">
+      <c r="J32" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K29" s="2" t="inlineStr">
+      <c r="K32" s="2" t="inlineStr">
         <is>
           <t>Сорокин Антон Павлович</t>
         </is>
       </c>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M29" s="2" t="inlineStr">
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
         <is>
           <t>71.12.2</t>
         </is>
       </c>
-      <c r="N29" s="2" t="inlineStr"/>
-      <c r="O29" s="2" t="inlineStr">
+      <c r="N32" s="2" t="inlineStr"/>
+      <c r="O32" s="2" t="inlineStr">
         <is>
           <t>24.06.2026 15:40 — 22.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P29" s="2" t="inlineStr">
+      <c r="P32" s="2" t="inlineStr">
         <is>
           <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
         </is>
       </c>
-      <c r="Q29" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=8f2b34eb3bfa17574b43f4dfd1edd9879569d029&amp;tsid=4501157003</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 22:48</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="Q32" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=d255ff9d8c195ac53abc2fedf2afd4988a73c57f&amp;tsid=4501157003</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr"/>
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>4499964</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>Автоматика и телемеханика движения поездов... , 13552-00-00В Дроссель-трансформатор (безперемычек) ДТМ-0,17-1000М ЮКЛЯ.672 ...</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>АО "Мосинжпроект"</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>АО "МОСИНЖПРОЕКТ"</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr">
         <is>
           <t>7701885820</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="J33" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K30" s="2" t="inlineStr">
+      <c r="K33" s="2" t="inlineStr">
         <is>
           <t>Сорокин Антон Павлович</t>
         </is>
       </c>
-      <c r="L30" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M30" s="2" t="inlineStr">
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
         <is>
           <t>71.12.2</t>
         </is>
       </c>
-      <c r="N30" s="2" t="inlineStr"/>
-      <c r="O30" s="2" t="inlineStr">
+      <c r="N33" s="2" t="inlineStr"/>
+      <c r="O33" s="2" t="inlineStr">
         <is>
           <t>24.06.2026 08:46 — 15.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P30" s="2" t="inlineStr">
+      <c r="P33" s="2" t="inlineStr">
         <is>
           <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
         </is>
       </c>
-      <c r="Q30" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=8f2b34eb3bfa17574b43f4dfd1edd9879569d029&amp;tsid=4499964003</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 22:48</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr"/>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="Q33" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=d255ff9d8c195ac53abc2fedf2afd4988a73c57f&amp;tsid=4499964003</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>4480614</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Плановое и аварийное техническое обслуживание зданий и сооружений (годовое обслуживание август 2026 - август 2027) ГК Логика молока, производственная площадка в г. Ялуторовске
 Обслуживание зданий и сооружений завода в г. Ялуторовске....  стен из газобетонных блоков Устройство металлическихперемычекс устройством штраб Усиление кирпичных стен ...</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>АО "ЭЙЧ ЭНД ЭН"</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>АО "ЭЙЧ ЭНД ЭН"</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>7714626332</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr">
+      <c r="J34" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K31" s="2" t="inlineStr">
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>Закриев Якуб Салманович</t>
         </is>
       </c>
-      <c r="L31" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M31" s="2" t="inlineStr">
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
         <is>
           <t>10.51.9</t>
         </is>
       </c>
-      <c r="N31" s="2" t="inlineStr"/>
-      <c r="O31" s="2" t="inlineStr">
+      <c r="N34" s="2" t="inlineStr"/>
+      <c r="O34" s="2" t="inlineStr">
         <is>
           <t>08.06.2026 14:44 — 08.07.2026 23:00</t>
         </is>
       </c>
-      <c r="P31" s="2" t="inlineStr">
+      <c r="P34" s="2" t="inlineStr">
         <is>
           <t>г Москва, ул Вятская, д 27 стр 13</t>
         </is>
       </c>
-      <c r="Q31" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/planovoe-i-avariinoe-tekhnicheskoe-obsluzhivanie-zdanii-i-sooruzhenii/tender-4480614/#btid=2&amp;sqh=8f2b34eb3bfa17574b43f4dfd1edd9879569d029&amp;tsid=4480614004</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 22:48</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="Q34" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/planovoe-i-avariinoe-tekhnicheskoe-obsluzhivanie-zdanii-i-sooruzhenii/tender-4480614/#btid=2&amp;sqh=d255ff9d8c195ac53abc2fedf2afd4988a73c57f&amp;tsid=4480614004</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr"/>
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>4512370</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>ТО Сплит систем Лабинск Эйч энд Эн... кондиционирования Техническое обслуживание внутреннегоблокакассетного типа мультизональной  ...блокакондиционера. Мойка теплообменника внутреннегоблокакондиционера Чистка фильтров внутреннегоблокакондиционера Чистка фильтров приточнойвентиляционной...</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>АО "ЭЙЧ ЭНД ЭН"</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>АО "ЭЙЧ ЭНД ЭН"</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="I35" s="2" t="inlineStr">
         <is>
           <t>7714626332</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr">
+      <c r="J35" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K32" s="2" t="inlineStr">
+      <c r="K35" s="2" t="inlineStr">
         <is>
           <t>Закриев Якуб Салманович</t>
         </is>
       </c>
-      <c r="L32" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M32" s="2" t="inlineStr">
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
         <is>
           <t>10.51.9</t>
         </is>
       </c>
-      <c r="N32" s="2" t="inlineStr"/>
-      <c r="O32" s="2" t="inlineStr">
+      <c r="N35" s="2" t="inlineStr"/>
+      <c r="O35" s="2" t="inlineStr">
         <is>
           <t>03.07.2026 12:40 — 14.07.2026 18:30</t>
         </is>
       </c>
-      <c r="P32" s="2" t="inlineStr">
+      <c r="P35" s="2" t="inlineStr">
         <is>
           <t>г Москва, ул Вятская, д 27 стр 13</t>
         </is>
       </c>
-      <c r="Q32" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=48fb12302dd23d97fd728136e7c312e5ed2dcf94&amp;tsid=4512370458</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 22:48</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr"/>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="Q35" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=e2af420114ba61a379eed65341d8a02e5f5e76cf&amp;tsid=4512370458</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>4501181</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Вентиляторы промышленные и оборудование общеобменной вентиляции...  5Ф РешёткавентиляционнаяАМР 600х300М РешёткавентиляционнаяАМР 150х150М РешёткавентиляционнаяАМР 300х200М  ... мм.; масса 0,65 кгБлокконтроля сопротивления БСК-3.1 Канальный ...  533Па, габаритные размеры 700х467х2230 мм,блоков/моноблоков 5/1, в составе: - ...</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>АО "Мосинжпроект"</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>АО "МОСИНЖПРОЕКТ"</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr">
+      <c r="I36" s="2" t="inlineStr">
         <is>
           <t>7701885820</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr">
+      <c r="J36" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K33" s="2" t="inlineStr">
+      <c r="K36" s="2" t="inlineStr">
         <is>
           <t>Сорокин Антон Павлович</t>
         </is>
       </c>
-      <c r="L33" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M33" s="2" t="inlineStr">
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
         <is>
           <t>71.12.2</t>
         </is>
       </c>
-      <c r="N33" s="2" t="inlineStr"/>
-      <c r="O33" s="2" t="inlineStr">
+      <c r="N36" s="2" t="inlineStr"/>
+      <c r="O36" s="2" t="inlineStr">
         <is>
           <t>24.06.2026 15:45 — 22.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P33" s="2" t="inlineStr">
+      <c r="P36" s="2" t="inlineStr">
         <is>
           <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
         </is>
       </c>
-      <c r="Q33" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=48fb12302dd23d97fd728136e7c312e5ed2dcf94&amp;tsid=4501181003</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 22:48</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="Q36" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=e2af420114ba61a379eed65341d8a02e5f5e76cf&amp;tsid=4501181003</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr"/>
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>4501483</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ
 Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ...  d 50x2", внутренняя резьба RTPБлокуправления наружной установки ICEFREE TR-16 ...  Оповещатель звуковой МАЯК-12-ЗМБлокуправления наружной установки ICEFREE TS- ... проводов КС-3 007004 Велос Переходвентиляционный150х100 - D150, из тонколистовой оцинкованной ...</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr">
+      <c r="I37" s="2" t="inlineStr">
         <is>
           <t>7805368914</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr">
+      <c r="J37" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург</t>
         </is>
       </c>
-      <c r="K34" s="2" t="inlineStr">
+      <c r="K37" s="2" t="inlineStr">
         <is>
           <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M34" s="2" t="inlineStr">
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
         <is>
           <t>46.90</t>
         </is>
       </c>
-      <c r="N34" s="2" t="inlineStr"/>
-      <c r="O34" s="2" t="inlineStr">
+      <c r="N37" s="2" t="inlineStr"/>
+      <c r="O37" s="2" t="inlineStr">
         <is>
           <t>25.06.2026 05:03 — 09.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P34" s="2" t="inlineStr">
+      <c r="P37" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
-      <c r="Q34" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=48fb12302dd23d97fd728136e7c312e5ed2dcf94&amp;tsid=4501483003</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 22:48</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr"/>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="Q37" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=e2af420114ba61a379eed65341d8a02e5f5e76cf&amp;tsid=4501483003</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>4500120</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Коммуникационное оборудование, компьютеры, комплектующие к ним, серверное оборудование и ПО...  и кабелей – 1 компл. Удаленныйблок(репитер) BSF414 , питание 220В,  ... 2х2 Комбайнер специализированный OMU Side (блок1) OMUSC1 Комбайнер специализированный OMU ... контроллер для мониторинга в FlexGain View,вентиляционнаяпанель с фильтрами, комплект кабелей, ...</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>АО "Мосинжпроект"</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>АО "МОСИНЖПРОЕКТ"</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr">
+      <c r="I38" s="2" t="inlineStr">
         <is>
           <t>7701885820</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr">
+      <c r="J38" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K35" s="2" t="inlineStr">
+      <c r="K38" s="2" t="inlineStr">
         <is>
           <t>Сорокин Антон Павлович</t>
         </is>
       </c>
-      <c r="L35" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M35" s="2" t="inlineStr">
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
         <is>
           <t>71.12.2</t>
         </is>
       </c>
-      <c r="N35" s="2" t="inlineStr"/>
-      <c r="O35" s="2" t="inlineStr">
+      <c r="N38" s="2" t="inlineStr"/>
+      <c r="O38" s="2" t="inlineStr">
         <is>
           <t>24.06.2026 09:48 — 15.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P35" s="2" t="inlineStr">
+      <c r="P38" s="2" t="inlineStr">
         <is>
           <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
         </is>
       </c>
-      <c r="Q35" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=48fb12302dd23d97fd728136e7c312e5ed2dcf94&amp;tsid=4500120003</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 22:48</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="Q38" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=e2af420114ba61a379eed65341d8a02e5f5e76cf&amp;tsid=4500120003</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr"/>
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>4496006</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп
 Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп... -316 ***Петля крепежная стальная ***Платаблокауправления ZC5 CAME ***Средство чистящее " ... /распылитель для чаши Генуя ***РешеткавентиляционнаяРВ-1 225Х225 ***Петля анкерная 0 ... мл ***Папка с зажимом ***РешеткавентиляционнаяРВ-1 325Х125 ***Папка на кольцах ...</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>ООО "СИБУР"</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>ООО "СИБУР"</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr">
+      <c r="I39" s="2" t="inlineStr">
         <is>
           <t>7727576505</t>
         </is>
       </c>
-      <c r="J36" s="2" t="inlineStr">
+      <c r="J39" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K36" s="2" t="inlineStr">
+      <c r="K39" s="2" t="inlineStr">
         <is>
           <t>Карисалов Михаил Юрьевич</t>
         </is>
       </c>
-      <c r="L36" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M36" s="2" t="inlineStr">
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
         <is>
           <t>70.10</t>
         </is>
       </c>
-      <c r="N36" s="2" t="inlineStr"/>
-      <c r="O36" s="2" t="inlineStr">
+      <c r="N39" s="2" t="inlineStr"/>
+      <c r="O39" s="2" t="inlineStr">
         <is>
           <t>20.06.2026 16:19 — 11.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P36" s="2" t="inlineStr">
+      <c r="P39" s="2" t="inlineStr">
         <is>
           <t>г Москва, ул Кржижановского, д 16 к 3</t>
         </is>
       </c>
-      <c r="Q36" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nelikvidnykh-tmts-tarelki-dlia-filtra-prokladki-dvigatel/tender-4496006/#btid=2&amp;sqh=48fb12302dd23d97fd728136e7c312e5ed2dcf94&amp;tsid=4496006003</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06 22:48</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr"/>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="Q39" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/prodazha-nelikvidnykh-tmts-tarelki-dlia-filtra-prokladki-dvigatel/tender-4496006/#btid=2&amp;sqh=e2af420114ba61a379eed65341d8a02e5f5e76cf&amp;tsid=4496006003</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:28</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>Работы</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>4129930</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Реализация материалов для ремонта (напольные покрытия, настенные покрытия, окна, двери и т.д.) с АО "Мальцовский портландцемент"Блокдверной балконныйБлокдверной филенчатый ДГ 21х9Блококонный 1500х1000 ммБлококонный 1770х1700 мм Желоб ...  Docke Рама оконная 3000х1200 мм Решеткавентиляционнаянаружная Ручка оконная ГОСТ 5087-80 ...</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr">
+      <c r="I40" s="2" t="inlineStr">
         <is>
           <t>7708117908</t>
         </is>
       </c>
-      <c r="J37" s="2" t="inlineStr">
+      <c r="J40" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K37" s="2" t="inlineStr">
+      <c r="K40" s="2" t="inlineStr">
         <is>
           <t>Шматов Вячеслав Вячеславович</t>
         </is>
       </c>
-      <c r="L37" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M37" s="2" t="inlineStr">
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
         <is>
           <t>23.51</t>
         </is>
       </c>
-      <c r="N37" s="2" t="inlineStr"/>
-      <c r="O37" s="2" t="inlineStr">
+      <c r="N40" s="2" t="inlineStr"/>
+      <c r="O40" s="2" t="inlineStr">
         <is>
           <t>06.08.2025 14:33 — 07.08.2026 12:00</t>
         </is>
       </c>
-      <c r="P37" s="2" t="inlineStr">
+      <c r="P40" s="2" t="inlineStr">
         <is>
           <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
         </is>
       </c>
-      <c r="Q37" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=48fb12302dd23d97fd728136e7c312e5ed2dcf94&amp;tsid=4129930003</t>
+      <c r="Q40" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=e2af420114ba61a379eed65341d8a02e5f5e76cf&amp;tsid=4129930003</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q37"/>
+  <autoFilter ref="A1:Q40"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -3417,6 +3655,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId39"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-07 19:21 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q40"/>
+  <dimension ref="A1:Q39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -622,14 +622,14 @@
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/stroitelnye-materialy-postavka-v-nakhodku-dlia-ooo-svetloe-postavka/tender-4515159/#btid=2&amp;sqh=4fab989164db7b10ecec829f6897bdac08350c55&amp;tsid=4515159004</t>
+          <t>https://www.b2b-center.ru/market/stroitelnye-materialy-postavka-v-nakhodku-dlia-ooo-svetloe-postavka/tender-4515159/#btid=2&amp;sqh=8e563bad4224f0e48f0af61695f5f4c8f562ba44&amp;tsid=4515159004</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -702,14 +702,14 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=4fab989164db7b10ecec829f6897bdac08350c55&amp;tsid=4510835003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=8e563bad4224f0e48f0af61695f5f4c8f562ba44&amp;tsid=4510835003</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -781,14 +781,14 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/remont-dorozhnoi-plitki-na-pod-ezdnoi-i-vyezdnoi-doroge-ot-glavnogo/tender-4506366/#btid=2&amp;sqh=4fab989164db7b10ecec829f6897bdac08350c55&amp;tsid=4506366458</t>
+          <t>https://www.b2b-center.ru/app/market-next/remont-dorozhnoi-plitki-na-pod-ezdnoi-i-vyezdnoi-doroge-ot-glavnogo/tender-4506366/#btid=2&amp;sqh=8e563bad4224f0e48f0af61695f5f4c8f562ba44&amp;tsid=4506366458</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -857,14 +857,14 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=4fab989164db7b10ecec829f6897bdac08350c55&amp;tsid=4503612458</t>
+          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=8e563bad4224f0e48f0af61695f5f4c8f562ba44&amp;tsid=4503612458</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -936,14 +936,14 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=4fab989164db7b10ecec829f6897bdac08350c55&amp;tsid=4130106003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=8e563bad4224f0e48f0af61695f5f4c8f562ba44&amp;tsid=4130106003</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1015,14 +1015,14 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=10aaad04274a74c975e4784773a70ef40b0bcff6&amp;tsid=4498936003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=c7e9a6366e60bddb02c708506fc1962f4e205a53&amp;tsid=4498936003</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1095,14 +1095,14 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=aebe24b8163e25d0928f7986e508a491655fa5fb&amp;tsid=4497016004</t>
+          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=587cba0d7823c00bf4cffa8986d257d91a51d340&amp;tsid=4497016004</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1170,14 +1170,14 @@
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=daff8080cf9b8da16c0725b58565f69b83594a24&amp;tsid=4512196458</t>
+          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=7dbda509515c8bcaf34ece759fdb41e1f4a74d2d&amp;tsid=4512196458</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1249,14 +1249,14 @@
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=daff8080cf9b8da16c0725b58565f69b83594a24&amp;tsid=4512292004</t>
+          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=7dbda509515c8bcaf34ece759fdb41e1f4a74d2d&amp;tsid=4512292004</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1331,14 +1331,14 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=3dd94215dadaf9910b48b26d09dfaa0e13a663da&amp;tsid=4475879003</t>
+          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=590be7cb5732e94d1262344f871803b3ef2abb29&amp;tsid=4475879003</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1410,14 +1410,14 @@
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=358aa82398996a91e344701708c2c096b691b14a&amp;tsid=4508331004</t>
+          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=5b1aeb5217f9925cfe184b7dc644e4672b8e7853&amp;tsid=4508331004</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1485,14 +1485,14 @@
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-plity-pdn-3-1-5/tender-4514583/#btid=2&amp;sqh=9509cf995bcfa53f7089eec3503c1a45f4370746&amp;tsid=4514583458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-plity-pdn-3-1-5/tender-4514583/#btid=2&amp;sqh=dc1fd934a3fc31dafe24919d7248ef2c5f3ef41c&amp;tsid=4514583458</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1508,12 +1508,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>4513278</t>
+          <t>4516217</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>ЖБИблоки ФБС</t>
+          <t>ТМЦЖБИи песок</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1550,7 +1550,7 @@
       <c r="N14" s="2" t="inlineStr"/>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>06.07.2026 04:17 — 09.07.2026 00:00</t>
+          <t>07.07.2026 14:31 — 10.07.2026 10:00</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -1560,14 +1560,14 @@
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-bloki-fbs/tender-4513278/#btid=2&amp;sqh=e231a923af9fe898f079520bf0b78e917c1dcd36&amp;tsid=4513278458</t>
+          <t>https://www.b2b-center.ru/app/market-next/tmts-zhbi-i-pesok/tender-4516217/#btid=2&amp;sqh=08a697ca4c161444f3d019ceaddceab59e726906&amp;tsid=4516217458</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1578,32 +1578,32 @@
       <c r="C15" s="2" t="inlineStr"/>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Поставка</t>
+          <t>Прочее</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>4514839</t>
+          <t>4513278</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>12-х-1 Заключение договора на поставку материалов для наружных сетей водоснабжения и водоотведения на объект строительства «Дальневосточный детский центр отдыха и оздоровления в Хабаровском крае». (9 лотов) Лот №1 ВодоснабжениеЖБИ</t>
+          <t>ЖБИблоки ФБС</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>ООО "ПРОМСТРОЙ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>ООО "ПРОМСТРОЙ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>9723169975</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -1611,11 +1611,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>Султанов Владислав Назипович</t>
-        </is>
-      </c>
+      <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1623,30 +1619,30 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>71.12.2</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr"/>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>06.07.2026 16:45 — 10.07.2026 11:00</t>
+          <t>06.07.2026 04:17 — 09.07.2026 00:00</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Волгоградский пр-кт, д 42 к 5, ком 9</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/12-kh-1-zakliuchenie-dogovora-na-postavku-materialov-dlia-naruzhnykh-setei/tender-4514839/#btid=2&amp;sqh=e231a923af9fe898f079520bf0b78e917c1dcd36&amp;tsid=4514839004</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-bloki-fbs/tender-4513278/#btid=2&amp;sqh=08a697ca4c161444f3d019ceaddceab59e726906&amp;tsid=4513278458</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1657,32 +1653,32 @@
       <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Поставка</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>4510341</t>
+          <t>4514839</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>ЖБИ(чеч 34\25 7510 \ 17338)</t>
+          <t>12-х-1 Заключение договора на поставку материалов для наружных сетей водоснабжения и водоотведения на объект строительства «Дальневосточный детский центр отдыха и оздоровления в Хабаровском крае». (9 лотов) Лот №1 ВодоснабжениеЖБИ</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "ПРОМСТРОЙ"</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "ПРОМСТРОЙ"</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>7724498866</t>
+          <t>9723169975</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1692,7 +1688,7 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Городний Анатолий Валерьевич</t>
+          <t>Султанов Владислав Назипович</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -1702,30 +1698,30 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>46.73</t>
+          <t>71.12.2</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr"/>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>02.07.2026 09:54 — 07.07.2026 16:00</t>
+          <t>06.07.2026 16:45 — 10.07.2026 11:00</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+          <t>г Москва, Волгоградский пр-кт, д 42 к 5, ком 9</t>
         </is>
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=e231a923af9fe898f079520bf0b78e917c1dcd36&amp;tsid=4510341459</t>
+          <t>https://www.b2b-center.ru/market/12-kh-1-zakliuchenie-dogovora-na-postavku-materialov-dlia-naruzhnykh-setei/tender-4514839/#btid=2&amp;sqh=08a697ca4c161444f3d019ceaddceab59e726906&amp;tsid=4514839004</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1741,27 +1737,27 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>4508347</t>
+          <t>4510341</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>ЖБИКЕМГРЭС</t>
+          <t>ЖБИ(чеч 34\25 7510 \ 17338)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>7724498866</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -1769,7 +1765,11 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1777,30 +1777,30 @@
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>46.73</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr"/>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>01.07.2026 05:45 — 10.07.2026 00:00</t>
+          <t>02.07.2026 09:54 — 08.07.2026 15:00</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
         </is>
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=e231a923af9fe898f079520bf0b78e917c1dcd36&amp;tsid=4508347458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=08a697ca4c161444f3d019ceaddceab59e726906&amp;tsid=4510341459</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1816,27 +1816,27 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>4489772</t>
+          <t>4508347</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы 1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы</t>
+          <t>ЖБИКЕМГРЭС</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>7736583259</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1844,11 +1844,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>Масько Александр Вадимович</t>
-        </is>
-      </c>
+      <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1856,30 +1852,30 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>70.10</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr"/>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>16.06.2026 11:00 — 16.07.2026 12:00</t>
+          <t>01.07.2026 05:45 — 10.07.2026 00:00</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Старая Басманная, д 12 стр 1</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=e231a923af9fe898f079520bf0b78e917c1dcd36&amp;tsid=4489772003</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=08a697ca4c161444f3d019ceaddceab59e726906&amp;tsid=4508347458</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1895,37 +1891,37 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>4474790</t>
+          <t>4489772</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
+          <t>1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы 1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>4704012472</t>
+          <t>7736583259</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Габидуллин Тимур Махмудович</t>
+          <t>Масько Александр Вадимович</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -1935,30 +1931,30 @@
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>17.12</t>
+          <t>70.10</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr"/>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>03.06.2026 09:59 — 30.07.2026 20:00</t>
+          <t>16.06.2026 11:00 — 16.07.2026 12:00</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+          <t>г Москва, ул Старая Басманная, д 12 стр 1</t>
         </is>
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=e231a923af9fe898f079520bf0b78e917c1dcd36&amp;tsid=4474790003</t>
+          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=08a697ca4c161444f3d019ceaddceab59e726906&amp;tsid=4489772003</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1974,37 +1970,37 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>4180328</t>
+          <t>4474790</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, г.Диксон). ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, ПГТ Диксон).</t>
+          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>7714456916</t>
+          <t>4704012472</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
+          <t>Ленинградская обл</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Наумов Андрей Александрович</t>
+          <t>Габидуллин Тимур Махмудович</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -2014,30 +2010,30 @@
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>70.22</t>
+          <t>17.12</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr"/>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>24.09.2025 15:32 — 23.07.2026 12:00</t>
+          <t>03.06.2026 09:59 — 30.07.2026 20:00</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Денежный пер, д 9/6</t>
+          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
         </is>
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=e231a923af9fe898f079520bf0b78e917c1dcd36&amp;tsid=4180328003</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=08a697ca4c161444f3d019ceaddceab59e726906&amp;tsid=4474790003</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -2053,37 +2049,37 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>3973258</t>
+          <t>4180328</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
+          <t>ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, г.Диксон). ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, ПГТ Диксон).</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>4704012472</t>
+          <t>7714456916</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Габидуллин Тимур Махмудович</t>
+          <t>Наумов Андрей Александрович</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -2093,30 +2089,30 @@
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>17.12</t>
+          <t>70.22</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr"/>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>10.03.2025 00:48 — 30.07.2026 23:00</t>
+          <t>24.09.2025 15:32 — 23.07.2026 12:00</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+          <t>г Москва, Денежный пер, д 9/6</t>
         </is>
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=e231a923af9fe898f079520bf0b78e917c1dcd36&amp;tsid=3973258003</t>
+          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=08a697ca4c161444f3d019ceaddceab59e726906&amp;tsid=4180328003</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2127,40 +2123,44 @@
       <c r="C22" s="2" t="inlineStr"/>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Поставка</t>
+          <t>Прочее</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>4513525</t>
+          <t>3973258</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Поставка модульных защитных сооруженийЗДАНИЕ ЗАЩИТНОЕ ДЛЯ УКРЫТИЯ 4,4*2,4*2,2МЖЕЛЕЗОБЕТОННОЕСБОРНОЕ</t>
+          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>4704012472</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr"/>
+          <t>Ленинградская обл</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Габидуллин Тимур Махмудович</t>
+        </is>
+      </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -2168,30 +2168,30 @@
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>17.12</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr"/>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>06.07.2026 08:36 — 10.07.2026 14:00</t>
+          <t>10.03.2025 00:48 — 30.07.2026 23:00</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
         </is>
       </c>
       <c r="Q22" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/postavka-modulnykh-zashchitnykh-sooruzhenii/tender-4513525/#btid=2&amp;sqh=c1daba5a5e59db9c1d36b293d05151486b52ae02&amp;tsid=4513525458</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=08a697ca4c161444f3d019ceaddceab59e726906&amp;tsid=3973258003</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2202,15 +2202,90 @@
       <c r="C23" s="2" t="inlineStr"/>
       <c r="D23" s="2" t="inlineStr">
         <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>4513525</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Поставка модульных защитных сооруженийЗДАНИЕ ЗАЩИТНОЕ ДЛЯ УКРЫТИЯ 4,4*2,4*2,2МЖЕЛЕЗОБЕТОННОЕСБОРНОЕ</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr"/>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>06.07.2026 08:36 — 10.07.2026 14:00</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/postavka-modulnykh-zashchitnykh-sooruzhenii/tender-4513525/#btid=2&amp;sqh=5ca340ddd1aafc75928e9226e262d7f80332171b&amp;tsid=4513525458</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 19:21</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>4513563</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Блок ФБС 12.4.6-Т-и
 Кольцо стеновое КС 20.9 ГОСТ 8020-2016
@@ -2219,137 +2294,62 @@
 Кольцо стеновое КС 20.9 ГОСТ 8020-20164513563 ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "ТОРГОВЫЙ ДОМ ПОЛИМЕТАЛЛ"Железобетонные изделия</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>7805368914</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr">
+      <c r="K24" s="2" t="inlineStr">
         <is>
           <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
-      <c r="L23" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M23" s="2" t="inlineStr">
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>46.90</t>
-        </is>
-      </c>
-      <c r="N23" s="2" t="inlineStr"/>
-      <c r="O23" s="2" t="inlineStr">
-        <is>
-          <t>06.07.2026 08:49 — 10.07.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P23" s="2" t="inlineStr">
-        <is>
-          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
-        </is>
-      </c>
-      <c r="Q23" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/blok-fbs-12-4-6-t-i-koltso-stenovoe-ks-20-9-gost-8020-2016-na-k-pm/tender-4513563/#btid=2&amp;sqh=c1daba5a5e59db9c1d36b293d05151486b52ae02&amp;tsid=4513563004</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-07 11:28</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Поставка</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>4512260</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>ТМЦ. Срочный отбор предложений на право заключения договора поставкижелезобетонных изделийдля нужд филиала «Канская теплосеть» АО «Енисейская ТГК (ТГК-13)».</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>9725042029</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr"/>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="inlineStr">
-        <is>
-          <t>64.20</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr"/>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 11:52 — 08.07.2026 12:00</t>
+          <t>06.07.2026 08:49 — 10.07.2026 12:00</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/tmts-srochnyi-otbor-predlozhenii-na-pravo-zakliucheniia-dogovora-postavki/tender-4512260/#btid=2&amp;sqh=c1daba5a5e59db9c1d36b293d05151486b52ae02&amp;tsid=4512260458</t>
+          <t>https://www.b2b-center.ru/market/blok-fbs-12-4-6-t-i-koltso-stenovoe-ks-20-9-gost-8020-2016-na-k-pm/tender-4513563/#btid=2&amp;sqh=5ca340ddd1aafc75928e9226e262d7f80332171b&amp;tsid=4513563004</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -2360,45 +2360,40 @@
       <c r="C25" s="2" t="inlineStr"/>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Поставка</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>4512082</t>
+          <t>4512260</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Оголовок с платформенным опиранием 4ОСП 32-3 серия 1.111.1-4 в. 2 для ООО "Сахавольфрам"
-Оголовок с платформенным опиранием 4ОСП 32-3 серия 1.111.1-4 в. 2 для ООО "Сахавольфрам"4512082 ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "ТОРГОВЫЙ ДОМ ПОЛИМЕТАЛЛ"Железобетонные изделия</t>
+          <t>ТМЦ. Срочный отбор предложений на право заключения договора поставкижелезобетонных изделийдля нужд филиала «Канская теплосеть» АО «Енисейская ТГК (ТГК-13)».</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>7805368914</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>г Санкт-Петербург</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
-        </is>
-      </c>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr"/>
       <c r="L25" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -2406,30 +2401,30 @@
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>46.90</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr"/>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 11:05 — 08.07.2026 12:00</t>
+          <t>03.07.2026 11:52 — 08.07.2026 12:00</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q25" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/ogolovok-s-platformennym-opiraniem-4osp-32-3-seriia-1-111-1-4-v-2-dlia/tender-4512082/#btid=2&amp;sqh=c1daba5a5e59db9c1d36b293d05151486b52ae02&amp;tsid=4512082004</t>
+          <t>https://www.b2b-center.ru/app/market-next/tmts-srochnyi-otbor-predlozhenii-na-pravo-zakliucheniia-dogovora-postavki/tender-4512260/#btid=2&amp;sqh=5ca340ddd1aafc75928e9226e262d7f80332171b&amp;tsid=4512260458</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2440,94 +2435,15 @@
       <c r="C26" s="2" t="inlineStr"/>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Поставка</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>4511065</t>
+          <t>4511621</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>Защитноежелезобетонноеукрытие 8.0х2.4</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>ООО "Группа Полипластик"</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>ООО "ГРУППА ПОЛИПЛАСТИК"</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>5021013384</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>Коржов Олег Викторович</t>
-        </is>
-      </c>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="inlineStr">
-        <is>
-          <t>22.21.9</t>
-        </is>
-      </c>
-      <c r="N26" s="2" t="inlineStr"/>
-      <c r="O26" s="2" t="inlineStr">
-        <is>
-          <t>02.07.2026 14:23 — 16.07.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P26" s="2" t="inlineStr">
-        <is>
-          <t>г Москва, Очаковское шоссе, д 18 стр 3, помещ 014</t>
-        </is>
-      </c>
-      <c r="Q26" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/zashchitnoe-zhelezobetonnoe-ukrytie-8-0kh2-4/tender-4511065/#btid=2&amp;sqh=c1daba5a5e59db9c1d36b293d05151486b52ae02&amp;tsid=4511065004</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-07 11:28</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr"/>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>Поставка</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>4511621</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>Закупка аккумуляторных батарей (залитых) для нужд АО "Павловск Неруд" с поставкой в Августе 2026г.
 Обязательная расценка стоимости доставки, возможен забор груза на условиях самовывоза.
@@ -2536,19 +2452,98 @@
 Заказчик АО "Павловск Неруд" предприятие АО "Национальная нерудная компания"Аккумулятор ТН-550Перемычкам/ц для АКБ 115,5мм ТН-550Перемычкам/ц для АКБ 212,0мм ТН-550 Транспортная услуга</t>
         </is>
       </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>АО "ННК"</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>АО "ННК-ОЙЛ"</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>5032049030</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Худайнатов Эдуард Юрьевич</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>70.22</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>03.07.2026 06:22 — 08.07.2026 11:00</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул 1-я Тверская-Ямская, д 5, помещ 1012</t>
+        </is>
+      </c>
+      <c r="Q26" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=e3415418c829f6295e8f7502db2a2c9dcace8ed4&amp;tsid=4511621004</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 19:21</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr"/>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>4511787</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>ЗЧ к автотранспорту... /66 ТЕРМОСТАТ ТС-107-1306100-06ПЕРЕМЫЧКААКБ КЛЕММА-КЛЕММА ПП 500-50 ...</t>
+        </is>
+      </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>АО "ННК"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>АО "ННК-ОЙЛ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>5032049030</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
@@ -2556,11 +2551,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>Худайнатов Эдуард Юрьевич</t>
-        </is>
-      </c>
+      <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -2568,30 +2559,30 @@
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>70.22</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr"/>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 06:22 — 08.07.2026 11:00</t>
+          <t>03.07.2026 08:32 — 08.07.2026 00:00</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул 1-я Тверская-Ямская, д 5, помещ 1012</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q27" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=d255ff9d8c195ac53abc2fedf2afd4988a73c57f&amp;tsid=4511621004</t>
+          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=e3415418c829f6295e8f7502db2a2c9dcace8ed4&amp;tsid=4511787458</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -2607,35 +2598,39 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>4511787</t>
+          <t>4512541</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>ЗЧ к автотранспорту... /66 ТЕРМОСТАТ ТС-107-1306100-06ПЕРЕМЫЧКААКБ КЛЕММА-КЛЕММА ПП 500-50 ...</t>
+          <t>Запасные части CAT.... -3748 Cat Опора 348-9537 CatПеремычка140-0860 Cat Скоба 8X-3130 ...</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>1004001744</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr"/>
+          <t>Респ Карелия</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "СЕВЕРСТАЛЬ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -2643,30 +2638,30 @@
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>07.10.2</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr"/>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 08:32 — 08.07.2026 00:00</t>
+          <t>03.07.2026 14:07 — 10.07.2026 11:00</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>Респ Карелия, г Костомукша, шоссе Горняков, стр 284</t>
         </is>
       </c>
       <c r="Q28" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=d255ff9d8c195ac53abc2fedf2afd4988a73c57f&amp;tsid=4511787458</t>
+          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=e3415418c829f6295e8f7502db2a2c9dcace8ed4&amp;tsid=4512541003</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -2682,37 +2677,38 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>4512541</t>
+          <t>4508230</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Запасные части CAT.... -3748 Cat Опора 348-9537 CatПеремычка140-0860 Cat Скоба 8X-3130 ...</t>
+          <t>Сборный (Изделия электроустановочные и монтажные, Ящики, щиты, шкафы, пункты и комплектующие к ним, Приборы электроизмерительные, реле)
+МГ-019742, МГ-019713, МГ-019696, МГ-019665, МГ-019621, МГ-019620, МГ-019619, МГ-017109... -HESI-EX (5X20), Phoenix Contact 1277638ПеремычкаFBS 10-5, Phoenix Contact 3030213 ...ПеремычкаFBS 10-5 BU, Phoenix Contact  ...</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
+          <t>АО "ИК "АРЛАН"</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
+          <t>АО "ИК "АРЛАН"</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>1004001744</t>
+          <t>7722220390</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Респ Карелия</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "СЕВЕРСТАЛЬ МЕНЕДЖМЕНТ"</t>
+          <t>Барилов Евгений Александрович</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
@@ -2722,30 +2718,30 @@
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>07.10.2</t>
+          <t>82.99</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr"/>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 14:07 — 10.07.2026 11:00</t>
+          <t>30.06.2026 17:59 — 09.07.2026 12:00</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>Респ Карелия, г Костомукша, шоссе Горняков, стр 284</t>
+          <t>г Москва, Романов пер, д 4</t>
         </is>
       </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=d255ff9d8c195ac53abc2fedf2afd4988a73c57f&amp;tsid=4512541003</t>
+          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=e3415418c829f6295e8f7502db2a2c9dcace8ed4&amp;tsid=4508230004</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -2761,28 +2757,27 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>4508230</t>
+          <t>4501157</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Сборный (Изделия электроустановочные и монтажные, Ящики, щиты, шкафы, пункты и комплектующие к ним, Приборы электроизмерительные, реле)
-МГ-019742, МГ-019713, МГ-019696, МГ-019665, МГ-019621, МГ-019620, МГ-019619, МГ-017109... -HESI-EX (5X20), Phoenix Contact 1277638ПеремычкаFBS 10-5, Phoenix Contact 3030213 ...ПеремычкаFBS 10-5 BU, Phoenix Contact  ...</t>
+          <t>Источники электропитания (ИБП, аккумуляторные батареи, блоки питания)...  х 1248 А·ч, включая соединительныеперемычки. Вид положительного электрода - трубчатая пластина ...  с коммутирующей арматурой, межэлементными и межряднымиперемычками, крепежами, комплектом для обслуживания АБ. Тип ...</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>АО "ИК "АРЛАН"</t>
+          <t>АО "Мосинжпроект"</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>АО "ИК "АРЛАН"</t>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>7722220390</t>
+          <t>7701885820</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -2792,7 +2787,7 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>Барилов Евгений Александрович</t>
+          <t>Сорокин Антон Павлович</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
@@ -2802,30 +2797,30 @@
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>82.99</t>
+          <t>71.12.2</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr"/>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>30.06.2026 17:59 — 09.07.2026 12:00</t>
+          <t>24.06.2026 15:40 — 22.07.2026 12:00</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Романов пер, д 4</t>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
         </is>
       </c>
       <c r="Q30" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=d255ff9d8c195ac53abc2fedf2afd4988a73c57f&amp;tsid=4508230004</t>
+          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=e3415418c829f6295e8f7502db2a2c9dcace8ed4&amp;tsid=4501157003</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -2841,150 +2836,150 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
+          <t>4499964</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Автоматика и телемеханика движения поездов... , 13552-00-00В Дроссель-трансформатор (безперемычек) ДТМ-0,17-1000М ЮКЛЯ.672 ...</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>АО "Мосинжпроект"</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>7701885820</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Сорокин Антон Павлович</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>71.12.2</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr"/>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>24.06.2026 08:46 — 15.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+        </is>
+      </c>
+      <c r="Q31" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=e3415418c829f6295e8f7502db2a2c9dcace8ed4&amp;tsid=4499964003</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 19:21</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
           <t>4504775</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники
 Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники...  Трубка пробная № 37-542-000 Соединитель-перемычка04182454 Кольцо стальное №CP48001-0305 Фильтр ...</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>7805368914</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr">
+      <c r="J32" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург</t>
         </is>
       </c>
-      <c r="K31" s="2" t="inlineStr">
+      <c r="K32" s="2" t="inlineStr">
         <is>
           <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
-      <c r="L31" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M31" s="2" t="inlineStr">
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
         <is>
           <t>46.90</t>
-        </is>
-      </c>
-      <c r="N31" s="2" t="inlineStr"/>
-      <c r="O31" s="2" t="inlineStr">
-        <is>
-          <t>27.06.2026 01:36 — 15.07.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P31" s="2" t="inlineStr">
-        <is>
-          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
-        </is>
-      </c>
-      <c r="Q31" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=d255ff9d8c195ac53abc2fedf2afd4988a73c57f&amp;tsid=4504775003</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-07 11:28</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>4501157</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Источники электропитания (ИБП, аккумуляторные батареи, блоки питания)...  х 1248 А·ч, включая соединительныеперемычки. Вид положительного электрода - трубчатая пластина ...  с коммутирующей арматурой, межэлементными и межряднымиперемычками, крепежами, комплектом для обслуживания АБ. Тип ...</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>АО "Мосинжпроект"</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>АО "МОСИНЖПРОЕКТ"</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>7701885820</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr">
-        <is>
-          <t>Сорокин Антон Павлович</t>
-        </is>
-      </c>
-      <c r="L32" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M32" s="2" t="inlineStr">
-        <is>
-          <t>71.12.2</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr"/>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 15:40 — 22.07.2026 12:00</t>
+          <t>27.06.2026 01:36 — 15.07.2026 12:00</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
       <c r="Q32" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=d255ff9d8c195ac53abc2fedf2afd4988a73c57f&amp;tsid=4501157003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=e3415418c829f6295e8f7502db2a2c9dcace8ed4&amp;tsid=4504775003</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -3000,27 +2995,28 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>4499964</t>
+          <t>4480614</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Автоматика и телемеханика движения поездов... , 13552-00-00В Дроссель-трансформатор (безперемычек) ДТМ-0,17-1000М ЮКЛЯ.672 ...</t>
+          <t>Плановое и аварийное техническое обслуживание зданий и сооружений (годовое обслуживание август 2026 - август 2027) ГК Логика молока, производственная площадка в г. Ялуторовске
+Обслуживание зданий и сооружений завода в г. Ялуторовске....  стен из газобетонных блоков Устройство металлическихперемычекс устройством штраб Усиление кирпичных стен ...</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>АО "Мосинжпроект"</t>
+          <t>АО "ЭЙЧ ЭНД ЭН"</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>АО "МОСИНЖПРОЕКТ"</t>
+          <t>АО "ЭЙЧ ЭНД ЭН"</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>7701885820</t>
+          <t>7714626332</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -3030,7 +3026,7 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Сорокин Антон Павлович</t>
+          <t>Закриев Якуб Салманович</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
@@ -3040,30 +3036,30 @@
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>71.12.2</t>
+          <t>10.51.9</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr"/>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 08:46 — 15.07.2026 12:00</t>
+          <t>08.06.2026 14:44 — 08.07.2026 23:00</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+          <t>г Москва, ул Вятская, д 27 стр 13</t>
         </is>
       </c>
       <c r="Q33" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=d255ff9d8c195ac53abc2fedf2afd4988a73c57f&amp;tsid=4499964003</t>
+          <t>https://www.b2b-center.ru/market/planovoe-i-avariinoe-tekhnicheskoe-obsluzhivanie-zdanii-i-sooruzhenii/tender-4480614/#btid=2&amp;sqh=e3415418c829f6295e8f7502db2a2c9dcace8ed4&amp;tsid=4480614004</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3079,13 +3075,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>4480614</t>
+          <t>4512370</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Плановое и аварийное техническое обслуживание зданий и сооружений (годовое обслуживание август 2026 - август 2027) ГК Логика молока, производственная площадка в г. Ялуторовске
-Обслуживание зданий и сооружений завода в г. Ялуторовске....  стен из газобетонных блоков Устройство металлическихперемычекс устройством штраб Усиление кирпичных стен ...</t>
+          <t>ТО Сплит систем Лабинск Эйч энд Эн... кондиционирования Техническое обслуживание внутреннегоблокакассетного типа мультизональной  ...блокакондиционера. Мойка теплообменника внутреннегоблокакондиционера Чистка фильтров внутреннегоблокакондиционера Чистка фильтров приточнойвентиляционной...</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3126,7 +3121,7 @@
       <c r="N34" s="2" t="inlineStr"/>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>08.06.2026 14:44 — 08.07.2026 23:00</t>
+          <t>03.07.2026 12:40 — 14.07.2026 18:30</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr">
@@ -3136,14 +3131,14 @@
       </c>
       <c r="Q34" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/planovoe-i-avariinoe-tekhnicheskoe-obsluzhivanie-zdanii-i-sooruzhenii/tender-4480614/#btid=2&amp;sqh=d255ff9d8c195ac53abc2fedf2afd4988a73c57f&amp;tsid=4480614004</t>
+          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=f38571f0054d6cc62726795ef661a590bb1229f1&amp;tsid=4512370458</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -3159,27 +3154,27 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>4512370</t>
+          <t>4501181</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>ТО Сплит систем Лабинск Эйч энд Эн... кондиционирования Техническое обслуживание внутреннегоблокакассетного типа мультизональной  ...блокакондиционера. Мойка теплообменника внутреннегоблокакондиционера Чистка фильтров внутреннегоблокакондиционера Чистка фильтров приточнойвентиляционной...</t>
+          <t>Вентиляторы промышленные и оборудование общеобменной вентиляции...  5Ф РешёткавентиляционнаяАМР 600х300М РешёткавентиляционнаяАМР 150х150М РешёткавентиляционнаяАМР 300х200М  ... мм.; масса 0,65 кгБлокконтроля сопротивления БСК-3.1 Канальный ...  533Па, габаритные размеры 700х467х2230 мм,блоков/моноблоков 5/1, в составе: - ...</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>АО "ЭЙЧ ЭНД ЭН"</t>
+          <t>АО "Мосинжпроект"</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>АО "ЭЙЧ ЭНД ЭН"</t>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>7714626332</t>
+          <t>7701885820</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -3189,7 +3184,7 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>Закриев Якуб Салманович</t>
+          <t>Сорокин Антон Павлович</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
@@ -3199,30 +3194,30 @@
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>10.51.9</t>
+          <t>71.12.2</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr"/>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 12:40 — 14.07.2026 18:30</t>
+          <t>24.06.2026 15:45 — 22.07.2026 12:00</t>
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Вятская, д 27 стр 13</t>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
         </is>
       </c>
       <c r="Q35" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=e2af420114ba61a379eed65341d8a02e5f5e76cf&amp;tsid=4512370458</t>
+          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=f38571f0054d6cc62726795ef661a590bb1229f1&amp;tsid=4501181003</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -3238,37 +3233,38 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>4501181</t>
+          <t>4501483</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Вентиляторы промышленные и оборудование общеобменной вентиляции...  5Ф РешёткавентиляционнаяАМР 600х300М РешёткавентиляционнаяАМР 150х150М РешёткавентиляционнаяАМР 300х200М  ... мм.; масса 0,65 кгБлокконтроля сопротивления БСК-3.1 Канальный ...  533Па, габаритные размеры 700х467х2230 мм,блоков/моноблоков 5/1, в составе: - ...</t>
+          <t>Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ
+Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ...  d 50x2", внутренняя резьба RTPБлокуправления наружной установки ICEFREE TR-16 ...  Оповещатель звуковой МАЯК-12-ЗМБлокуправления наружной установки ICEFREE TS- ... проводов КС-3 007004 Велос Переходвентиляционный150х100 - D150, из тонколистовой оцинкованной ...</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>АО "Мосинжпроект"</t>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>АО "МОСИНЖПРОЕКТ"</t>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>7701885820</t>
+          <t>7805368914</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
+          <t>г Санкт-Петербург</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>Сорокин Антон Павлович</t>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
@@ -3278,30 +3274,30 @@
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>71.12.2</t>
+          <t>46.90</t>
         </is>
       </c>
       <c r="N36" s="2" t="inlineStr"/>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 15:45 — 22.07.2026 12:00</t>
+          <t>25.06.2026 05:03 — 09.07.2026 12:00</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
       <c r="Q36" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=e2af420114ba61a379eed65341d8a02e5f5e76cf&amp;tsid=4501181003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=f38571f0054d6cc62726795ef661a590bb1229f1&amp;tsid=4501483003</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -3317,38 +3313,37 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>4501483</t>
+          <t>4500120</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ
-Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ...  d 50x2", внутренняя резьба RTPБлокуправления наружной установки ICEFREE TR-16 ...  Оповещатель звуковой МАЯК-12-ЗМБлокуправления наружной установки ICEFREE TS- ... проводов КС-3 007004 Велос Переходвентиляционный150х100 - D150, из тонколистовой оцинкованной ...</t>
+          <t>Коммуникационное оборудование, компьютеры, комплектующие к ним, серверное оборудование и ПО...  и кабелей – 1 компл. Удаленныйблок(репитер) BSF414 , питание 220В,  ... 2х2 Комбайнер специализированный OMU Side (блок1) OMUSC1 Комбайнер специализированный OMU ... контроллер для мониторинга в FlexGain View,вентиляционнаяпанель с фильтрами, комплект кабелей, ...</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+          <t>АО "Мосинжпроект"</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>7805368914</t>
+          <t>7701885820</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>г Санкт-Петербург</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
+          <t>Сорокин Антон Павлович</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
@@ -3358,30 +3353,30 @@
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>46.90</t>
+          <t>71.12.2</t>
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr"/>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>25.06.2026 05:03 — 09.07.2026 12:00</t>
+          <t>24.06.2026 09:48 — 15.07.2026 12:00</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
         </is>
       </c>
       <c r="Q37" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=e2af420114ba61a379eed65341d8a02e5f5e76cf&amp;tsid=4501483003</t>
+          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=f38571f0054d6cc62726795ef661a590bb1229f1&amp;tsid=4500120003</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -3397,27 +3392,28 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>4500120</t>
+          <t>4496006</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Коммуникационное оборудование, компьютеры, комплектующие к ним, серверное оборудование и ПО...  и кабелей – 1 компл. Удаленныйблок(репитер) BSF414 , питание 220В,  ... 2х2 Комбайнер специализированный OMU Side (блок1) OMUSC1 Комбайнер специализированный OMU ... контроллер для мониторинга в FlexGain View,вентиляционнаяпанель с фильтрами, комплект кабелей, ...</t>
+          <t>Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп
+Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп... -316 ***Петля крепежная стальная ***Платаблокауправления ZC5 CAME ***Средство чистящее " ... /распылитель для чаши Генуя ***РешеткавентиляционнаяРВ-1 225Х225 ***Петля анкерная 0 ... мл ***Папка с зажимом ***РешеткавентиляционнаяРВ-1 325Х125 ***Папка на кольцах ...</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>АО "Мосинжпроект"</t>
+          <t>ООО "СИБУР"</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>АО "МОСИНЖПРОЕКТ"</t>
+          <t>ООО "СИБУР"</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>7701885820</t>
+          <t>7727576505</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -3427,7 +3423,7 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>Сорокин Антон Павлович</t>
+          <t>Карисалов Михаил Юрьевич</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
@@ -3437,30 +3433,30 @@
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>71.12.2</t>
+          <t>70.10</t>
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr"/>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 09:48 — 15.07.2026 12:00</t>
+          <t>20.06.2026 16:19 — 11.07.2026 12:00</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+          <t>г Москва, ул Кржижановского, д 16 к 3</t>
         </is>
       </c>
       <c r="Q38" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=e2af420114ba61a379eed65341d8a02e5f5e76cf&amp;tsid=4500120003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-nelikvidnykh-tmts-tarelki-dlia-filtra-prokladki-dvigatel/tender-4496006/#btid=2&amp;sqh=f38571f0054d6cc62726795ef661a590bb1229f1&amp;tsid=4496006003</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:28</t>
+          <t>2026-07-07 19:21</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -3471,33 +3467,32 @@
       <c r="C39" s="2" t="inlineStr"/>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Работы</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>4496006</t>
+          <t>4129930</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп
-Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп... -316 ***Петля крепежная стальная ***Платаблокауправления ZC5 CAME ***Средство чистящее " ... /распылитель для чаши Генуя ***РешеткавентиляционнаяРВ-1 225Х225 ***Петля анкерная 0 ... мл ***Папка с зажимом ***РешеткавентиляционнаяРВ-1 325Х125 ***Папка на кольцах ...</t>
+          <t>Реализация материалов для ремонта (напольные покрытия, настенные покрытия, окна, двери и т.д.) с АО "Мальцовский портландцемент"Блокдверной балконныйБлокдверной филенчатый ДГ 21х9Блококонный 1500х1000 ммБлококонный 1770х1700 мм Желоб ...  Docke Рама оконная 3000х1200 мм Решеткавентиляционнаянаружная Ручка оконная ГОСТ 5087-80 ...</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>ООО "СИБУР"</t>
+          <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>ООО "СИБУР"</t>
+          <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>7727576505</t>
+          <t>7708117908</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
@@ -3507,7 +3502,7 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Карисалов Михаил Юрьевич</t>
+          <t>Шматов Вячеслав Вячеславович</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
@@ -3517,107 +3512,28 @@
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>70.10</t>
+          <t>23.51</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr"/>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>20.06.2026 16:19 — 11.07.2026 12:00</t>
+          <t>06.08.2025 14:33 — 07.08.2026 12:00</t>
         </is>
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Кржижановского, д 16 к 3</t>
+          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
         </is>
       </c>
       <c r="Q39" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nelikvidnykh-tmts-tarelki-dlia-filtra-prokladki-dvigatel/tender-4496006/#btid=2&amp;sqh=e2af420114ba61a379eed65341d8a02e5f5e76cf&amp;tsid=4496006003</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-07 11:28</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>Работы</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>4129930</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>Реализация материалов для ремонта (напольные покрытия, настенные покрытия, окна, двери и т.д.) с АО "Мальцовский портландцемент"Блокдверной балконныйБлокдверной филенчатый ДГ 21х9Блококонный 1500х1000 ммБлококонный 1770х1700 мм Желоб ...  Docke Рама оконная 3000х1200 мм Решеткавентиляционнаянаружная Ручка оконная ГОСТ 5087-80 ...</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>АО "ЦЕМРОС"</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr">
-        <is>
-          <t>АО "ЦЕМРОС"</t>
-        </is>
-      </c>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>7708117908</t>
-        </is>
-      </c>
-      <c r="J40" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K40" s="2" t="inlineStr">
-        <is>
-          <t>Шматов Вячеслав Вячеславович</t>
-        </is>
-      </c>
-      <c r="L40" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M40" s="2" t="inlineStr">
-        <is>
-          <t>23.51</t>
-        </is>
-      </c>
-      <c r="N40" s="2" t="inlineStr"/>
-      <c r="O40" s="2" t="inlineStr">
-        <is>
-          <t>06.08.2025 14:33 — 07.08.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P40" s="2" t="inlineStr">
-        <is>
-          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
-        </is>
-      </c>
-      <c r="Q40" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=e2af420114ba61a379eed65341d8a02e5f5e76cf&amp;tsid=4129930003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=f38571f0054d6cc62726795ef661a590bb1229f1&amp;tsid=4129930003</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q40"/>
+  <autoFilter ref="A1:Q39"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -3657,7 +3573,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId39"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-08 09:22 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -622,14 +622,14 @@
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/stroitelnye-materialy-postavka-v-nakhodku-dlia-ooo-svetloe-postavka/tender-4515159/#btid=2&amp;sqh=8e563bad4224f0e48f0af61695f5f4c8f562ba44&amp;tsid=4515159004</t>
+          <t>https://www.b2b-center.ru/market/stroitelnye-materialy-postavka-v-nakhodku-dlia-ooo-svetloe-postavka/tender-4515159/#btid=2&amp;sqh=e7a55a0d5d41409a139acf7b95567d4018bbe91b&amp;tsid=4515159004</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -702,14 +702,14 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=8e563bad4224f0e48f0af61695f5f4c8f562ba44&amp;tsid=4510835003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=e7a55a0d5d41409a139acf7b95567d4018bbe91b&amp;tsid=4510835003</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -781,14 +781,14 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/remont-dorozhnoi-plitki-na-pod-ezdnoi-i-vyezdnoi-doroge-ot-glavnogo/tender-4506366/#btid=2&amp;sqh=8e563bad4224f0e48f0af61695f5f4c8f562ba44&amp;tsid=4506366458</t>
+          <t>https://www.b2b-center.ru/app/market-next/remont-dorozhnoi-plitki-na-pod-ezdnoi-i-vyezdnoi-doroge-ot-glavnogo/tender-4506366/#btid=2&amp;sqh=e7a55a0d5d41409a139acf7b95567d4018bbe91b&amp;tsid=4506366458</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -857,14 +857,14 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=8e563bad4224f0e48f0af61695f5f4c8f562ba44&amp;tsid=4503612458</t>
+          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=e7a55a0d5d41409a139acf7b95567d4018bbe91b&amp;tsid=4503612458</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -936,14 +936,14 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=8e563bad4224f0e48f0af61695f5f4c8f562ba44&amp;tsid=4130106003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=e7a55a0d5d41409a139acf7b95567d4018bbe91b&amp;tsid=4130106003</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1015,14 +1015,14 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=c7e9a6366e60bddb02c708506fc1962f4e205a53&amp;tsid=4498936003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=65b3211d179906b2f900c53c4e6927f2f19c4f5e&amp;tsid=4498936003</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1095,14 +1095,14 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=587cba0d7823c00bf4cffa8986d257d91a51d340&amp;tsid=4497016004</t>
+          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=51ed30504898ec176bd44a7009092b0697483118&amp;tsid=4497016004</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1170,14 +1170,14 @@
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=7dbda509515c8bcaf34ece759fdb41e1f4a74d2d&amp;tsid=4512196458</t>
+          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=a5886426bebe1763852434306a3c3797e5a69302&amp;tsid=4512196458</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1249,14 +1249,14 @@
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=7dbda509515c8bcaf34ece759fdb41e1f4a74d2d&amp;tsid=4512292004</t>
+          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=a5886426bebe1763852434306a3c3797e5a69302&amp;tsid=4512292004</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1331,14 +1331,14 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=590be7cb5732e94d1262344f871803b3ef2abb29&amp;tsid=4475879003</t>
+          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=611fe3fb002a9aabd1dc3af49ad2af72c1d00d53&amp;tsid=4475879003</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1354,39 +1354,35 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>4508331</t>
+          <t>4514583</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Плита ПАГ-14А600ГОСТ 25912-2015 для ООО ГРК Амикан. Требуется жесткая упаковка по ГОСТу КП по форме ТД Полиметалл. В цену включить стоимость доставки до адреса в г. Лесосибирск и обрешетки. При подаче аналогов необходимо приложить тех. документацию</t>
+          <t>Закупка ЖБИ (плитыПДН3*1,5)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>7805368914</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>г Санкт-Петербург</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
-        </is>
-      </c>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1394,30 +1390,30 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>46.90</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr"/>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>01.07.2026 05:44 — 08.07.2026 10:00</t>
+          <t>06.07.2026 15:00 — 09.07.2026 12:00</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/plita-pag-14a600-gost-25912-2015-dlia-ooo-grk-amikan-trebuetsia/tender-4508331/#btid=2&amp;sqh=5b1aeb5217f9925cfe184b7dc644e4672b8e7853&amp;tsid=4508331004</t>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-plity-pdn-3-1-5/tender-4514583/#btid=2&amp;sqh=f177e1e5925ec7c45574fa0eba249b0b78a6969c&amp;tsid=4514583458</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1433,12 +1429,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>4514583</t>
+          <t>4516217</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Закупка ЖБИ (плитыПДН3*1,5)</t>
+          <t>ТМЦЖБИи песок</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1475,7 +1471,7 @@
       <c r="N13" s="2" t="inlineStr"/>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>06.07.2026 15:00 — 09.07.2026 12:00</t>
+          <t>07.07.2026 14:31 — 10.07.2026 10:00</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -1485,14 +1481,14 @@
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-plity-pdn-3-1-5/tender-4514583/#btid=2&amp;sqh=dc1fd934a3fc31dafe24919d7248ef2c5f3ef41c&amp;tsid=4514583458</t>
+          <t>https://www.b2b-center.ru/app/market-next/tmts-zhbi-i-pesok/tender-4516217/#btid=2&amp;sqh=ca0badfa5ad2b3baf05984ac65950e28246e3eac&amp;tsid=4516217458</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1508,12 +1504,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>4516217</t>
+          <t>4513278</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>ТМЦЖБИи песок</t>
+          <t>ЖБИблоки ФБС</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1550,7 +1546,7 @@
       <c r="N14" s="2" t="inlineStr"/>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>07.07.2026 14:31 — 10.07.2026 10:00</t>
+          <t>06.07.2026 04:17 — 09.07.2026 00:00</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -1560,14 +1556,14 @@
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/tmts-zhbi-i-pesok/tender-4516217/#btid=2&amp;sqh=08a697ca4c161444f3d019ceaddceab59e726906&amp;tsid=4516217458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-bloki-fbs/tender-4513278/#btid=2&amp;sqh=ca0badfa5ad2b3baf05984ac65950e28246e3eac&amp;tsid=4513278458</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1578,32 +1574,32 @@
       <c r="C15" s="2" t="inlineStr"/>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Поставка</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>4513278</t>
+          <t>4514839</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>ЖБИблоки ФБС</t>
+          <t>12-х-1 Заключение договора на поставку материалов для наружных сетей водоснабжения и водоотведения на объект строительства «Дальневосточный детский центр отдыха и оздоровления в Хабаровском крае». (9 лотов) Лот №1 ВодоснабжениеЖБИ</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "ПРОМСТРОЙ"</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "ПРОМСТРОЙ"</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>9723169975</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -1611,7 +1607,11 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Султанов Владислав Назипович</t>
+        </is>
+      </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1619,30 +1619,30 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>71.12.2</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr"/>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>06.07.2026 04:17 — 09.07.2026 00:00</t>
+          <t>06.07.2026 16:45 — 10.07.2026 11:00</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Москва, Волгоградский пр-кт, д 42 к 5, ком 9</t>
         </is>
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-bloki-fbs/tender-4513278/#btid=2&amp;sqh=08a697ca4c161444f3d019ceaddceab59e726906&amp;tsid=4513278458</t>
+          <t>https://www.b2b-center.ru/market/12-kh-1-zakliuchenie-dogovora-na-postavku-materialov-dlia-naruzhnykh-setei/tender-4514839/#btid=2&amp;sqh=ca0badfa5ad2b3baf05984ac65950e28246e3eac&amp;tsid=4514839004</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1653,32 +1653,32 @@
       <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Поставка</t>
+          <t>Прочее</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>4514839</t>
+          <t>4510341</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>12-х-1 Заключение договора на поставку материалов для наружных сетей водоснабжения и водоотведения на объект строительства «Дальневосточный детский центр отдыха и оздоровления в Хабаровском крае». (9 лотов) Лот №1 ВодоснабжениеЖБИ</t>
+          <t>ЖБИ(чеч 34\25 7510 \ 17338)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>ООО "ПРОМСТРОЙ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>ООО "ПРОМСТРОЙ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>9723169975</t>
+          <t>7724498866</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Султанов Владислав Назипович</t>
+          <t>Городний Анатолий Валерьевич</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -1698,30 +1698,30 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>71.12.2</t>
+          <t>46.73</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr"/>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>06.07.2026 16:45 — 10.07.2026 11:00</t>
+          <t>02.07.2026 09:54 — 08.07.2026 15:00</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Волгоградский пр-кт, д 42 к 5, ком 9</t>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
         </is>
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/12-kh-1-zakliuchenie-dogovora-na-postavku-materialov-dlia-naruzhnykh-setei/tender-4514839/#btid=2&amp;sqh=08a697ca4c161444f3d019ceaddceab59e726906&amp;tsid=4514839004</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=ca0badfa5ad2b3baf05984ac65950e28246e3eac&amp;tsid=4510341459</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1737,12 +1737,12 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>4510341</t>
+          <t>4510662</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>ЖБИ(чеч 34\25 7510 \ 17338)</t>
+          <t>(ЖБИизделия/кольца колодезные, плиты ПК15)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1783,7 +1783,7 @@
       <c r="N17" s="2" t="inlineStr"/>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>02.07.2026 09:54 — 08.07.2026 15:00</t>
+          <t>02.07.2026 12:00 — 09.07.2026 13:00</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -1793,14 +1793,14 @@
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=08a697ca4c161444f3d019ceaddceab59e726906&amp;tsid=4510341459</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-izdeliia-koltsa-kolodeznye-plity-pk15/tender-4510662/#btid=2&amp;sqh=ca0badfa5ad2b3baf05984ac65950e28246e3eac&amp;tsid=4510662459</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1816,27 +1816,27 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>4508347</t>
+          <t>4510504</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>ЖБИКЕМГРЭС</t>
+          <t>(Заявка № ДОР-17560) Лестницы/ЖБИ</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>7724498866</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1844,7 +1844,11 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1852,30 +1856,30 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>46.73</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr"/>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>01.07.2026 05:45 — 10.07.2026 00:00</t>
+          <t>02.07.2026 10:55 — 09.07.2026 13:00</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
         </is>
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=08a697ca4c161444f3d019ceaddceab59e726906&amp;tsid=4508347458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zaiavka-dor-17560-lestnitsy-zhbi/tender-4510504/#btid=2&amp;sqh=ca0badfa5ad2b3baf05984ac65950e28246e3eac&amp;tsid=4510504459</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1891,27 +1895,27 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>4489772</t>
+          <t>4508347</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы 1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы</t>
+          <t>ЖБИКЕМГРЭС</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>7736583259</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -1919,11 +1923,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>Масько Александр Вадимович</t>
-        </is>
-      </c>
+      <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1931,30 +1931,30 @@
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>70.10</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr"/>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>16.06.2026 11:00 — 16.07.2026 12:00</t>
+          <t>01.07.2026 05:45 — 10.07.2026 00:00</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Старая Басманная, д 12 стр 1</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=08a697ca4c161444f3d019ceaddceab59e726906&amp;tsid=4489772003</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=ca0badfa5ad2b3baf05984ac65950e28246e3eac&amp;tsid=4508347458</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1970,37 +1970,37 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>4474790</t>
+          <t>4489772</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
+          <t>1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы 1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>4704012472</t>
+          <t>7736583259</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Габидуллин Тимур Махмудович</t>
+          <t>Масько Александр Вадимович</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -2010,30 +2010,30 @@
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>17.12</t>
+          <t>70.10</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr"/>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>03.06.2026 09:59 — 30.07.2026 20:00</t>
+          <t>16.06.2026 11:00 — 16.07.2026 12:00</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+          <t>г Москва, ул Старая Басманная, д 12 стр 1</t>
         </is>
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=08a697ca4c161444f3d019ceaddceab59e726906&amp;tsid=4474790003</t>
+          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=ca0badfa5ad2b3baf05984ac65950e28246e3eac&amp;tsid=4489772003</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -2049,37 +2049,37 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>4180328</t>
+          <t>4474790</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, г.Диксон). ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, ПГТ Диксон).</t>
+          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>7714456916</t>
+          <t>4704012472</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
+          <t>Ленинградская обл</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Наумов Андрей Александрович</t>
+          <t>Габидуллин Тимур Махмудович</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -2089,30 +2089,30 @@
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>70.22</t>
+          <t>17.12</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr"/>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>24.09.2025 15:32 — 23.07.2026 12:00</t>
+          <t>03.06.2026 09:59 — 30.07.2026 20:00</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Денежный пер, д 9/6</t>
+          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
         </is>
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=08a697ca4c161444f3d019ceaddceab59e726906&amp;tsid=4180328003</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=ca0badfa5ad2b3baf05984ac65950e28246e3eac&amp;tsid=4474790003</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2128,37 +2128,37 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>3973258</t>
+          <t>4180328</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
+          <t>ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, г.Диксон). ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, ПГТ Диксон).</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>4704012472</t>
+          <t>7714456916</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Габидуллин Тимур Махмудович</t>
+          <t>Наумов Андрей Александрович</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
@@ -2168,30 +2168,30 @@
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>17.12</t>
+          <t>70.22</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr"/>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>10.03.2025 00:48 — 30.07.2026 23:00</t>
+          <t>24.09.2025 15:32 — 23.07.2026 12:00</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+          <t>г Москва, Денежный пер, д 9/6</t>
         </is>
       </c>
       <c r="Q22" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=08a697ca4c161444f3d019ceaddceab59e726906&amp;tsid=3973258003</t>
+          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=ca0badfa5ad2b3baf05984ac65950e28246e3eac&amp;tsid=4180328003</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2202,40 +2202,44 @@
       <c r="C23" s="2" t="inlineStr"/>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Поставка</t>
+          <t>Прочее</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>4513525</t>
+          <t>3973258</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Поставка модульных защитных сооруженийЗДАНИЕ ЗАЩИТНОЕ ДЛЯ УКРЫТИЯ 4,4*2,4*2,2МЖЕЛЕЗОБЕТОННОЕСБОРНОЕ</t>
+          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>4704012472</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr"/>
+          <t>Ленинградская обл</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Габидуллин Тимур Махмудович</t>
+        </is>
+      </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -2243,30 +2247,30 @@
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>17.12</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr"/>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>06.07.2026 08:36 — 10.07.2026 14:00</t>
+          <t>10.03.2025 00:48 — 30.07.2026 23:00</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
         </is>
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/postavka-modulnykh-zashchitnykh-sooruzhenii/tender-4513525/#btid=2&amp;sqh=5ca340ddd1aafc75928e9226e262d7f80332171b&amp;tsid=4513525458</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=ca0badfa5ad2b3baf05984ac65950e28246e3eac&amp;tsid=3973258003</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2277,15 +2281,90 @@
       <c r="C24" s="2" t="inlineStr"/>
       <c r="D24" s="2" t="inlineStr">
         <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>4513525</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Поставка модульных защитных сооруженийЗДАНИЕ ЗАЩИТНОЕ ДЛЯ УКРЫТИЯ 4,4*2,4*2,2МЖЕЛЕЗОБЕТОННОЕСБОРНОЕ</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>06.07.2026 08:36 — 10.07.2026 14:00</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q24" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/postavka-modulnykh-zashchitnykh-sooruzhenii/tender-4513525/#btid=2&amp;sqh=f2ccdf8699fcd02c28a40854bc3aff3687fb23e1&amp;tsid=4513525458</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08 09:22</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr"/>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>4513563</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>Блок ФБС 12.4.6-Т-и
 Кольцо стеновое КС 20.9 ГОСТ 8020-2016
@@ -2294,137 +2373,62 @@
 Кольцо стеновое КС 20.9 ГОСТ 8020-20164513563 ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "ТОРГОВЫЙ ДОМ ПОЛИМЕТАЛЛ"Железобетонные изделия</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="I25" s="2" t="inlineStr">
         <is>
           <t>7805368914</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="J25" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr">
+      <c r="K25" s="2" t="inlineStr">
         <is>
           <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="inlineStr">
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
         <is>
           <t>46.90</t>
-        </is>
-      </c>
-      <c r="N24" s="2" t="inlineStr"/>
-      <c r="O24" s="2" t="inlineStr">
-        <is>
-          <t>06.07.2026 08:49 — 10.07.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P24" s="2" t="inlineStr">
-        <is>
-          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
-        </is>
-      </c>
-      <c r="Q24" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/blok-fbs-12-4-6-t-i-koltso-stenovoe-ks-20-9-gost-8020-2016-na-k-pm/tender-4513563/#btid=2&amp;sqh=5ca340ddd1aafc75928e9226e262d7f80332171b&amp;tsid=4513563004</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-07 19:21</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr"/>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>Поставка</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>4512260</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>ТМЦ. Срочный отбор предложений на право заключения договора поставкижелезобетонных изделийдля нужд филиала «Канская теплосеть» АО «Енисейская ТГК (ТГК-13)».</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>9725042029</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr"/>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M25" s="2" t="inlineStr">
-        <is>
-          <t>64.20</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr"/>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 11:52 — 08.07.2026 12:00</t>
+          <t>06.07.2026 08:49 — 10.07.2026 12:00</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
       <c r="Q25" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/tmts-srochnyi-otbor-predlozhenii-na-pravo-zakliucheniia-dogovora-postavki/tender-4512260/#btid=2&amp;sqh=5ca340ddd1aafc75928e9226e262d7f80332171b&amp;tsid=4512260458</t>
+          <t>https://www.b2b-center.ru/market/blok-fbs-12-4-6-t-i-koltso-stenovoe-ks-20-9-gost-8020-2016-na-k-pm/tender-4513563/#btid=2&amp;sqh=f2ccdf8699fcd02c28a40854bc3aff3687fb23e1&amp;tsid=4513563004</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2435,36 +2439,32 @@
       <c r="C26" s="2" t="inlineStr"/>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Поставка</t>
+          <t>Прочее</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>4511621</t>
+          <t>4517499</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Закупка аккумуляторных батарей (залитых) для нужд АО "Павловск Неруд" с поставкой в Августе 2026г.
-Обязательная расценка стоимости доставки, возможен забор груза на условиях самовывоза.
-В ТКП просьба отразить локацию склада отгрузки.
-ТКП БЕЗ указания стоимости доставки рассматриваться НЕ БУДУТ.
-Заказчик АО "Павловск Неруд" предприятие АО "Национальная нерудная компания"Аккумулятор ТН-550Перемычкам/ц для АКБ 115,5мм ТН-550Перемычкам/ц для АКБ 212,0мм ТН-550 Транспортная услуга</t>
+          <t>КРЫШКА-ПАТРУБОК 200-Т-535СБ ПК-40; ЗАГЛУШКА НА КЛАПАН СД К-5976.00.00 СБ; КРЫШКА 200-Т-525СБ ПК-40;ПЕРЕМЫЧКАД/ПРОДУВКИ ППХ 200-Т-530 СБ</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>АО "ННК"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>АО "ННК-ОЙЛ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>5032049030</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -2472,11 +2472,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>Худайнатов Эдуард Юрьевич</t>
-        </is>
-      </c>
+      <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -2484,30 +2480,30 @@
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>70.22</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr"/>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 06:22 — 08.07.2026 11:00</t>
+          <t>08.07.2026 10:53 — 10.07.2026 12:00</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул 1-я Тверская-Ямская, д 5, помещ 1012</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q26" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zakupka-akkumuliatornykh-batarei-zalitykh-dlia-nuzhd-ao-pavlovsk-nerud/tender-4511621/#btid=2&amp;sqh=e3415418c829f6295e8f7502db2a2c9dcace8ed4&amp;tsid=4511621004</t>
+          <t>https://www.b2b-center.ru/app/market-next/kryshka-patrubok-200-t-535sb-pk-40-zaglushka-na-klapan-sd-k-5976-00-00/tender-4517499/#btid=2&amp;sqh=a741c4d6737d6b95143fe98c39a13a7a3c409e1a&amp;tsid=4517499458</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -2523,35 +2519,39 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>4511787</t>
+          <t>4512541</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>ЗЧ к автотранспорту... /66 ТЕРМОСТАТ ТС-107-1306100-06ПЕРЕМЫЧКААКБ КЛЕММА-КЛЕММА ПП 500-50 ...</t>
+          <t>Запасные части CAT.... -3748 Cat Опора 348-9537 CatПеремычка140-0860 Cat Скоба 8X-3130 ...</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>1004001744</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr"/>
+          <t>Респ Карелия</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "СЕВЕРСТАЛЬ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -2559,30 +2559,30 @@
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>07.10.2</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr"/>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 08:32 — 08.07.2026 00:00</t>
+          <t>03.07.2026 14:07 — 10.07.2026 11:00</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>Респ Карелия, г Костомукша, шоссе Горняков, стр 284</t>
         </is>
       </c>
       <c r="Q27" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zch-k-avtotransportu/tender-4511787/#btid=2&amp;sqh=e3415418c829f6295e8f7502db2a2c9dcace8ed4&amp;tsid=4511787458</t>
+          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=a741c4d6737d6b95143fe98c39a13a7a3c409e1a&amp;tsid=4512541003</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -2598,37 +2598,38 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>4512541</t>
+          <t>4508230</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Запасные части CAT.... -3748 Cat Опора 348-9537 CatПеремычка140-0860 Cat Скоба 8X-3130 ...</t>
+          <t>Сборный (Изделия электроустановочные и монтажные, Ящики, щиты, шкафы, пункты и комплектующие к ним, Приборы электроизмерительные, реле)
+МГ-019742, МГ-019713, МГ-019696, МГ-019665, МГ-019621, МГ-019620, МГ-019619, МГ-017109... -HESI-EX (5X20), Phoenix Contact 1277638ПеремычкаFBS 10-5, Phoenix Contact 3030213 ...ПеремычкаFBS 10-5 BU, Phoenix Contact  ...</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
+          <t>АО "ИК "АРЛАН"</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
+          <t>АО "ИК "АРЛАН"</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>1004001744</t>
+          <t>7722220390</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>Респ Карелия</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "СЕВЕРСТАЛЬ МЕНЕДЖМЕНТ"</t>
+          <t>Барилов Евгений Александрович</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
@@ -2638,30 +2639,30 @@
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>07.10.2</t>
+          <t>82.99</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr"/>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 14:07 — 10.07.2026 11:00</t>
+          <t>30.06.2026 17:59 — 09.07.2026 12:00</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>Респ Карелия, г Костомукша, шоссе Горняков, стр 284</t>
+          <t>г Москва, Романов пер, д 4</t>
         </is>
       </c>
       <c r="Q28" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=e3415418c829f6295e8f7502db2a2c9dcace8ed4&amp;tsid=4512541003</t>
+          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=a741c4d6737d6b95143fe98c39a13a7a3c409e1a&amp;tsid=4508230004</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -2677,28 +2678,27 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>4508230</t>
+          <t>4501157</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Сборный (Изделия электроустановочные и монтажные, Ящики, щиты, шкафы, пункты и комплектующие к ним, Приборы электроизмерительные, реле)
-МГ-019742, МГ-019713, МГ-019696, МГ-019665, МГ-019621, МГ-019620, МГ-019619, МГ-017109... -HESI-EX (5X20), Phoenix Contact 1277638ПеремычкаFBS 10-5, Phoenix Contact 3030213 ...ПеремычкаFBS 10-5 BU, Phoenix Contact  ...</t>
+          <t>Источники электропитания (ИБП, аккумуляторные батареи, блоки питания)...  х 1248 А·ч, включая соединительныеперемычки. Вид положительного электрода - трубчатая пластина ...  с коммутирующей арматурой, межэлементными и межряднымиперемычками, крепежами, комплектом для обслуживания АБ. Тип ...</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>АО "ИК "АРЛАН"</t>
+          <t>АО "Мосинжпроект"</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>АО "ИК "АРЛАН"</t>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>7722220390</t>
+          <t>7701885820</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>Барилов Евгений Александрович</t>
+          <t>Сорокин Антон Павлович</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
@@ -2718,30 +2718,30 @@
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>82.99</t>
+          <t>71.12.2</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr"/>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>30.06.2026 17:59 — 09.07.2026 12:00</t>
+          <t>24.06.2026 15:40 — 22.07.2026 12:00</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Романов пер, д 4</t>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
         </is>
       </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=e3415418c829f6295e8f7502db2a2c9dcace8ed4&amp;tsid=4508230004</t>
+          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=a741c4d6737d6b95143fe98c39a13a7a3c409e1a&amp;tsid=4501157003</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -2757,12 +2757,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>4501157</t>
+          <t>4499964</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Источники электропитания (ИБП, аккумуляторные батареи, блоки питания)...  х 1248 А·ч, включая соединительныеперемычки. Вид положительного электрода - трубчатая пластина ...  с коммутирующей арматурой, межэлементными и межряднымиперемычками, крепежами, комплектом для обслуживания АБ. Тип ...</t>
+          <t>Автоматика и телемеханика движения поездов... , 13552-00-00В Дроссель-трансформатор (безперемычек) ДТМ-0,17-1000М ЮКЛЯ.672 ...</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -2803,7 +2803,7 @@
       <c r="N30" s="2" t="inlineStr"/>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 15:40 — 22.07.2026 12:00</t>
+          <t>24.06.2026 08:46 — 15.07.2026 12:00</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
@@ -2813,14 +2813,14 @@
       </c>
       <c r="Q30" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=e3415418c829f6295e8f7502db2a2c9dcace8ed4&amp;tsid=4501157003</t>
+          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=a741c4d6737d6b95143fe98c39a13a7a3c409e1a&amp;tsid=4499964003</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -2836,37 +2836,38 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>4499964</t>
+          <t>4504775</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Автоматика и телемеханика движения поездов... , 13552-00-00В Дроссель-трансформатор (безперемычек) ДТМ-0,17-1000М ЮКЛЯ.672 ...</t>
+          <t>Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники
+Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники...  Трубка пробная № 37-542-000 Соединитель-перемычка04182454 Кольцо стальное №CP48001-0305 Фильтр ...</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>АО "Мосинжпроект"</t>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>АО "МОСИНЖПРОЕКТ"</t>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>7701885820</t>
+          <t>7805368914</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
+          <t>г Санкт-Петербург</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>Сорокин Антон Павлович</t>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
@@ -2876,30 +2877,30 @@
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>71.12.2</t>
+          <t>46.90</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr"/>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 08:46 — 15.07.2026 12:00</t>
+          <t>27.06.2026 01:36 — 15.07.2026 12:00</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
       <c r="Q31" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=e3415418c829f6295e8f7502db2a2c9dcace8ed4&amp;tsid=4499964003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=a741c4d6737d6b95143fe98c39a13a7a3c409e1a&amp;tsid=4504775003</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -2915,38 +2916,38 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>4504775</t>
+          <t>4480614</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники
-Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники...  Трубка пробная № 37-542-000 Соединитель-перемычка04182454 Кольцо стальное №CP48001-0305 Фильтр ...</t>
+          <t>Плановое и аварийное техническое обслуживание зданий и сооружений (годовое обслуживание август 2026 - август 2027) ГК Логика молока, производственная площадка в г. Ялуторовске
+Обслуживание зданий и сооружений завода в г. Ялуторовске....  стен из газобетонных блоков Устройство металлическихперемычекс устройством штраб Усиление кирпичных стен ...</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+          <t>АО "ЭЙЧ ЭНД ЭН"</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+          <t>АО "ЭЙЧ ЭНД ЭН"</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>7805368914</t>
+          <t>7714626332</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>г Санкт-Петербург</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
+          <t>Закриев Якуб Салманович</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
@@ -2956,30 +2957,30 @@
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>46.90</t>
+          <t>10.51.9</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr"/>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>27.06.2026 01:36 — 15.07.2026 12:00</t>
+          <t>08.06.2026 14:44 — 08.07.2026 23:00</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
+          <t>г Москва, ул Вятская, д 27 стр 13</t>
         </is>
       </c>
       <c r="Q32" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=e3415418c829f6295e8f7502db2a2c9dcace8ed4&amp;tsid=4504775003</t>
+          <t>https://www.b2b-center.ru/market/planovoe-i-avariinoe-tekhnicheskoe-obsluzhivanie-zdanii-i-sooruzhenii/tender-4480614/#btid=2&amp;sqh=a741c4d6737d6b95143fe98c39a13a7a3c409e1a&amp;tsid=4480614004</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -2995,28 +2996,28 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>4480614</t>
+          <t>4449201</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Плановое и аварийное техническое обслуживание зданий и сооружений (годовое обслуживание август 2026 - август 2027) ГК Логика молока, производственная площадка в г. Ялуторовске
-Обслуживание зданий и сооружений завода в г. Ялуторовске....  стен из газобетонных блоков Устройство металлическихперемычекс устройством штраб Усиление кирпичных стен ...</t>
+          <t>Реализация НВИ, Оборудование теплообменное; Оборудование емкостное; Запчасти и узлы теплообменного оборудования; Запчасти и узлы емкостного оборудования;
+Продажа НВИ согласно прилагаемого перечня. 110-Емкостное и теп-ое об-е; 136-Запчасти и узлы емкостного и теплообПрокладка сперемычкамидля теплообменников ПУТГм-Б-09-01( ... . Е-21504.05.06 Прокладка сперемычкамидля теплообменников ПУТГм-Б-09-01 ...</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>АО "ЭЙЧ ЭНД ЭН"</t>
+          <t>ООО "СИБУР"</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>АО "ЭЙЧ ЭНД ЭН"</t>
+          <t>ООО "СИБУР"</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>7714626332</t>
+          <t>7727576505</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -3026,7 +3027,7 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Закриев Якуб Салманович</t>
+          <t>Карисалов Михаил Юрьевич</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
@@ -3036,30 +3037,30 @@
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>10.51.9</t>
+          <t>70.10</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr"/>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>08.06.2026 14:44 — 08.07.2026 23:00</t>
+          <t>15.05.2026 06:57 — 10.07.2026 12:00</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Вятская, д 27 стр 13</t>
+          <t>г Москва, ул Кржижановского, д 16 к 3</t>
         </is>
       </c>
       <c r="Q33" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/planovoe-i-avariinoe-tekhnicheskoe-obsluzhivanie-zdanii-i-sooruzhenii/tender-4480614/#btid=2&amp;sqh=e3415418c829f6295e8f7502db2a2c9dcace8ed4&amp;tsid=4480614004</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nvi-oborudovanie-teploobmennoe-oborudovanie-emkostnoe/tender-4449201/#btid=2&amp;sqh=a741c4d6737d6b95143fe98c39a13a7a3c409e1a&amp;tsid=4449201003</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3131,14 +3132,14 @@
       </c>
       <c r="Q34" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=f38571f0054d6cc62726795ef661a590bb1229f1&amp;tsid=4512370458</t>
+          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=ad5c728ff17738e7bd83d093069a0c2a65996cc5&amp;tsid=4512370458</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -3210,14 +3211,14 @@
       </c>
       <c r="Q35" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=f38571f0054d6cc62726795ef661a590bb1229f1&amp;tsid=4501181003</t>
+          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=ad5c728ff17738e7bd83d093069a0c2a65996cc5&amp;tsid=4501181003</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -3290,14 +3291,14 @@
       </c>
       <c r="Q36" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=f38571f0054d6cc62726795ef661a590bb1229f1&amp;tsid=4501483003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=ad5c728ff17738e7bd83d093069a0c2a65996cc5&amp;tsid=4501483003</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -3369,14 +3370,14 @@
       </c>
       <c r="Q37" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=f38571f0054d6cc62726795ef661a590bb1229f1&amp;tsid=4500120003</t>
+          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=ad5c728ff17738e7bd83d093069a0c2a65996cc5&amp;tsid=4500120003</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -3449,14 +3450,14 @@
       </c>
       <c r="Q38" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nelikvidnykh-tmts-tarelki-dlia-filtra-prokladki-dvigatel/tender-4496006/#btid=2&amp;sqh=f38571f0054d6cc62726795ef661a590bb1229f1&amp;tsid=4496006003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-nelikvidnykh-tmts-tarelki-dlia-filtra-prokladki-dvigatel/tender-4496006/#btid=2&amp;sqh=ad5c728ff17738e7bd83d093069a0c2a65996cc5&amp;tsid=4496006003</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07 19:21</t>
+          <t>2026-07-08 09:22</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -3528,7 +3529,7 @@
       </c>
       <c r="Q39" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=f38571f0054d6cc62726795ef661a590bb1229f1&amp;tsid=4129930003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=ad5c728ff17738e7bd83d093069a0c2a65996cc5&amp;tsid=4129930003</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
leads: обновление 2026-07-08 17:16 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q39"/>
+  <dimension ref="A1:Q41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 09:22</t>
+          <t>2026-07-08 17:16</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -560,235 +560,235 @@
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>4518085</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>ГК АО Логика Молока МК  Казань - Выполнение работ по текущему ремонту зданий и сооружений... конструкций технологического оборудования Демонтаж железобетоннойплитыпола Демонтаж бетонных полов  ... Укладка асфальта, включая: - устройстводорожногокорыта, h=0,40 м; ... , ворот, дверей, фасонки, опорныеплиты, опорные элементы фонарей, рамы, вентиляторов ...</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЭЙЧ ЭНД ЭН"</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЭЙЧ ЭНД ЭН"</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>7714626332</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Закриев Якуб Салманович</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>10.51.9</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>08.07.2026 14:53 — 15.07.2026 10:00</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Вятская, д 27 стр 13</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/gk-ao-logika-moloka-mk-kazan-vypolnenie-rabot-po-tekushchemu-remontu/tender-4518085/#btid=2&amp;sqh=205eb0da7eb9426cf1073846adc5ae6e8e3f427a&amp;tsid=4518085458</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08 17:16</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>Поставка</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>4515159</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Строительные материалы (поставка в Находку/Для ООО Светлое) поставка в срок до 10.09.2026
 Строительные материалы... -021 серый Краска ПФ-115 белаяПлита дорожнаяпостоянная железобетонная 1ПДН-14 6000х2000х140 мм ...</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>7805368914</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>46.90</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>07.07.2026 05:38 — 13.07.2026 10:00</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/stroitelnye-materialy-postavka-v-nakhodku-dlia-ooo-svetloe-postavka/tender-4515159/#btid=2&amp;sqh=e7a55a0d5d41409a139acf7b95567d4018bbe91b&amp;tsid=4515159004</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 09:22</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/stroitelnye-materialy-postavka-v-nakhodku-dlia-ooo-svetloe-postavka/tender-4515159/#btid=2&amp;sqh=205eb0da7eb9426cf1073846adc5ae6e8e3f427a&amp;tsid=4515159004</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08 17:16</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>4510835</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Реализация. Невостребованные складские остатки (не б/у). Запасные части для ГТО (для автосамосвалов, автобусов, легкового транспорта, бульдозеров, экскаваторов, грейдеров)
 Реализация. Запасные части для автосамосвалов HOWO, БЕЛАЗ, КАМАЗ, SCANIA; бульдозеров Cat 834, D9R, DT10T, KOMATSU WD600, PR754, Т-25; грейдера САТ140М; экскаваторов Bucyrus RH120E, Hyundai R520LC, ЭО, ЭШ, ЭКГ, ЕК-400, Liebherr R984C....  2445 V-ACS 32-R1195-9Дорожныйзнак "Осторожно газопровод" ДПТ-М  ... КАТУШКА электромагнитная 1317540-74030 Керамогранитплита300х600мм Керамогранитплита600х600мм Килоамперметр М42301 1, ... 90/460 У2Плита75570-8608180Плитаднища 1080.52.101Плиталотков ПТ  ...</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>ООО "УК "СИБАНТРАЦИТ"</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>ООО "УК "СИБАНТРАЦИТ"</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>9703160290</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Мельников Сергей Владимирович</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>70.22</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr"/>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>02.07.2026 13:09 — 16.07.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>г Москва, ул Усачёва, д 2 стр 1, помещ 2/1</t>
-        </is>
-      </c>
-      <c r="Q3" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=e7a55a0d5d41409a139acf7b95567d4018bbe91b&amp;tsid=4510835003</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 09:22</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Работы</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>4506366</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Ремонтдорожнойплитки на подъездной и выездной дороге от главного входа гостиницы</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>АО "ЛОТТЕ РУС"</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>АО "ЛОТТЕ РУС"</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>7704169180</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>Андерсен Мортен Бундгорд</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>55.10</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr"/>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>29.06.2026 16:30 — 09.07.2026 17:18</t>
+          <t>02.07.2026 13:09 — 16.07.2026 12:00</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Новинский б-р, д 8 стр 2</t>
+          <t>г Москва, ул Усачёва, д 2 стр 1, помещ 2/1</t>
         </is>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/remont-dorozhnoi-plitki-na-pod-ezdnoi-i-vyezdnoi-doroge-ot-glavnogo/tender-4506366/#btid=2&amp;sqh=e7a55a0d5d41409a139acf7b95567d4018bbe91b&amp;tsid=4506366458</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=205eb0da7eb9426cf1073846adc5ae6e8e3f427a&amp;tsid=4510835003</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 09:22</t>
+          <t>2026-07-08 17:16</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -799,33 +799,32 @@
       <c r="C5" s="2" t="inlineStr"/>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Поставка</t>
+          <t>Работы</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>4503612</t>
+          <t>4506366</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>RUNEV-11652 на выполнение работ по сортировке, разделке и вывозу демонтированных 
-трубопроводов и металлоконструкций на склад хранения. Вывозу строительного мусора на утилизацию с площадки Б-9 АО «Невинномысский Азот»....  площадки 600м² для выполнения работ, издорожных плит(60 шт, поставка заказчика), с выравниванием ...</t>
+          <t>Ремонтдорожнойплитки на подъездной и выездной дороге от главного входа гостиницы</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>АО "ЛОТТЕ РУС"</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>АО "ЛОТТЕ РУС"</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>7704169180</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -833,7 +832,11 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Андерсен Мортен Бундгорд</t>
+        </is>
+      </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -841,30 +844,30 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>55.10</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr"/>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>26.06.2026 10:29 — 08.07.2026 17:00</t>
+          <t>29.06.2026 16:30 — 09.07.2026 17:18</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Москва, Новинский б-р, д 8 стр 2</t>
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=e7a55a0d5d41409a139acf7b95567d4018bbe91b&amp;tsid=4503612458</t>
+          <t>https://www.b2b-center.ru/app/market-next/remont-dorozhnoi-plitki-na-pod-ezdnoi-i-vyezdnoi-doroge-ot-glavnogo/tender-4506366/#btid=2&amp;sqh=205eb0da7eb9426cf1073846adc5ae6e8e3f427a&amp;tsid=4506366458</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 09:22</t>
+          <t>2026-07-08 17:16</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -936,14 +939,14 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=e7a55a0d5d41409a139acf7b95567d4018bbe91b&amp;tsid=4130106003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=205eb0da7eb9426cf1073846adc5ae6e8e3f427a&amp;tsid=4130106003</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 09:22</t>
+          <t>2026-07-08 17:16</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1015,14 +1018,14 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=65b3211d179906b2f900c53c4e6927f2f19c4f5e&amp;tsid=4498936003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=20f081afdcf5d4216fe7f7d55028026da25573b4&amp;tsid=4498936003</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 09:22</t>
+          <t>2026-07-08 17:16</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1095,14 +1098,14 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=51ed30504898ec176bd44a7009092b0697483118&amp;tsid=4497016004</t>
+          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=932f29f78b9e46c99545830aafd6fbf41b0a25c1&amp;tsid=4497016004</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 09:22</t>
+          <t>2026-07-08 17:16</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1118,27 +1121,27 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>4512196</t>
+          <t>4518573</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>ОПОРА ЛЭПЛИСТВ НЕПРОПИТАН 22-28СМ L11</t>
+          <t>2228 ОпрыЛЭПпо заявке МГ-019766</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>АО "ИК "АРЛАН"</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>АО "ИК "АРЛАН"</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>7722220390</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1146,7 +1149,11 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Барилов Евгений Александрович</t>
+        </is>
+      </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1154,30 +1161,30 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>82.99</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr"/>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 11:30 — 09.07.2026 00:00</t>
+          <t>08.07.2026 18:39 — 14.07.2026 12:00</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Москва, Романов пер, д 4</t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=a5886426bebe1763852434306a3c3797e5a69302&amp;tsid=4512196458</t>
+          <t>https://www.b2b-center.ru/market/2228-opry-lep-po-zaiavke-mg-019766/tender-4518573/#btid=2&amp;sqh=d419ff3a6d419d91b36995ba662568dcb7bb8545&amp;tsid=4518573004</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 09:22</t>
+          <t>2026-07-08 17:16</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1188,32 +1195,32 @@
       <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Работы</t>
+          <t>Прочее</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>4512292</t>
+          <t>4512196</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>ТЕХНИЧЕСКОЕ ЗАДАНИЕ на строительствоЛЭП-6кВдля электроснабжения электрогидравлического экскаватора Liebherr 9200Е Работы по строительствуЛЭП-6кВдля электроснабжения электрогидравлического экскаватора Liebherr 9200Е.</t>
+          <t>ОПОРА ЛЭПЛИСТВ НЕПРОПИТАН 22-28СМ L11</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>ООО "СЕРВИС ПЛЮС"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>ООО "СЕРВИС ПЛЮС"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>7704643931</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1221,11 +1228,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>Иванов Владимир Ильич</t>
-        </is>
-      </c>
+      <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1233,30 +1236,30 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>68.32</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr"/>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 12:19 — 14.07.2026 12:00</t>
+          <t>03.07.2026 11:30 — 09.07.2026 00:00</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Пречистенка, д 40/2 стр 4, помещ I, ком 2А</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=a5886426bebe1763852434306a3c3797e5a69302&amp;tsid=4512292004</t>
+          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=d419ff3a6d419d91b36995ba662568dcb7bb8545&amp;tsid=4512196458</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 09:22</t>
+          <t>2026-07-08 17:16</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1267,15 +1270,173 @@
       <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="2" t="inlineStr">
         <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>4512292</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>ТЕХНИЧЕСКОЕ ЗАДАНИЕ на строительствоЛЭП-6кВдля электроснабжения электрогидравлического экскаватора Liebherr 9200Е Работы по строительствуЛЭП-6кВдля электроснабжения электрогидравлического экскаватора Liebherr 9200Е.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СЕРВИС ПЛЮС"</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СЕРВИС ПЛЮС"</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>7704643931</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Иванов Владимир Ильич</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>68.32</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>03.07.2026 12:19 — 14.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Пречистенка, д 40/2 стр 4, помещ I, ком 2А</t>
+        </is>
+      </c>
+      <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=d419ff3a6d419d91b36995ba662568dcb7bb8545&amp;tsid=4512292004</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08 17:16</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>4517766</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Заявка № ДОР-17519 ( /ЖБИ изделия/)Плиты перекрытия ПК-15КольцоК-7-1КольцоК-7-3КольцоК-7-5 ...  крышка ДКЛКольцоВГ-15КольцоК-15-10КольцоК-15-8КольцоК-15 ... -7КольцоК-15-6Кольцо...  К-15-5 Плита днища ДДК-8КолодецВД ...</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>7724498866</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>46.73</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>08.07.2026 12:34 — 09.07.2026 16:00</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+        </is>
+      </c>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zaiavka-dor-17519-zhbi-izdeliia/tender-4517766/#btid=2&amp;sqh=09c932b695968d7bb9663ffc840a0f8be026b09f&amp;tsid=4517766459</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08 17:16</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>4475879</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Электро/пневмо и ручной инструмент/Электроизм. инструмент/Расходные мат-лы
 РТИ, РВД, шланги, ремни
@@ -1283,212 +1444,62 @@
 Уплотнительный материал (прокладки, паронит, набивка сальниковая)...  Шина цепной пилы Oregon 752HSFL104Кольцостопор. нар. 210х5 DIN471 Andritz ... клин для бревен Sandvik 1401КольцоAbicor Binzel 757.D007 вихреобразующее ...  Kron ЦПВС-5 RAL7012 КрышкаколодцаП10 ж/б Игла клапана ... Kron ПСВС-3 RAL7012 О-кольцо11,3х2,4 NBR70 Ремень ...</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>4704012472</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>Ленинградская обл</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>Габидуллин Тимур Махмудович</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>17.12</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="inlineStr"/>
-      <c r="O11" s="2" t="inlineStr">
-        <is>
-          <t>03.06.2026 15:56 — 30.07.2026 20:00</t>
-        </is>
-      </c>
-      <c r="P11" s="2" t="inlineStr">
-        <is>
-          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
-        </is>
-      </c>
-      <c r="Q11" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=611fe3fb002a9aabd1dc3af49ad2af72c1d00d53&amp;tsid=4475879003</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 09:22</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>4514583</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Закупка ЖБИ (плитыПДН3*1,5)</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>9725042029</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>64.20</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr"/>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>06.07.2026 15:00 — 09.07.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
-        </is>
-      </c>
-      <c r="Q12" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-plity-pdn-3-1-5/tender-4514583/#btid=2&amp;sqh=f177e1e5925ec7c45574fa0eba249b0b78a6969c&amp;tsid=4514583458</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 09:22</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr"/>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>4516217</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>ТМЦЖБИи песок</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>9725042029</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>64.20</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr"/>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>07.07.2026 14:31 — 10.07.2026 10:00</t>
+          <t>03.06.2026 15:56 — 30.07.2026 20:00</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
         </is>
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/tmts-zhbi-i-pesok/tender-4516217/#btid=2&amp;sqh=ca0badfa5ad2b3baf05984ac65950e28246e3eac&amp;tsid=4516217458</t>
+          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=09c932b695968d7bb9663ffc840a0f8be026b09f&amp;tsid=4475879003</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 09:22</t>
+          <t>2026-07-08 17:16</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1504,12 +1515,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>4513278</t>
+          <t>4514583</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>ЖБИблоки ФБС</t>
+          <t>Закупка ЖБИ (плитыПДН3*1,5)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1546,7 +1557,7 @@
       <c r="N14" s="2" t="inlineStr"/>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>06.07.2026 04:17 — 09.07.2026 00:00</t>
+          <t>06.07.2026 15:00 — 09.07.2026 12:00</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -1556,14 +1567,14 @@
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-bloki-fbs/tender-4513278/#btid=2&amp;sqh=ca0badfa5ad2b3baf05984ac65950e28246e3eac&amp;tsid=4513278458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-plity-pdn-3-1-5/tender-4514583/#btid=2&amp;sqh=cf1203dbd9ec1ad5b95e895ff4f06dd4c715c086&amp;tsid=4514583458</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 09:22</t>
+          <t>2026-07-08 17:16</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1574,32 +1585,32 @@
       <c r="C15" s="2" t="inlineStr"/>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Поставка</t>
+          <t>Прочее</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>4514839</t>
+          <t>4517935</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>12-х-1 Заключение договора на поставку материалов для наружных сетей водоснабжения и водоотведения на объект строительства «Дальневосточный детский центр отдыха и оздоровления в Хабаровском крае». (9 лотов) Лот №1 ВодоснабжениеЖБИ</t>
+          <t>ЖБИ(Дор № 17559)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>ООО "ПРОМСТРОЙ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>ООО "ПРОМСТРОЙ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>9723169975</t>
+          <t>7724498866</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -1609,7 +1620,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Султанов Владислав Назипович</t>
+          <t>Городний Анатолий Валерьевич</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1619,30 +1630,30 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>71.12.2</t>
+          <t>46.73</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr"/>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>06.07.2026 16:45 — 10.07.2026 11:00</t>
+          <t>08.07.2026 13:40 — 09.07.2026 17:00</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Волгоградский пр-кт, д 42 к 5, ком 9</t>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
         </is>
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/12-kh-1-zakliuchenie-dogovora-na-postavku-materialov-dlia-naruzhnykh-setei/tender-4514839/#btid=2&amp;sqh=ca0badfa5ad2b3baf05984ac65950e28246e3eac&amp;tsid=4514839004</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-dor-17559/tender-4517935/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=4517935459</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 09:22</t>
+          <t>2026-07-08 17:16</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1658,27 +1669,27 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>4510341</t>
+          <t>4516217</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>ЖБИ(чеч 34\25 7510 \ 17338)</t>
+          <t>ТМЦЖБИи песок</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>7724498866</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1686,11 +1697,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>Городний Анатолий Валерьевич</t>
-        </is>
-      </c>
+      <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1698,30 +1705,30 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>46.73</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr"/>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>02.07.2026 09:54 — 08.07.2026 15:00</t>
+          <t>07.07.2026 14:31 — 10.07.2026 10:00</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-chech-34-25-7510-17338/tender-4510341/#btid=2&amp;sqh=ca0badfa5ad2b3baf05984ac65950e28246e3eac&amp;tsid=4510341459</t>
+          <t>https://www.b2b-center.ru/app/market-next/tmts-zhbi-i-pesok/tender-4516217/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=4516217458</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 09:22</t>
+          <t>2026-07-08 17:16</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1737,27 +1744,27 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>4510662</t>
+          <t>4513278</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>(ЖБИизделия/кольца колодезные, плиты ПК15)</t>
+          <t>ЖБИблоки ФБС</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>7724498866</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -1765,11 +1772,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>Городний Анатолий Валерьевич</t>
-        </is>
-      </c>
+      <c r="K17" s="2" t="inlineStr"/>
       <c r="L17" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1777,30 +1780,30 @@
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>46.73</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr"/>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>02.07.2026 12:00 — 09.07.2026 13:00</t>
+          <t>06.07.2026 04:17 — 09.07.2026 00:00</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-izdeliia-koltsa-kolodeznye-plity-pk15/tender-4510662/#btid=2&amp;sqh=ca0badfa5ad2b3baf05984ac65950e28246e3eac&amp;tsid=4510662459</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-bloki-fbs/tender-4513278/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=4513278458</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 09:22</t>
+          <t>2026-07-08 17:16</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1811,32 +1814,32 @@
       <c r="C18" s="2" t="inlineStr"/>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Поставка</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>4510504</t>
+          <t>4514839</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>(Заявка № ДОР-17560) Лестницы/ЖБИ</t>
+          <t>12-х-1 Заключение договора на поставку материалов для наружных сетей водоснабжения и водоотведения на объект строительства «Дальневосточный детский центр отдыха и оздоровления в Хабаровском крае». (9 лотов) Лот №1 ВодоснабжениеЖБИ</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "ПРОМСТРОЙ"</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "ПРОМСТРОЙ"</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>7724498866</t>
+          <t>9723169975</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1846,7 +1849,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Городний Анатолий Валерьевич</t>
+          <t>Султанов Владислав Назипович</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -1856,30 +1859,30 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>46.73</t>
+          <t>71.12.2</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr"/>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>02.07.2026 10:55 — 09.07.2026 13:00</t>
+          <t>06.07.2026 16:45 — 10.07.2026 11:00</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+          <t>г Москва, Волгоградский пр-кт, д 42 к 5, ком 9</t>
         </is>
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zaiavka-dor-17560-lestnitsy-zhbi/tender-4510504/#btid=2&amp;sqh=ca0badfa5ad2b3baf05984ac65950e28246e3eac&amp;tsid=4510504459</t>
+          <t>https://www.b2b-center.ru/market/12-kh-1-zakliuchenie-dogovora-na-postavku-materialov-dlia-naruzhnykh-setei/tender-4514839/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=4514839004</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 09:22</t>
+          <t>2026-07-08 17:16</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1895,27 +1898,27 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>4508347</t>
+          <t>4510662</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>ЖБИКЕМГРЭС</t>
+          <t>(ЖБИизделия/кольца колодезные, плиты ПК15)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>7724498866</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -1923,7 +1926,11 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1931,30 +1938,30 @@
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>46.73</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr"/>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>01.07.2026 05:45 — 10.07.2026 00:00</t>
+          <t>02.07.2026 12:00 — 09.07.2026 13:00</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
         </is>
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=ca0badfa5ad2b3baf05984ac65950e28246e3eac&amp;tsid=4508347458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-izdeliia-koltsa-kolodeznye-plity-pk15/tender-4510662/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=4510662459</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 09:22</t>
+          <t>2026-07-08 17:16</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1970,27 +1977,27 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>4489772</t>
+          <t>4510504</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы 1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы</t>
+          <t>(Заявка № ДОР-17560) Лестницы/ЖБИ</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>7736583259</t>
+          <t>7724498866</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -2000,7 +2007,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Масько Александр Вадимович</t>
+          <t>Городний Анатолий Валерьевич</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -2010,30 +2017,30 @@
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>70.10</t>
+          <t>46.73</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr"/>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>16.06.2026 11:00 — 16.07.2026 12:00</t>
+          <t>02.07.2026 10:55 — 09.07.2026 13:00</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Старая Басманная, д 12 стр 1</t>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
         </is>
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=ca0badfa5ad2b3baf05984ac65950e28246e3eac&amp;tsid=4489772003</t>
+          <t>https://www.b2b-center.ru/app/market-next/zaiavka-dor-17560-lestnitsy-zhbi/tender-4510504/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=4510504459</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 09:22</t>
+          <t>2026-07-08 17:16</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -2049,37 +2056,37 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>4474790</t>
+          <t>4510823</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
+          <t>(ДОР-17553)ЖБИ/Лестницы ВЛ-2/Скоба</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>4704012472</t>
+          <t>7724498866</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Габидуллин Тимур Махмудович</t>
+          <t>Городний Анатолий Валерьевич</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -2089,30 +2096,30 @@
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>17.12</t>
+          <t>46.73</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr"/>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>03.06.2026 09:59 — 30.07.2026 20:00</t>
+          <t>02.07.2026 12:55 — 09.07.2026 11:00</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
         </is>
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=ca0badfa5ad2b3baf05984ac65950e28246e3eac&amp;tsid=4474790003</t>
+          <t>https://www.b2b-center.ru/app/market-next/dor-17553-zhbi-lestnitsy-vl-2-skoba/tender-4510823/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=4510823459</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 09:22</t>
+          <t>2026-07-08 17:16</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2128,27 +2135,27 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>4180328</t>
+          <t>4508347</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, г.Диксон). ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, ПГТ Диксон).</t>
+          <t>ЖБИКЕМГРЭС</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>7714456916</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -2156,11 +2163,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>Наумов Андрей Александрович</t>
-        </is>
-      </c>
+      <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -2168,30 +2171,30 @@
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>70.22</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr"/>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>24.09.2025 15:32 — 23.07.2026 12:00</t>
+          <t>01.07.2026 05:45 — 10.07.2026 00:00</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Денежный пер, д 9/6</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q22" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=ca0badfa5ad2b3baf05984ac65950e28246e3eac&amp;tsid=4180328003</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=4508347458</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 09:22</t>
+          <t>2026-07-08 17:16</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2207,37 +2210,37 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>3973258</t>
+          <t>4489772</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
+          <t>1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы 1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>4704012472</t>
+          <t>7736583259</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Габидуллин Тимур Махмудович</t>
+          <t>Масько Александр Вадимович</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
@@ -2247,30 +2250,30 @@
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>17.12</t>
+          <t>70.10</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr"/>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>10.03.2025 00:48 — 30.07.2026 23:00</t>
+          <t>16.06.2026 11:00 — 16.07.2026 12:00</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+          <t>г Москва, ул Старая Басманная, д 12 стр 1</t>
         </is>
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=ca0badfa5ad2b3baf05984ac65950e28246e3eac&amp;tsid=3973258003</t>
+          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=4489772003</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 09:22</t>
+          <t>2026-07-08 17:16</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2281,40 +2284,44 @@
       <c r="C24" s="2" t="inlineStr"/>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Поставка</t>
+          <t>Прочее</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>4513525</t>
+          <t>4474790</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Поставка модульных защитных сооруженийЗДАНИЕ ЗАЩИТНОЕ ДЛЯ УКРЫТИЯ 4,4*2,4*2,2МЖЕЛЕЗОБЕТОННОЕСБОРНОЕ</t>
+          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>4704012472</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr"/>
+          <t>Ленинградская обл</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Габидуллин Тимур Махмудович</t>
+        </is>
+      </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -2322,30 +2329,30 @@
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>17.12</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr"/>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>06.07.2026 08:36 — 10.07.2026 14:00</t>
+          <t>03.06.2026 09:59 — 30.07.2026 20:00</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
         </is>
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/postavka-modulnykh-zashchitnykh-sooruzhenii/tender-4513525/#btid=2&amp;sqh=f2ccdf8699fcd02c28a40854bc3aff3687fb23e1&amp;tsid=4513525458</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=4474790003</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 09:22</t>
+          <t>2026-07-08 17:16</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -2361,10 +2368,243 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
+          <t>4180328</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, г.Диксон). ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, ПГТ Диксон).</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>7714456916</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Наумов Андрей Александрович</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>70.22</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr"/>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>24.09.2025 15:32 — 23.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Денежный пер, д 9/6</t>
+        </is>
+      </c>
+      <c r="Q25" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=4180328003</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08 17:16</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>3973258</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>4704012472</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Ленинградская обл</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Габидуллин Тимур Махмудович</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>17.12</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>10.03.2025 00:48 — 30.07.2026 23:00</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+        </is>
+      </c>
+      <c r="Q26" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=3973258003</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08 17:16</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr"/>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>4513525</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Поставка модульных защитных сооруженийЗДАНИЕ ЗАЩИТНОЕ ДЛЯ УКРЫТИЯ 4,4*2,4*2,2МЖЕЛЕЗОБЕТОННОЕСБОРНОЕ</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr"/>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>06.07.2026 08:36 — 10.07.2026 14:00</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/postavka-modulnykh-zashchitnykh-sooruzhenii/tender-4513525/#btid=2&amp;sqh=39868999b159823b02130aa6f265a3a7ff3e9512&amp;tsid=4513525458</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08 17:16</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
           <t>4513563</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Блок ФБС 12.4.6-Т-и
 Кольцо стеновое КС 20.9 ГОСТ 8020-2016
@@ -2373,852 +2613,614 @@
 Кольцо стеновое КС 20.9 ГОСТ 8020-20164513563 ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "ТОРГОВЫЙ ДОМ ПОЛИМЕТАЛЛ"Железобетонные изделия</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>7805368914</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
+      <c r="J28" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург</t>
         </is>
       </c>
-      <c r="K25" s="2" t="inlineStr">
+      <c r="K28" s="2" t="inlineStr">
         <is>
           <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M25" s="2" t="inlineStr">
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
         <is>
           <t>46.90</t>
         </is>
       </c>
-      <c r="N25" s="2" t="inlineStr"/>
-      <c r="O25" s="2" t="inlineStr">
+      <c r="N28" s="2" t="inlineStr"/>
+      <c r="O28" s="2" t="inlineStr">
         <is>
           <t>06.07.2026 08:49 — 10.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P25" s="2" t="inlineStr">
+      <c r="P28" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
-      <c r="Q25" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/blok-fbs-12-4-6-t-i-koltso-stenovoe-ks-20-9-gost-8020-2016-na-k-pm/tender-4513563/#btid=2&amp;sqh=f2ccdf8699fcd02c28a40854bc3aff3687fb23e1&amp;tsid=4513563004</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 09:22</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="Q28" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/blok-fbs-12-4-6-t-i-koltso-stenovoe-ks-20-9-gost-8020-2016-na-k-pm/tender-4513563/#btid=2&amp;sqh=39868999b159823b02130aa6f265a3a7ff3e9512&amp;tsid=4513563004</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08 17:16</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr"/>
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>4517499</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>КРЫШКА-ПАТРУБОК 200-Т-535СБ ПК-40; ЗАГЛУШКА НА КЛАПАН СД К-5976.00.00 СБ; КРЫШКА 200-Т-525СБ ПК-40;ПЕРЕМЫЧКАД/ПРОДУВКИ ППХ 200-Т-530 СБ</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>9725042029</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="J29" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr"/>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="inlineStr">
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
         <is>
           <t>64.20</t>
         </is>
       </c>
-      <c r="N26" s="2" t="inlineStr"/>
-      <c r="O26" s="2" t="inlineStr">
+      <c r="N29" s="2" t="inlineStr"/>
+      <c r="O29" s="2" t="inlineStr">
         <is>
           <t>08.07.2026 10:53 — 10.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P26" s="2" t="inlineStr">
+      <c r="P29" s="2" t="inlineStr">
         <is>
           <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
-      <c r="Q26" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/app/market-next/kryshka-patrubok-200-t-535sb-pk-40-zaglushka-na-klapan-sd-k-5976-00-00/tender-4517499/#btid=2&amp;sqh=a741c4d6737d6b95143fe98c39a13a7a3c409e1a&amp;tsid=4517499458</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 09:22</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr"/>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="Q29" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/kryshka-patrubok-200-t-535sb-pk-40-zaglushka-na-klapan-sd-k-5976-00-00/tender-4517499/#btid=2&amp;sqh=4ba4cb5de9195180187222c70541fed058c879ca&amp;tsid=4517499458</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08 17:16</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>4512541</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Запасные части CAT.... -3748 Cat Опора 348-9537 CatПеремычка140-0860 Cat Скоба 8X-3130 ...</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>1004001744</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="J30" s="2" t="inlineStr">
         <is>
           <t>Респ Карелия</t>
         </is>
       </c>
-      <c r="K27" s="2" t="inlineStr">
+      <c r="K30" s="2" t="inlineStr">
         <is>
           <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "СЕВЕРСТАЛЬ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M27" s="2" t="inlineStr">
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
         <is>
           <t>07.10.2</t>
         </is>
       </c>
-      <c r="N27" s="2" t="inlineStr"/>
-      <c r="O27" s="2" t="inlineStr">
+      <c r="N30" s="2" t="inlineStr"/>
+      <c r="O30" s="2" t="inlineStr">
         <is>
           <t>03.07.2026 14:07 — 10.07.2026 11:00</t>
         </is>
       </c>
-      <c r="P27" s="2" t="inlineStr">
+      <c r="P30" s="2" t="inlineStr">
         <is>
           <t>Респ Карелия, г Костомукша, шоссе Горняков, стр 284</t>
         </is>
       </c>
-      <c r="Q27" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=a741c4d6737d6b95143fe98c39a13a7a3c409e1a&amp;tsid=4512541003</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 09:22</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="Q30" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=4ba4cb5de9195180187222c70541fed058c879ca&amp;tsid=4512541003</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08 17:16</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr"/>
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>4508230</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>Сборный (Изделия электроустановочные и монтажные, Ящики, щиты, шкафы, пункты и комплектующие к ним, Приборы электроизмерительные, реле)
 МГ-019742, МГ-019713, МГ-019696, МГ-019665, МГ-019621, МГ-019620, МГ-019619, МГ-017109... -HESI-EX (5X20), Phoenix Contact 1277638ПеремычкаFBS 10-5, Phoenix Contact 3030213 ...ПеремычкаFBS 10-5 BU, Phoenix Contact  ...</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>АО "ИК "АРЛАН"</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>АО "ИК "АРЛАН"</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>7722220390</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="J31" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K28" s="2" t="inlineStr">
+      <c r="K31" s="2" t="inlineStr">
         <is>
           <t>Барилов Евгений Александрович</t>
         </is>
       </c>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M28" s="2" t="inlineStr">
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
         <is>
           <t>82.99</t>
         </is>
       </c>
-      <c r="N28" s="2" t="inlineStr"/>
-      <c r="O28" s="2" t="inlineStr">
+      <c r="N31" s="2" t="inlineStr"/>
+      <c r="O31" s="2" t="inlineStr">
         <is>
           <t>30.06.2026 17:59 — 09.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P28" s="2" t="inlineStr">
+      <c r="P31" s="2" t="inlineStr">
         <is>
           <t>г Москва, Романов пер, д 4</t>
         </is>
       </c>
-      <c r="Q28" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=a741c4d6737d6b95143fe98c39a13a7a3c409e1a&amp;tsid=4508230004</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 09:22</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr"/>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="Q31" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=4ba4cb5de9195180187222c70541fed058c879ca&amp;tsid=4508230004</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08 17:16</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>4501157</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Источники электропитания (ИБП, аккумуляторные батареи, блоки питания)...  х 1248 А·ч, включая соединительныеперемычки. Вид положительного электрода - трубчатая пластина ...  с коммутирующей арматурой, межэлементными и межряднымиперемычками, крепежами, комплектом для обслуживания АБ. Тип ...</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>АО "Мосинжпроект"</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>АО "МОСИНЖПРОЕКТ"</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>7701885820</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr">
+      <c r="J32" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K29" s="2" t="inlineStr">
+      <c r="K32" s="2" t="inlineStr">
         <is>
           <t>Сорокин Антон Павлович</t>
         </is>
       </c>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M29" s="2" t="inlineStr">
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
         <is>
           <t>71.12.2</t>
         </is>
       </c>
-      <c r="N29" s="2" t="inlineStr"/>
-      <c r="O29" s="2" t="inlineStr">
+      <c r="N32" s="2" t="inlineStr"/>
+      <c r="O32" s="2" t="inlineStr">
         <is>
           <t>24.06.2026 15:40 — 22.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P29" s="2" t="inlineStr">
+      <c r="P32" s="2" t="inlineStr">
         <is>
           <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
         </is>
       </c>
-      <c r="Q29" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=a741c4d6737d6b95143fe98c39a13a7a3c409e1a&amp;tsid=4501157003</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 09:22</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="Q32" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=4ba4cb5de9195180187222c70541fed058c879ca&amp;tsid=4501157003</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08 17:16</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr"/>
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>4499964</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>Автоматика и телемеханика движения поездов... , 13552-00-00В Дроссель-трансформатор (безперемычек) ДТМ-0,17-1000М ЮКЛЯ.672 ...</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>АО "Мосинжпроект"</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>АО "МОСИНЖПРОЕКТ"</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr">
         <is>
           <t>7701885820</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="J33" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K30" s="2" t="inlineStr">
+      <c r="K33" s="2" t="inlineStr">
         <is>
           <t>Сорокин Антон Павлович</t>
         </is>
       </c>
-      <c r="L30" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M30" s="2" t="inlineStr">
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
         <is>
           <t>71.12.2</t>
         </is>
       </c>
-      <c r="N30" s="2" t="inlineStr"/>
-      <c r="O30" s="2" t="inlineStr">
+      <c r="N33" s="2" t="inlineStr"/>
+      <c r="O33" s="2" t="inlineStr">
         <is>
           <t>24.06.2026 08:46 — 15.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P30" s="2" t="inlineStr">
+      <c r="P33" s="2" t="inlineStr">
         <is>
           <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
         </is>
       </c>
-      <c r="Q30" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=a741c4d6737d6b95143fe98c39a13a7a3c409e1a&amp;tsid=4499964003</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 09:22</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr"/>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="Q33" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=4ba4cb5de9195180187222c70541fed058c879ca&amp;tsid=4499964003</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08 17:16</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>4504775</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники
 Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники...  Трубка пробная № 37-542-000 Соединитель-перемычка04182454 Кольцо стальное №CP48001-0305 Фильтр ...</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>7805368914</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr">
+      <c r="J34" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург</t>
         </is>
       </c>
-      <c r="K31" s="2" t="inlineStr">
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
-      <c r="L31" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M31" s="2" t="inlineStr">
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
         <is>
           <t>46.90</t>
         </is>
       </c>
-      <c r="N31" s="2" t="inlineStr"/>
-      <c r="O31" s="2" t="inlineStr">
+      <c r="N34" s="2" t="inlineStr"/>
+      <c r="O34" s="2" t="inlineStr">
         <is>
           <t>27.06.2026 01:36 — 15.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P31" s="2" t="inlineStr">
+      <c r="P34" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
-      <c r="Q31" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=a741c4d6737d6b95143fe98c39a13a7a3c409e1a&amp;tsid=4504775003</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 09:22</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="Q34" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=4ba4cb5de9195180187222c70541fed058c879ca&amp;tsid=4504775003</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08 17:16</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr"/>
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>4480614</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>Плановое и аварийное техническое обслуживание зданий и сооружений (годовое обслуживание август 2026 - август 2027) ГК Логика молока, производственная площадка в г. Ялуторовске
 Обслуживание зданий и сооружений завода в г. Ялуторовске....  стен из газобетонных блоков Устройство металлическихперемычекс устройством штраб Усиление кирпичных стен ...</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>АО "ЭЙЧ ЭНД ЭН"</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>АО "ЭЙЧ ЭНД ЭН"</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="I35" s="2" t="inlineStr">
         <is>
           <t>7714626332</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr">
+      <c r="J35" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K32" s="2" t="inlineStr">
+      <c r="K35" s="2" t="inlineStr">
         <is>
           <t>Закриев Якуб Салманович</t>
         </is>
       </c>
-      <c r="L32" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M32" s="2" t="inlineStr">
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
         <is>
           <t>10.51.9</t>
-        </is>
-      </c>
-      <c r="N32" s="2" t="inlineStr"/>
-      <c r="O32" s="2" t="inlineStr">
-        <is>
-          <t>08.06.2026 14:44 — 08.07.2026 23:00</t>
-        </is>
-      </c>
-      <c r="P32" s="2" t="inlineStr">
-        <is>
-          <t>г Москва, ул Вятская, д 27 стр 13</t>
-        </is>
-      </c>
-      <c r="Q32" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/planovoe-i-avariinoe-tekhnicheskoe-obsluzhivanie-zdanii-i-sooruzhenii/tender-4480614/#btid=2&amp;sqh=a741c4d6737d6b95143fe98c39a13a7a3c409e1a&amp;tsid=4480614004</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 09:22</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr"/>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>4449201</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>Реализация НВИ, Оборудование теплообменное; Оборудование емкостное; Запчасти и узлы теплообменного оборудования; Запчасти и узлы емкостного оборудования;
-Продажа НВИ согласно прилагаемого перечня. 110-Емкостное и теп-ое об-е; 136-Запчасти и узлы емкостного и теплообПрокладка сперемычкамидля теплообменников ПУТГм-Б-09-01( ... . Е-21504.05.06 Прокладка сперемычкамидля теплообменников ПУТГм-Б-09-01 ...</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>ООО "СИБУР"</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>ООО "СИБУР"</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>7727576505</t>
-        </is>
-      </c>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>Карисалов Михаил Юрьевич</t>
-        </is>
-      </c>
-      <c r="L33" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M33" s="2" t="inlineStr">
-        <is>
-          <t>70.10</t>
-        </is>
-      </c>
-      <c r="N33" s="2" t="inlineStr"/>
-      <c r="O33" s="2" t="inlineStr">
-        <is>
-          <t>15.05.2026 06:57 — 10.07.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P33" s="2" t="inlineStr">
-        <is>
-          <t>г Москва, ул Кржижановского, д 16 к 3</t>
-        </is>
-      </c>
-      <c r="Q33" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nvi-oborudovanie-teploobmennoe-oborudovanie-emkostnoe/tender-4449201/#btid=2&amp;sqh=a741c4d6737d6b95143fe98c39a13a7a3c409e1a&amp;tsid=4449201003</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 09:22</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>4512370</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>ТО Сплит систем Лабинск Эйч энд Эн... кондиционирования Техническое обслуживание внутреннегоблокакассетного типа мультизональной  ...блокакондиционера. Мойка теплообменника внутреннегоблокакондиционера Чистка фильтров внутреннегоблокакондиционера Чистка фильтров приточнойвентиляционной...</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>АО "ЭЙЧ ЭНД ЭН"</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>АО "ЭЙЧ ЭНД ЭН"</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>7714626332</t>
-        </is>
-      </c>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>Закриев Якуб Салманович</t>
-        </is>
-      </c>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M34" s="2" t="inlineStr">
-        <is>
-          <t>10.51.9</t>
-        </is>
-      </c>
-      <c r="N34" s="2" t="inlineStr"/>
-      <c r="O34" s="2" t="inlineStr">
-        <is>
-          <t>03.07.2026 12:40 — 14.07.2026 18:30</t>
-        </is>
-      </c>
-      <c r="P34" s="2" t="inlineStr">
-        <is>
-          <t>г Москва, ул Вятская, д 27 стр 13</t>
-        </is>
-      </c>
-      <c r="Q34" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=ad5c728ff17738e7bd83d093069a0c2a65996cc5&amp;tsid=4512370458</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 09:22</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr"/>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>4501181</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>Вентиляторы промышленные и оборудование общеобменной вентиляции...  5Ф РешёткавентиляционнаяАМР 600х300М РешёткавентиляционнаяАМР 150х150М РешёткавентиляционнаяАМР 300х200М  ... мм.; масса 0,65 кгБлокконтроля сопротивления БСК-3.1 Канальный ...  533Па, габаритные размеры 700х467х2230 мм,блоков/моноблоков 5/1, в составе: - ...</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>АО "Мосинжпроект"</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>АО "МОСИНЖПРОЕКТ"</t>
-        </is>
-      </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>7701885820</t>
-        </is>
-      </c>
-      <c r="J35" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="inlineStr">
-        <is>
-          <t>Сорокин Антон Павлович</t>
-        </is>
-      </c>
-      <c r="L35" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M35" s="2" t="inlineStr">
-        <is>
-          <t>71.12.2</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr"/>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 15:45 — 22.07.2026 12:00</t>
+          <t>08.06.2026 14:44 — 08.07.2026 23:00</t>
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+          <t>г Москва, ул Вятская, д 27 стр 13</t>
         </is>
       </c>
       <c r="Q35" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=ad5c728ff17738e7bd83d093069a0c2a65996cc5&amp;tsid=4501181003</t>
+          <t>https://www.b2b-center.ru/market/planovoe-i-avariinoe-tekhnicheskoe-obsluzhivanie-zdanii-i-sooruzhenii/tender-4480614/#btid=2&amp;sqh=4ba4cb5de9195180187222c70541fed058c879ca&amp;tsid=4480614004</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 09:22</t>
+          <t>2026-07-08 17:16</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -3234,307 +3236,465 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
+          <t>4512370</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>ТО Сплит систем Лабинск Эйч энд Эн... кондиционирования Техническое обслуживание внутреннегоблокакассетного типа мультизональной  ...блокакондиционера. Мойка теплообменника внутреннегоблокакондиционера Чистка фильтров внутреннегоблокакондиционера Чистка фильтров приточнойвентиляционной...</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЭЙЧ ЭНД ЭН"</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЭЙЧ ЭНД ЭН"</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>7714626332</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>Закриев Якуб Салманович</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>10.51.9</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr"/>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>03.07.2026 12:40 — 14.07.2026 18:30</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Вятская, д 27 стр 13</t>
+        </is>
+      </c>
+      <c r="Q36" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=c61084f649b6de8adb87da7e7712cbd359326b47&amp;tsid=4512370458</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08 17:16</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr"/>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>4501181</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Вентиляторы промышленные и оборудование общеобменной вентиляции...  5Ф РешёткавентиляционнаяАМР 600х300М РешёткавентиляционнаяАМР 150х150М РешёткавентиляционнаяАМР 300х200М  ... мм.; масса 0,65 кгБлокконтроля сопротивления БСК-3.1 Канальный ...  533Па, габаритные размеры 700х467х2230 мм,блоков/моноблоков 5/1, в составе: - ...</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>АО "Мосинжпроект"</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>7701885820</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Сорокин Антон Павлович</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>71.12.2</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr"/>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>24.06.2026 15:45 — 22.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P37" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+        </is>
+      </c>
+      <c r="Q37" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=c61084f649b6de8adb87da7e7712cbd359326b47&amp;tsid=4501181003</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08 17:16</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
           <t>4501483</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ
 Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ...  d 50x2", внутренняя резьба RTPБлокуправления наружной установки ICEFREE TR-16 ...  Оповещатель звуковой МАЯК-12-ЗМБлокуправления наружной установки ICEFREE TS- ... проводов КС-3 007004 Велос Переходвентиляционный150х100 - D150, из тонколистовой оцинкованной ...</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr">
+      <c r="I38" s="2" t="inlineStr">
         <is>
           <t>7805368914</t>
         </is>
       </c>
-      <c r="J36" s="2" t="inlineStr">
+      <c r="J38" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург</t>
         </is>
       </c>
-      <c r="K36" s="2" t="inlineStr">
+      <c r="K38" s="2" t="inlineStr">
         <is>
           <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
-      <c r="L36" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M36" s="2" t="inlineStr">
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
         <is>
           <t>46.90</t>
         </is>
       </c>
-      <c r="N36" s="2" t="inlineStr"/>
-      <c r="O36" s="2" t="inlineStr">
+      <c r="N38" s="2" t="inlineStr"/>
+      <c r="O38" s="2" t="inlineStr">
         <is>
           <t>25.06.2026 05:03 — 09.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P36" s="2" t="inlineStr">
+      <c r="P38" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
-      <c r="Q36" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=ad5c728ff17738e7bd83d093069a0c2a65996cc5&amp;tsid=4501483003</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 09:22</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr"/>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="Q38" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=c61084f649b6de8adb87da7e7712cbd359326b47&amp;tsid=4501483003</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08 17:16</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr"/>
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>4500120</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>Коммуникационное оборудование, компьютеры, комплектующие к ним, серверное оборудование и ПО...  и кабелей – 1 компл. Удаленныйблок(репитер) BSF414 , питание 220В,  ... 2х2 Комбайнер специализированный OMU Side (блок1) OMUSC1 Комбайнер специализированный OMU ... контроллер для мониторинга в FlexGain View,вентиляционнаяпанель с фильтрами, комплект кабелей, ...</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>АО "Мосинжпроект"</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>АО "МОСИНЖПРОЕКТ"</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr">
+      <c r="I39" s="2" t="inlineStr">
         <is>
           <t>7701885820</t>
         </is>
       </c>
-      <c r="J37" s="2" t="inlineStr">
+      <c r="J39" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K37" s="2" t="inlineStr">
+      <c r="K39" s="2" t="inlineStr">
         <is>
           <t>Сорокин Антон Павлович</t>
         </is>
       </c>
-      <c r="L37" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M37" s="2" t="inlineStr">
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
         <is>
           <t>71.12.2</t>
         </is>
       </c>
-      <c r="N37" s="2" t="inlineStr"/>
-      <c r="O37" s="2" t="inlineStr">
+      <c r="N39" s="2" t="inlineStr"/>
+      <c r="O39" s="2" t="inlineStr">
         <is>
           <t>24.06.2026 09:48 — 15.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P37" s="2" t="inlineStr">
+      <c r="P39" s="2" t="inlineStr">
         <is>
           <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
         </is>
       </c>
-      <c r="Q37" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=ad5c728ff17738e7bd83d093069a0c2a65996cc5&amp;tsid=4500120003</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 09:22</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="Q39" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=c61084f649b6de8adb87da7e7712cbd359326b47&amp;tsid=4500120003</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08 17:16</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>4496006</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп
 Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп... -316 ***Петля крепежная стальная ***Платаблокауправления ZC5 CAME ***Средство чистящее " ... /распылитель для чаши Генуя ***РешеткавентиляционнаяРВ-1 225Х225 ***Петля анкерная 0 ... мл ***Папка с зажимом ***РешеткавентиляционнаяРВ-1 325Х125 ***Папка на кольцах ...</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>ООО "СИБУР"</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>ООО "СИБУР"</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr">
+      <c r="I40" s="2" t="inlineStr">
         <is>
           <t>7727576505</t>
         </is>
       </c>
-      <c r="J38" s="2" t="inlineStr">
+      <c r="J40" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K38" s="2" t="inlineStr">
+      <c r="K40" s="2" t="inlineStr">
         <is>
           <t>Карисалов Михаил Юрьевич</t>
         </is>
       </c>
-      <c r="L38" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M38" s="2" t="inlineStr">
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
         <is>
           <t>70.10</t>
         </is>
       </c>
-      <c r="N38" s="2" t="inlineStr"/>
-      <c r="O38" s="2" t="inlineStr">
+      <c r="N40" s="2" t="inlineStr"/>
+      <c r="O40" s="2" t="inlineStr">
         <is>
           <t>20.06.2026 16:19 — 11.07.2026 12:00</t>
         </is>
       </c>
-      <c r="P38" s="2" t="inlineStr">
+      <c r="P40" s="2" t="inlineStr">
         <is>
           <t>г Москва, ул Кржижановского, д 16 к 3</t>
         </is>
       </c>
-      <c r="Q38" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nelikvidnykh-tmts-tarelki-dlia-filtra-prokladki-dvigatel/tender-4496006/#btid=2&amp;sqh=ad5c728ff17738e7bd83d093069a0c2a65996cc5&amp;tsid=4496006003</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 09:22</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr"/>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="Q40" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/prodazha-nelikvidnykh-tmts-tarelki-dlia-filtra-prokladki-dvigatel/tender-4496006/#btid=2&amp;sqh=c61084f649b6de8adb87da7e7712cbd359326b47&amp;tsid=4496006003</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08 17:16</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr"/>
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>Работы</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>4129930</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>Реализация материалов для ремонта (напольные покрытия, настенные покрытия, окна, двери и т.д.) с АО "Мальцовский портландцемент"Блокдверной балконныйБлокдверной филенчатый ДГ 21х9Блококонный 1500х1000 ммБлококонный 1770х1700 мм Желоб ...  Docke Рама оконная 3000х1200 мм Решеткавентиляционнаянаружная Ручка оконная ГОСТ 5087-80 ...</t>
         </is>
       </c>
-      <c r="G39" s="2" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
-      <c r="H39" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
-      <c r="I39" s="2" t="inlineStr">
+      <c r="I41" s="2" t="inlineStr">
         <is>
           <t>7708117908</t>
         </is>
       </c>
-      <c r="J39" s="2" t="inlineStr">
+      <c r="J41" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K39" s="2" t="inlineStr">
+      <c r="K41" s="2" t="inlineStr">
         <is>
           <t>Шматов Вячеслав Вячеславович</t>
         </is>
       </c>
-      <c r="L39" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M39" s="2" t="inlineStr">
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
         <is>
           <t>23.51</t>
         </is>
       </c>
-      <c r="N39" s="2" t="inlineStr"/>
-      <c r="O39" s="2" t="inlineStr">
+      <c r="N41" s="2" t="inlineStr"/>
+      <c r="O41" s="2" t="inlineStr">
         <is>
           <t>06.08.2025 14:33 — 07.08.2026 12:00</t>
         </is>
       </c>
-      <c r="P39" s="2" t="inlineStr">
+      <c r="P41" s="2" t="inlineStr">
         <is>
           <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
         </is>
       </c>
-      <c r="Q39" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=ad5c728ff17738e7bd83d093069a0c2a65996cc5&amp;tsid=4129930003</t>
+      <c r="Q41" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=c61084f649b6de8adb87da7e7712cbd359326b47&amp;tsid=4129930003</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q39"/>
+  <autoFilter ref="A1:Q41"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -3574,6 +3734,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId40"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-08 21:54 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q41"/>
+  <dimension ref="A1:Q40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -621,14 +621,14 @@
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/gk-ao-logika-moloka-mk-kazan-vypolnenie-rabot-po-tekushchemu-remontu/tender-4518085/#btid=2&amp;sqh=205eb0da7eb9426cf1073846adc5ae6e8e3f427a&amp;tsid=4518085458</t>
+          <t>https://www.b2b-center.ru/app/market-next/gk-ao-logika-moloka-mk-kazan-vypolnenie-rabot-po-tekushchemu-remontu/tender-4518085/#btid=2&amp;sqh=7e7f430ea309d9e7ba9d92330037515147bd2b2f&amp;tsid=4518085458</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -701,14 +701,14 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/stroitelnye-materialy-postavka-v-nakhodku-dlia-ooo-svetloe-postavka/tender-4515159/#btid=2&amp;sqh=205eb0da7eb9426cf1073846adc5ae6e8e3f427a&amp;tsid=4515159004</t>
+          <t>https://www.b2b-center.ru/market/stroitelnye-materialy-postavka-v-nakhodku-dlia-ooo-svetloe-postavka/tender-4515159/#btid=2&amp;sqh=7e7f430ea309d9e7ba9d92330037515147bd2b2f&amp;tsid=4515159004</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -781,14 +781,14 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=205eb0da7eb9426cf1073846adc5ae6e8e3f427a&amp;tsid=4510835003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=7e7f430ea309d9e7ba9d92330037515147bd2b2f&amp;tsid=4510835003</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -860,14 +860,14 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/remont-dorozhnoi-plitki-na-pod-ezdnoi-i-vyezdnoi-doroge-ot-glavnogo/tender-4506366/#btid=2&amp;sqh=205eb0da7eb9426cf1073846adc5ae6e8e3f427a&amp;tsid=4506366458</t>
+          <t>https://www.b2b-center.ru/app/market-next/remont-dorozhnoi-plitki-na-pod-ezdnoi-i-vyezdnoi-doroge-ot-glavnogo/tender-4506366/#btid=2&amp;sqh=7e7f430ea309d9e7ba9d92330037515147bd2b2f&amp;tsid=4506366458</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -939,14 +939,14 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=205eb0da7eb9426cf1073846adc5ae6e8e3f427a&amp;tsid=4130106003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=7e7f430ea309d9e7ba9d92330037515147bd2b2f&amp;tsid=4130106003</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1018,14 +1018,14 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=20f081afdcf5d4216fe7f7d55028026da25573b4&amp;tsid=4498936003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=7ca8303a65c1a30cbea65c4ff3722aa91162da88&amp;tsid=4498936003</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1098,14 +1098,14 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=932f29f78b9e46c99545830aafd6fbf41b0a25c1&amp;tsid=4497016004</t>
+          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=74802e65efe7c97e35b3d92d42e9245e0dd2fb1e&amp;tsid=4497016004</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1177,14 +1177,14 @@
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/2228-opry-lep-po-zaiavke-mg-019766/tender-4518573/#btid=2&amp;sqh=d419ff3a6d419d91b36995ba662568dcb7bb8545&amp;tsid=4518573004</t>
+          <t>https://www.b2b-center.ru/market/2228-opry-lep-po-zaiavke-mg-019766/tender-4518573/#btid=2&amp;sqh=126d75d692f2ff393304d4fd68020dcaed2781ca&amp;tsid=4518573004</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1195,32 +1195,32 @@
       <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Работы</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>4512196</t>
+          <t>4512292</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>ОПОРА ЛЭПЛИСТВ НЕПРОПИТАН 22-28СМ L11</t>
+          <t>ТЕХНИЧЕСКОЕ ЗАДАНИЕ на строительствоЛЭП-6кВдля электроснабжения электрогидравлического экскаватора Liebherr 9200Е Работы по строительствуЛЭП-6кВдля электроснабжения электрогидравлического экскаватора Liebherr 9200Е.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "СЕРВИС ПЛЮС"</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "СЕРВИС ПЛЮС"</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>7704643931</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1228,7 +1228,11 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Иванов Владимир Ильич</t>
+        </is>
+      </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1236,30 +1240,30 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>68.32</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr"/>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 11:30 — 09.07.2026 00:00</t>
+          <t>03.07.2026 12:19 — 14.07.2026 12:00</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Москва, ул Пречистенка, д 40/2 стр 4, помещ I, ком 2А</t>
         </is>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/opora-lep-listv-nepropitan-22-28sm-l11/tender-4512196/#btid=2&amp;sqh=d419ff3a6d419d91b36995ba662568dcb7bb8545&amp;tsid=4512196458</t>
+          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=126d75d692f2ff393304d4fd68020dcaed2781ca&amp;tsid=4512292004</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1270,32 +1274,32 @@
       <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Работы</t>
+          <t>Прочее</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>4512292</t>
+          <t>4517766</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>ТЕХНИЧЕСКОЕ ЗАДАНИЕ на строительствоЛЭП-6кВдля электроснабжения электрогидравлического экскаватора Liebherr 9200Е Работы по строительствуЛЭП-6кВдля электроснабжения электрогидравлического экскаватора Liebherr 9200Е.</t>
+          <t>Заявка № ДОР-17519 ( /ЖБИ изделия/)Плиты перекрытия ПК-15КольцоК-7-1КольцоК-7-3КольцоК-7-5 ...  крышка ДКЛКольцоВГ-15КольцоК-15-10КольцоК-15-8КольцоК-15 ... -7КольцоК-15-6Кольцо...  К-15-5 Плита днища ДДК-8КолодецВД ...</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>ООО "СЕРВИС ПЛЮС"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>ООО "СЕРВИС ПЛЮС"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>7704643931</t>
+          <t>7724498866</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -1305,7 +1309,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Иванов Владимир Ильич</t>
+          <t>Городний Анатолий Валерьевич</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1315,30 +1319,30 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>68.32</t>
+          <t>46.73</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr"/>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 12:19 — 14.07.2026 12:00</t>
+          <t>08.07.2026 12:34 — 09.07.2026 16:00</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Пречистенка, д 40/2 стр 4, помещ I, ком 2А</t>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
         </is>
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=d419ff3a6d419d91b36995ba662568dcb7bb8545&amp;tsid=4512292004</t>
+          <t>https://www.b2b-center.ru/app/market-next/zaiavka-dor-17519-zhbi-izdeliia/tender-4517766/#btid=2&amp;sqh=30b662768b6c3c0e209a92625a122c3aaba5749e&amp;tsid=4517766459</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1354,89 +1358,10 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>4517766</t>
+          <t>4475879</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Заявка № ДОР-17519 ( /ЖБИ изделия/)Плиты перекрытия ПК-15КольцоК-7-1КольцоК-7-3КольцоК-7-5 ...  крышка ДКЛКольцоВГ-15КольцоК-15-10КольцоК-15-8КольцоК-15 ... -7КольцоК-15-6Кольцо...  К-15-5 Плита днища ДДК-8КолодецВД ...</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>7724498866</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>Городний Анатолий Валерьевич</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>46.73</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr"/>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>08.07.2026 12:34 — 09.07.2026 16:00</t>
-        </is>
-      </c>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
-        </is>
-      </c>
-      <c r="Q12" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/app/market-next/zaiavka-dor-17519-zhbi-izdeliia/tender-4517766/#btid=2&amp;sqh=09c932b695968d7bb9663ffc840a0f8be026b09f&amp;tsid=4517766459</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 17:16</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr"/>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>4475879</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Электро/пневмо и ручной инструмент/Электроизм. инструмент/Расходные мат-лы
 РТИ, РВД, шланги, ремни
@@ -1444,31 +1369,106 @@
 Уплотнительный материал (прокладки, паронит, набивка сальниковая)...  Шина цепной пилы Oregon 752HSFL104Кольцостопор. нар. 210х5 DIN471 Andritz ... клин для бревен Sandvik 1401КольцоAbicor Binzel 757.D007 вихреобразующее ...  Kron ЦПВС-5 RAL7012 КрышкаколодцаП10 ж/б Игла клапана ... Kron ПСВС-3 RAL7012 О-кольцо11,3х2,4 NBR70 Ремень ...</t>
         </is>
       </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>4704012472</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Ленинградская обл</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Габидуллин Тимур Махмудович</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>17.12</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>03.06.2026 15:56 — 30.07.2026 20:00</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+        </is>
+      </c>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=30b662768b6c3c0e209a92625a122c3aaba5749e&amp;tsid=4475879003</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08 21:54</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>4514583</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Закупка ЖБИ (плитыПДН3*1,5)</t>
+        </is>
+      </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>4704012472</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>Габидуллин Тимур Махмудович</t>
-        </is>
-      </c>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr"/>
       <c r="L13" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1476,30 +1476,30 @@
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>17.12</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr"/>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>03.06.2026 15:56 — 30.07.2026 20:00</t>
+          <t>06.07.2026 15:00 — 09.07.2026 12:00</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=09c932b695968d7bb9663ffc840a0f8be026b09f&amp;tsid=4475879003</t>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-plity-pdn-3-1-5/tender-4514583/#btid=2&amp;sqh=644cf4698c56cc8fb64e2ac70ee7d36bb390047a&amp;tsid=4514583458</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1515,27 +1515,27 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>4514583</t>
+          <t>4517935</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Закупка ЖБИ (плитыПДН3*1,5)</t>
+          <t>ЖБИ(Дор № 17559)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>7724498866</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1543,7 +1543,11 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1551,30 +1555,30 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>46.73</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr"/>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>06.07.2026 15:00 — 09.07.2026 12:00</t>
+          <t>08.07.2026 13:40 — 09.07.2026 17:00</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
         </is>
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-plity-pdn-3-1-5/tender-4514583/#btid=2&amp;sqh=cf1203dbd9ec1ad5b95e895ff4f06dd4c715c086&amp;tsid=4514583458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-dor-17559/tender-4517935/#btid=2&amp;sqh=b76aab64d3a1e08073d515c107772aa3df2cfd7a&amp;tsid=4517935459</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1590,27 +1594,27 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>4517935</t>
+          <t>4516217</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>ЖБИ(Дор № 17559)</t>
+          <t>ТМЦЖБИи песок</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>7724498866</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -1618,11 +1622,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>Городний Анатолий Валерьевич</t>
-        </is>
-      </c>
+      <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1630,30 +1630,30 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>46.73</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr"/>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>08.07.2026 13:40 — 09.07.2026 17:00</t>
+          <t>07.07.2026 14:31 — 10.07.2026 10:00</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-dor-17559/tender-4517935/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=4517935459</t>
+          <t>https://www.b2b-center.ru/app/market-next/tmts-zhbi-i-pesok/tender-4516217/#btid=2&amp;sqh=b76aab64d3a1e08073d515c107772aa3df2cfd7a&amp;tsid=4516217458</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1664,32 +1664,32 @@
       <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Поставка</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>4516217</t>
+          <t>4514839</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>ТМЦЖБИи песок</t>
+          <t>12-х-1 Заключение договора на поставку материалов для наружных сетей водоснабжения и водоотведения на объект строительства «Дальневосточный детский центр отдыха и оздоровления в Хабаровском крае». (9 лотов) Лот №1 ВодоснабжениеЖБИ</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "ПРОМСТРОЙ"</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "ПРОМСТРОЙ"</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>9723169975</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1697,7 +1697,11 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Султанов Владислав Назипович</t>
+        </is>
+      </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1705,30 +1709,30 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>71.12.2</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr"/>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>07.07.2026 14:31 — 10.07.2026 10:00</t>
+          <t>06.07.2026 16:45 — 10.07.2026 11:00</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Москва, Волгоградский пр-кт, д 42 к 5, ком 9</t>
         </is>
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/tmts-zhbi-i-pesok/tender-4516217/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=4516217458</t>
+          <t>https://www.b2b-center.ru/market/12-kh-1-zakliuchenie-dogovora-na-postavku-materialov-dlia-naruzhnykh-setei/tender-4514839/#btid=2&amp;sqh=b76aab64d3a1e08073d515c107772aa3df2cfd7a&amp;tsid=4514839004</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1744,27 +1748,27 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>4513278</t>
+          <t>4510662</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>ЖБИблоки ФБС</t>
+          <t>(ЖБИизделия/кольца колодезные, плиты ПК15)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>7724498866</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -1772,7 +1776,11 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1780,30 +1788,30 @@
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>46.73</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr"/>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>06.07.2026 04:17 — 09.07.2026 00:00</t>
+          <t>02.07.2026 12:00 — 09.07.2026 13:00</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
         </is>
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-bloki-fbs/tender-4513278/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=4513278458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-izdeliia-koltsa-kolodeznye-plity-pk15/tender-4510662/#btid=2&amp;sqh=b76aab64d3a1e08073d515c107772aa3df2cfd7a&amp;tsid=4510662459</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1814,32 +1822,32 @@
       <c r="C18" s="2" t="inlineStr"/>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Поставка</t>
+          <t>Прочее</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>4514839</t>
+          <t>4510504</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>12-х-1 Заключение договора на поставку материалов для наружных сетей водоснабжения и водоотведения на объект строительства «Дальневосточный детский центр отдыха и оздоровления в Хабаровском крае». (9 лотов) Лот №1 ВодоснабжениеЖБИ</t>
+          <t>(Заявка № ДОР-17560) Лестницы/ЖБИ</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>ООО "ПРОМСТРОЙ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>ООО "ПРОМСТРОЙ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>9723169975</t>
+          <t>7724498866</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1849,7 +1857,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Султанов Владислав Назипович</t>
+          <t>Городний Анатолий Валерьевич</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -1859,30 +1867,30 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>71.12.2</t>
+          <t>46.73</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr"/>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>06.07.2026 16:45 — 10.07.2026 11:00</t>
+          <t>02.07.2026 10:55 — 09.07.2026 13:00</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Волгоградский пр-кт, д 42 к 5, ком 9</t>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
         </is>
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/12-kh-1-zakliuchenie-dogovora-na-postavku-materialov-dlia-naruzhnykh-setei/tender-4514839/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=4514839004</t>
+          <t>https://www.b2b-center.ru/app/market-next/zaiavka-dor-17560-lestnitsy-zhbi/tender-4510504/#btid=2&amp;sqh=b76aab64d3a1e08073d515c107772aa3df2cfd7a&amp;tsid=4510504459</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1898,12 +1906,12 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>4510662</t>
+          <t>4510823</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>(ЖБИизделия/кольца колодезные, плиты ПК15)</t>
+          <t>(ДОР-17553)ЖБИ/Лестницы ВЛ-2/Скоба</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1944,7 +1952,7 @@
       <c r="N19" s="2" t="inlineStr"/>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>02.07.2026 12:00 — 09.07.2026 13:00</t>
+          <t>02.07.2026 12:55 — 09.07.2026 11:00</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -1954,14 +1962,14 @@
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-izdeliia-koltsa-kolodeznye-plity-pk15/tender-4510662/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=4510662459</t>
+          <t>https://www.b2b-center.ru/app/market-next/dor-17553-zhbi-lestnitsy-vl-2-skoba/tender-4510823/#btid=2&amp;sqh=b76aab64d3a1e08073d515c107772aa3df2cfd7a&amp;tsid=4510823459</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1977,27 +1985,27 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>4510504</t>
+          <t>4508347</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>(Заявка № ДОР-17560) Лестницы/ЖБИ</t>
+          <t>ЖБИКЕМГРЭС</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>7724498866</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -2005,11 +2013,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>Городний Анатолий Валерьевич</t>
-        </is>
-      </c>
+      <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -2017,30 +2021,30 @@
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>46.73</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr"/>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>02.07.2026 10:55 — 09.07.2026 13:00</t>
+          <t>01.07.2026 05:45 — 10.07.2026 00:00</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zaiavka-dor-17560-lestnitsy-zhbi/tender-4510504/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=4510504459</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=b76aab64d3a1e08073d515c107772aa3df2cfd7a&amp;tsid=4508347458</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -2056,27 +2060,27 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>4510823</t>
+          <t>4489772</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>(ДОР-17553)ЖБИ/Лестницы ВЛ-2/Скоба</t>
+          <t>1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы 1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>7724498866</t>
+          <t>7736583259</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -2086,7 +2090,7 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Городний Анатолий Валерьевич</t>
+          <t>Масько Александр Вадимович</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -2096,30 +2100,30 @@
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>46.73</t>
+          <t>70.10</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr"/>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>02.07.2026 12:55 — 09.07.2026 11:00</t>
+          <t>16.06.2026 11:00 — 16.07.2026 12:00</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+          <t>г Москва, ул Старая Басманная, д 12 стр 1</t>
         </is>
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/dor-17553-zhbi-lestnitsy-vl-2-skoba/tender-4510823/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=4510823459</t>
+          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=b76aab64d3a1e08073d515c107772aa3df2cfd7a&amp;tsid=4489772003</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2135,35 +2139,39 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>4508347</t>
+          <t>4474790</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>ЖБИКЕМГРЭС</t>
+          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>4704012472</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr"/>
+          <t>Ленинградская обл</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Габидуллин Тимур Махмудович</t>
+        </is>
+      </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -2171,30 +2179,30 @@
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>17.12</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr"/>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>01.07.2026 05:45 — 10.07.2026 00:00</t>
+          <t>03.06.2026 09:59 — 30.07.2026 20:00</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
         </is>
       </c>
       <c r="Q22" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=4508347458</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=b76aab64d3a1e08073d515c107772aa3df2cfd7a&amp;tsid=4474790003</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2210,27 +2218,27 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>4489772</t>
+          <t>4180328</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы 1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы</t>
+          <t>ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, г.Диксон). ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, ПГТ Диксон).</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
+          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
+          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>7736583259</t>
+          <t>7714456916</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
@@ -2240,7 +2248,7 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Масько Александр Вадимович</t>
+          <t>Наумов Андрей Александрович</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
@@ -2250,30 +2258,30 @@
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>70.10</t>
+          <t>70.22</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr"/>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>16.06.2026 11:00 — 16.07.2026 12:00</t>
+          <t>24.09.2025 15:32 — 23.07.2026 12:00</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Старая Басманная, д 12 стр 1</t>
+          <t>г Москва, Денежный пер, д 9/6</t>
         </is>
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=4489772003</t>
+          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=b76aab64d3a1e08073d515c107772aa3df2cfd7a&amp;tsid=4180328003</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2289,7 +2297,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>4474790</t>
+          <t>3973258</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2335,7 +2343,7 @@
       <c r="N24" s="2" t="inlineStr"/>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>03.06.2026 09:59 — 30.07.2026 20:00</t>
+          <t>10.03.2025 00:48 — 30.07.2026 23:00</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -2345,14 +2353,14 @@
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=4474790003</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=b76aab64d3a1e08073d515c107772aa3df2cfd7a&amp;tsid=3973258003</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -2368,37 +2376,40 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>4180328</t>
+          <t>4517919</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, г.Диксон). ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, ПГТ Диксон).</t>
+          <t>Кольцо опорное с днищем для нужд ООО ГРК Амикан. Требуется жесткая упаковка по ГОСТу
+КП по форме ТД Полиметалл.
+В цену включить стоимость доставки до адреса в г. Лесосибирск и обрешетки.
+При подаче аналогов необходимо приложить тех. документацию.4517919 ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "ТОРГОВЫЙ ДОМ ПОЛИМЕТАЛЛ"Железобетонные изделия</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>7714456916</t>
+          <t>7805368914</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
+          <t>г Санкт-Петербург</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Наумов Андрей Александрович</t>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
@@ -2408,30 +2419,30 @@
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>70.22</t>
+          <t>46.90</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr"/>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>24.09.2025 15:32 — 23.07.2026 12:00</t>
+          <t>08.07.2026 14:18 — 15.07.2026 10:00</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Денежный пер, д 9/6</t>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
       <c r="Q25" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=4180328003</t>
+          <t>https://www.b2b-center.ru/market/koltso-opornoe-s-dnishchem-dlia-nuzhd-ooo-grk-amikan-trebuetsia-zhestkaia/tender-4517919/#btid=2&amp;sqh=89742f9ad89f2d0628eb6c8f37f8a3612ae1205c&amp;tsid=4517919004</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2442,44 +2453,40 @@
       <c r="C26" s="2" t="inlineStr"/>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Поставка</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>3973258</t>
+          <t>4513525</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
+          <t>Поставка модульных защитных сооруженийЗДАНИЕ ЗАЩИТНОЕ ДЛЯ УКРЫТИЯ 4,4*2,4*2,2МЖЕЛЕЗОБЕТОННОЕСБОРНОЕ</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>4704012472</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>Габидуллин Тимур Махмудович</t>
-        </is>
-      </c>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -2487,30 +2494,30 @@
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>17.12</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr"/>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>10.03.2025 00:48 — 30.07.2026 23:00</t>
+          <t>06.07.2026 08:36 — 10.07.2026 14:00</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q26" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=836a6cc7975ce27f733d610c25121da4d37c43a8&amp;tsid=3973258003</t>
+          <t>https://www.b2b-center.ru/app/market-next/postavka-modulnykh-zashchitnykh-sooruzhenii/tender-4513525/#btid=2&amp;sqh=89742f9ad89f2d0628eb6c8f37f8a3612ae1205c&amp;tsid=4513525458</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -2521,90 +2528,15 @@
       <c r="C27" s="2" t="inlineStr"/>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Поставка</t>
+          <t>Прочее</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>4513525</t>
+          <t>4513563</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>Поставка модульных защитных сооруженийЗДАНИЕ ЗАЩИТНОЕ ДЛЯ УКРЫТИЯ 4,4*2,4*2,2МЖЕЛЕЗОБЕТОННОЕСБОРНОЕ</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>9725042029</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr"/>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M27" s="2" t="inlineStr">
-        <is>
-          <t>64.20</t>
-        </is>
-      </c>
-      <c r="N27" s="2" t="inlineStr"/>
-      <c r="O27" s="2" t="inlineStr">
-        <is>
-          <t>06.07.2026 08:36 — 10.07.2026 14:00</t>
-        </is>
-      </c>
-      <c r="P27" s="2" t="inlineStr">
-        <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
-        </is>
-      </c>
-      <c r="Q27" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/app/market-next/postavka-modulnykh-zashchitnykh-sooruzhenii/tender-4513525/#btid=2&amp;sqh=39868999b159823b02130aa6f265a3a7ff3e9512&amp;tsid=4513525458</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 17:16</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>4513563</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Блок ФБС 12.4.6-Т-и
 Кольцо стеновое КС 20.9 ГОСТ 8020-2016
@@ -2613,31 +2545,106 @@
 Кольцо стеновое КС 20.9 ГОСТ 8020-20164513563 ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "ТОРГОВЫЙ ДОМ ПОЛИМЕТАЛЛ"Железобетонные изделия</t>
         </is>
       </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>7805368914</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>46.90</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr"/>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>06.07.2026 08:49 — 10.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
+        </is>
+      </c>
+      <c r="Q27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/blok-fbs-12-4-6-t-i-koltso-stenovoe-ks-20-9-gost-8020-2016-na-k-pm/tender-4513563/#btid=2&amp;sqh=89742f9ad89f2d0628eb6c8f37f8a3612ae1205c&amp;tsid=4513563004</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08 21:54</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>4517499</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>КРЫШКА-ПАТРУБОК 200-Т-535СБ ПК-40; ЗАГЛУШКА НА КЛАПАН СД К-5976.00.00 СБ; КРЫШКА 200-Т-525СБ ПК-40;ПЕРЕМЫЧКАД/ПРОДУВКИ ППХ 200-Т-530 СБ</t>
+        </is>
+      </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>7805368914</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>г Санкт-Петербург</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
-        </is>
-      </c>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -2645,30 +2652,30 @@
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>46.90</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr"/>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>06.07.2026 08:49 — 10.07.2026 12:00</t>
+          <t>08.07.2026 10:53 — 10.07.2026 12:00</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q28" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/blok-fbs-12-4-6-t-i-koltso-stenovoe-ks-20-9-gost-8020-2016-na-k-pm/tender-4513563/#btid=2&amp;sqh=39868999b159823b02130aa6f265a3a7ff3e9512&amp;tsid=4513563004</t>
+          <t>https://www.b2b-center.ru/app/market-next/kryshka-patrubok-200-t-535sb-pk-40-zaglushka-na-klapan-sd-k-5976-00-00/tender-4517499/#btid=2&amp;sqh=c47fd9ae2b92e169b8e2d5a0e25b7d57701224bc&amp;tsid=4517499458</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -2684,35 +2691,39 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>4517499</t>
+          <t>4512541</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>КРЫШКА-ПАТРУБОК 200-Т-535СБ ПК-40; ЗАГЛУШКА НА КЛАПАН СД К-5976.00.00 СБ; КРЫШКА 200-Т-525СБ ПК-40;ПЕРЕМЫЧКАД/ПРОДУВКИ ППХ 200-Т-530 СБ</t>
+          <t>Запасные части CAT.... -3748 Cat Опора 348-9537 CatПеремычка140-0860 Cat Скоба 8X-3130 ...</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>1004001744</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K29" s="2" t="inlineStr"/>
+          <t>Респ Карелия</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "СЕВЕРСТАЛЬ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -2720,30 +2731,30 @@
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>07.10.2</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr"/>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>08.07.2026 10:53 — 10.07.2026 12:00</t>
+          <t>03.07.2026 14:07 — 10.07.2026 11:00</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>Респ Карелия, г Костомукша, шоссе Горняков, стр 284</t>
         </is>
       </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/kryshka-patrubok-200-t-535sb-pk-40-zaglushka-na-klapan-sd-k-5976-00-00/tender-4517499/#btid=2&amp;sqh=4ba4cb5de9195180187222c70541fed058c879ca&amp;tsid=4517499458</t>
+          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=c47fd9ae2b92e169b8e2d5a0e25b7d57701224bc&amp;tsid=4512541003</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -2759,37 +2770,38 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>4512541</t>
+          <t>4508230</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Запасные части CAT.... -3748 Cat Опора 348-9537 CatПеремычка140-0860 Cat Скоба 8X-3130 ...</t>
+          <t>Сборный (Изделия электроустановочные и монтажные, Ящики, щиты, шкафы, пункты и комплектующие к ним, Приборы электроизмерительные, реле)
+МГ-019742, МГ-019713, МГ-019696, МГ-019665, МГ-019621, МГ-019620, МГ-019619, МГ-017109... -HESI-EX (5X20), Phoenix Contact 1277638ПеремычкаFBS 10-5, Phoenix Contact 3030213 ...ПеремычкаFBS 10-5 BU, Phoenix Contact  ...</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
+          <t>АО "ИК "АРЛАН"</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
+          <t>АО "ИК "АРЛАН"</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>1004001744</t>
+          <t>7722220390</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>Респ Карелия</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "СЕВЕРСТАЛЬ МЕНЕДЖМЕНТ"</t>
+          <t>Барилов Евгений Александрович</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
@@ -2799,30 +2811,30 @@
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>07.10.2</t>
+          <t>82.99</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr"/>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 14:07 — 10.07.2026 11:00</t>
+          <t>30.06.2026 17:59 — 09.07.2026 12:00</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>Респ Карелия, г Костомукша, шоссе Горняков, стр 284</t>
+          <t>г Москва, Романов пер, д 4</t>
         </is>
       </c>
       <c r="Q30" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=4ba4cb5de9195180187222c70541fed058c879ca&amp;tsid=4512541003</t>
+          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=c47fd9ae2b92e169b8e2d5a0e25b7d57701224bc&amp;tsid=4508230004</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -2838,28 +2850,27 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>4508230</t>
+          <t>4501157</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Сборный (Изделия электроустановочные и монтажные, Ящики, щиты, шкафы, пункты и комплектующие к ним, Приборы электроизмерительные, реле)
-МГ-019742, МГ-019713, МГ-019696, МГ-019665, МГ-019621, МГ-019620, МГ-019619, МГ-017109... -HESI-EX (5X20), Phoenix Contact 1277638ПеремычкаFBS 10-5, Phoenix Contact 3030213 ...ПеремычкаFBS 10-5 BU, Phoenix Contact  ...</t>
+          <t>Источники электропитания (ИБП, аккумуляторные батареи, блоки питания)...  х 1248 А·ч, включая соединительныеперемычки. Вид положительного электрода - трубчатая пластина ...  с коммутирующей арматурой, межэлементными и межряднымиперемычками, крепежами, комплектом для обслуживания АБ. Тип ...</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>АО "ИК "АРЛАН"</t>
+          <t>АО "Мосинжпроект"</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>АО "ИК "АРЛАН"</t>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>7722220390</t>
+          <t>7701885820</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
@@ -2869,7 +2880,7 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>Барилов Евгений Александрович</t>
+          <t>Сорокин Антон Павлович</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
@@ -2879,30 +2890,30 @@
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>82.99</t>
+          <t>71.12.2</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr"/>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>30.06.2026 17:59 — 09.07.2026 12:00</t>
+          <t>24.06.2026 15:40 — 22.07.2026 12:00</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Романов пер, д 4</t>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
         </is>
       </c>
       <c r="Q31" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=4ba4cb5de9195180187222c70541fed058c879ca&amp;tsid=4508230004</t>
+          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=c47fd9ae2b92e169b8e2d5a0e25b7d57701224bc&amp;tsid=4501157003</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -2918,12 +2929,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>4501157</t>
+          <t>4499964</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Источники электропитания (ИБП, аккумуляторные батареи, блоки питания)...  х 1248 А·ч, включая соединительныеперемычки. Вид положительного электрода - трубчатая пластина ...  с коммутирующей арматурой, межэлементными и межряднымиперемычками, крепежами, комплектом для обслуживания АБ. Тип ...</t>
+          <t>Автоматика и телемеханика движения поездов... , 13552-00-00В Дроссель-трансформатор (безперемычек) ДТМ-0,17-1000М ЮКЛЯ.672 ...</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -2964,7 +2975,7 @@
       <c r="N32" s="2" t="inlineStr"/>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 15:40 — 22.07.2026 12:00</t>
+          <t>24.06.2026 08:46 — 15.07.2026 12:00</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
@@ -2974,14 +2985,14 @@
       </c>
       <c r="Q32" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=4ba4cb5de9195180187222c70541fed058c879ca&amp;tsid=4501157003</t>
+          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=c47fd9ae2b92e169b8e2d5a0e25b7d57701224bc&amp;tsid=4499964003</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -2997,37 +3008,38 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>4499964</t>
+          <t>4504775</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Автоматика и телемеханика движения поездов... , 13552-00-00В Дроссель-трансформатор (безперемычек) ДТМ-0,17-1000М ЮКЛЯ.672 ...</t>
+          <t>Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники
+Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники...  Трубка пробная № 37-542-000 Соединитель-перемычка04182454 Кольцо стальное №CP48001-0305 Фильтр ...</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>АО "Мосинжпроект"</t>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>АО "МОСИНЖПРОЕКТ"</t>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>7701885820</t>
+          <t>7805368914</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
+          <t>г Санкт-Петербург</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Сорокин Антон Павлович</t>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
@@ -3037,30 +3049,30 @@
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>71.12.2</t>
+          <t>46.90</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr"/>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 08:46 — 15.07.2026 12:00</t>
+          <t>27.06.2026 01:36 — 15.07.2026 12:00</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
       <c r="Q33" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=4ba4cb5de9195180187222c70541fed058c879ca&amp;tsid=4499964003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=c47fd9ae2b92e169b8e2d5a0e25b7d57701224bc&amp;tsid=4504775003</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3076,38 +3088,38 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>4504775</t>
+          <t>4449201</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники
-Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники...  Трубка пробная № 37-542-000 Соединитель-перемычка04182454 Кольцо стальное №CP48001-0305 Фильтр ...</t>
+          <t>Реализация НВИ, Оборудование теплообменное; Оборудование емкостное; Запчасти и узлы теплообменного оборудования; Запчасти и узлы емкостного оборудования;
+Продажа НВИ согласно прилагаемого перечня. 110-Емкостное и теп-ое об-е; 136-Запчасти и узлы емкостного и теплообПрокладка сперемычкамидля теплообменников ПУТГм-Б-09-01( ... . Е-21504.05.06 Прокладка сперемычкамидля теплообменников ПУТГм-Б-09-01 ...</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+          <t>ООО "СИБУР"</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+          <t>ООО "СИБУР"</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>7805368914</t>
+          <t>7727576505</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>г Санкт-Петербург</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
+          <t>Карисалов Михаил Юрьевич</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
@@ -3117,30 +3129,30 @@
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>46.90</t>
+          <t>70.10</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr"/>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>27.06.2026 01:36 — 15.07.2026 12:00</t>
+          <t>15.05.2026 06:57 — 10.07.2026 12:00</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
+          <t>г Москва, ул Кржижановского, д 16 к 3</t>
         </is>
       </c>
       <c r="Q34" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=4ba4cb5de9195180187222c70541fed058c879ca&amp;tsid=4504775003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nvi-oborudovanie-teploobmennoe-oborudovanie-emkostnoe/tender-4449201/#btid=2&amp;sqh=c47fd9ae2b92e169b8e2d5a0e25b7d57701224bc&amp;tsid=4449201003</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -3156,13 +3168,12 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>4480614</t>
+          <t>4512370</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Плановое и аварийное техническое обслуживание зданий и сооружений (годовое обслуживание август 2026 - август 2027) ГК Логика молока, производственная площадка в г. Ялуторовске
-Обслуживание зданий и сооружений завода в г. Ялуторовске....  стен из газобетонных блоков Устройство металлическихперемычекс устройством штраб Усиление кирпичных стен ...</t>
+          <t>ТО Сплит систем Лабинск Эйч энд Эн... кондиционирования Техническое обслуживание внутреннегоблокакассетного типа мультизональной  ...блокакондиционера. Мойка теплообменника внутреннегоблокакондиционера Чистка фильтров внутреннегоблокакондиционера Чистка фильтров приточнойвентиляционной...</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -3203,7 +3214,7 @@
       <c r="N35" s="2" t="inlineStr"/>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>08.06.2026 14:44 — 08.07.2026 23:00</t>
+          <t>03.07.2026 12:40 — 14.07.2026 18:30</t>
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr">
@@ -3213,14 +3224,14 @@
       </c>
       <c r="Q35" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/planovoe-i-avariinoe-tekhnicheskoe-obsluzhivanie-zdanii-i-sooruzhenii/tender-4480614/#btid=2&amp;sqh=4ba4cb5de9195180187222c70541fed058c879ca&amp;tsid=4480614004</t>
+          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=81d361b3df721ca4c08106d95f9fd6e553bf88c0&amp;tsid=4512370458</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -3236,27 +3247,27 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>4512370</t>
+          <t>4501181</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>ТО Сплит систем Лабинск Эйч энд Эн... кондиционирования Техническое обслуживание внутреннегоблокакассетного типа мультизональной  ...блокакондиционера. Мойка теплообменника внутреннегоблокакондиционера Чистка фильтров внутреннегоблокакондиционера Чистка фильтров приточнойвентиляционной...</t>
+          <t>Вентиляторы промышленные и оборудование общеобменной вентиляции...  5Ф РешёткавентиляционнаяАМР 600х300М РешёткавентиляционнаяАМР 150х150М РешёткавентиляционнаяАМР 300х200М  ... мм.; масса 0,65 кгБлокконтроля сопротивления БСК-3.1 Канальный ...  533Па, габаритные размеры 700х467х2230 мм,блоков/моноблоков 5/1, в составе: - ...</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>АО "ЭЙЧ ЭНД ЭН"</t>
+          <t>АО "Мосинжпроект"</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>АО "ЭЙЧ ЭНД ЭН"</t>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>7714626332</t>
+          <t>7701885820</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -3266,7 +3277,7 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>Закриев Якуб Салманович</t>
+          <t>Сорокин Антон Павлович</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
@@ -3276,30 +3287,30 @@
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>10.51.9</t>
+          <t>71.12.2</t>
         </is>
       </c>
       <c r="N36" s="2" t="inlineStr"/>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 12:40 — 14.07.2026 18:30</t>
+          <t>24.06.2026 15:45 — 22.07.2026 12:00</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Вятская, д 27 стр 13</t>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
         </is>
       </c>
       <c r="Q36" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=c61084f649b6de8adb87da7e7712cbd359326b47&amp;tsid=4512370458</t>
+          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=81d361b3df721ca4c08106d95f9fd6e553bf88c0&amp;tsid=4501181003</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -3315,37 +3326,38 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>4501181</t>
+          <t>4501483</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Вентиляторы промышленные и оборудование общеобменной вентиляции...  5Ф РешёткавентиляционнаяАМР 600х300М РешёткавентиляционнаяАМР 150х150М РешёткавентиляционнаяАМР 300х200М  ... мм.; масса 0,65 кгБлокконтроля сопротивления БСК-3.1 Канальный ...  533Па, габаритные размеры 700х467х2230 мм,блоков/моноблоков 5/1, в составе: - ...</t>
+          <t>Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ
+Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ...  d 50x2", внутренняя резьба RTPБлокуправления наружной установки ICEFREE TR-16 ...  Оповещатель звуковой МАЯК-12-ЗМБлокуправления наружной установки ICEFREE TS- ... проводов КС-3 007004 Велос Переходвентиляционный150х100 - D150, из тонколистовой оцинкованной ...</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>АО "Мосинжпроект"</t>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>АО "МОСИНЖПРОЕКТ"</t>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>7701885820</t>
+          <t>7805368914</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
+          <t>г Санкт-Петербург</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>Сорокин Антон Павлович</t>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
@@ -3355,30 +3367,30 @@
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>71.12.2</t>
+          <t>46.90</t>
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr"/>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 15:45 — 22.07.2026 12:00</t>
+          <t>25.06.2026 05:03 — 09.07.2026 12:00</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
       <c r="Q37" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=c61084f649b6de8adb87da7e7712cbd359326b47&amp;tsid=4501181003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=81d361b3df721ca4c08106d95f9fd6e553bf88c0&amp;tsid=4501483003</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -3394,38 +3406,37 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>4501483</t>
+          <t>4500120</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ
-Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ...  d 50x2", внутренняя резьба RTPБлокуправления наружной установки ICEFREE TR-16 ...  Оповещатель звуковой МАЯК-12-ЗМБлокуправления наружной установки ICEFREE TS- ... проводов КС-3 007004 Велос Переходвентиляционный150х100 - D150, из тонколистовой оцинкованной ...</t>
+          <t>Коммуникационное оборудование, компьютеры, комплектующие к ним, серверное оборудование и ПО...  и кабелей – 1 компл. Удаленныйблок(репитер) BSF414 , питание 220В,  ... 2х2 Комбайнер специализированный OMU Side (блок1) OMUSC1 Комбайнер специализированный OMU ... контроллер для мониторинга в FlexGain View,вентиляционнаяпанель с фильтрами, комплект кабелей, ...</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+          <t>АО "Мосинжпроект"</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>7805368914</t>
+          <t>7701885820</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>г Санкт-Петербург</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
+          <t>Сорокин Антон Павлович</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
@@ -3435,30 +3446,30 @@
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>46.90</t>
+          <t>71.12.2</t>
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr"/>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>25.06.2026 05:03 — 09.07.2026 12:00</t>
+          <t>24.06.2026 09:48 — 15.07.2026 12:00</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
         </is>
       </c>
       <c r="Q38" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=c61084f649b6de8adb87da7e7712cbd359326b47&amp;tsid=4501483003</t>
+          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=81d361b3df721ca4c08106d95f9fd6e553bf88c0&amp;tsid=4500120003</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -3474,27 +3485,28 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>4500120</t>
+          <t>4496006</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Коммуникационное оборудование, компьютеры, комплектующие к ним, серверное оборудование и ПО...  и кабелей – 1 компл. Удаленныйблок(репитер) BSF414 , питание 220В,  ... 2х2 Комбайнер специализированный OMU Side (блок1) OMUSC1 Комбайнер специализированный OMU ... контроллер для мониторинга в FlexGain View,вентиляционнаяпанель с фильтрами, комплект кабелей, ...</t>
+          <t>Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп
+Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп... -316 ***Петля крепежная стальная ***Платаблокауправления ZC5 CAME ***Средство чистящее " ... /распылитель для чаши Генуя ***РешеткавентиляционнаяРВ-1 225Х225 ***Петля анкерная 0 ... мл ***Папка с зажимом ***РешеткавентиляционнаяРВ-1 325Х125 ***Папка на кольцах ...</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>АО "Мосинжпроект"</t>
+          <t>ООО "СИБУР"</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>АО "МОСИНЖПРОЕКТ"</t>
+          <t>ООО "СИБУР"</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>7701885820</t>
+          <t>7727576505</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
@@ -3504,7 +3516,7 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Сорокин Антон Павлович</t>
+          <t>Карисалов Михаил Юрьевич</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
@@ -3514,30 +3526,30 @@
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>71.12.2</t>
+          <t>70.10</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr"/>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 09:48 — 15.07.2026 12:00</t>
+          <t>20.06.2026 16:19 — 11.07.2026 12:00</t>
         </is>
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+          <t>г Москва, ул Кржижановского, д 16 к 3</t>
         </is>
       </c>
       <c r="Q39" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=c61084f649b6de8adb87da7e7712cbd359326b47&amp;tsid=4500120003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-nelikvidnykh-tmts-tarelki-dlia-filtra-prokladki-dvigatel/tender-4496006/#btid=2&amp;sqh=81d361b3df721ca4c08106d95f9fd6e553bf88c0&amp;tsid=4496006003</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:16</t>
+          <t>2026-07-08 21:54</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -3548,33 +3560,32 @@
       <c r="C40" s="2" t="inlineStr"/>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Работы</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>4496006</t>
+          <t>4129930</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп
-Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп... -316 ***Петля крепежная стальная ***Платаблокауправления ZC5 CAME ***Средство чистящее " ... /распылитель для чаши Генуя ***РешеткавентиляционнаяРВ-1 225Х225 ***Петля анкерная 0 ... мл ***Папка с зажимом ***РешеткавентиляционнаяРВ-1 325Х125 ***Папка на кольцах ...</t>
+          <t>Реализация материалов для ремонта (напольные покрытия, настенные покрытия, окна, двери и т.д.) с АО "Мальцовский портландцемент"Блокдверной балконныйБлокдверной филенчатый ДГ 21х9Блококонный 1500х1000 ммБлококонный 1770х1700 мм Желоб ...  Docke Рама оконная 3000х1200 мм Решеткавентиляционнаянаружная Ручка оконная ГОСТ 5087-80 ...</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>ООО "СИБУР"</t>
+          <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>ООО "СИБУР"</t>
+          <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>7727576505</t>
+          <t>7708117908</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -3584,7 +3595,7 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>Карисалов Михаил Юрьевич</t>
+          <t>Шматов Вячеслав Вячеславович</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
@@ -3594,107 +3605,28 @@
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>70.10</t>
+          <t>23.51</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr"/>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>20.06.2026 16:19 — 11.07.2026 12:00</t>
+          <t>06.08.2025 14:33 — 07.08.2026 12:00</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Кржижановского, д 16 к 3</t>
+          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
         </is>
       </c>
       <c r="Q40" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nelikvidnykh-tmts-tarelki-dlia-filtra-prokladki-dvigatel/tender-4496006/#btid=2&amp;sqh=c61084f649b6de8adb87da7e7712cbd359326b47&amp;tsid=4496006003</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 17:16</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr"/>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>Работы</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>4129930</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>Реализация материалов для ремонта (напольные покрытия, настенные покрытия, окна, двери и т.д.) с АО "Мальцовский портландцемент"Блокдверной балконныйБлокдверной филенчатый ДГ 21х9Блококонный 1500х1000 ммБлококонный 1770х1700 мм Желоб ...  Docke Рама оконная 3000х1200 мм Решеткавентиляционнаянаружная Ручка оконная ГОСТ 5087-80 ...</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>АО "ЦЕМРОС"</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>АО "ЦЕМРОС"</t>
-        </is>
-      </c>
-      <c r="I41" s="2" t="inlineStr">
-        <is>
-          <t>7708117908</t>
-        </is>
-      </c>
-      <c r="J41" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K41" s="2" t="inlineStr">
-        <is>
-          <t>Шматов Вячеслав Вячеславович</t>
-        </is>
-      </c>
-      <c r="L41" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M41" s="2" t="inlineStr">
-        <is>
-          <t>23.51</t>
-        </is>
-      </c>
-      <c r="N41" s="2" t="inlineStr"/>
-      <c r="O41" s="2" t="inlineStr">
-        <is>
-          <t>06.08.2025 14:33 — 07.08.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P41" s="2" t="inlineStr">
-        <is>
-          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
-        </is>
-      </c>
-      <c r="Q41" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=c61084f649b6de8adb87da7e7712cbd359326b47&amp;tsid=4129930003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=81d361b3df721ca4c08106d95f9fd6e553bf88c0&amp;tsid=4129930003</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q41"/>
+  <autoFilter ref="A1:Q40"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -3735,7 +3667,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId40"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-09 06:24 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q40"/>
+  <dimension ref="A1:Q41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -621,14 +621,14 @@
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/gk-ao-logika-moloka-mk-kazan-vypolnenie-rabot-po-tekushchemu-remontu/tender-4518085/#btid=2&amp;sqh=7e7f430ea309d9e7ba9d92330037515147bd2b2f&amp;tsid=4518085458</t>
+          <t>https://www.b2b-center.ru/app/market-next/gk-ao-logika-moloka-mk-kazan-vypolnenie-rabot-po-tekushchemu-remontu/tender-4518085/#btid=2&amp;sqh=df656b471d512af3cbdfd310cfc48e3283748109&amp;tsid=4518085458</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -701,14 +701,14 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/stroitelnye-materialy-postavka-v-nakhodku-dlia-ooo-svetloe-postavka/tender-4515159/#btid=2&amp;sqh=7e7f430ea309d9e7ba9d92330037515147bd2b2f&amp;tsid=4515159004</t>
+          <t>https://www.b2b-center.ru/market/stroitelnye-materialy-postavka-v-nakhodku-dlia-ooo-svetloe-postavka/tender-4515159/#btid=2&amp;sqh=df656b471d512af3cbdfd310cfc48e3283748109&amp;tsid=4515159004</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -781,14 +781,14 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=7e7f430ea309d9e7ba9d92330037515147bd2b2f&amp;tsid=4510835003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannye-skladskie-ostatki-ne-b-u-zapasnye/tender-4510835/#btid=2&amp;sqh=df656b471d512af3cbdfd310cfc48e3283748109&amp;tsid=4510835003</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -860,14 +860,14 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/remont-dorozhnoi-plitki-na-pod-ezdnoi-i-vyezdnoi-doroge-ot-glavnogo/tender-4506366/#btid=2&amp;sqh=7e7f430ea309d9e7ba9d92330037515147bd2b2f&amp;tsid=4506366458</t>
+          <t>https://www.b2b-center.ru/app/market-next/remont-dorozhnoi-plitki-na-pod-ezdnoi-i-vyezdnoi-doroge-ot-glavnogo/tender-4506366/#btid=2&amp;sqh=df656b471d512af3cbdfd310cfc48e3283748109&amp;tsid=4506366458</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -878,32 +878,33 @@
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Поставка</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>4130106</t>
+          <t>4503612</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Реализация ЖБИ изделий с АО "Мальцовский портландцемент"Бордюрдорожный1000х300х150мм Ясногорский завод строительных материалов Кольца  ...  КС-7-3 ЖБИ 24/7Плитаопорная ОП-1К ПС-334-08 ...Плитаперекрытия колодца 1ПП-20-2 D2200  ...</t>
+          <t>RUNEV-11652 на выполнение работ по сортировке, разделке и вывозу демонтированных 
+трубопроводов и металлоконструкций на склад хранения. Вывозу строительного мусора на утилизацию с площадки Б-9 АО «Невинномысский Азот»....  площадки 600м² для выполнения работ, издорожных плит(60 шт, поставка заказчика), с выравниванием ...</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>АО "ЦЕМРОС"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>АО "ЦЕМРОС"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>7708117908</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -911,11 +912,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>Шматов Вячеслав Вячеславович</t>
-        </is>
-      </c>
+      <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -923,30 +920,30 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>23.51</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr"/>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>06.08.2025 15:30 — 07.08.2026 12:00</t>
+          <t>26.06.2026 10:29 — 10.07.2026 12:00</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=7e7f430ea309d9e7ba9d92330037515147bd2b2f&amp;tsid=4130106003</t>
+          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=df656b471d512af3cbdfd310cfc48e3283748109&amp;tsid=4503612458</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -962,27 +959,27 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>4498936</t>
+          <t>4130106</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Продажа невостребованных ТМЦ -Плиты аэродромные, Фильтр сетчатый МИГ, Ролик лебедки Материалы с хранения. Перечень ориентировочный, может измениться в меньшую сторону за счет возможной востребованности.</t>
+          <t>Реализация ЖБИ изделий с АО "Мальцовский портландцемент"Бордюрдорожный1000х300х150мм Ясногорский завод строительных материалов Кольца  ...  КС-7-3 ЖБИ 24/7Плитаопорная ОП-1К ПС-334-08 ...Плитаперекрытия колодца 1ПП-20-2 D2200  ...</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>ООО "СИБУР"</t>
+          <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>ООО "СИБУР"</t>
+          <t>АО "ЦЕМРОС"</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>7727576505</t>
+          <t>7708117908</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -992,7 +989,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Карисалов Михаил Юрьевич</t>
+          <t>Шматов Вячеслав Вячеславович</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -1002,30 +999,30 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>70.10</t>
+          <t>23.51</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr"/>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>23.06.2026 13:41 — 14.07.2026 12:00</t>
+          <t>06.08.2025 15:30 — 07.08.2026 12:00</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Кржижановского, д 16 к 3</t>
+          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=7ca8303a65c1a30cbea65c4ff3722aa91162da88&amp;tsid=4498936003</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-zhbi-izdelii-s-ao-maltsovskii-portlandtsement/tender-4130106/#btid=2&amp;sqh=df656b471d512af3cbdfd310cfc48e3283748109&amp;tsid=4130106003</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1036,155 +1033,155 @@
       <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="2" t="inlineStr">
         <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>4498936</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Продажа невостребованных ТМЦ -Плиты аэродромные, Фильтр сетчатый МИГ, Ролик лебедки Материалы с хранения. Перечень ориентировочный, может измениться в меньшую сторону за счет возможной востребованности.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СИБУР"</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СИБУР"</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>7727576505</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Карисалов Михаил Юрьевич</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>70.10</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr"/>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>23.06.2026 13:41 — 14.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Кржижановского, д 16 к 3</t>
+        </is>
+      </c>
+      <c r="Q8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/prodazha-nevostrebovannykh-tmts-plity-aerodromnye-filtr-setchatyi/tender-4498936/#btid=2&amp;sqh=d42e225725fa7c567a2e4c416bd52a2de1f89d8a&amp;tsid=4498936003</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09 06:24</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
           <t>Работы</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>4497016</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>BOX_00514 Выполнение работ по строительству общежития №4 на 80 койко-мест временного вахтового поселка на месторождении «Бараньевское»
 Выполнение работ по строительству общежития №4 на 80 койко-мест временного вахтового поселка АО «Камчатское золото», на месторождении «Бараньевское»ЛОТ №1: Монтаж фундамента (висячиезабивные сваииз стальных труб 219×5 мм)  ...</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>ООО «Фокси-Бокс»</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>ООО "ФОКСИ-БОКС"</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>7805780074</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>Василенко Иван Михайлович</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>46.73</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr"/>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>22.06.2026 16:20 — 09.07.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P8" s="2" t="inlineStr">
-        <is>
-          <t>196006, Г.САНКТ-ПЕТЕРБУРГ, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОСКОВСКАЯ ЗАСТАВА, УЛ ЗАСТАВСКАЯ, Д. 7, ЛИТЕРА А, ПОМЕЩ. 1-Н, ПОМЕЩ. № 157</t>
-        </is>
-      </c>
-      <c r="Q8" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=74802e65efe7c97e35b3d92d42e9245e0dd2fb1e&amp;tsid=4497016004</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 21:54</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>4518573</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>2228 ОпрыЛЭПпо заявке МГ-019766</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>АО "ИК "АРЛАН"</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>АО "ИК "АРЛАН"</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>7722220390</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>Барилов Евгений Александрович</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>82.99</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr"/>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>08.07.2026 18:39 — 14.07.2026 12:00</t>
+          <t>22.06.2026 16:20 — 09.07.2026 12:00</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Романов пер, д 4</t>
+          <t>196006, Г.САНКТ-ПЕТЕРБУРГ, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОСКОВСКАЯ ЗАСТАВА, УЛ ЗАСТАВСКАЯ, Д. 7, ЛИТЕРА А, ПОМЕЩ. 1-Н, ПОМЕЩ. № 157</t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/2228-opry-lep-po-zaiavke-mg-019766/tender-4518573/#btid=2&amp;sqh=126d75d692f2ff393304d4fd68020dcaed2781ca&amp;tsid=4518573004</t>
+          <t>https://www.b2b-center.ru/market/box-00514-vypolnenie-rabot-po-stroitelstvu-obshchezhitiia-4-na-80/tender-4497016/#btid=2&amp;sqh=a4ba2a86521186dc9f61cf0473bf34152a47bd90&amp;tsid=4497016004</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1195,32 +1192,32 @@
       <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Работы</t>
+          <t>Прочее</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>4512292</t>
+          <t>4518573</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>ТЕХНИЧЕСКОЕ ЗАДАНИЕ на строительствоЛЭП-6кВдля электроснабжения электрогидравлического экскаватора Liebherr 9200Е Работы по строительствуЛЭП-6кВдля электроснабжения электрогидравлического экскаватора Liebherr 9200Е.</t>
+          <t>2228 ОпрыЛЭПпо заявке МГ-019766</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>ООО "СЕРВИС ПЛЮС"</t>
+          <t>АО "ИК "АРЛАН"</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>ООО "СЕРВИС ПЛЮС"</t>
+          <t>АО "ИК "АРЛАН"</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>7704643931</t>
+          <t>7722220390</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1230,7 +1227,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Иванов Владимир Ильич</t>
+          <t>Барилов Евгений Александрович</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1240,30 +1237,30 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>68.32</t>
+          <t>82.99</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr"/>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 12:19 — 14.07.2026 12:00</t>
+          <t>08.07.2026 18:39 — 14.07.2026 12:00</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Пречистенка, д 40/2 стр 4, помещ I, ком 2А</t>
+          <t>г Москва, Романов пер, д 4</t>
         </is>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=126d75d692f2ff393304d4fd68020dcaed2781ca&amp;tsid=4512292004</t>
+          <t>https://www.b2b-center.ru/market/2228-opry-lep-po-zaiavke-mg-019766/tender-4518573/#btid=2&amp;sqh=a10b7e7f46ffd6b21e4533147ea487f8de128fa3&amp;tsid=4518573004</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1274,32 +1271,32 @@
       <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Работы</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>4517766</t>
+          <t>4512292</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Заявка № ДОР-17519 ( /ЖБИ изделия/)Плиты перекрытия ПК-15КольцоК-7-1КольцоК-7-3КольцоК-7-5 ...  крышка ДКЛКольцоВГ-15КольцоК-15-10КольцоК-15-8КольцоК-15 ... -7КольцоК-15-6Кольцо...  К-15-5 Плита днища ДДК-8КолодецВД ...</t>
+          <t>ТЕХНИЧЕСКОЕ ЗАДАНИЕ на строительствоЛЭП-6кВдля электроснабжения электрогидравлического экскаватора Liebherr 9200Е Работы по строительствуЛЭП-6кВдля электроснабжения электрогидравлического экскаватора Liebherr 9200Е.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "СЕРВИС ПЛЮС"</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "СЕРВИС ПЛЮС"</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>7724498866</t>
+          <t>7704643931</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -1309,7 +1306,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Городний Анатолий Валерьевич</t>
+          <t>Иванов Владимир Ильич</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1319,30 +1316,30 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>46.73</t>
+          <t>68.32</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr"/>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>08.07.2026 12:34 — 09.07.2026 16:00</t>
+          <t>03.07.2026 12:19 — 14.07.2026 12:00</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+          <t>г Москва, ул Пречистенка, д 40/2 стр 4, помещ I, ком 2А</t>
         </is>
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zaiavka-dor-17519-zhbi-izdeliia/tender-4517766/#btid=2&amp;sqh=30b662768b6c3c0e209a92625a122c3aaba5749e&amp;tsid=4517766459</t>
+          <t>https://www.b2b-center.ru/market/tekhnicheskoe-zadanie-na-stroitelstvo-lep-6kv-dlia-elektrosnabzheniia/tender-4512292/#btid=2&amp;sqh=a10b7e7f46ffd6b21e4533147ea487f8de128fa3&amp;tsid=4512292004</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1358,10 +1355,89 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
+          <t>4517766</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Заявка № ДОР-17519 ( /ЖБИ изделия/)Плиты перекрытия ПК-15КольцоК-7-1КольцоК-7-3КольцоК-7-5 ...  крышка ДКЛКольцоВГ-15КольцоК-15-10КольцоК-15-8КольцоК-15 ... -7КольцоК-15-6Кольцо...  К-15-5 Плита днища ДДК-8КолодецВД ...</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>7724498866</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>46.73</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>08.07.2026 12:34 — 09.07.2026 16:00</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+        </is>
+      </c>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zaiavka-dor-17519-zhbi-izdeliia/tender-4517766/#btid=2&amp;sqh=2158895c26a3e5dc80e9d72b11368437bfb8a600&amp;tsid=4517766459</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09 06:24</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
           <t>4475879</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Электро/пневмо и ручной инструмент/Электроизм. инструмент/Расходные мат-лы
 РТИ, РВД, шланги, ремни
@@ -1369,137 +1445,62 @@
 Уплотнительный материал (прокладки, паронит, набивка сальниковая)...  Шина цепной пилы Oregon 752HSFL104Кольцостопор. нар. 210х5 DIN471 Andritz ... клин для бревен Sandvik 1401КольцоAbicor Binzel 757.D007 вихреобразующее ...  Kron ЦПВС-5 RAL7012 КрышкаколодцаП10 ж/б Игла клапана ... Kron ПСВС-3 RAL7012 О-кольцо11,3х2,4 NBR70 Ремень ...</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>4704012472</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>Ленинградская обл</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>Габидуллин Тимур Махмудович</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>17.12</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr"/>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>03.06.2026 15:56 — 30.07.2026 20:00</t>
-        </is>
-      </c>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
-        </is>
-      </c>
-      <c r="Q12" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=30b662768b6c3c0e209a92625a122c3aaba5749e&amp;tsid=4475879003</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 21:54</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr"/>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>4514583</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Закупка ЖБИ (плитыПДН3*1,5)</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>9725042029</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>64.20</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr"/>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>06.07.2026 15:00 — 09.07.2026 12:00</t>
+          <t>03.06.2026 15:56 — 30.07.2026 20:00</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
         </is>
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-plity-pdn-3-1-5/tender-4514583/#btid=2&amp;sqh=644cf4698c56cc8fb64e2ac70ee7d36bb390047a&amp;tsid=4514583458</t>
+          <t>https://www.b2b-center.ru/market/elektro-pnevmo-i-ruchnoi-instrument-elektroizm-instrument-raskhodnye/tender-4475879/#btid=2&amp;sqh=2158895c26a3e5dc80e9d72b11368437bfb8a600&amp;tsid=4475879003</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1515,27 +1516,27 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>4517935</t>
+          <t>4514583</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>ЖБИ(Дор № 17559)</t>
+          <t>Закупка ЖБИ (плитыПДН3*1,5)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>7724498866</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1543,11 +1544,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>Городний Анатолий Валерьевич</t>
-        </is>
-      </c>
+      <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1555,30 +1552,30 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>46.73</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr"/>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>08.07.2026 13:40 — 09.07.2026 17:00</t>
+          <t>06.07.2026 15:00 — 09.07.2026 12:00</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-dor-17559/tender-4517935/#btid=2&amp;sqh=b76aab64d3a1e08073d515c107772aa3df2cfd7a&amp;tsid=4517935459</t>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-plity-pdn-3-1-5/tender-4514583/#btid=2&amp;sqh=4f6fd525536919c5d52fb0844080b8b430dbfe97&amp;tsid=4514583458</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1594,27 +1591,27 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>4516217</t>
+          <t>4517935</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>ТМЦЖБИи песок</t>
+          <t>ЖБИ(Дор № 17559)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>7724498866</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -1622,7 +1619,11 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1630,30 +1631,30 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>46.73</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr"/>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>07.07.2026 14:31 — 10.07.2026 10:00</t>
+          <t>08.07.2026 13:40 — 09.07.2026 17:00</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
         </is>
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/tmts-zhbi-i-pesok/tender-4516217/#btid=2&amp;sqh=b76aab64d3a1e08073d515c107772aa3df2cfd7a&amp;tsid=4516217458</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-dor-17559/tender-4517935/#btid=2&amp;sqh=078c38c6b7dbfe2faeed2697847f177e03ada8c9&amp;tsid=4517935459</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1664,32 +1665,32 @@
       <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Поставка</t>
+          <t>Прочее</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>4514839</t>
+          <t>4516217</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>12-х-1 Заключение договора на поставку материалов для наружных сетей водоснабжения и водоотведения на объект строительства «Дальневосточный детский центр отдыха и оздоровления в Хабаровском крае». (9 лотов) Лот №1 ВодоснабжениеЖБИ</t>
+          <t>ТМЦЖБИи песок</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>ООО "ПРОМСТРОЙ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>ООО "ПРОМСТРОЙ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>9723169975</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1697,11 +1698,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>Султанов Владислав Назипович</t>
-        </is>
-      </c>
+      <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -1709,30 +1706,30 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>71.12.2</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr"/>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>06.07.2026 16:45 — 10.07.2026 11:00</t>
+          <t>07.07.2026 14:31 — 10.07.2026 10:00</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Волгоградский пр-кт, д 42 к 5, ком 9</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/12-kh-1-zakliuchenie-dogovora-na-postavku-materialov-dlia-naruzhnykh-setei/tender-4514839/#btid=2&amp;sqh=b76aab64d3a1e08073d515c107772aa3df2cfd7a&amp;tsid=4514839004</t>
+          <t>https://www.b2b-center.ru/app/market-next/tmts-zhbi-i-pesok/tender-4516217/#btid=2&amp;sqh=078c38c6b7dbfe2faeed2697847f177e03ada8c9&amp;tsid=4516217458</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1743,32 +1740,32 @@
       <c r="C17" s="2" t="inlineStr"/>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Поставка</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>4510662</t>
+          <t>4514839</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>(ЖБИизделия/кольца колодезные, плиты ПК15)</t>
+          <t>12-х-1 Заключение договора на поставку материалов для наружных сетей водоснабжения и водоотведения на объект строительства «Дальневосточный детский центр отдыха и оздоровления в Хабаровском крае». (9 лотов) Лот №1 ВодоснабжениеЖБИ</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "ПРОМСТРОЙ"</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+          <t>ООО "ПРОМСТРОЙ"</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>7724498866</t>
+          <t>9723169975</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -1778,7 +1775,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Городний Анатолий Валерьевич</t>
+          <t>Султанов Владислав Назипович</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -1788,30 +1785,30 @@
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>46.73</t>
+          <t>71.12.2</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr"/>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>02.07.2026 12:00 — 09.07.2026 13:00</t>
+          <t>06.07.2026 16:45 — 10.07.2026 11:00</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+          <t>г Москва, Волгоградский пр-кт, д 42 к 5, ком 9</t>
         </is>
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-izdeliia-koltsa-kolodeznye-plity-pk15/tender-4510662/#btid=2&amp;sqh=b76aab64d3a1e08073d515c107772aa3df2cfd7a&amp;tsid=4510662459</t>
+          <t>https://www.b2b-center.ru/market/12-kh-1-zakliuchenie-dogovora-na-postavku-materialov-dlia-naruzhnykh-setei/tender-4514839/#btid=2&amp;sqh=078c38c6b7dbfe2faeed2697847f177e03ada8c9&amp;tsid=4514839004</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1827,12 +1824,12 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>4510504</t>
+          <t>4510662</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>(Заявка № ДОР-17560) Лестницы/ЖБИ</t>
+          <t>(ЖБИизделия/кольца колодезные, плиты ПК15)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1873,7 +1870,7 @@
       <c r="N18" s="2" t="inlineStr"/>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>02.07.2026 10:55 — 09.07.2026 13:00</t>
+          <t>02.07.2026 12:00 — 09.07.2026 13:00</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
@@ -1883,14 +1880,14 @@
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zaiavka-dor-17560-lestnitsy-zhbi/tender-4510504/#btid=2&amp;sqh=b76aab64d3a1e08073d515c107772aa3df2cfd7a&amp;tsid=4510504459</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-izdeliia-koltsa-kolodeznye-plity-pk15/tender-4510662/#btid=2&amp;sqh=078c38c6b7dbfe2faeed2697847f177e03ada8c9&amp;tsid=4510662459</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1906,12 +1903,12 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>4510823</t>
+          <t>4510504</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>(ДОР-17553)ЖБИ/Лестницы ВЛ-2/Скоба</t>
+          <t>(Заявка № ДОР-17560) Лестницы/ЖБИ</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1952,7 +1949,7 @@
       <c r="N19" s="2" t="inlineStr"/>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>02.07.2026 12:55 — 09.07.2026 11:00</t>
+          <t>02.07.2026 10:55 — 09.07.2026 13:00</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -1962,14 +1959,14 @@
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/dor-17553-zhbi-lestnitsy-vl-2-skoba/tender-4510823/#btid=2&amp;sqh=b76aab64d3a1e08073d515c107772aa3df2cfd7a&amp;tsid=4510823459</t>
+          <t>https://www.b2b-center.ru/app/market-next/zaiavka-dor-17560-lestnitsy-zhbi/tender-4510504/#btid=2&amp;sqh=078c38c6b7dbfe2faeed2697847f177e03ada8c9&amp;tsid=4510504459</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1985,27 +1982,27 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>4508347</t>
+          <t>4510823</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>ЖБИКЕМГРЭС</t>
+          <t>(ДОР-17553)ЖБИ/Лестницы ВЛ-2/Скоба</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>9725042029</t>
+          <t>7724498866</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -2013,7 +2010,11 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -2021,30 +2022,30 @@
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>64.20</t>
+          <t>46.73</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr"/>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>01.07.2026 05:45 — 10.07.2026 00:00</t>
+          <t>02.07.2026 12:55 — 09.07.2026 11:00</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
         </is>
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=b76aab64d3a1e08073d515c107772aa3df2cfd7a&amp;tsid=4508347458</t>
+          <t>https://www.b2b-center.ru/app/market-next/dor-17553-zhbi-lestnitsy-vl-2-skoba/tender-4510823/#btid=2&amp;sqh=078c38c6b7dbfe2faeed2697847f177e03ada8c9&amp;tsid=4510823459</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -2060,27 +2061,27 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>4489772</t>
+          <t>4508347</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы 1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы</t>
+          <t>ЖБИКЕМГРЭС</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>7736583259</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -2088,11 +2089,7 @@
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>Масько Александр Вадимович</t>
-        </is>
-      </c>
+      <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -2100,30 +2097,30 @@
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>70.10</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr"/>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>16.06.2026 11:00 — 16.07.2026 12:00</t>
+          <t>01.07.2026 05:45 — 10.07.2026 00:00</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Старая Басманная, д 12 стр 1</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=b76aab64d3a1e08073d515c107772aa3df2cfd7a&amp;tsid=4489772003</t>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-kemgres/tender-4508347/#btid=2&amp;sqh=078c38c6b7dbfe2faeed2697847f177e03ada8c9&amp;tsid=4508347458</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2139,37 +2136,37 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>4474790</t>
+          <t>4489772</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
+          <t>1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы 1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>4704012472</t>
+          <t>7736583259</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Габидуллин Тимур Махмудович</t>
+          <t>Масько Александр Вадимович</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
@@ -2179,30 +2176,30 @@
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>17.12</t>
+          <t>70.10</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr"/>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>03.06.2026 09:59 — 30.07.2026 20:00</t>
+          <t>16.06.2026 11:00 — 16.07.2026 12:00</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+          <t>г Москва, ул Старая Басманная, д 12 стр 1</t>
         </is>
       </c>
       <c r="Q22" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=b76aab64d3a1e08073d515c107772aa3df2cfd7a&amp;tsid=4474790003</t>
+          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4489772/#btid=2&amp;sqh=078c38c6b7dbfe2faeed2697847f177e03ada8c9&amp;tsid=4489772003</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2218,37 +2215,37 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>4180328</t>
+          <t>4474790</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, г.Диксон). ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, ПГТ Диксон).</t>
+          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>7714456916</t>
+          <t>4704012472</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>г Москва</t>
+          <t>Ленинградская обл</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Наумов Андрей Александрович</t>
+          <t>Габидуллин Тимур Махмудович</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
@@ -2258,30 +2255,30 @@
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>70.22</t>
+          <t>17.12</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr"/>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>24.09.2025 15:32 — 23.07.2026 12:00</t>
+          <t>03.06.2026 09:59 — 30.07.2026 20:00</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Денежный пер, д 9/6</t>
+          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
         </is>
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=b76aab64d3a1e08073d515c107772aa3df2cfd7a&amp;tsid=4180328003</t>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-4474790/#btid=2&amp;sqh=078c38c6b7dbfe2faeed2697847f177e03ada8c9&amp;tsid=4474790003</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2297,37 +2294,37 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>3973258</t>
+          <t>4180328</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
+          <t>ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, г.Диксон). ПродаютсяЖБИ, плиты 1ПДН-18, ГОСТ Р 56600-2015, новые с хранения, паспорт качества имеется (находятся на п-ов Таймыр, ПГТ Диксон).</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+          <t>ООО ГРУППА "РУССКАЯ ЭНЕРГИЯ"</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>4704012472</t>
+          <t>7714456916</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл</t>
+          <t>г Москва</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Габидуллин Тимур Махмудович</t>
+          <t>Богданов Дмитрий Юрьевич</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
@@ -2337,30 +2334,30 @@
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>17.12</t>
+          <t>70.22</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr"/>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>10.03.2025 00:48 — 30.07.2026 23:00</t>
+          <t>24.09.2025 15:32 — 23.07.2026 12:00</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+          <t>г Москва, Денежный пер, д 9/6</t>
         </is>
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=b76aab64d3a1e08073d515c107772aa3df2cfd7a&amp;tsid=3973258003</t>
+          <t>https://www.b2b-center.ru/market/prodaiutsia-zhbi-plity-1pdn-18-gost-r-56600-2015-novye-s-khraneniia/tender-4180328/#btid=2&amp;sqh=078c38c6b7dbfe2faeed2697847f177e03ada8c9&amp;tsid=4180328003</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -2376,10 +2373,89 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
+          <t>3973258</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Общестроительные, изоляционные и нерудные материалы:ЖБИ/кирпич/блоки/цемент/мас</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>НПАО "СВЕТОГОРСКИЙ ЦБК"</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>4704012472</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Ленинградская обл</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Габидуллин Тимур Махмудович</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>17.12</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr"/>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>10.03.2025 00:48 — 30.07.2026 23:00</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>Ленинградская обл, Выборгский р-н, г Светогорск, ул Заводская, д 17</t>
+        </is>
+      </c>
+      <c r="Q25" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/obshchestroitelnye-izoliatsionnye-i-nerudnye-materialy/tender-3973258/#btid=2&amp;sqh=078c38c6b7dbfe2faeed2697847f177e03ada8c9&amp;tsid=3973258003</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09 06:24</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
           <t>4517919</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Кольцо опорное с днищем для нужд ООО ГРК Амикан. Требуется жесткая упаковка по ГОСТу
 КП по форме ТД Полиметалл.
@@ -2387,137 +2463,62 @@
 При подаче аналогов необходимо приложить тех. документацию.4517919 ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "ТОРГОВЫЙ ДОМ ПОЛИМЕТАЛЛ"Железобетонные изделия</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>7805368914</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург</t>
         </is>
       </c>
-      <c r="K25" s="2" t="inlineStr">
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M25" s="2" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
         <is>
           <t>46.90</t>
-        </is>
-      </c>
-      <c r="N25" s="2" t="inlineStr"/>
-      <c r="O25" s="2" t="inlineStr">
-        <is>
-          <t>08.07.2026 14:18 — 15.07.2026 10:00</t>
-        </is>
-      </c>
-      <c r="P25" s="2" t="inlineStr">
-        <is>
-          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
-        </is>
-      </c>
-      <c r="Q25" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/koltso-opornoe-s-dnishchem-dlia-nuzhd-ooo-grk-amikan-trebuetsia-zhestkaia/tender-4517919/#btid=2&amp;sqh=89742f9ad89f2d0628eb6c8f37f8a3612ae1205c&amp;tsid=4517919004</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 21:54</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>Поставка</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>4513525</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>Поставка модульных защитных сооруженийЗДАНИЕ ЗАЩИТНОЕ ДЛЯ УКРЫТИЯ 4,4*2,4*2,2МЖЕЛЕЗОБЕТОННОЕСБОРНОЕ</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>9725042029</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr"/>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="inlineStr">
-        <is>
-          <t>64.20</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr"/>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>06.07.2026 08:36 — 10.07.2026 14:00</t>
+          <t>08.07.2026 14:18 — 15.07.2026 10:00</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
       <c r="Q26" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/postavka-modulnykh-zashchitnykh-sooruzhenii/tender-4513525/#btid=2&amp;sqh=89742f9ad89f2d0628eb6c8f37f8a3612ae1205c&amp;tsid=4513525458</t>
+          <t>https://www.b2b-center.ru/market/koltso-opornoe-s-dnishchem-dlia-nuzhd-ooo-grk-amikan-trebuetsia-zhestkaia/tender-4517919/#btid=2&amp;sqh=ed7ea99079e69087fa26f57f1c8c0092034dffe1&amp;tsid=4517919004</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -2528,15 +2529,90 @@
       <c r="C27" s="2" t="inlineStr"/>
       <c r="D27" s="2" t="inlineStr">
         <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>4513525</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Поставка модульных защитных сооруженийЗДАНИЕ ЗАЩИТНОЕ ДЛЯ УКРЫТИЯ 4,4*2,4*2,2МЖЕЛЕЗОБЕТОННОЕСБОРНОЕ</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr"/>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>06.07.2026 08:36 — 10.07.2026 14:00</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/postavka-modulnykh-zashchitnykh-sooruzhenii/tender-4513525/#btid=2&amp;sqh=ed7ea99079e69087fa26f57f1c8c0092034dffe1&amp;tsid=4513525458</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09 06:24</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
           <t>Прочее</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>4513563</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Блок ФБС 12.4.6-Т-и
 Кольцо стеновое КС 20.9 ГОСТ 8020-2016
@@ -2545,137 +2621,62 @@
 Кольцо стеновое КС 20.9 ГОСТ 8020-20164513563 ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "ТОРГОВЫЙ ДОМ ПОЛИМЕТАЛЛ"Железобетонные изделия</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>7805368914</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="J28" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург</t>
         </is>
       </c>
-      <c r="K27" s="2" t="inlineStr">
+      <c r="K28" s="2" t="inlineStr">
         <is>
           <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M27" s="2" t="inlineStr">
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
         <is>
           <t>46.90</t>
-        </is>
-      </c>
-      <c r="N27" s="2" t="inlineStr"/>
-      <c r="O27" s="2" t="inlineStr">
-        <is>
-          <t>06.07.2026 08:49 — 10.07.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P27" s="2" t="inlineStr">
-        <is>
-          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
-        </is>
-      </c>
-      <c r="Q27" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/blok-fbs-12-4-6-t-i-koltso-stenovoe-ks-20-9-gost-8020-2016-na-k-pm/tender-4513563/#btid=2&amp;sqh=89742f9ad89f2d0628eb6c8f37f8a3612ae1205c&amp;tsid=4513563004</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 21:54</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>4517499</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>КРЫШКА-ПАТРУБОК 200-Т-535СБ ПК-40; ЗАГЛУШКА НА КЛАПАН СД К-5976.00.00 СБ; КРЫШКА 200-Т-525СБ ПК-40;ПЕРЕМЫЧКАД/ПРОДУВКИ ППХ 200-Т-530 СБ</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>9725042029</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr"/>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M28" s="2" t="inlineStr">
-        <is>
-          <t>64.20</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr"/>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>08.07.2026 10:53 — 10.07.2026 12:00</t>
+          <t>06.07.2026 08:49 — 10.07.2026 12:00</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
       <c r="Q28" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/kryshka-patrubok-200-t-535sb-pk-40-zaglushka-na-klapan-sd-k-5976-00-00/tender-4517499/#btid=2&amp;sqh=c47fd9ae2b92e169b8e2d5a0e25b7d57701224bc&amp;tsid=4517499458</t>
+          <t>https://www.b2b-center.ru/market/blok-fbs-12-4-6-t-i-koltso-stenovoe-ks-20-9-gost-8020-2016-na-k-pm/tender-4513563/#btid=2&amp;sqh=ed7ea99079e69087fa26f57f1c8c0092034dffe1&amp;tsid=4513563004</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -2691,39 +2692,35 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>4512541</t>
+          <t>4518697</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Запасные части CAT.... -3748 Cat Опора 348-9537 CatПеремычка140-0860 Cat Скоба 8X-3130 ...</t>
+          <t>Реле, электропривод,перемычка</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>1004001744</t>
+          <t>9725042029</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Респ Карелия</t>
-        </is>
-      </c>
-      <c r="K29" s="2" t="inlineStr">
-        <is>
-          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "СЕВЕРСТАЛЬ МЕНЕДЖМЕНТ"</t>
-        </is>
-      </c>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr"/>
       <c r="L29" s="2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
@@ -2731,30 +2728,30 @@
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>07.10.2</t>
+          <t>64.20</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr"/>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 14:07 — 10.07.2026 11:00</t>
+          <t>09.07.2026 06:57 — 15.07.2026 00:00</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>Респ Карелия, г Костомукша, шоссе Горняков, стр 284</t>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
         </is>
       </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=c47fd9ae2b92e169b8e2d5a0e25b7d57701224bc&amp;tsid=4512541003</t>
+          <t>https://www.b2b-center.ru/app/market-next/rele-elektroprivod-peremychka/tender-4518697/#btid=2&amp;sqh=3cbbb8c8331f397240a1125edf87ead8bb7f9c01&amp;tsid=4518697458</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -2770,229 +2767,225 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
+          <t>4517499</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>КРЫШКА-ПАТРУБОК 200-Т-535СБ ПК-40; ЗАГЛУШКА НА КЛАПАН СД К-5976.00.00 СБ; КРЫШКА 200-Т-525СБ ПК-40;ПЕРЕМЫЧКАД/ПРОДУВКИ ППХ 200-Т-530 СБ</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr"/>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>08.07.2026 10:53 — 10.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q30" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/kryshka-patrubok-200-t-535sb-pk-40-zaglushka-na-klapan-sd-k-5976-00-00/tender-4517499/#btid=2&amp;sqh=3cbbb8c8331f397240a1125edf87ead8bb7f9c01&amp;tsid=4517499458</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09 06:24</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr"/>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>4512541</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Запасные части CAT.... -3748 Cat Опора 348-9537 CatПеремычка140-0860 Cat Скоба 8X-3130 ...</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>АО "КАРЕЛЬСКИЙ ОКАТЫШ"</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>1004001744</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Респ Карелия</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "СЕВЕРСТАЛЬ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>07.10.2</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr"/>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>03.07.2026 14:07 — 10.07.2026 11:00</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>Респ Карелия, г Костомукша, шоссе Горняков, стр 284</t>
+        </is>
+      </c>
+      <c r="Q31" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/zapasnye-chasti-cat/tender-4512541/#btid=2&amp;sqh=3cbbb8c8331f397240a1125edf87ead8bb7f9c01&amp;tsid=4512541003</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09 06:24</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
           <t>4508230</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Сборный (Изделия электроустановочные и монтажные, Ящики, щиты, шкафы, пункты и комплектующие к ним, Приборы электроизмерительные, реле)
 МГ-019742, МГ-019713, МГ-019696, МГ-019665, МГ-019621, МГ-019620, МГ-019619, МГ-017109... -HESI-EX (5X20), Phoenix Contact 1277638ПеремычкаFBS 10-5, Phoenix Contact 3030213 ...ПеремычкаFBS 10-5 BU, Phoenix Contact  ...</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>АО "ИК "АРЛАН"</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>АО "ИК "АРЛАН"</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>7722220390</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="J32" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K30" s="2" t="inlineStr">
+      <c r="K32" s="2" t="inlineStr">
         <is>
           <t>Барилов Евгений Александрович</t>
         </is>
       </c>
-      <c r="L30" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M30" s="2" t="inlineStr">
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
         <is>
           <t>82.99</t>
-        </is>
-      </c>
-      <c r="N30" s="2" t="inlineStr"/>
-      <c r="O30" s="2" t="inlineStr">
-        <is>
-          <t>30.06.2026 17:59 — 09.07.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P30" s="2" t="inlineStr">
-        <is>
-          <t>г Москва, Романов пер, д 4</t>
-        </is>
-      </c>
-      <c r="Q30" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=c47fd9ae2b92e169b8e2d5a0e25b7d57701224bc&amp;tsid=4508230004</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 21:54</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr"/>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>4501157</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>Источники электропитания (ИБП, аккумуляторные батареи, блоки питания)...  х 1248 А·ч, включая соединительныеперемычки. Вид положительного электрода - трубчатая пластина ...  с коммутирующей арматурой, межэлементными и межряднымиперемычками, крепежами, комплектом для обслуживания АБ. Тип ...</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>АО "Мосинжпроект"</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>АО "МОСИНЖПРОЕКТ"</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>7701885820</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>Сорокин Антон Павлович</t>
-        </is>
-      </c>
-      <c r="L31" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M31" s="2" t="inlineStr">
-        <is>
-          <t>71.12.2</t>
-        </is>
-      </c>
-      <c r="N31" s="2" t="inlineStr"/>
-      <c r="O31" s="2" t="inlineStr">
-        <is>
-          <t>24.06.2026 15:40 — 22.07.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P31" s="2" t="inlineStr">
-        <is>
-          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
-        </is>
-      </c>
-      <c r="Q31" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=c47fd9ae2b92e169b8e2d5a0e25b7d57701224bc&amp;tsid=4501157003</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 21:54</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>4499964</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Автоматика и телемеханика движения поездов... , 13552-00-00В Дроссель-трансформатор (безперемычек) ДТМ-0,17-1000М ЮКЛЯ.672 ...</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>АО "Мосинжпроект"</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>АО "МОСИНЖПРОЕКТ"</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>7701885820</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr">
-        <is>
-          <t>Сорокин Антон Павлович</t>
-        </is>
-      </c>
-      <c r="L32" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M32" s="2" t="inlineStr">
-        <is>
-          <t>71.12.2</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr"/>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 08:46 — 15.07.2026 12:00</t>
+          <t>30.06.2026 17:59 — 09.07.2026 12:00</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+          <t>г Москва, Романов пер, д 4</t>
         </is>
       </c>
       <c r="Q32" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=c47fd9ae2b92e169b8e2d5a0e25b7d57701224bc&amp;tsid=4499964003</t>
+          <t>https://www.b2b-center.ru/market/sbornyi-izdeliia-elektroustanovochnye-i-montazhnye-iashchiki-shchity-shkafy/tender-4508230/#btid=2&amp;sqh=3cbbb8c8331f397240a1125edf87ead8bb7f9c01&amp;tsid=4508230004</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -3008,230 +3001,229 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
+          <t>4501157</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Источники электропитания (ИБП, аккумуляторные батареи, блоки питания)...  х 1248 А·ч, включая соединительныеперемычки. Вид положительного электрода - трубчатая пластина ...  с коммутирующей арматурой, межэлементными и межряднымиперемычками, крепежами, комплектом для обслуживания АБ. Тип ...</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>АО "Мосинжпроект"</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>7701885820</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Сорокин Антон Павлович</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>71.12.2</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr"/>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>24.06.2026 15:40 — 22.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+        </is>
+      </c>
+      <c r="Q33" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4501157/#btid=2&amp;sqh=3cbbb8c8331f397240a1125edf87ead8bb7f9c01&amp;tsid=4501157003</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09 06:24</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>4499964</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Автоматика и телемеханика движения поездов... , 13552-00-00В Дроссель-трансформатор (безперемычек) ДТМ-0,17-1000М ЮКЛЯ.672 ...</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>АО "Мосинжпроект"</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>7701885820</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Сорокин Антон Павлович</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>71.12.2</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr"/>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>24.06.2026 08:46 — 15.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+        </is>
+      </c>
+      <c r="Q34" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov/tender-4499964/#btid=2&amp;sqh=3cbbb8c8331f397240a1125edf87ead8bb7f9c01&amp;tsid=4499964003</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09 06:24</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr"/>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
           <t>4504775</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники
 Реализация неликвидных ТМЦ Буровой инструмент и запчасти для буровой техники...  Трубка пробная № 37-542-000 Соединитель-перемычка04182454 Кольцо стальное №CP48001-0305 Фильтр ...</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr">
+      <c r="I35" s="2" t="inlineStr">
         <is>
           <t>7805368914</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr">
+      <c r="J35" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург</t>
         </is>
       </c>
-      <c r="K33" s="2" t="inlineStr">
+      <c r="K35" s="2" t="inlineStr">
         <is>
           <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
-      <c r="L33" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M33" s="2" t="inlineStr">
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
         <is>
           <t>46.90</t>
-        </is>
-      </c>
-      <c r="N33" s="2" t="inlineStr"/>
-      <c r="O33" s="2" t="inlineStr">
-        <is>
-          <t>27.06.2026 01:36 — 15.07.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P33" s="2" t="inlineStr">
-        <is>
-          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
-        </is>
-      </c>
-      <c r="Q33" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=c47fd9ae2b92e169b8e2d5a0e25b7d57701224bc&amp;tsid=4504775003</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 21:54</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>4449201</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>Реализация НВИ, Оборудование теплообменное; Оборудование емкостное; Запчасти и узлы теплообменного оборудования; Запчасти и узлы емкостного оборудования;
-Продажа НВИ согласно прилагаемого перечня. 110-Емкостное и теп-ое об-е; 136-Запчасти и узлы емкостного и теплообПрокладка сперемычкамидля теплообменников ПУТГм-Б-09-01( ... . Е-21504.05.06 Прокладка сперемычкамидля теплообменников ПУТГм-Б-09-01 ...</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>ООО "СИБУР"</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>ООО "СИБУР"</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>7727576505</t>
-        </is>
-      </c>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>Карисалов Михаил Юрьевич</t>
-        </is>
-      </c>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M34" s="2" t="inlineStr">
-        <is>
-          <t>70.10</t>
-        </is>
-      </c>
-      <c r="N34" s="2" t="inlineStr"/>
-      <c r="O34" s="2" t="inlineStr">
-        <is>
-          <t>15.05.2026 06:57 — 10.07.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P34" s="2" t="inlineStr">
-        <is>
-          <t>г Москва, ул Кржижановского, д 16 к 3</t>
-        </is>
-      </c>
-      <c r="Q34" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-nvi-oborudovanie-teploobmennoe-oborudovanie-emkostnoe/tender-4449201/#btid=2&amp;sqh=c47fd9ae2b92e169b8e2d5a0e25b7d57701224bc&amp;tsid=4449201003</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 21:54</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr"/>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>4512370</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>ТО Сплит систем Лабинск Эйч энд Эн... кондиционирования Техническое обслуживание внутреннегоблокакассетного типа мультизональной  ...блокакондиционера. Мойка теплообменника внутреннегоблокакондиционера Чистка фильтров внутреннегоблокакондиционера Чистка фильтров приточнойвентиляционной...</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>АО "ЭЙЧ ЭНД ЭН"</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>АО "ЭЙЧ ЭНД ЭН"</t>
-        </is>
-      </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>7714626332</t>
-        </is>
-      </c>
-      <c r="J35" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="inlineStr">
-        <is>
-          <t>Закриев Якуб Салманович</t>
-        </is>
-      </c>
-      <c r="L35" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M35" s="2" t="inlineStr">
-        <is>
-          <t>10.51.9</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr"/>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>03.07.2026 12:40 — 14.07.2026 18:30</t>
+          <t>27.06.2026 01:36 — 15.07.2026 12:00</t>
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>г Москва, ул Вятская, д 27 стр 13</t>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
       <c r="Q35" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=81d361b3df721ca4c08106d95f9fd6e553bf88c0&amp;tsid=4512370458</t>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nelikvidnykh-tmts-burovoi-instrument-i-zapchasti-dlia-burovoi/tender-4504775/#btid=2&amp;sqh=3cbbb8c8331f397240a1125edf87ead8bb7f9c01&amp;tsid=4504775003</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -3247,27 +3239,27 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>4501181</t>
+          <t>4512370</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Вентиляторы промышленные и оборудование общеобменной вентиляции...  5Ф РешёткавентиляционнаяАМР 600х300М РешёткавентиляционнаяАМР 150х150М РешёткавентиляционнаяАМР 300х200М  ... мм.; масса 0,65 кгБлокконтроля сопротивления БСК-3.1 Канальный ...  533Па, габаритные размеры 700х467х2230 мм,блоков/моноблоков 5/1, в составе: - ...</t>
+          <t>ТО Сплит систем Лабинск Эйч энд Эн... кондиционирования Техническое обслуживание внутреннегоблокакассетного типа мультизональной  ...блокакондиционера. Мойка теплообменника внутреннегоблокакондиционера Чистка фильтров внутреннегоблокакондиционера Чистка фильтров приточнойвентиляционной...</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>АО "Мосинжпроект"</t>
+          <t>АО "ЭЙЧ ЭНД ЭН"</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>АО "МОСИНЖПРОЕКТ"</t>
+          <t>АО "ЭЙЧ ЭНД ЭН"</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>7701885820</t>
+          <t>7714626332</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -3277,7 +3269,7 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>Сорокин Антон Павлович</t>
+          <t>Закриев Якуб Салманович</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
@@ -3287,30 +3279,30 @@
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>71.12.2</t>
+          <t>10.51.9</t>
         </is>
       </c>
       <c r="N36" s="2" t="inlineStr"/>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 15:45 — 22.07.2026 12:00</t>
+          <t>03.07.2026 12:40 — 14.07.2026 18:30</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+          <t>г Москва, ул Вятская, д 27 стр 13</t>
         </is>
       </c>
       <c r="Q36" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=81d361b3df721ca4c08106d95f9fd6e553bf88c0&amp;tsid=4501181003</t>
+          <t>https://www.b2b-center.ru/app/market-next/to-split-sistem-labinsk-eich-end-en/tender-4512370/#btid=2&amp;sqh=a73f8537856e727662d95990e30903f60b3a8637&amp;tsid=4512370458</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -3326,150 +3318,150 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
+          <t>4501181</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Вентиляторы промышленные и оборудование общеобменной вентиляции...  5Ф РешёткавентиляционнаяАМР 600х300М РешёткавентиляционнаяАМР 150х150М РешёткавентиляционнаяАМР 300х200М  ... мм.; масса 0,65 кгБлокконтроля сопротивления БСК-3.1 Канальный ...  533Па, габаритные размеры 700х467х2230 мм,блоков/моноблоков 5/1, в составе: - ...</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>АО "Мосинжпроект"</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>7701885820</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Сорокин Антон Павлович</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>71.12.2</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr"/>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>24.06.2026 15:45 — 22.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P37" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+        </is>
+      </c>
+      <c r="Q37" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4501181/#btid=2&amp;sqh=a73f8537856e727662d95990e30903f60b3a8637&amp;tsid=4501181003</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09 06:24</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
           <t>4501483</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ
 Продажа запасных частей, стройматериалов, электротехнического оборудования, прочее ТМЦ...  d 50x2", внутренняя резьба RTPБлокуправления наружной установки ICEFREE TR-16 ...  Оповещатель звуковой МАЯК-12-ЗМБлокуправления наружной установки ICEFREE TS- ... проводов КС-3 007004 Велос Переходвентиляционный150х100 - D150, из тонколистовой оцинкованной ...</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr">
+      <c r="I38" s="2" t="inlineStr">
         <is>
           <t>7805368914</t>
         </is>
       </c>
-      <c r="J37" s="2" t="inlineStr">
+      <c r="J38" s="2" t="inlineStr">
         <is>
           <t>г Санкт-Петербург</t>
         </is>
       </c>
-      <c r="K37" s="2" t="inlineStr">
+      <c r="K38" s="2" t="inlineStr">
         <is>
           <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
         </is>
       </c>
-      <c r="L37" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M37" s="2" t="inlineStr">
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
         <is>
           <t>46.90</t>
-        </is>
-      </c>
-      <c r="N37" s="2" t="inlineStr"/>
-      <c r="O37" s="2" t="inlineStr">
-        <is>
-          <t>25.06.2026 05:03 — 09.07.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P37" s="2" t="inlineStr">
-        <is>
-          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
-        </is>
-      </c>
-      <c r="Q37" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=81d361b3df721ca4c08106d95f9fd6e553bf88c0&amp;tsid=4501483003</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 21:54</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>Прочее</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>4500120</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>Коммуникационное оборудование, компьютеры, комплектующие к ним, серверное оборудование и ПО...  и кабелей – 1 компл. Удаленныйблок(репитер) BSF414 , питание 220В,  ... 2х2 Комбайнер специализированный OMU Side (блок1) OMUSC1 Комбайнер специализированный OMU ... контроллер для мониторинга в FlexGain View,вентиляционнаяпанель с фильтрами, комплект кабелей, ...</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>АО "Мосинжпроект"</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>АО "МОСИНЖПРОЕКТ"</t>
-        </is>
-      </c>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t>7701885820</t>
-        </is>
-      </c>
-      <c r="J38" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K38" s="2" t="inlineStr">
-        <is>
-          <t>Сорокин Антон Павлович</t>
-        </is>
-      </c>
-      <c r="L38" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M38" s="2" t="inlineStr">
-        <is>
-          <t>71.12.2</t>
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr"/>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>24.06.2026 09:48 — 15.07.2026 12:00</t>
+          <t>25.06.2026 05:03 — 09.07.2026 12:00</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
         </is>
       </c>
       <c r="Q38" s="3" t="inlineStr">
         <is>
-          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=81d361b3df721ca4c08106d95f9fd6e553bf88c0&amp;tsid=4500120003</t>
+          <t>https://www.b2b-center.ru/market/prodazha-zapasnykh-chastei-stroimaterialov-elektrotekhnicheskogo/tender-4501483/#btid=2&amp;sqh=a73f8537856e727662d95990e30903f60b3a8637&amp;tsid=4501483003</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 21:54</t>
+          <t>2026-07-09 06:24</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -3485,148 +3477,227 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
+          <t>4500120</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Коммуникационное оборудование, компьютеры, комплектующие к ним, серверное оборудование и ПО...  и кабелей – 1 компл. Удаленныйблок(репитер) BSF414 , питание 220В,  ... 2х2 Комбайнер специализированный OMU Side (блок1) OMUSC1 Комбайнер специализированный OMU ... контроллер для мониторинга в FlexGain View,вентиляционнаяпанель с фильтрами, комплект кабелей, ...</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>АО "Мосинжпроект"</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>7701885820</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>Сорокин Антон Павлович</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>71.12.2</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr"/>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>24.06.2026 09:48 — 15.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P39" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+        </is>
+      </c>
+      <c r="Q39" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4500120/#btid=2&amp;sqh=a73f8537856e727662d95990e30903f60b3a8637&amp;tsid=4500120003</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09 06:24</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
           <t>4496006</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп
 Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп... -316 ***Петля крепежная стальная ***Платаблокауправления ZC5 CAME ***Средство чистящее " ... /распылитель для чаши Генуя ***РешеткавентиляционнаяРВ-1 225Х225 ***Петля анкерная 0 ... мл ***Папка с зажимом ***РешеткавентиляционнаяРВ-1 325Х125 ***Папка на кольцах ...</t>
         </is>
       </c>
-      <c r="G39" s="2" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>ООО "СИБУР"</t>
         </is>
       </c>
-      <c r="H39" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>ООО "СИБУР"</t>
         </is>
       </c>
-      <c r="I39" s="2" t="inlineStr">
+      <c r="I40" s="2" t="inlineStr">
         <is>
           <t>7727576505</t>
         </is>
       </c>
-      <c r="J39" s="2" t="inlineStr">
+      <c r="J40" s="2" t="inlineStr">
         <is>
           <t>г Москва</t>
         </is>
       </c>
-      <c r="K39" s="2" t="inlineStr">
+      <c r="K40" s="2" t="inlineStr">
         <is>
           <t>Карисалов Михаил Юрьевич</t>
         </is>
       </c>
-      <c r="L39" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M39" s="2" t="inlineStr">
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
         <is>
           <t>70.10</t>
-        </is>
-      </c>
-      <c r="N39" s="2" t="inlineStr"/>
-      <c r="O39" s="2" t="inlineStr">
-        <is>
-          <t>20.06.2026 16:19 — 11.07.2026 12:00</t>
-        </is>
-      </c>
-      <c r="P39" s="2" t="inlineStr">
-        <is>
-          <t>г Москва, ул Кржижановского, д 16 к 3</t>
-        </is>
-      </c>
-      <c r="Q39" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/prodazha-nelikvidnykh-tmts-tarelki-dlia-filtra-prokladki-dvigatel/tender-4496006/#btid=2&amp;sqh=81d361b3df721ca4c08106d95f9fd6e553bf88c0&amp;tsid=4496006003</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08 21:54</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>b2b-center</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>Работы</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>4129930</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>Реализация материалов для ремонта (напольные покрытия, настенные покрытия, окна, двери и т.д.) с АО "Мальцовский портландцемент"Блокдверной балконныйБлокдверной филенчатый ДГ 21х9Блококонный 1500х1000 ммБлококонный 1770х1700 мм Желоб ...  Docke Рама оконная 3000х1200 мм Решеткавентиляционнаянаружная Ручка оконная ГОСТ 5087-80 ...</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>АО "ЦЕМРОС"</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr">
-        <is>
-          <t>АО "ЦЕМРОС"</t>
-        </is>
-      </c>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>7708117908</t>
-        </is>
-      </c>
-      <c r="J40" s="2" t="inlineStr">
-        <is>
-          <t>г Москва</t>
-        </is>
-      </c>
-      <c r="K40" s="2" t="inlineStr">
-        <is>
-          <t>Шматов Вячеслав Вячеславович</t>
-        </is>
-      </c>
-      <c r="L40" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="M40" s="2" t="inlineStr">
-        <is>
-          <t>23.51</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr"/>
       <c r="O40" s="2" t="inlineStr">
         <is>
+          <t>20.06.2026 16:19 — 11.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Кржижановского, д 16 к 3</t>
+        </is>
+      </c>
+      <c r="Q40" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/prodazha-nelikvidnykh-tmts-tarelki-dlia-filtra-prokladki-dvigatel/tender-4496006/#btid=2&amp;sqh=a73f8537856e727662d95990e30903f60b3a8637&amp;tsid=4496006003</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09 06:24</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr"/>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>4129930</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Реализация материалов для ремонта (напольные покрытия, настенные покрытия, окна, двери и т.д.) с АО "Мальцовский портландцемент"Блокдверной балконныйБлокдверной филенчатый ДГ 21х9Блококонный 1500х1000 ммБлококонный 1770х1700 мм Желоб ...  Docke Рама оконная 3000х1200 мм Решеткавентиляционнаянаружная Ручка оконная ГОСТ 5087-80 ...</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЦЕМРОС"</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЦЕМРОС"</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>7708117908</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>Шматов Вячеслав Вячеславович</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>23.51</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr"/>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
           <t>06.08.2025 14:33 — 07.08.2026 12:00</t>
         </is>
       </c>
-      <c r="P40" s="2" t="inlineStr">
+      <c r="P41" s="2" t="inlineStr">
         <is>
           <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
         </is>
       </c>
-      <c r="Q40" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=81d361b3df721ca4c08106d95f9fd6e553bf88c0&amp;tsid=4129930003</t>
+      <c r="Q41" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/realizatsiia-materialov-dlia-remonta-napolnye-pokrytiia-nastennye/tender-4129930/#btid=2&amp;sqh=a73f8537856e727662d95990e30903f60b3a8637&amp;tsid=4129930003</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q40"/>
+  <autoFilter ref="A1:Q41"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -3667,6 +3738,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId40"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-09 10:58 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q41"/>
+  <dimension ref="A1:Q44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3696,8 +3696,242 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09 10:58</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>4493774</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>ЖБИ</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>7724498866</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>46.73</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr"/>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>18.06.2026 13:28 — 09.07.2026 17:00</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+        </is>
+      </c>
+      <c r="Q42" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi/tender-4493774/#btid=2&amp;sqh=4de110662536ea4efa61dc7fd0ead6d66e928ea0&amp;tsid=4493774459</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09 10:58</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr"/>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>4519105</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Железобетонные изделия</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr"/>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr"/>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>09.07.2026 10:37 — 15.07.2026 15:00</t>
+        </is>
+      </c>
+      <c r="P43" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q43" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zhelezobetonnye-izdeliia/tender-4519105/#btid=2&amp;sqh=287337b5de2fe9bff123ad9ecef89e4caf81547f&amp;tsid=4519105458</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09 10:58</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>4449201</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Реализация НВИ, Оборудование теплообменное; Оборудование емкостное; Запчасти и узлы теплообменного оборудования; Запчасти и узлы емкостного оборудования;
+Продажа НВИ согласно прилагаемого перечня. 110-Емкостное и теп-ое об-е; 136-Запчасти и узлы емкостного и теплообПрокладка сперемычкамидля теплообменников ПУТГм-Б-09-01( ... . Е-21504.05.06 Прокладка сперемычкамидля теплообменников ПУТГм-Б-09-01 ...</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СИБУР"</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СИБУР"</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>7727576505</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>Карисалов Михаил Юрьевич</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>70.10</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr"/>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>15.05.2026 06:57 — 10.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P44" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Кржижановского, д 16 к 3</t>
+        </is>
+      </c>
+      <c r="Q44" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nvi-oborudovanie-teploobmennoe-oborudovanie-emkostnoe/tender-4449201/#btid=2&amp;sqh=d70958974e87d5dafee5868f84dad6b87e725d49&amp;tsid=4449201003</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q41"/>
+  <autoFilter ref="A1:Q44"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -3739,6 +3973,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId43"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-09 11:30 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q44"/>
+  <dimension ref="A1:Q45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3930,8 +3930,87 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09 11:30</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr"/>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>4439437</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>ПРОДАМПеремычкаАКБ 469-3724094 короткая 25см - 1 ШТ ПРОДАМПеремычкаАКБ 469-3724094 короткая 25см - 1 ШТ</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>АО "ГРУППА "ИЛИМ"</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>АО "ГРУППА "ИЛИМ"</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>7840346335</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>Ломко Алексей Петрович</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>17.11.1</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr"/>
+      <c r="O45" s="2" t="inlineStr">
+        <is>
+          <t>06.05.2026 12:59 — 31.08.2026 16:00</t>
+        </is>
+      </c>
+      <c r="P45" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург, ул Марата, д 17</t>
+        </is>
+      </c>
+      <c r="Q45" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/prodam-peremychka-akb-469-3724094-korotkaia-25sm-1-sht/tender-4439437/#btid=2&amp;sqh=0e692f3403aae112de65642cd62cf456eaf7ab36&amp;tsid=4439437003</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q44"/>
+  <autoFilter ref="A1:Q45"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -3976,6 +4055,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId44"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-09 18:33 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$48</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q45"/>
+  <dimension ref="A1:Q48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4009,8 +4009,246 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09 18:33</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>4520151</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>2236 ОНК и ПЭ по заявкам МГ-019723, МГ-019274...  Ду200 для прохода через ж/бколодец Кольцоопорно-направляющее ОНК-110-325 Манжета ...  герметизирующая МГ 110/325Кольцоопорно-направляющее ОНК-110-426 Манжета ...</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>АО "ИК "АРЛАН"</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>АО "ИК "АРЛАН"</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>7722220390</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>Барилов Евгений Александрович</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>82.99</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr"/>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>09.07.2026 18:16 — 15.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P46" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Романов пер, д 4</t>
+        </is>
+      </c>
+      <c r="Q46" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/2236-onk-i-pe-po-zaiavkam-mg-019723-mg-019274/tender-4520151/#btid=2&amp;sqh=165eb0d6fb0cf7b4abad0695cde7b8da40291638&amp;tsid=4520151004</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09 18:33</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr"/>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>4519859</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Ж/б сваи Чер25А (железобетон)4519859 ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "АРТСТРОЙТЕХНОЛОГИЯ"Железобетонные изделия</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>7724498866</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M47" s="2" t="inlineStr">
+        <is>
+          <t>46.73</t>
+        </is>
+      </c>
+      <c r="N47" s="2" t="inlineStr"/>
+      <c r="O47" s="2" t="inlineStr">
+        <is>
+          <t>09.07.2026 15:23 — 13.07.2026 13:00</t>
+        </is>
+      </c>
+      <c r="P47" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+        </is>
+      </c>
+      <c r="Q47" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zh-b-svai-cher25a-zhelezobeton/tender-4519859/#btid=2&amp;sqh=097c65a167793ef3a0141f4334315d5f05fcb3b1&amp;tsid=4519859459</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09 18:33</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>4441588</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Реализация запасных частей и расходных материалов железнодорожной техники и верхнего строения пути со всех карьеров группы компаний АО "ННК"
+Реализация запасных частей и расходных материалов железнодорожной техники и верхнего строения пути со всех карьеров группы компаний АО "ННК"... ) Вал кулачковый Д50.27.079-3Перемычкапутевого ящика 1548.00.000-01 ...</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>АО "ННК"</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>АО "ННК-ОЙЛ"</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>5032049030</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>Худайнатов Эдуард Юрьевич</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>70.22</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr"/>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>07.05.2026 15:26 — 27.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P48" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул 1-я Тверская-Ямская, д 5, помещ 1012</t>
+        </is>
+      </c>
+      <c r="Q48" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/realizatsiia-zapasnykh-chastei-i-raskhodnykh-materialov-zheleznodorozhnoi/tender-4441588/#btid=2&amp;sqh=dcd2120f4ac7e8c75161ce303c945415e285054e&amp;tsid=4441588003</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q45"/>
+  <autoFilter ref="A1:Q48"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -4056,6 +4294,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId47"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-10 07:19 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q48"/>
+  <dimension ref="A1:Q49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4247,8 +4247,83 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10 07:19</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr"/>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>4520332</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>ТМЦЖБИПодножник ПЖД-4 СУЭК-Кузбасс</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr"/>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N49" s="2" t="inlineStr"/>
+      <c r="O49" s="2" t="inlineStr">
+        <is>
+          <t>10.07.2026 06:58 — 16.07.2026 11:00</t>
+        </is>
+      </c>
+      <c r="P49" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q49" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/tmts-zhbi-podnozhnik-pzhd-4-suek-kuzbass/tender-4520332/#btid=2&amp;sqh=1d86b3d7a6d902f8f947badf5f5c055a8377828f&amp;tsid=4520332458</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q48"/>
+  <autoFilter ref="A1:Q49"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -4297,6 +4372,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId48"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-10 11:37 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$174</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$176</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q174"/>
+  <dimension ref="A1:Q176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -12170,7 +12170,7 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M142" s="2" t="n"/>
+      <c r="M142" s="2" t="inlineStr"/>
       <c r="N142" s="2" t="inlineStr">
         <is>
           <t>222 500,00 ₽</t>
@@ -12247,7 +12247,7 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M143" s="2" t="n"/>
+      <c r="M143" s="2" t="inlineStr"/>
       <c r="N143" s="2" t="inlineStr">
         <is>
           <t>222 500,00 ₽</t>
@@ -12324,7 +12324,7 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M144" s="2" t="n"/>
+      <c r="M144" s="2" t="inlineStr"/>
       <c r="N144" s="2" t="inlineStr">
         <is>
           <t>222 500,00 ₽</t>
@@ -12401,7 +12401,7 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M145" s="2" t="n"/>
+      <c r="M145" s="2" t="inlineStr"/>
       <c r="N145" s="2" t="inlineStr">
         <is>
           <t>126 250,00 ₽</t>
@@ -14888,8 +14888,162 @@
         </is>
       </c>
     </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10 11:37</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="inlineStr"/>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E175" s="2" t="inlineStr">
+        <is>
+          <t>4509622</t>
+        </is>
+      </c>
+      <c r="F175" s="2" t="inlineStr">
+        <is>
+          <t>Услуги по переработке ломажелезобетонных изделийдля получения вторичного щебня</t>
+        </is>
+      </c>
+      <c r="G175" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H175" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I175" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J175" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K175" s="2" t="inlineStr"/>
+      <c r="L175" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M175" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N175" s="2" t="inlineStr"/>
+      <c r="O175" s="2" t="inlineStr">
+        <is>
+          <t>01.07.2026 16:05 — 16.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P175" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q175" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/uslugi-po-pererabotke-loma-zhelezobetonnykh-izdelii-dlia-polucheniia/tender-4509622/#btid=2&amp;sqh=3839600186317e7cd9dd4fc4e37b1326ae2dea3d&amp;tsid=4509622458</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10 11:37</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="inlineStr"/>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E176" s="2" t="inlineStr">
+        <is>
+          <t>4511065</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="inlineStr">
+        <is>
+          <t>Защитноежелезобетонноеукрытие 8.0х2.4</t>
+        </is>
+      </c>
+      <c r="G176" s="2" t="inlineStr">
+        <is>
+          <t>ООО "Группа Полипластик"</t>
+        </is>
+      </c>
+      <c r="H176" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ГРУППА ПОЛИПЛАСТИК"</t>
+        </is>
+      </c>
+      <c r="I176" s="2" t="inlineStr">
+        <is>
+          <t>5021013384</t>
+        </is>
+      </c>
+      <c r="J176" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K176" s="2" t="inlineStr">
+        <is>
+          <t>Коржов Олег Викторович</t>
+        </is>
+      </c>
+      <c r="L176" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M176" s="2" t="inlineStr">
+        <is>
+          <t>22.21.9</t>
+        </is>
+      </c>
+      <c r="N176" s="2" t="inlineStr"/>
+      <c r="O176" s="2" t="inlineStr">
+        <is>
+          <t>02.07.2026 14:23 — 16.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P176" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Очаковское шоссе, д 18 стр 3, помещ 014</t>
+        </is>
+      </c>
+      <c r="Q176" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/zashchitnoe-zhelezobetonnoe-ukrytie-8-0kh2-4/tender-4511065/#btid=2&amp;sqh=3839600186317e7cd9dd4fc4e37b1326ae2dea3d&amp;tsid=4511065004</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q174"/>
+  <autoFilter ref="A1:Q176"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -15064,6 +15218,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q172" r:id="rId171"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q173" r:id="rId172"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q174" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q175" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q176" r:id="rId175"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-13 11:54 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$161</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$168</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q161"/>
+  <dimension ref="A1:Q168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8394,7 +8394,7 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M94" s="2" t="n"/>
+      <c r="M94" s="2" t="inlineStr"/>
       <c r="N94" s="2" t="inlineStr">
         <is>
           <t>222 500,00 ₽</t>
@@ -8471,7 +8471,7 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M95" s="2" t="n"/>
+      <c r="M95" s="2" t="inlineStr"/>
       <c r="N95" s="2" t="inlineStr">
         <is>
           <t>222 500,00 ₽</t>
@@ -8548,7 +8548,7 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M96" s="2" t="n"/>
+      <c r="M96" s="2" t="inlineStr"/>
       <c r="N96" s="2" t="inlineStr">
         <is>
           <t>222 500,00 ₽</t>
@@ -8625,7 +8625,7 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="M97" s="2" t="n"/>
+      <c r="M97" s="2" t="inlineStr"/>
       <c r="N97" s="2" t="inlineStr">
         <is>
           <t>126 250,00 ₽</t>
@@ -13864,8 +13864,552 @@
         </is>
       </c>
     </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 11:54</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr"/>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E162" s="2" t="inlineStr">
+        <is>
+          <t>4503612</t>
+        </is>
+      </c>
+      <c r="F162" s="2" t="inlineStr">
+        <is>
+          <t>RUNEV-11652 на выполнение работ по сортировке, разделке и вывозу демонтированных 
+трубопроводов и металлоконструкций на склад хранения. Вывозу строительного мусора на утилизацию с площадки Б-9 АО «Невинномысский Азот»....  площадки 600м² для выполнения работ, издорожных плит(60 шт, поставка заказчика), с выравниванием ...</t>
+        </is>
+      </c>
+      <c r="G162" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H162" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I162" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J162" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K162" s="2" t="inlineStr"/>
+      <c r="L162" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M162" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N162" s="2" t="inlineStr"/>
+      <c r="O162" s="2" t="inlineStr">
+        <is>
+          <t>26.06.2026 10:29 — 16.07.2026 16:00</t>
+        </is>
+      </c>
+      <c r="P162" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q162" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/runev-11652-na-vypolnenie-rabot-po-sortirovke-razdelke-i-vyvozu/tender-4503612/#btid=2&amp;sqh=21d8274a03653123aad467ce3240de2439960421&amp;tsid=4503612458</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 11:54</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr"/>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E163" s="2" t="inlineStr">
+        <is>
+          <t>4522896</t>
+        </is>
+      </c>
+      <c r="F163" s="2" t="inlineStr">
+        <is>
+          <t>Закупка ЖБИ(плиты, блоки)(ЗнЗ 0581)
+Закупка ЖБИ(плиты, блоки)(ЗнЗ 0581)ПлитаПДН14 Ш*Д*В (2000*8000*140) Блок фундаментный ФБС 24.4.6-т Д*Ш*В (2380х400х580)</t>
+        </is>
+      </c>
+      <c r="G163" s="2" t="inlineStr">
+        <is>
+          <t>ООО "МАСТЕРМАЙН"</t>
+        </is>
+      </c>
+      <c r="H163" s="2" t="inlineStr">
+        <is>
+          <t>ООО "МАСТЕРМАЙН"</t>
+        </is>
+      </c>
+      <c r="I163" s="2" t="inlineStr">
+        <is>
+          <t>9703156495</t>
+        </is>
+      </c>
+      <c r="J163" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K163" s="2" t="inlineStr">
+        <is>
+          <t>Шулик Николай Русланович</t>
+        </is>
+      </c>
+      <c r="L163" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M163" s="2" t="inlineStr">
+        <is>
+          <t>09.90</t>
+        </is>
+      </c>
+      <c r="N163" s="2" t="inlineStr"/>
+      <c r="O163" s="2" t="inlineStr">
+        <is>
+          <t>13.07.2026 14:30 — 16.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P163" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, пер Капранова, д 3 стр 4</t>
+        </is>
+      </c>
+      <c r="Q163" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/zakupka-zhbi-plity-bloki-znz-0581/tender-4522896/#btid=2&amp;sqh=ba85439fa962bb3921acdce890afc237b30341d3&amp;tsid=4522896004</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 11:54</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr"/>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>4522244</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr">
+        <is>
+          <t>ЗакупкаЖБИ- лотки, плиты, бруски, блоки</t>
+        </is>
+      </c>
+      <c r="G164" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H164" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I164" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J164" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K164" s="2" t="inlineStr"/>
+      <c r="L164" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M164" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N164" s="2" t="inlineStr"/>
+      <c r="O164" s="2" t="inlineStr">
+        <is>
+          <t>13.07.2026 10:16 — 16.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P164" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q164" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-lotki-plity-bruski-bloki/tender-4522244/#btid=2&amp;sqh=e2c6b1daf3f654ca099d2c23cb8b465c860eccb0&amp;tsid=4522244458</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 11:54</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr"/>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E165" s="2" t="inlineStr">
+        <is>
+          <t>4522375</t>
+        </is>
+      </c>
+      <c r="F165" s="2" t="inlineStr">
+        <is>
+          <t>ЗакупкаЖБИ(кольца, ФБС)</t>
+        </is>
+      </c>
+      <c r="G165" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H165" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I165" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J165" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K165" s="2" t="inlineStr"/>
+      <c r="L165" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M165" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N165" s="2" t="inlineStr"/>
+      <c r="O165" s="2" t="inlineStr">
+        <is>
+          <t>13.07.2026 11:12 — 16.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P165" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q165" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-koltsa-fbs/tender-4522375/#btid=2&amp;sqh=e2c6b1daf3f654ca099d2c23cb8b465c860eccb0&amp;tsid=4522375458</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 11:54</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr"/>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>4517935</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr">
+        <is>
+          <t>ЖБИ(Дор № 17559)</t>
+        </is>
+      </c>
+      <c r="G166" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="H166" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="I166" s="2" t="inlineStr">
+        <is>
+          <t>7724498866</t>
+        </is>
+      </c>
+      <c r="J166" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K166" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
+      <c r="L166" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M166" s="2" t="inlineStr">
+        <is>
+          <t>46.73</t>
+        </is>
+      </c>
+      <c r="N166" s="2" t="inlineStr"/>
+      <c r="O166" s="2" t="inlineStr">
+        <is>
+          <t>08.07.2026 13:40 — 13.07.2026 17:00</t>
+        </is>
+      </c>
+      <c r="P166" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+        </is>
+      </c>
+      <c r="Q166" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi-dor-17559/tender-4517935/#btid=2&amp;sqh=e2c6b1daf3f654ca099d2c23cb8b465c860eccb0&amp;tsid=4517935459</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 11:54</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C167" s="2" t="inlineStr"/>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E167" s="2" t="inlineStr">
+        <is>
+          <t>4493774</t>
+        </is>
+      </c>
+      <c r="F167" s="2" t="inlineStr">
+        <is>
+          <t>ЖБИ</t>
+        </is>
+      </c>
+      <c r="G167" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="H167" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="I167" s="2" t="inlineStr">
+        <is>
+          <t>7724498866</t>
+        </is>
+      </c>
+      <c r="J167" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K167" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
+      <c r="L167" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M167" s="2" t="inlineStr">
+        <is>
+          <t>46.73</t>
+        </is>
+      </c>
+      <c r="N167" s="2" t="inlineStr"/>
+      <c r="O167" s="2" t="inlineStr">
+        <is>
+          <t>18.06.2026 13:28 — 13.07.2026 17:00</t>
+        </is>
+      </c>
+      <c r="P167" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+        </is>
+      </c>
+      <c r="Q167" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi/tender-4493774/#btid=2&amp;sqh=e2c6b1daf3f654ca099d2c23cb8b465c860eccb0&amp;tsid=4493774459</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 11:54</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr"/>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E168" s="2" t="inlineStr">
+        <is>
+          <t>4184850</t>
+        </is>
+      </c>
+      <c r="F168" s="2" t="inlineStr">
+        <is>
+          <t>Распродажа склада электронных компонентов: Schneider Electric, Phoenix Contact, Harting, Schroff, Finder, Ferraz Shawmut, Duplomatic, Axon, Schlemmer, BRALO, ABB, Wago, Weidmuller
+Распродажа склада электронных компонентов: Schneider Electric, Phoenix Contact, Harting, Schroff, Finder, Ferraz Shawmut, Duplomatic, Axon, Schlemmer, BRALO, ABB, Wago, Weidmuller... высокого тока - UKH 50 Проволочнаяперемычка- FBSW 2-5/250MM ...Перемычка- FBS 3-5Перемычка- FBS 10-5 ...  - D-UT 2,5/10Перемычка- FBS-PV UT Клемма с ... ,5-3 /WH Скобы Проходные клеммыПеремычкаКоробка датчика Клемма Концевая крышка Маркировочные ...</t>
+        </is>
+      </c>
+      <c r="G168" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СОЮЗИМПОРТ ИНЖИНИРИНГ"</t>
+        </is>
+      </c>
+      <c r="H168" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СОЮЗИМПОРТ ИНЖИНИРИНГ"</t>
+        </is>
+      </c>
+      <c r="I168" s="2" t="inlineStr">
+        <is>
+          <t>7743180170</t>
+        </is>
+      </c>
+      <c r="J168" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K168" s="2" t="inlineStr">
+        <is>
+          <t>Капитонов Михаил Александрович</t>
+        </is>
+      </c>
+      <c r="L168" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M168" s="2" t="inlineStr">
+        <is>
+          <t>46.62</t>
+        </is>
+      </c>
+      <c r="N168" s="2" t="inlineStr"/>
+      <c r="O168" s="2" t="inlineStr">
+        <is>
+          <t>29.09.2025 17:00 — 29.09.2027 12:00</t>
+        </is>
+      </c>
+      <c r="P168" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Михалковская, д 63Б стр 2, помещ XVI, ком 14</t>
+        </is>
+      </c>
+      <c r="Q168" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/rasprodazha-sklada-elektronnykh-komponentov-schneider-electric/tender-4184850/#btid=2&amp;sqh=af227beb640f55be02dd1ebd99ccc5d25ff48fd7&amp;tsid=4184850003</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q161"/>
+  <autoFilter ref="A1:Q168"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -14027,6 +14571,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q159" r:id="rId158"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q160" r:id="rId159"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q161" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q162" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q163" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q164" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q165" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q166" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q167" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q168" r:id="rId167"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-13 18:39 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$168</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$169</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q168"/>
+  <dimension ref="A1:Q169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14408,8 +14408,88 @@
         </is>
       </c>
     </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 18:39</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C169" s="2" t="inlineStr"/>
+      <c r="D169" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E169" s="2" t="inlineStr">
+        <is>
+          <t>4480614</t>
+        </is>
+      </c>
+      <c r="F169" s="2" t="inlineStr">
+        <is>
+          <t>Плановое и аварийное техническое обслуживание зданий и сооружений (годовое обслуживание август 2026 - август 2027) ГК Логика молока, производственная площадка в г. Ялуторовске
+Обслуживание зданий и сооружений завода в г. Ялуторовске....  стен из газобетонных блоков Устройство металлическихперемычекс устройством штраб Усиление кирпичных стен ...</t>
+        </is>
+      </c>
+      <c r="G169" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЭЙЧ ЭНД ЭН"</t>
+        </is>
+      </c>
+      <c r="H169" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЭЙЧ ЭНД ЭН"</t>
+        </is>
+      </c>
+      <c r="I169" s="2" t="inlineStr">
+        <is>
+          <t>7714626332</t>
+        </is>
+      </c>
+      <c r="J169" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K169" s="2" t="inlineStr">
+        <is>
+          <t>Закриев Якуб Салманович</t>
+        </is>
+      </c>
+      <c r="L169" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M169" s="2" t="inlineStr">
+        <is>
+          <t>10.51.9</t>
+        </is>
+      </c>
+      <c r="N169" s="2" t="inlineStr"/>
+      <c r="O169" s="2" t="inlineStr">
+        <is>
+          <t>08.06.2026 14:44 — 16.07.2026 14:00</t>
+        </is>
+      </c>
+      <c r="P169" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Вятская, д 27 стр 13</t>
+        </is>
+      </c>
+      <c r="Q169" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/planovoe-i-avariinoe-tekhnicheskoe-obsluzhivanie-zdanii-i-sooruzhenii/tender-4480614/#btid=2&amp;sqh=cfde69d3b6b8b27ab12976db6c1d5204da8619d6&amp;tsid=4480614004</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q168"/>
+  <autoFilter ref="A1:Q169"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -14578,6 +14658,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q166" r:id="rId165"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q167" r:id="rId166"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q168" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q169" r:id="rId168"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-14 07:56 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$169</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$173</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q169"/>
+  <dimension ref="A1:Q173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14488,8 +14488,333 @@
         </is>
       </c>
     </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14 07:56</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E170" s="2" t="inlineStr">
+        <is>
+          <t>32616202178</t>
+        </is>
+      </c>
+      <c r="F170" s="2" t="inlineStr">
+        <is>
+          <t>Поставкаплитаэродромных железобетонных на объекты строительства Московского метрополитена.</t>
+        </is>
+      </c>
+      <c r="G170" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "УПРАВЛЕНИЕ РАЗВИТИЯ СТРОИТЕЛЬНЫХ ТЕХНОЛОГИЙ"</t>
+        </is>
+      </c>
+      <c r="H170" s="2" t="inlineStr">
+        <is>
+          <t>АО "УРСТ"</t>
+        </is>
+      </c>
+      <c r="I170" s="2" t="inlineStr">
+        <is>
+          <t>7703800010</t>
+        </is>
+      </c>
+      <c r="J170" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K170" s="2" t="inlineStr">
+        <is>
+          <t>Смирнов Игорь Анатольевич</t>
+        </is>
+      </c>
+      <c r="L170" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M170" s="2" t="inlineStr">
+        <is>
+          <t>41.20.9</t>
+        </is>
+      </c>
+      <c r="N170" s="2" t="inlineStr">
+        <is>
+          <t>49 998 526,14 ₽</t>
+        </is>
+      </c>
+      <c r="O170" s="2" t="inlineStr">
+        <is>
+          <t>14.07.2026 | 14.07.2026 | 30.07.2026</t>
+        </is>
+      </c>
+      <c r="P170" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Климашкина, д 22 стр 2</t>
+        </is>
+      </c>
+      <c r="Q170" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/223/purchase/public/purchase/info/common-info.html?regNumber=32616202178</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14 07:56</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C171" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D171" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E171" s="2" t="inlineStr">
+        <is>
+          <t>32616202028</t>
+        </is>
+      </c>
+      <c r="F171" s="2" t="inlineStr">
+        <is>
+          <t>225455_ПоставкааэродромныхплитПАГ-14 на КПО «Островский» для нужд АО «Невский экологический оператор»</t>
+        </is>
+      </c>
+      <c r="G171" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "НЕВСКИЙ ЭКОЛОГИЧЕСКИЙ ОПЕРАТОР"</t>
+        </is>
+      </c>
+      <c r="H171" s="2" t="inlineStr">
+        <is>
+          <t>АО "НЕВСКИЙ ЭКОЛОГИЧЕСКИЙ ОПЕРАТОР"</t>
+        </is>
+      </c>
+      <c r="I171" s="2" t="inlineStr">
+        <is>
+          <t>7804678913</t>
+        </is>
+      </c>
+      <c r="J171" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="K171" s="2" t="inlineStr">
+        <is>
+          <t>Горшкова Екатерина Сергеевна</t>
+        </is>
+      </c>
+      <c r="L171" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M171" s="2" t="inlineStr">
+        <is>
+          <t>38.22.9</t>
+        </is>
+      </c>
+      <c r="N171" s="2" t="inlineStr">
+        <is>
+          <t>4 495 966,48 ₽</t>
+        </is>
+      </c>
+      <c r="O171" s="2" t="inlineStr">
+        <is>
+          <t>14.07.2026 | 14.07.2026 | 22.07.2026</t>
+        </is>
+      </c>
+      <c r="P171" s="2" t="inlineStr">
+        <is>
+          <t>195009, Г.САНКТ-ПЕТЕРБУРГ, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ФИНЛЯНДСКИЙ ОКРУГ, УЛ АРСЕНАЛЬНАЯ, Д. 1, К. 2, ЛИТЕРА А, ПОМЕЩ. 1Н-23(ЧАСТЬ)</t>
+        </is>
+      </c>
+      <c r="Q171" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/223/purchase/public/purchase/info/common-info.html?regNumber=32616202028</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14 07:56</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr"/>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E172" s="2" t="inlineStr">
+        <is>
+          <t>4523550</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="inlineStr">
+        <is>
+          <t>Перевозка автотранспортнаяопоры ЛЭП</t>
+        </is>
+      </c>
+      <c r="G172" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H172" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I172" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J172" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K172" s="2" t="inlineStr"/>
+      <c r="L172" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M172" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N172" s="2" t="inlineStr"/>
+      <c r="O172" s="2" t="inlineStr">
+        <is>
+          <t>14.07.2026 08:18 — 20.07.2026 00:00</t>
+        </is>
+      </c>
+      <c r="P172" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q172" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/perevozka-avtotransportnaia-opory-lep/tender-4523550/#btid=2&amp;sqh=a09a6c4af435ba909329daeec03fd9101d4da898&amp;tsid=4523550458</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14 07:56</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C173" s="2" t="inlineStr"/>
+      <c r="D173" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E173" s="2" t="inlineStr">
+        <is>
+          <t>4496006</t>
+        </is>
+      </c>
+      <c r="F173" s="2" t="inlineStr">
+        <is>
+          <t>Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп
+Продажа неликвидных ТМЦ Тарелки для фильтра, прокладки, двигатель, фильтры и тп... -316 ***Петля крепежная стальная ***Платаблокауправления ZC5 CAME ***Средство чистящее " ... /распылитель для чаши Генуя ***РешеткавентиляционнаяРВ-1 225Х225 ***Петля анкерная 0 ... мл ***Папка с зажимом ***РешеткавентиляционнаяРВ-1 325Х125 ***Папка на кольцах ...</t>
+        </is>
+      </c>
+      <c r="G173" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СИБУР"</t>
+        </is>
+      </c>
+      <c r="H173" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СИБУР"</t>
+        </is>
+      </c>
+      <c r="I173" s="2" t="inlineStr">
+        <is>
+          <t>7727576505</t>
+        </is>
+      </c>
+      <c r="J173" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K173" s="2" t="inlineStr">
+        <is>
+          <t>Карисалов Михаил Юрьевич</t>
+        </is>
+      </c>
+      <c r="L173" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M173" s="2" t="inlineStr">
+        <is>
+          <t>70.10</t>
+        </is>
+      </c>
+      <c r="N173" s="2" t="inlineStr"/>
+      <c r="O173" s="2" t="inlineStr">
+        <is>
+          <t>20.06.2026 16:19 — 21.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P173" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Кржижановского, д 16 к 3</t>
+        </is>
+      </c>
+      <c r="Q173" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/prodazha-nelikvidnykh-tmts-tarelki-dlia-filtra-prokladki-dvigatel/tender-4496006/#btid=2&amp;sqh=506d0ed21264de4e33f9bb105b3632d1a2e8d2ca&amp;tsid=4496006003</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q169"/>
+  <autoFilter ref="A1:Q173"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -14659,6 +14984,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q167" r:id="rId166"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q168" r:id="rId167"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q169" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q170" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q171" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q172" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q173" r:id="rId172"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-14 17:05 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$173</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$182</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q173"/>
+  <dimension ref="A1:Q182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14813,8 +14813,733 @@
         </is>
       </c>
     </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14 17:05</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C174" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D174" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E174" s="2" t="inlineStr">
+        <is>
+          <t>32616203149</t>
+        </is>
+      </c>
+      <c r="F174" s="2" t="inlineStr">
+        <is>
+          <t>Плитыдорожныежелезобетонные</t>
+        </is>
+      </c>
+      <c r="G174" s="2" t="inlineStr">
+        <is>
+          <t>ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ АВТО-БЕРКУТ</t>
+        </is>
+      </c>
+      <c r="H174" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АВТО-БЕРКУТ-ВОЛХОВ"</t>
+        </is>
+      </c>
+      <c r="I174" s="2" t="inlineStr">
+        <is>
+          <t>4702013150</t>
+        </is>
+      </c>
+      <c r="J174" s="2" t="inlineStr">
+        <is>
+          <t>Ленинградская обл</t>
+        </is>
+      </c>
+      <c r="K174" s="2" t="inlineStr">
+        <is>
+          <t>Петрова Марина Владимировна</t>
+        </is>
+      </c>
+      <c r="L174" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M174" s="2" t="inlineStr">
+        <is>
+          <t>49.4</t>
+        </is>
+      </c>
+      <c r="N174" s="2" t="inlineStr">
+        <is>
+          <t>4 000 000,00 ₽</t>
+        </is>
+      </c>
+      <c r="O174" s="2" t="inlineStr">
+        <is>
+          <t>14.07.2026 | 14.07.2026 | 14.07.2026</t>
+        </is>
+      </c>
+      <c r="P174" s="2" t="inlineStr">
+        <is>
+          <t>Ленинградская обл, Волховский р-н, деревня Кисельня, ул Центральная, д 5А, офис 5</t>
+        </is>
+      </c>
+      <c r="Q174" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/223/purchase/public/purchase/info/common-info.html?regNumber=32616203149</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14 17:05</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E175" s="2" t="inlineStr">
+        <is>
+          <t>32616204549</t>
+        </is>
+      </c>
+      <c r="F175" s="2" t="inlineStr">
+        <is>
+          <t>ЛОТ 581-СЗК ПоставкаплитПАГ-14 ГОСТ 25912-2015</t>
+        </is>
+      </c>
+      <c r="G175" s="2" t="inlineStr">
+        <is>
+          <t>ФЕДЕРАЛЬНОЕ ГОСУДАРСТВЕННОЕ УНИТАРНОЕ ПРЕДПРИЯТИЕ "ГЛАВНОЕ УПРАВЛЕНИЕ СПЕЦИАЛЬНОГО СТРОИТЕЛЬСТВА"</t>
+        </is>
+      </c>
+      <c r="H175" s="2" t="inlineStr">
+        <is>
+          <t>ФГУП "ГУСС"</t>
+        </is>
+      </c>
+      <c r="I175" s="2" t="inlineStr">
+        <is>
+          <t>2315078029</t>
+        </is>
+      </c>
+      <c r="J175" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K175" s="2" t="inlineStr">
+        <is>
+          <t>Волков Николай Алексеевич</t>
+        </is>
+      </c>
+      <c r="L175" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M175" s="2" t="inlineStr">
+        <is>
+          <t>41.20.9</t>
+        </is>
+      </c>
+      <c r="N175" s="2" t="inlineStr">
+        <is>
+          <t>10 939 200,00 ₽</t>
+        </is>
+      </c>
+      <c r="O175" s="2" t="inlineStr">
+        <is>
+          <t>14.07.2026 | 14.07.2026 | 20.07.2026</t>
+        </is>
+      </c>
+      <c r="P175" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, пер Померанцев, д 8 стр 1</t>
+        </is>
+      </c>
+      <c r="Q175" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/223/purchase/public/purchase/info/common-info.html?regNumber=32616204549</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14 17:05</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E176" s="2" t="inlineStr">
+        <is>
+          <t>32616204386</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="inlineStr">
+        <is>
+          <t>Железобетонныеизделия</t>
+        </is>
+      </c>
+      <c r="G176" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ДОРОЖНАЯ СЛУЖБА"</t>
+        </is>
+      </c>
+      <c r="H176" s="2" t="inlineStr">
+        <is>
+          <t>АО "ДСИО"</t>
+        </is>
+      </c>
+      <c r="I176" s="2" t="inlineStr">
+        <is>
+          <t>3808166080</t>
+        </is>
+      </c>
+      <c r="J176" s="2" t="inlineStr">
+        <is>
+          <t>Иркутская обл</t>
+        </is>
+      </c>
+      <c r="K176" s="2" t="inlineStr">
+        <is>
+          <t>Аксаментов Владимир Сергеевич</t>
+        </is>
+      </c>
+      <c r="L176" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M176" s="2" t="inlineStr">
+        <is>
+          <t>52.21.22</t>
+        </is>
+      </c>
+      <c r="N176" s="2" t="inlineStr">
+        <is>
+          <t>135 000,00 ₽</t>
+        </is>
+      </c>
+      <c r="O176" s="2" t="inlineStr">
+        <is>
+          <t>14.07.2026 | 14.07.2026</t>
+        </is>
+      </c>
+      <c r="P176" s="2" t="inlineStr">
+        <is>
+          <t>г Иркутск, ул Декабрьских Событий, д 88</t>
+        </is>
+      </c>
+      <c r="Q176" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/223/purchase/public/purchase/info/common-info.html?regNumber=32616204386</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14 17:05</t>
+        </is>
+      </c>
+      <c r="B177" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C177" s="2" t="inlineStr"/>
+      <c r="D177" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E177" s="2" t="inlineStr">
+        <is>
+          <t>4524027</t>
+        </is>
+      </c>
+      <c r="F177" s="2" t="inlineStr">
+        <is>
+          <t>Дорожные плиты.</t>
+        </is>
+      </c>
+      <c r="G177" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ГК ФСК"</t>
+        </is>
+      </c>
+      <c r="H177" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ГК ФСК"</t>
+        </is>
+      </c>
+      <c r="I177" s="2" t="inlineStr">
+        <is>
+          <t>7708332091</t>
+        </is>
+      </c>
+      <c r="J177" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K177" s="2" t="inlineStr">
+        <is>
+          <t>Трубников Дмитрий Александрович</t>
+        </is>
+      </c>
+      <c r="L177" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M177" s="2" t="inlineStr">
+        <is>
+          <t>64.99</t>
+        </is>
+      </c>
+      <c r="N177" s="2" t="inlineStr"/>
+      <c r="O177" s="2" t="inlineStr">
+        <is>
+          <t>14.07.2026 10:54 — 15.07.2026 11:00</t>
+        </is>
+      </c>
+      <c r="P177" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Каланчевская, д 32, помещ 4/2П</t>
+        </is>
+      </c>
+      <c r="Q177" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/dorozhnye-plity/tender-4524027/#btid=2&amp;sqh=c663ffddb049e0e4e9b5fc9c1361168fd882b152&amp;tsid=4524027004</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14 17:05</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C178" s="2" t="inlineStr"/>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E178" s="2" t="inlineStr">
+        <is>
+          <t>4524100</t>
+        </is>
+      </c>
+      <c r="F178" s="2" t="inlineStr">
+        <is>
+          <t>Герметизация стыковдорожных плит(ДМЗ) для нужд ГК Агропромкомплектация (ООО "ДМЗ"). См. подробнее графу закупочные позиции и закупочную документацию</t>
+        </is>
+      </c>
+      <c r="G178" s="2" t="inlineStr">
+        <is>
+          <t>ООО «АГРОПРОМКОМПЛЕКТАЦИЯ»</t>
+        </is>
+      </c>
+      <c r="H178" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АГРОПРОМКОМПЛЕКТАЦИЯ"</t>
+        </is>
+      </c>
+      <c r="I178" s="2" t="inlineStr">
+        <is>
+          <t>7735004043</t>
+        </is>
+      </c>
+      <c r="J178" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K178" s="2" t="inlineStr">
+        <is>
+          <t>Новиков Сергей Анатольевич</t>
+        </is>
+      </c>
+      <c r="L178" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M178" s="2" t="inlineStr">
+        <is>
+          <t>70.22</t>
+        </is>
+      </c>
+      <c r="N178" s="2" t="inlineStr"/>
+      <c r="O178" s="2" t="inlineStr">
+        <is>
+          <t>14.07.2026 11:46 — 21.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P178" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, г Зеленоград, к 313Б</t>
+        </is>
+      </c>
+      <c r="Q178" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/germetizatsiia-stykov-dorozhnykh-plit-dmz-dlia-nuzhd-gk/tender-4524100/#btid=2&amp;sqh=c663ffddb049e0e4e9b5fc9c1361168fd882b152&amp;tsid=4524100004</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14 17:05</t>
+        </is>
+      </c>
+      <c r="B179" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="inlineStr"/>
+      <c r="D179" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E179" s="2" t="inlineStr">
+        <is>
+          <t>4524381</t>
+        </is>
+      </c>
+      <c r="F179" s="2" t="inlineStr">
+        <is>
+          <t>Участок Коксовый_ЖБИ_внепл.август...  20 Серия 3.900-1-14Плитажелезобетоннаядорожнаяпредварительно напряженная 1 ПДН-18 ... .60.20.1,8 ГОСТ 56600-2015Плита... -1 Серия 3.900-1-14Плитапредварительно напряженная ПАГ-14 Для аэродромных ...</t>
+        </is>
+      </c>
+      <c r="G179" s="2" t="inlineStr">
+        <is>
+          <t>ООО УК "ПМХ"</t>
+        </is>
+      </c>
+      <c r="H179" s="2" t="inlineStr">
+        <is>
+          <t>ООО УК "ПМХ"</t>
+        </is>
+      </c>
+      <c r="I179" s="2" t="inlineStr">
+        <is>
+          <t>0411075740</t>
+        </is>
+      </c>
+      <c r="J179" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K179" s="2" t="inlineStr">
+        <is>
+          <t>Зубицкий Евгений Борисович</t>
+        </is>
+      </c>
+      <c r="L179" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M179" s="2" t="inlineStr">
+        <is>
+          <t>70.10</t>
+        </is>
+      </c>
+      <c r="N179" s="2" t="inlineStr"/>
+      <c r="O179" s="2" t="inlineStr">
+        <is>
+          <t>14.07.2026 13:15 — 24.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P179" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, 2-й Верхний Михайловский проезд, д 9</t>
+        </is>
+      </c>
+      <c r="Q179" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/uchastok-koksovyi-zhbi-vnepl-avgust/tender-4524381/#btid=2&amp;sqh=c663ffddb049e0e4e9b5fc9c1361168fd882b152&amp;tsid=4524381004</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14 17:05</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr"/>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E180" s="2" t="inlineStr">
+        <is>
+          <t>4524517</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>Закупка плит ПД 30.18-17 ГОСТ33148-20144524517 ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "АИМ МЕНЕДЖМЕНТ"Железобетонные изделия</t>
+        </is>
+      </c>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H180" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I180" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J180" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K180" s="2" t="inlineStr"/>
+      <c r="L180" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M180" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N180" s="2" t="inlineStr"/>
+      <c r="O180" s="2" t="inlineStr">
+        <is>
+          <t>14.07.2026 14:15 — 16.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P180" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q180" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-plit-pd-30-18-17-gost33148-2014/tender-4524517/#btid=2&amp;sqh=9b8b2657faf73f75bfc2aa323f2cf256d32da280&amp;tsid=4524517458</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14 17:05</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr"/>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E181" s="2" t="inlineStr">
+        <is>
+          <t>4516552</t>
+        </is>
+      </c>
+      <c r="F181" s="2" t="inlineStr">
+        <is>
+          <t>поставка МВСП для нужд ООО «НХТК» в 2027 году: Лот Шпалыжелезобетонныебез скреплений (новые и б/у)</t>
+        </is>
+      </c>
+      <c r="G181" s="2" t="inlineStr">
+        <is>
+          <t>ООО "НХТК"</t>
+        </is>
+      </c>
+      <c r="H181" s="2" t="inlineStr">
+        <is>
+          <t>ООО "НХТК"</t>
+        </is>
+      </c>
+      <c r="I181" s="2" t="inlineStr">
+        <is>
+          <t>7727344230</t>
+        </is>
+      </c>
+      <c r="J181" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K181" s="2" t="inlineStr">
+        <is>
+          <t>Сапронов Александр Алексеевич</t>
+        </is>
+      </c>
+      <c r="L181" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M181" s="2" t="inlineStr">
+        <is>
+          <t>52.29</t>
+        </is>
+      </c>
+      <c r="N181" s="2" t="inlineStr"/>
+      <c r="O181" s="2" t="inlineStr">
+        <is>
+          <t>07.07.2026 16:41 — 22.07.2026 15:00</t>
+        </is>
+      </c>
+      <c r="P181" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Академика Пилюгина, д 22, помещ XL, ком 10</t>
+        </is>
+      </c>
+      <c r="Q181" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/postavka-mvsp-dlia-nuzhd-ooo-nkhtk-v-2027-godu-lot-shpaly/tender-4516552/#btid=2&amp;sqh=9b8b2657faf73f75bfc2aa323f2cf256d32da280&amp;tsid=4516552458</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14 17:05</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr"/>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E182" s="2" t="inlineStr">
+        <is>
+          <t>4516662</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="inlineStr">
+        <is>
+          <t>поставка МВСП для нужд ООО «НХТК» в 2027 году: Лот Шпалыжелезобетонныесо скреплениями (новые и б/у)</t>
+        </is>
+      </c>
+      <c r="G182" s="2" t="inlineStr">
+        <is>
+          <t>ООО "НХТК"</t>
+        </is>
+      </c>
+      <c r="H182" s="2" t="inlineStr">
+        <is>
+          <t>ООО "НХТК"</t>
+        </is>
+      </c>
+      <c r="I182" s="2" t="inlineStr">
+        <is>
+          <t>7727344230</t>
+        </is>
+      </c>
+      <c r="J182" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K182" s="2" t="inlineStr">
+        <is>
+          <t>Сапронов Александр Алексеевич</t>
+        </is>
+      </c>
+      <c r="L182" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M182" s="2" t="inlineStr">
+        <is>
+          <t>52.29</t>
+        </is>
+      </c>
+      <c r="N182" s="2" t="inlineStr"/>
+      <c r="O182" s="2" t="inlineStr">
+        <is>
+          <t>07.07.2026 17:27 — 22.07.2026 15:00</t>
+        </is>
+      </c>
+      <c r="P182" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Академика Пилюгина, д 22, помещ XL, ком 10</t>
+        </is>
+      </c>
+      <c r="Q182" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/postavka-mvsp-dlia-nuzhd-ooo-nkhtk-v-2027-godu-lot-shpaly/tender-4516662/#btid=2&amp;sqh=9b8b2657faf73f75bfc2aa323f2cf256d32da280&amp;tsid=4516662458</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q173"/>
+  <autoFilter ref="A1:Q182"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -14988,6 +15713,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q171" r:id="rId170"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q172" r:id="rId171"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q173" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q174" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q175" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q176" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q177" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q178" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q179" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q180" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q181" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q182" r:id="rId181"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-15 07:54 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$182</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$183</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q182"/>
+  <dimension ref="A1:Q183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -15538,8 +15538,93 @@
         </is>
       </c>
     </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-15 07:54</t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E183" s="2" t="inlineStr">
+        <is>
+          <t>32616205599</t>
+        </is>
+      </c>
+      <c r="F183" s="2" t="inlineStr">
+        <is>
+          <t>ПоставкаЖБИдля ПО АО "ИЭСК" ЗЭС в 2026г.</t>
+        </is>
+      </c>
+      <c r="G183" s="2" t="inlineStr">
+        <is>
+          <t>ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "ЭН+ ТОРГОВЫЙ ДОМ"</t>
+        </is>
+      </c>
+      <c r="H183" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ЭН+ ТОРГОВЫЙ ДОМ"</t>
+        </is>
+      </c>
+      <c r="I183" s="2" t="inlineStr">
+        <is>
+          <t>3808118560</t>
+        </is>
+      </c>
+      <c r="J183" s="2" t="inlineStr">
+        <is>
+          <t>Иркутская обл</t>
+        </is>
+      </c>
+      <c r="K183" s="2" t="inlineStr">
+        <is>
+          <t>Лазарева Мария Анатольевна</t>
+        </is>
+      </c>
+      <c r="L183" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M183" s="2" t="inlineStr">
+        <is>
+          <t>46.69.9</t>
+        </is>
+      </c>
+      <c r="N183" s="2" t="inlineStr">
+        <is>
+          <t>0,00 ₽</t>
+        </is>
+      </c>
+      <c r="O183" s="2" t="inlineStr">
+        <is>
+          <t>15.07.2026 | 15.07.2026 | 03.08.2026</t>
+        </is>
+      </c>
+      <c r="P183" s="2" t="inlineStr">
+        <is>
+          <t>г Иркутск, ул Рабочая, стр 22, офис 509</t>
+        </is>
+      </c>
+      <c r="Q183" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/223/purchase/public/purchase/info/common-info.html?regNumber=32616205599</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q182"/>
+  <autoFilter ref="A1:Q183"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -15722,6 +15807,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q180" r:id="rId179"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q181" r:id="rId180"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q182" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q183" r:id="rId182"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-15 14:21 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$183</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$191</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q183"/>
+  <dimension ref="A1:Q191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -15623,8 +15623,646 @@
         </is>
       </c>
     </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-15 14:21</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t>32616208754</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="inlineStr">
+        <is>
+          <t>Выполнение ПИР, СМР, ПНР полным иждивением Подрядчика по титулу: Реконструкция ЗТП-10/0,4 кВ №200 с заменой РУ-0,4 кВ, строительствоЛЭП-0,4 кВ (по сущ.опорам) от РУ-0,4 кВ ЗТП-200, ПС №605 "Бронницы", в т.ч. ПИР, МО, г.о. Бронницы, г. Бронницы, ул. Красная, д 24 Ю8-26-303-305070(291721) для нужд филиала ПАО «Россети Московский регион» - Южные электрические сети</t>
+        </is>
+      </c>
+      <c r="G184" s="2" t="inlineStr">
+        <is>
+          <t>ПУБЛИЧНОЕ АКЦИОНЕРНОЕ ОБЩЕСТВО "РОССЕТИ МОСКОВСКИЙ РЕГИОН"</t>
+        </is>
+      </c>
+      <c r="H184" s="2" t="inlineStr">
+        <is>
+          <t>ПАО "РОССЕТИ МОСКОВСКИЙ РЕГИОН", ПАО "РОССЕТИ МР"</t>
+        </is>
+      </c>
+      <c r="I184" s="2" t="inlineStr">
+        <is>
+          <t>5036065113</t>
+        </is>
+      </c>
+      <c r="J184" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K184" s="2" t="inlineStr">
+        <is>
+          <t>Пятигор Александр Михайлович</t>
+        </is>
+      </c>
+      <c r="L184" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M184" s="2" t="inlineStr">
+        <is>
+          <t>35.12.1</t>
+        </is>
+      </c>
+      <c r="N184" s="2" t="inlineStr">
+        <is>
+          <t>762 787,35 ₽</t>
+        </is>
+      </c>
+      <c r="O184" s="2" t="inlineStr">
+        <is>
+          <t>15.07.2026 | 15.07.2026 | 20.07.2026</t>
+        </is>
+      </c>
+      <c r="P184" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, 2-й Павелецкий проезд, д 3 стр 2</t>
+        </is>
+      </c>
+      <c r="Q184" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/223/purchase/public/purchase/info/common-info.html?regNumber=32616208754</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-15 14:21</t>
+        </is>
+      </c>
+      <c r="B185" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C185" s="2" t="inlineStr"/>
+      <c r="D185" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E185" s="2" t="inlineStr">
+        <is>
+          <t>4525630</t>
+        </is>
+      </c>
+      <c r="F185" s="2" t="inlineStr">
+        <is>
+          <t>Дорожные плиты.</t>
+        </is>
+      </c>
+      <c r="G185" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ГК ФСК"</t>
+        </is>
+      </c>
+      <c r="H185" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ГК ФСК"</t>
+        </is>
+      </c>
+      <c r="I185" s="2" t="inlineStr">
+        <is>
+          <t>7708332091</t>
+        </is>
+      </c>
+      <c r="J185" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K185" s="2" t="inlineStr">
+        <is>
+          <t>Трубников Дмитрий Александрович</t>
+        </is>
+      </c>
+      <c r="L185" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M185" s="2" t="inlineStr">
+        <is>
+          <t>64.99</t>
+        </is>
+      </c>
+      <c r="N185" s="2" t="inlineStr"/>
+      <c r="O185" s="2" t="inlineStr">
+        <is>
+          <t>15.07.2026 11:39 — 15.07.2026 17:15</t>
+        </is>
+      </c>
+      <c r="P185" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Каланчевская, д 32, помещ 4/2П</t>
+        </is>
+      </c>
+      <c r="Q185" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/dorozhnye-plity/tender-4525630/#btid=2&amp;sqh=0a56759641bcb40a7dfc484218183077c6795c3f&amp;tsid=4525630004</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-15 14:21</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr"/>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E186" s="2" t="inlineStr">
+        <is>
+          <t>4525310</t>
+        </is>
+      </c>
+      <c r="F186" s="2" t="inlineStr">
+        <is>
+          <t>Благоустройство территории (Заменадорожных плит, бетонные работы) РЦ Кемерово</t>
+        </is>
+      </c>
+      <c r="G186" s="2" t="inlineStr">
+        <is>
+          <t>АО "ТАНДЕР"</t>
+        </is>
+      </c>
+      <c r="H186" s="2" t="inlineStr">
+        <is>
+          <t>АО "ТАНДЕР"</t>
+        </is>
+      </c>
+      <c r="I186" s="2" t="inlineStr">
+        <is>
+          <t>2310031475</t>
+        </is>
+      </c>
+      <c r="J186" s="2" t="inlineStr">
+        <is>
+          <t>Краснодарский край</t>
+        </is>
+      </c>
+      <c r="K186" s="2" t="inlineStr">
+        <is>
+          <t>Мелешина Анна Юрьевна</t>
+        </is>
+      </c>
+      <c r="L186" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M186" s="2" t="inlineStr">
+        <is>
+          <t>47.11</t>
+        </is>
+      </c>
+      <c r="N186" s="2" t="inlineStr"/>
+      <c r="O186" s="2" t="inlineStr">
+        <is>
+          <t>15.07.2026 11:59 — 22.07.2026 14:00</t>
+        </is>
+      </c>
+      <c r="P186" s="2" t="inlineStr">
+        <is>
+          <t>г Краснодар, ул им. Леваневского, д 185</t>
+        </is>
+      </c>
+      <c r="Q186" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/blagoustroistvo-territorii-zamena-dorozhnykh-plit-betonnye-raboty-rts/tender-4525310/#btid=2&amp;sqh=0a56759641bcb40a7dfc484218183077c6795c3f&amp;tsid=4525310458</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-15 14:21</t>
+        </is>
+      </c>
+      <c r="B187" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C187" s="2" t="inlineStr"/>
+      <c r="D187" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E187" s="2" t="inlineStr">
+        <is>
+          <t>4525507</t>
+        </is>
+      </c>
+      <c r="F187" s="2" t="inlineStr">
+        <is>
+          <t>СМР. Выполнение полного комплекса строительно-монтажных и пусконаладочных работ по следующим системам объекта «Маслохозяйство». «Амурский газохимический комплекс. Титул 7416» 
+(Холодный склад материалов разового потребления)....  тротуарного Опалубка для фундаментов/ фундаментныхплитОпалубка для оснований, высотой до  ... и трамбовками Бетонирование фундаментов, ростверков,плити т.д., прочность на сжатие ...  армирования A 240 Монтаж ж/бплит дорожных(ПАГ/ПДН) Опалубка для оснований, ...</t>
+        </is>
+      </c>
+      <c r="G187" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ИСК ФАВОРИТ"</t>
+        </is>
+      </c>
+      <c r="H187" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ИСК ФАВОРИТ"</t>
+        </is>
+      </c>
+      <c r="I187" s="2" t="inlineStr">
+        <is>
+          <t>2312200175</t>
+        </is>
+      </c>
+      <c r="J187" s="2" t="inlineStr">
+        <is>
+          <t>Краснодарский край</t>
+        </is>
+      </c>
+      <c r="K187" s="2" t="inlineStr">
+        <is>
+          <t>Иваныш Василий Николаевич</t>
+        </is>
+      </c>
+      <c r="L187" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M187" s="2" t="inlineStr">
+        <is>
+          <t>41.20</t>
+        </is>
+      </c>
+      <c r="N187" s="2" t="inlineStr"/>
+      <c r="O187" s="2" t="inlineStr">
+        <is>
+          <t>15.07.2026 10:44 — 22.07.2026 17:00</t>
+        </is>
+      </c>
+      <c r="P187" s="2" t="inlineStr">
+        <is>
+          <t>г Краснодар, ул Комсомольская, д 15, офис 32</t>
+        </is>
+      </c>
+      <c r="Q187" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/smr-vypolnenie-polnogo-kompleksa-stroitelno-montazhnykh-i/tender-4525507/#btid=2&amp;sqh=0a56759641bcb40a7dfc484218183077c6795c3f&amp;tsid=4525507458</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-15 14:21</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="inlineStr"/>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
+          <t>4208488</t>
+        </is>
+      </c>
+      <c r="F188" s="2" t="inlineStr">
+        <is>
+          <t>Реализация столбов электрических и кронштейнов от Воронежского филиала АО "ЦЕМРОС"
+1.Столб электрический (мачта освещения) круглый H9м-10 шт;
+2.Столб электрический 8-гранный H9м-8 шт
+3.Кронштейн 100 мм-900 штСтолб электрический (мачта освещения) круглый H9м Столб электрический 8-гранный H9м Кронштейн 100 ммОпора ЛЭПСВ 110-5-А</t>
+        </is>
+      </c>
+      <c r="G188" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЦЕМРОС"</t>
+        </is>
+      </c>
+      <c r="H188" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЦЕМРОС"</t>
+        </is>
+      </c>
+      <c r="I188" s="2" t="inlineStr">
+        <is>
+          <t>7708117908</t>
+        </is>
+      </c>
+      <c r="J188" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K188" s="2" t="inlineStr">
+        <is>
+          <t>Шматов Вячеслав Вячеславович</t>
+        </is>
+      </c>
+      <c r="L188" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M188" s="2" t="inlineStr">
+        <is>
+          <t>23.51</t>
+        </is>
+      </c>
+      <c r="N188" s="2" t="inlineStr"/>
+      <c r="O188" s="2" t="inlineStr">
+        <is>
+          <t>20.10.2025 15:44 — 27.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P188" s="2" t="inlineStr">
+        <is>
+          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
+        </is>
+      </c>
+      <c r="Q188" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/realizatsiia-stolbov-elektricheskikh-i-kronshteinov-ot-voronezhskogo/tender-4208488/#btid=2&amp;sqh=67abfe6b1b0b314cc08bebf6c0606fb0e6793b3f&amp;tsid=4208488003</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-15 14:21</t>
+        </is>
+      </c>
+      <c r="B189" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C189" s="2" t="inlineStr"/>
+      <c r="D189" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E189" s="2" t="inlineStr">
+        <is>
+          <t>4525841</t>
+        </is>
+      </c>
+      <c r="F189" s="2" t="inlineStr">
+        <is>
+          <t>В2В для заполнения и публикации4525841 ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "АИМ МЕНЕДЖМЕНТ"Железобетонные изделия</t>
+        </is>
+      </c>
+      <c r="G189" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H189" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I189" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J189" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K189" s="2" t="inlineStr"/>
+      <c r="L189" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M189" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N189" s="2" t="inlineStr"/>
+      <c r="O189" s="2" t="inlineStr">
+        <is>
+          <t>15.07.2026 12:24 — 20.07.2026 00:00</t>
+        </is>
+      </c>
+      <c r="P189" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q189" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/v2v-dlia-zapolneniia-i-publikatsii/tender-4525841/#btid=2&amp;sqh=8ec20d9a79c431a7e4e65ecfdafc00287d064504&amp;tsid=4525841458</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-15 14:21</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr"/>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>4525859</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="inlineStr">
+        <is>
+          <t>Перемычки на Пушкина 89а, г. Пермь4525859 ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "КИНЕТИКА"Железобетонные изделия</t>
+        </is>
+      </c>
+      <c r="G190" s="2" t="inlineStr">
+        <is>
+          <t>ООО "КИНЕТИКА"</t>
+        </is>
+      </c>
+      <c r="H190" s="2" t="inlineStr">
+        <is>
+          <t>ООО "КИНЕТИКА"</t>
+        </is>
+      </c>
+      <c r="I190" s="2" t="inlineStr">
+        <is>
+          <t>9703136308</t>
+        </is>
+      </c>
+      <c r="J190" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K190" s="2" t="inlineStr">
+        <is>
+          <t>Широкова Анастасия Вячеславовна</t>
+        </is>
+      </c>
+      <c r="L190" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M190" s="2" t="inlineStr">
+        <is>
+          <t>62.01</t>
+        </is>
+      </c>
+      <c r="N190" s="2" t="inlineStr"/>
+      <c r="O190" s="2" t="inlineStr">
+        <is>
+          <t>15.07.2026 12:31 — 17.07.2026 13:00</t>
+        </is>
+      </c>
+      <c r="P190" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ЗАМОСКВОРЕЧЬЕ, УЛ. ДУБИНИНСКАЯ, Д. 11/17, СТР. 3, ПОМЕЩ. 66А/Ч</t>
+        </is>
+      </c>
+      <c r="Q190" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/peremychki-na-pushkina-89a-g-perm/tender-4525859/#btid=2&amp;sqh=8ec20d9a79c431a7e4e65ecfdafc00287d064504&amp;tsid=4525859458</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-15 14:21</t>
+        </is>
+      </c>
+      <c r="B191" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C191" s="2" t="inlineStr"/>
+      <c r="D191" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E191" s="2" t="inlineStr">
+        <is>
+          <t>4525010</t>
+        </is>
+      </c>
+      <c r="F191" s="2" t="inlineStr">
+        <is>
+          <t>Выбор поставщикавентиляционногооборудования для нужд ТС «Перекрёсток»</t>
+        </is>
+      </c>
+      <c r="G191" s="2" t="inlineStr">
+        <is>
+          <t>ПАО "КОРПОРАТИВНЫЙ ЦЕНТР ИКС 5"</t>
+        </is>
+      </c>
+      <c r="H191" s="2" t="inlineStr">
+        <is>
+          <t>ПАО "КОРПОРАТИВНЫЙ ЦЕНТР ИКС 5"</t>
+        </is>
+      </c>
+      <c r="I191" s="2" t="inlineStr">
+        <is>
+          <t>9722079341</t>
+        </is>
+      </c>
+      <c r="J191" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K191" s="2" t="inlineStr">
+        <is>
+          <t>Шехтерман Игорь Владимирович</t>
+        </is>
+      </c>
+      <c r="L191" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M191" s="2" t="inlineStr">
+        <is>
+          <t>70.10</t>
+        </is>
+      </c>
+      <c r="N191" s="2" t="inlineStr"/>
+      <c r="O191" s="2" t="inlineStr">
+        <is>
+          <t>15.07.2026 13:12 — 24.07.2026 15:00</t>
+        </is>
+      </c>
+      <c r="P191" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Средняя Калитниковская, д 28 стр 4</t>
+        </is>
+      </c>
+      <c r="Q191" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/vybor-postavshchika-ventiliatsionnogo-oborudovaniia-dlia-nuzhd-ts/tender-4525010/#btid=2&amp;sqh=129dee572ed9ad796269df19c88f3ebdaa08ea24&amp;tsid=4525010458</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q183"/>
+  <autoFilter ref="A1:Q191"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -15808,6 +16446,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q181" r:id="rId180"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q182" r:id="rId181"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q183" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q184" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q185" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q186" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q187" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q188" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q189" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q190" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q191" r:id="rId190"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-15 19:36 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$191</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$192</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q191"/>
+  <dimension ref="A1:Q192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -16261,8 +16261,87 @@
         </is>
       </c>
     </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-15 19:36</t>
+        </is>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C192" s="2" t="inlineStr"/>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E192" s="2" t="inlineStr">
+        <is>
+          <t>4526077</t>
+        </is>
+      </c>
+      <c r="F192" s="2" t="inlineStr">
+        <is>
+          <t>ЖЕЛЕЗОБЕТОННЫЕ И БЕТОННЫЕ ИЗДЕЛИЯ: изделия КПД, блоки бетонные для стен подвалов,плиты дорожные, сваи, колонны, ригели непреднапряженные ЖЕЛЕЗОБЕТОННЫЕ И БЕТОННЫЕ ИЗДЕЛИЯ</t>
+        </is>
+      </c>
+      <c r="G192" s="2" t="inlineStr">
+        <is>
+          <t>АО ХК "ГВСУ "ЦЕНТР"</t>
+        </is>
+      </c>
+      <c r="H192" s="2" t="inlineStr">
+        <is>
+          <t>АО ХК "ГВСУ "ЦЕНТР"</t>
+        </is>
+      </c>
+      <c r="I192" s="2" t="inlineStr">
+        <is>
+          <t>7709261816</t>
+        </is>
+      </c>
+      <c r="J192" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K192" s="2" t="inlineStr">
+        <is>
+          <t>Голубничий Виталий Александрович</t>
+        </is>
+      </c>
+      <c r="L192" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M192" s="2" t="inlineStr">
+        <is>
+          <t>41.20.9</t>
+        </is>
+      </c>
+      <c r="N192" s="2" t="inlineStr"/>
+      <c r="O192" s="2" t="inlineStr">
+        <is>
+          <t>15.07.2026 20:30 — 31.12.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P192" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Воронцовская, д 21А стр 1</t>
+        </is>
+      </c>
+      <c r="Q192" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/zhelezobetonnye-i-betonnye-izdeliia-izdeliia-kpd-bloki-betonnye-dlia/tender-4526077/#btid=2&amp;sqh=63cabe33c523ad964d53549282468210fa4c268b&amp;tsid=4526077003</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q191"/>
+  <autoFilter ref="A1:Q192"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -16454,6 +16533,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q189" r:id="rId188"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q190" r:id="rId189"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q191" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q192" r:id="rId191"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-16 08:45 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$192</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$195</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q192"/>
+  <dimension ref="A1:Q195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -16340,8 +16340,245 @@
         </is>
       </c>
     </row>
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16 08:45</t>
+        </is>
+      </c>
+      <c r="B193" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C193" s="2" t="inlineStr"/>
+      <c r="D193" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E193" s="2" t="inlineStr">
+        <is>
+          <t>4526398</t>
+        </is>
+      </c>
+      <c r="F193" s="2" t="inlineStr">
+        <is>
+          <t>Капитальный ремонт наружнойтеплотрассыОбъекта ГМ Краснодар 9, 40-летия Победы</t>
+        </is>
+      </c>
+      <c r="G193" s="2" t="inlineStr">
+        <is>
+          <t>АО "ТАНДЕР"</t>
+        </is>
+      </c>
+      <c r="H193" s="2" t="inlineStr">
+        <is>
+          <t>АО "ТАНДЕР"</t>
+        </is>
+      </c>
+      <c r="I193" s="2" t="inlineStr">
+        <is>
+          <t>2310031475</t>
+        </is>
+      </c>
+      <c r="J193" s="2" t="inlineStr">
+        <is>
+          <t>Краснодарский край</t>
+        </is>
+      </c>
+      <c r="K193" s="2" t="inlineStr">
+        <is>
+          <t>Мелешина Анна Юрьевна</t>
+        </is>
+      </c>
+      <c r="L193" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M193" s="2" t="inlineStr">
+        <is>
+          <t>47.11</t>
+        </is>
+      </c>
+      <c r="N193" s="2" t="inlineStr"/>
+      <c r="O193" s="2" t="inlineStr">
+        <is>
+          <t>16.07.2026 09:20 — 23.07.2026 14:00</t>
+        </is>
+      </c>
+      <c r="P193" s="2" t="inlineStr">
+        <is>
+          <t>г Краснодар, ул им. Леваневского, д 185</t>
+        </is>
+      </c>
+      <c r="Q193" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/kapitalnyi-remont-naruzhnoi-teplotrassy-ob-ekta-gm-krasnodar-9/tender-4526398/#btid=2&amp;sqh=132288a85a43b177b236513a9279258c884f99a8&amp;tsid=4526398458</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16 08:45</t>
+        </is>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C194" s="2" t="inlineStr"/>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E194" s="2" t="inlineStr">
+        <is>
+          <t>4510823</t>
+        </is>
+      </c>
+      <c r="F194" s="2" t="inlineStr">
+        <is>
+          <t>(ДОР-17553)ЖБИ/Лестницы ВЛ-2/Скоба</t>
+        </is>
+      </c>
+      <c r="G194" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="H194" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="I194" s="2" t="inlineStr">
+        <is>
+          <t>7724498866</t>
+        </is>
+      </c>
+      <c r="J194" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K194" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
+      <c r="L194" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M194" s="2" t="inlineStr">
+        <is>
+          <t>46.73</t>
+        </is>
+      </c>
+      <c r="N194" s="2" t="inlineStr"/>
+      <c r="O194" s="2" t="inlineStr">
+        <is>
+          <t>02.07.2026 12:55 — 16.07.2026 15:00</t>
+        </is>
+      </c>
+      <c r="P194" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+        </is>
+      </c>
+      <c r="Q194" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/dor-17553-zhbi-lestnitsy-vl-2-skoba/tender-4510823/#btid=2&amp;sqh=b77094e8012c199faa06bef33da50033bec8ffea&amp;tsid=4510823459</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16 08:45</t>
+        </is>
+      </c>
+      <c r="B195" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C195" s="2" t="inlineStr"/>
+      <c r="D195" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E195" s="2" t="inlineStr">
+        <is>
+          <t>4524140</t>
+        </is>
+      </c>
+      <c r="F195" s="2" t="inlineStr">
+        <is>
+          <t>Запасные части для Komatsu HD785 (ЗНЗ_0588)...  KOMATSU Втулка распорная 04254-11645 KOMATSUБлок427-T46-1420 KOMATSU Гайка 01580 ...  топливного бака 19M-04-11220 KOMATSUВентиляционноеотверстие 21T-04-31130 KOMATSU Аккумуляторная ...</t>
+        </is>
+      </c>
+      <c r="G195" s="2" t="inlineStr">
+        <is>
+          <t>ООО "МАСТЕРМАЙН"</t>
+        </is>
+      </c>
+      <c r="H195" s="2" t="inlineStr">
+        <is>
+          <t>ООО "МАСТЕРМАЙН"</t>
+        </is>
+      </c>
+      <c r="I195" s="2" t="inlineStr">
+        <is>
+          <t>9703156495</t>
+        </is>
+      </c>
+      <c r="J195" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K195" s="2" t="inlineStr">
+        <is>
+          <t>Шулик Николай Русланович</t>
+        </is>
+      </c>
+      <c r="L195" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M195" s="2" t="inlineStr">
+        <is>
+          <t>09.90</t>
+        </is>
+      </c>
+      <c r="N195" s="2" t="inlineStr"/>
+      <c r="O195" s="2" t="inlineStr">
+        <is>
+          <t>16.07.2026 08:41 — 22.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P195" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, пер Капранова, д 3 стр 4</t>
+        </is>
+      </c>
+      <c r="Q195" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zapasnye-chasti-dlia-komatsu-hd785-znz-0588/tender-4524140/#btid=2&amp;sqh=0f0f63b154c8c9dba084d8d7d9fe4755015f3a48&amp;tsid=4524140458</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q192"/>
+  <autoFilter ref="A1:Q195"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -16534,6 +16771,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q190" r:id="rId189"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q191" r:id="rId190"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q192" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q193" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q194" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q195" r:id="rId194"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-16 14:28 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$195</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$196</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q195"/>
+  <dimension ref="A1:Q196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -16577,8 +16577,93 @@
         </is>
       </c>
     </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16 14:28</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C196" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E196" s="2" t="inlineStr">
+        <is>
+          <t>0273100000126000080</t>
+        </is>
+      </c>
+      <c r="F196" s="2" t="inlineStr">
+        <is>
+          <t>Оказание услуг по очистке и дезинфекции кондиционеров и систем вентиляции</t>
+        </is>
+      </c>
+      <c r="G196" s="2" t="inlineStr">
+        <is>
+          <t>ФОНД ПЕНСИОННОГО И СОЦИАЛЬНОГО СТРАХОВАНИЯ РОССИЙСКОЙ ФЕДЕРАЦИИ</t>
+        </is>
+      </c>
+      <c r="H196" s="2" t="inlineStr">
+        <is>
+          <t>МИЦ СФР</t>
+        </is>
+      </c>
+      <c r="I196" s="2" t="inlineStr">
+        <is>
+          <t>9715226210</t>
+        </is>
+      </c>
+      <c r="J196" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K196" s="2" t="inlineStr">
+        <is>
+          <t>Бровков Дмитрий Александрович</t>
+        </is>
+      </c>
+      <c r="L196" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M196" s="2" t="inlineStr">
+        <is>
+          <t>63.11.1</t>
+        </is>
+      </c>
+      <c r="N196" s="2" t="inlineStr">
+        <is>
+          <t>1 751 137,16 ₽</t>
+        </is>
+      </c>
+      <c r="O196" s="2" t="inlineStr">
+        <is>
+          <t>16.07.2026 | 16.07.2026 | 23.07.2026</t>
+        </is>
+      </c>
+      <c r="P196" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Сущёвский Вал, д 1</t>
+        </is>
+      </c>
+      <c r="Q196" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/epz/order/notice/zk20/view/common-info.html?regNumber=0273100000126000080</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q195"/>
+  <autoFilter ref="A1:Q196"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -16774,6 +16859,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q193" r:id="rId192"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q194" r:id="rId193"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q195" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q196" r:id="rId195"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-17 03:35 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$196</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$200</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q196"/>
+  <dimension ref="A1:Q200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -16662,8 +16662,332 @@
         </is>
       </c>
     </row>
+    <row r="197">
+      <c r="A197" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17 03:35</t>
+        </is>
+      </c>
+      <c r="B197" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C197" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D197" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E197" s="2" t="inlineStr">
+        <is>
+          <t>0134100009926000062</t>
+        </is>
+      </c>
+      <c r="F197" s="2" t="inlineStr">
+        <is>
+          <t>Оказание услуг по техническому обслуживанию и ремонту автотранспортных средств в г. Иркутск</t>
+        </is>
+      </c>
+      <c r="G197" s="2" t="inlineStr">
+        <is>
+          <t>ГЛАВНОЕ УПРАВЛЕНИЕ ФЕДЕРАЛЬНОЙ СЛУЖБЫ СУДЕБНЫХ ПРИСТАВОВ ПО ИРКУТСКОЙ ОБЛАСТИ</t>
+        </is>
+      </c>
+      <c r="H197" s="2" t="inlineStr">
+        <is>
+          <t>ГУФССП РОССИИ ПО ИРКУТСКОЙ ОБЛАСТИ</t>
+        </is>
+      </c>
+      <c r="I197" s="2" t="inlineStr">
+        <is>
+          <t>3811085917</t>
+        </is>
+      </c>
+      <c r="J197" s="2" t="inlineStr">
+        <is>
+          <t>Иркутская обл</t>
+        </is>
+      </c>
+      <c r="K197" s="2" t="inlineStr">
+        <is>
+          <t>Безызвестных Татьяна Георгиевна</t>
+        </is>
+      </c>
+      <c r="L197" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M197" s="2" t="inlineStr">
+        <is>
+          <t>84.11.13</t>
+        </is>
+      </c>
+      <c r="N197" s="2" t="inlineStr">
+        <is>
+          <t>600 000,00 ₽</t>
+        </is>
+      </c>
+      <c r="O197" s="2" t="inlineStr">
+        <is>
+          <t>17.07.2026 | 17.07.2026 | 27.07.2026</t>
+        </is>
+      </c>
+      <c r="P197" s="2" t="inlineStr">
+        <is>
+          <t>г Иркутск, ул Партизанская, д 79</t>
+        </is>
+      </c>
+      <c r="Q197" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/epz/order/notice/ea20/view/common-info.html?regNumber=0134100009926000062</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17 03:35</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C198" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E198" s="2" t="inlineStr">
+        <is>
+          <t>32616213826</t>
+        </is>
+      </c>
+      <c r="F198" s="2" t="inlineStr">
+        <is>
+          <t>Поставкажелезобетонныхизделий</t>
+        </is>
+      </c>
+      <c r="G198" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "БРАТСКАЯ ЭЛЕКТРОСЕТЕВАЯ КОМПАНИЯ"</t>
+        </is>
+      </c>
+      <c r="H198" s="2" t="inlineStr">
+        <is>
+          <t>АО "БЭСК"</t>
+        </is>
+      </c>
+      <c r="I198" s="2" t="inlineStr">
+        <is>
+          <t>3804009506</t>
+        </is>
+      </c>
+      <c r="J198" s="2" t="inlineStr">
+        <is>
+          <t>Иркутская обл</t>
+        </is>
+      </c>
+      <c r="K198" s="2" t="inlineStr">
+        <is>
+          <t>Катнов Александр Анатольевич</t>
+        </is>
+      </c>
+      <c r="L198" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M198" s="2" t="inlineStr">
+        <is>
+          <t>35.12.1</t>
+        </is>
+      </c>
+      <c r="N198" s="2" t="inlineStr">
+        <is>
+          <t>2 356 950,86 ₽</t>
+        </is>
+      </c>
+      <c r="O198" s="2" t="inlineStr">
+        <is>
+          <t>17.07.2026 | 17.07.2026 | 27.07.2026</t>
+        </is>
+      </c>
+      <c r="P198" s="2" t="inlineStr">
+        <is>
+          <t>г Иркутск, ул Лермонтова, д 279/10</t>
+        </is>
+      </c>
+      <c r="Q198" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/223/purchase/public/purchase/info/common-info.html?regNumber=32616213826</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17 03:35</t>
+        </is>
+      </c>
+      <c r="B199" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C199" s="2" t="inlineStr"/>
+      <c r="D199" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E199" s="2" t="inlineStr">
+        <is>
+          <t>4528242</t>
+        </is>
+      </c>
+      <c r="F199" s="2" t="inlineStr">
+        <is>
+          <t>ЖБИизделия, ограждение для строительства Воздухоснабжение. Обдувка стрелочных переводов для ООО "КАРБО-Л" ст. "Восточная"ЖБИизделия, ограждение для строительства Воздухоснабжение. Обдувка стрелочных переводов для ООО "КАРБО-Л" ст. "Восточная"</t>
+        </is>
+      </c>
+      <c r="G199" s="2" t="inlineStr">
+        <is>
+          <t>ООО "УК "СИБАНТРАЦИТ"</t>
+        </is>
+      </c>
+      <c r="H199" s="2" t="inlineStr">
+        <is>
+          <t>ООО "УК "СИБАНТРАЦИТ"</t>
+        </is>
+      </c>
+      <c r="I199" s="2" t="inlineStr">
+        <is>
+          <t>9703160290</t>
+        </is>
+      </c>
+      <c r="J199" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K199" s="2" t="inlineStr">
+        <is>
+          <t>Мельников Сергей Владимирович</t>
+        </is>
+      </c>
+      <c r="L199" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M199" s="2" t="inlineStr">
+        <is>
+          <t>70.22</t>
+        </is>
+      </c>
+      <c r="N199" s="2" t="inlineStr"/>
+      <c r="O199" s="2" t="inlineStr">
+        <is>
+          <t>17.07.2026 04:35 — 20.07.2026 10:00</t>
+        </is>
+      </c>
+      <c r="P199" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Усачёва, д 2 стр 1, помещ 2/1</t>
+        </is>
+      </c>
+      <c r="Q199" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/zhbi-izdeliia-ograzhdenie-dlia-stroitelstva-vozdukhosnabzhenie-obduvka/tender-4528242/#btid=2&amp;sqh=ba867e67b53291934a8ae1f4483c7ec4dc1678a9&amp;tsid=4528242004</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17 03:35</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C200" s="2" t="inlineStr"/>
+      <c r="D200" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E200" s="2" t="inlineStr">
+        <is>
+          <t>4528211</t>
+        </is>
+      </c>
+      <c r="F200" s="2" t="inlineStr">
+        <is>
+          <t>осветительные и эл. установ., ДПМ... -4000-K01 4ВТ IP20 200-240ВПЕРЕМЫЧКАПГС 50*900 У2.5 ZETA ...</t>
+        </is>
+      </c>
+      <c r="G200" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H200" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I200" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J200" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K200" s="2" t="inlineStr"/>
+      <c r="L200" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M200" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N200" s="2" t="inlineStr"/>
+      <c r="O200" s="2" t="inlineStr">
+        <is>
+          <t>17.07.2026 03:03 — 21.07.2026 00:00</t>
+        </is>
+      </c>
+      <c r="P200" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q200" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/osvetitelnye-i-el-ustanov-dpm/tender-4528211/#btid=2&amp;sqh=ff05b75de13b83fbcb90133a7b34ed7458097ec8&amp;tsid=4528211458</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q196"/>
+  <autoFilter ref="A1:Q200"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -16860,6 +17184,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q194" r:id="rId193"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q195" r:id="rId194"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q196" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q197" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q198" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q199" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q200" r:id="rId199"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-17 08:31 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$200</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$202</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q200"/>
+  <dimension ref="A1:Q202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -16986,8 +16986,166 @@
         </is>
       </c>
     </row>
+    <row r="201">
+      <c r="A201" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17 08:31</t>
+        </is>
+      </c>
+      <c r="B201" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C201" s="2" t="inlineStr"/>
+      <c r="D201" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E201" s="2" t="inlineStr">
+        <is>
+          <t>4156098</t>
+        </is>
+      </c>
+      <c r="F201" s="2" t="inlineStr">
+        <is>
+          <t>Реализация. Линия погрузки угля Б/У (ЛК-60Т 2022 г.в.). Конвейер ленточный подающий ЛК-60Т, линия погрузки угля, бункер приемный, кровельные металлоконструкции. Год ввода в эксплуатацию 2022. Исправное тех.состояние. Продажа бездорожных плит. Демонтаж и самовывоз силами и за счет покупателя.</t>
+        </is>
+      </c>
+      <c r="G201" s="2" t="inlineStr">
+        <is>
+          <t>ООО "УК "СИБАНТРАЦИТ"</t>
+        </is>
+      </c>
+      <c r="H201" s="2" t="inlineStr">
+        <is>
+          <t>ООО "УК "СИБАНТРАЦИТ"</t>
+        </is>
+      </c>
+      <c r="I201" s="2" t="inlineStr">
+        <is>
+          <t>9703160290</t>
+        </is>
+      </c>
+      <c r="J201" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K201" s="2" t="inlineStr">
+        <is>
+          <t>Мельников Сергей Владимирович</t>
+        </is>
+      </c>
+      <c r="L201" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M201" s="2" t="inlineStr">
+        <is>
+          <t>70.22</t>
+        </is>
+      </c>
+      <c r="N201" s="2" t="inlineStr"/>
+      <c r="O201" s="2" t="inlineStr">
+        <is>
+          <t>02.09.2025 11:51 — 31.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P201" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Усачёва, д 2 стр 1, помещ 2/1</t>
+        </is>
+      </c>
+      <c r="Q201" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/realizatsiia-liniia-pogruzki-uglia-b-u-lk-60t-2022-g-v/tender-4156098/#btid=2&amp;sqh=4aef30b600509c4e9a1cf22f4c37ce8b432c4794&amp;tsid=4156098003</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17 08:31</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C202" s="2" t="inlineStr"/>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E202" s="2" t="inlineStr">
+        <is>
+          <t>4528607</t>
+        </is>
+      </c>
+      <c r="F202" s="2" t="inlineStr">
+        <is>
+          <t>ЖБИ изделия,плиты, ригель для строительства ООО "Сибантрацит Майнинг", Разрез Колыванский АО ЖБИ изделия,плиты, ригель для строительства ООО "Сибантрацит Майнинг", Разрез Колыванский АО (ID: 21.12.0508.02)</t>
+        </is>
+      </c>
+      <c r="G202" s="2" t="inlineStr">
+        <is>
+          <t>ООО "УК "СИБАНТРАЦИТ"</t>
+        </is>
+      </c>
+      <c r="H202" s="2" t="inlineStr">
+        <is>
+          <t>ООО "УК "СИБАНТРАЦИТ"</t>
+        </is>
+      </c>
+      <c r="I202" s="2" t="inlineStr">
+        <is>
+          <t>9703160290</t>
+        </is>
+      </c>
+      <c r="J202" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K202" s="2" t="inlineStr">
+        <is>
+          <t>Мельников Сергей Владимирович</t>
+        </is>
+      </c>
+      <c r="L202" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M202" s="2" t="inlineStr">
+        <is>
+          <t>70.22</t>
+        </is>
+      </c>
+      <c r="N202" s="2" t="inlineStr"/>
+      <c r="O202" s="2" t="inlineStr">
+        <is>
+          <t>17.07.2026 09:53 — 21.07.2026 10:00</t>
+        </is>
+      </c>
+      <c r="P202" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Усачёва, д 2 стр 1, помещ 2/1</t>
+        </is>
+      </c>
+      <c r="Q202" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/zhbi-izdeliia-plity-rigel-dlia-stroitelstva-ooo-sibantratsit/tender-4528607/#btid=2&amp;sqh=1fac29ec22cc18056bf69981278eaec76ed27b48&amp;tsid=4528607004</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q200"/>
+  <autoFilter ref="A1:Q202"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -17188,6 +17346,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q198" r:id="rId197"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q199" r:id="rId198"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q200" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q201" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q202" r:id="rId201"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-17 14:04 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$202</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$203</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q202"/>
+  <dimension ref="A1:Q203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -17144,8 +17144,88 @@
         </is>
       </c>
     </row>
+    <row r="203">
+      <c r="A203" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17 14:04</t>
+        </is>
+      </c>
+      <c r="B203" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C203" s="2" t="inlineStr"/>
+      <c r="D203" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E203" s="2" t="inlineStr">
+        <is>
+          <t>4528233</t>
+        </is>
+      </c>
+      <c r="F203" s="2" t="inlineStr">
+        <is>
+          <t>ТМЦ трехлучевые фундаменты
+ТМЦ трехлучевые фундаменты4528233 Общество с ограниченной ответственностью "Управляющая компания "Колмар"Железобетонные изделия</t>
+        </is>
+      </c>
+      <c r="G203" s="2" t="inlineStr">
+        <is>
+          <t>ООО "УК "Колмар"</t>
+        </is>
+      </c>
+      <c r="H203" s="2" t="inlineStr">
+        <is>
+          <t>ООО "УК "КОЛМАР"</t>
+        </is>
+      </c>
+      <c r="I203" s="2" t="inlineStr">
+        <is>
+          <t>7701924275</t>
+        </is>
+      </c>
+      <c r="J203" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K203" s="2" t="inlineStr">
+        <is>
+          <t>Цивилев Валерий Евгеньевич</t>
+        </is>
+      </c>
+      <c r="L203" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M203" s="2" t="inlineStr">
+        <is>
+          <t>69.20.2</t>
+        </is>
+      </c>
+      <c r="N203" s="2" t="inlineStr"/>
+      <c r="O203" s="2" t="inlineStr">
+        <is>
+          <t>17.07.2026 04:33 — 21.07.2026 21:00</t>
+        </is>
+      </c>
+      <c r="P203" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, 1-й Красногвардейский проезд, д 21 стр 1, помещ I, ком 26</t>
+        </is>
+      </c>
+      <c r="Q203" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/tmts-trekhluchevye-fundamenty/tender-4528233/#btid=2&amp;sqh=65dbf63b79619a660bbda2040d343752d4033e23&amp;tsid=4528233004</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q202"/>
+  <autoFilter ref="A1:Q203"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -17348,6 +17428,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q200" r:id="rId199"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q201" r:id="rId200"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q202" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q203" r:id="rId202"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-20 09:38 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$203</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$205</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q203"/>
+  <dimension ref="A1:Q205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -17224,8 +17224,166 @@
         </is>
       </c>
     </row>
+    <row r="204">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20 09:38</t>
+        </is>
+      </c>
+      <c r="B204" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C204" s="2" t="inlineStr"/>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E204" s="2" t="inlineStr">
+        <is>
+          <t>4530331</t>
+        </is>
+      </c>
+      <c r="F204" s="2" t="inlineStr">
+        <is>
+          <t>1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы 1. Запасные части и комплектующие для портовых погрузотранспортных механизмов (новые с хранения) 2. Смонтированные Сплит-системы, водонагреватели, формы для изготовления массивовЖБИ(б/у) 3. Павильоны из профильной трубы</t>
+        </is>
+      </c>
+      <c r="G204" s="2" t="inlineStr">
+        <is>
+          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
+        </is>
+      </c>
+      <c r="H204" s="2" t="inlineStr">
+        <is>
+          <t>ООО "УПРАВЛЕНИЕ ТРАНСПОРТНЫМИ АКТИВАМИ"</t>
+        </is>
+      </c>
+      <c r="I204" s="2" t="inlineStr">
+        <is>
+          <t>7736583259</t>
+        </is>
+      </c>
+      <c r="J204" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K204" s="2" t="inlineStr">
+        <is>
+          <t>Масько Александр Вадимович</t>
+        </is>
+      </c>
+      <c r="L204" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M204" s="2" t="inlineStr">
+        <is>
+          <t>70.10</t>
+        </is>
+      </c>
+      <c r="N204" s="2" t="inlineStr"/>
+      <c r="O204" s="2" t="inlineStr">
+        <is>
+          <t>20.07.2026 11:05 — 20.08.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P204" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Старая Басманная, д 12 стр 1</t>
+        </is>
+      </c>
+      <c r="Q204" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/1-zapasnye-chasti-i-komplektuiushchie-dlia-portovykh-pogruzotransportnykh/tender-4530331/#btid=2&amp;sqh=198aea343f6f5ab2a1adc3ec03d1b93fd036ce1e&amp;tsid=4530331003</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20 09:38</t>
+        </is>
+      </c>
+      <c r="B205" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C205" s="2" t="inlineStr"/>
+      <c r="D205" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E205" s="2" t="inlineStr">
+        <is>
+          <t>4529901</t>
+        </is>
+      </c>
+      <c r="F205" s="2" t="inlineStr">
+        <is>
+          <t>ЗакупкаЖБИдля объекта г. Краснокамск, "Зал бокса". Закупка проходит в 1 круг тендерной процедуры. Предусмотрена переторжка с продлением тендера на 15 минут. По результатам данной процедуры будет определен победитель.</t>
+        </is>
+      </c>
+      <c r="G205" s="2" t="inlineStr">
+        <is>
+          <t>ООО "КИНЕТИКА"</t>
+        </is>
+      </c>
+      <c r="H205" s="2" t="inlineStr">
+        <is>
+          <t>ООО "КИНЕТИКА"</t>
+        </is>
+      </c>
+      <c r="I205" s="2" t="inlineStr">
+        <is>
+          <t>9703136308</t>
+        </is>
+      </c>
+      <c r="J205" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K205" s="2" t="inlineStr">
+        <is>
+          <t>Широкова Анастасия Вячеславовна</t>
+        </is>
+      </c>
+      <c r="L205" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M205" s="2" t="inlineStr">
+        <is>
+          <t>62.01</t>
+        </is>
+      </c>
+      <c r="N205" s="2" t="inlineStr"/>
+      <c r="O205" s="2" t="inlineStr">
+        <is>
+          <t>20.07.2026 09:25 — 27.07.2026 10:00</t>
+        </is>
+      </c>
+      <c r="P205" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ЗАМОСКВОРЕЧЬЕ, УЛ. ДУБИНИНСКАЯ, Д. 11/17, СТР. 3, ПОМЕЩ. 66А/Ч</t>
+        </is>
+      </c>
+      <c r="Q205" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi-dlia-ob-ekta-g-krasnokamsk-zal-boksa-zakupka-prokhodit/tender-4529901/#btid=2&amp;sqh=198aea343f6f5ab2a1adc3ec03d1b93fd036ce1e&amp;tsid=4529901458</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q203"/>
+  <autoFilter ref="A1:Q205"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -17429,6 +17587,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q201" r:id="rId200"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q202" r:id="rId201"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q203" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q204" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q205" r:id="rId204"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-20 14:35 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$205</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$206</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q205"/>
+  <dimension ref="A1:Q206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -17382,8 +17382,87 @@
         </is>
       </c>
     </row>
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20 14:35</t>
+        </is>
+      </c>
+      <c r="B206" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C206" s="2" t="inlineStr"/>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E206" s="2" t="inlineStr">
+        <is>
+          <t>4530281</t>
+        </is>
+      </c>
+      <c r="F206" s="2" t="inlineStr">
+        <is>
+          <t>Дорожные плиты. (Заявка 8097).</t>
+        </is>
+      </c>
+      <c r="G206" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ГК ФСК"</t>
+        </is>
+      </c>
+      <c r="H206" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ГК ФСК"</t>
+        </is>
+      </c>
+      <c r="I206" s="2" t="inlineStr">
+        <is>
+          <t>7708332091</t>
+        </is>
+      </c>
+      <c r="J206" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K206" s="2" t="inlineStr">
+        <is>
+          <t>Трубников Дмитрий Александрович</t>
+        </is>
+      </c>
+      <c r="L206" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M206" s="2" t="inlineStr">
+        <is>
+          <t>64.99</t>
+        </is>
+      </c>
+      <c r="N206" s="2" t="inlineStr"/>
+      <c r="O206" s="2" t="inlineStr">
+        <is>
+          <t>20.07.2026 12:34 — 21.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P206" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Каланчевская, д 32, помещ 4/2П</t>
+        </is>
+      </c>
+      <c r="Q206" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/dorozhnye-plity-zaiavka-8097/tender-4530281/#btid=2&amp;sqh=706cd3403e8bcdedc863efbb2163546e893b8f2b&amp;tsid=4530281004</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q205"/>
+  <autoFilter ref="A1:Q206"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -17589,6 +17668,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q203" r:id="rId202"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q204" r:id="rId203"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q205" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q206" r:id="rId205"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-21 08:48 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$206</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$209</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q206"/>
+  <dimension ref="A1:Q209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -17461,8 +17461,247 @@
         </is>
       </c>
     </row>
+    <row r="207">
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21 08:48</t>
+        </is>
+      </c>
+      <c r="B207" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C207" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D207" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E207" s="2" t="inlineStr">
+        <is>
+          <t>32616222187</t>
+        </is>
+      </c>
+      <c r="F207" s="2" t="inlineStr">
+        <is>
+          <t>Выполнение работ по разработке проекта производства работ (ППР) в т.ч. технологические карты (ТК) при пересеченииЛЭП«Тамтачет-Полинчет-Кондратьево» в пролётеопор№ 33 и № 34 с железнодорожными путями и воздушной линии 10кВ АО «РЖД», на 148 км ПК 1+12,7 перегона Тамтачет – Чунояр Красноярской железной дороги; строительства 2 КЛ-10кВ отопоры№1АЛЭП«Тамтачет-Полинчет-Кондратьево» до ячейки № 18 КРУН-10кВ ПС № 17 «Тамтачет» филиала ПАО «Россети Сибирь» - «Красноярскэнерго» по территории ПС «Тамтачет»</t>
+        </is>
+      </c>
+      <c r="G207" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "БРАТСКАЯ ЭЛЕКТРОСЕТЕВАЯ КОМПАНИЯ"</t>
+        </is>
+      </c>
+      <c r="H207" s="2" t="inlineStr">
+        <is>
+          <t>АО "БЭСК"</t>
+        </is>
+      </c>
+      <c r="I207" s="2" t="inlineStr">
+        <is>
+          <t>3804009506</t>
+        </is>
+      </c>
+      <c r="J207" s="2" t="inlineStr">
+        <is>
+          <t>Иркутская обл</t>
+        </is>
+      </c>
+      <c r="K207" s="2" t="inlineStr">
+        <is>
+          <t>Катнов Александр Анатольевич</t>
+        </is>
+      </c>
+      <c r="L207" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M207" s="2" t="inlineStr">
+        <is>
+          <t>35.12.1</t>
+        </is>
+      </c>
+      <c r="N207" s="2" t="inlineStr">
+        <is>
+          <t>55 666,67 ₽</t>
+        </is>
+      </c>
+      <c r="O207" s="2" t="inlineStr">
+        <is>
+          <t>21.07.2026 | 21.07.2026 | 28.07.2026</t>
+        </is>
+      </c>
+      <c r="P207" s="2" t="inlineStr">
+        <is>
+          <t>г Иркутск, ул Лермонтова, д 279/10</t>
+        </is>
+      </c>
+      <c r="Q207" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/223/purchase/public/purchase/info/common-info.html?regNumber=32616222187</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21 08:48</t>
+        </is>
+      </c>
+      <c r="B208" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C208" s="2" t="inlineStr"/>
+      <c r="D208" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E208" s="2" t="inlineStr">
+        <is>
+          <t>4510504</t>
+        </is>
+      </c>
+      <c r="F208" s="2" t="inlineStr">
+        <is>
+          <t>(Заявка № ДОР-17560) Лестницы/ЖБИ</t>
+        </is>
+      </c>
+      <c r="G208" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="H208" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="I208" s="2" t="inlineStr">
+        <is>
+          <t>7724498866</t>
+        </is>
+      </c>
+      <c r="J208" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K208" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
+      <c r="L208" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M208" s="2" t="inlineStr">
+        <is>
+          <t>46.73</t>
+        </is>
+      </c>
+      <c r="N208" s="2" t="inlineStr"/>
+      <c r="O208" s="2" t="inlineStr">
+        <is>
+          <t>02.07.2026 10:55 — 21.07.2026 15:00</t>
+        </is>
+      </c>
+      <c r="P208" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+        </is>
+      </c>
+      <c r="Q208" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zaiavka-dor-17560-lestnitsy-zhbi/tender-4510504/#btid=2&amp;sqh=78f48de2716a8021d5cd8c9fc9c0814cf1859492&amp;tsid=4510504459</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21 08:48</t>
+        </is>
+      </c>
+      <c r="B209" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C209" s="2" t="inlineStr"/>
+      <c r="D209" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E209" s="2" t="inlineStr">
+        <is>
+          <t>4531456</t>
+        </is>
+      </c>
+      <c r="F209" s="2" t="inlineStr">
+        <is>
+          <t>Закупка плит ПД4531456 ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "АИМ МЕНЕДЖМЕНТ"Железобетонные изделия</t>
+        </is>
+      </c>
+      <c r="G209" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H209" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I209" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J209" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K209" s="2" t="inlineStr"/>
+      <c r="L209" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M209" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N209" s="2" t="inlineStr"/>
+      <c r="O209" s="2" t="inlineStr">
+        <is>
+          <t>21.07.2026 06:46 — 24.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P209" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q209" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-plit-pd/tender-4531456/#btid=2&amp;sqh=ba1746f21dc0aab28065200078889d5aeff6b44a&amp;tsid=4531456458</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q206"/>
+  <autoFilter ref="A1:Q209"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -17669,6 +17908,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q204" r:id="rId203"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q205" r:id="rId204"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q206" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q207" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q208" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q209" r:id="rId208"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-22 08:49 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$209</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$210</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q209"/>
+  <dimension ref="A1:Q210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -17700,8 +17700,87 @@
         </is>
       </c>
     </row>
+    <row r="210">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22 08:49</t>
+        </is>
+      </c>
+      <c r="B210" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C210" s="2" t="inlineStr"/>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E210" s="2" t="inlineStr">
+        <is>
+          <t>4529727</t>
+        </is>
+      </c>
+      <c r="F210" s="2" t="inlineStr">
+        <is>
+          <t>Железобетонные изделияПлита перекрытия лотков П22-15И Плитка 2400*1500*160 б/у Плита перекрытия ПК 60-12 б/у</t>
+        </is>
+      </c>
+      <c r="G210" s="2" t="inlineStr">
+        <is>
+          <t>ПАО "Коршуновский ГОК"</t>
+        </is>
+      </c>
+      <c r="H210" s="2" t="inlineStr">
+        <is>
+          <t>ПАО "КОРШУНОВСКИЙ ГОК"</t>
+        </is>
+      </c>
+      <c r="I210" s="2" t="inlineStr">
+        <is>
+          <t>3834002314</t>
+        </is>
+      </c>
+      <c r="J210" s="2" t="inlineStr">
+        <is>
+          <t>Иркутская обл</t>
+        </is>
+      </c>
+      <c r="K210" s="2" t="inlineStr">
+        <is>
+          <t>Иванов Алексей Васильевич</t>
+        </is>
+      </c>
+      <c r="L210" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M210" s="2" t="inlineStr">
+        <is>
+          <t>07.10.2</t>
+        </is>
+      </c>
+      <c r="N210" s="2" t="inlineStr"/>
+      <c r="O210" s="2" t="inlineStr">
+        <is>
+          <t>22.07.2026 10:26 — 18.08.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P210" s="2" t="inlineStr">
+        <is>
+          <t>Иркутская обл, г Железногорск-Илимский, ул Иващенко, д 9А/1</t>
+        </is>
+      </c>
+      <c r="Q210" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/zhelezobetonnye-izdeliia/tender-4529727/#btid=2&amp;sqh=3973675c8038d4e5117112b1cd639f1f6856bab1&amp;tsid=4529727003</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q209"/>
+  <autoFilter ref="A1:Q210"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -17911,6 +17990,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q207" r:id="rId206"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q208" r:id="rId207"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q209" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q210" r:id="rId209"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-22 14:23 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$210</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$213</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q210"/>
+  <dimension ref="A1:Q213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -17779,8 +17779,241 @@
         </is>
       </c>
     </row>
+    <row r="211">
+      <c r="A211" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22 14:23</t>
+        </is>
+      </c>
+      <c r="B211" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C211" s="2" t="inlineStr"/>
+      <c r="D211" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E211" s="2" t="inlineStr">
+        <is>
+          <t>4534470</t>
+        </is>
+      </c>
+      <c r="F211" s="2" t="inlineStr">
+        <is>
+          <t>Железобетонные изделия...  ПЛИТА ПОКРЫТИЯКОЛОДЦЕВ1ПП-15-2 С.З.900.1-14.1КОЛЬЦОЖ ... .3.006.1-2.87 В2КОЛЬЦОКЦ-15-9 СЕРИЯ3.900-3 ...</t>
+        </is>
+      </c>
+      <c r="G211" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H211" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I211" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J211" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K211" s="2" t="inlineStr"/>
+      <c r="L211" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M211" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N211" s="2" t="inlineStr"/>
+      <c r="O211" s="2" t="inlineStr">
+        <is>
+          <t>22.07.2026 15:20 — 05.08.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P211" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q211" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zhelezobetonnye-izdeliia/tender-4534470/#btid=2&amp;sqh=da1070473860f60c15bd67903055d8c8bb7a4b41&amp;tsid=4534470458</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22 14:23</t>
+        </is>
+      </c>
+      <c r="B212" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C212" s="2" t="inlineStr"/>
+      <c r="D212" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E212" s="2" t="inlineStr">
+        <is>
+          <t>4534536</t>
+        </is>
+      </c>
+      <c r="F212" s="2" t="inlineStr">
+        <is>
+          <t>Поставка Кирпича КР-р-по 250*120*65/1НФ/150/2/50 по ГОСТ 530-2012... .038.1-1, в.1Перемычка5ПБ 21-27 1.038.1 ... -1, в.1Перемычка5ПБ 25-27 1.038.1 ... -1, в.1Перемычка3ПБ 16-37 1.038.1 ... -1, в.1Перемычка3ПБ 13-37 1.038.1 ... 038.1-1, в.1Перемычка5ПБ 34-20 1.038.1 ... -1, в.1Перемычка3ПБ 34-4 Балка монолитная БМ ...</t>
+        </is>
+      </c>
+      <c r="G212" s="2" t="inlineStr">
+        <is>
+          <t>ООО "Энергострой"</t>
+        </is>
+      </c>
+      <c r="H212" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ЭНЕРГОСТРОЙ"</t>
+        </is>
+      </c>
+      <c r="I212" s="2" t="inlineStr">
+        <is>
+          <t>7842436640</t>
+        </is>
+      </c>
+      <c r="J212" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K212" s="2" t="inlineStr">
+        <is>
+          <t>Тевис Александр Валентинович</t>
+        </is>
+      </c>
+      <c r="L212" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M212" s="2" t="inlineStr">
+        <is>
+          <t>42.21</t>
+        </is>
+      </c>
+      <c r="N212" s="2" t="inlineStr"/>
+      <c r="O212" s="2" t="inlineStr">
+        <is>
+          <t>22.07.2026 16:24 — 27.07.2026 16:27</t>
+        </is>
+      </c>
+      <c r="P212" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Нижняя Красносельская, д 40/12 к 20, офис 614</t>
+        </is>
+      </c>
+      <c r="Q212" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/postavka-kirpicha-kr-r-po-250-120-65-1nf-150-2-50-po-gost-530-2012/tender-4534536/#btid=2&amp;sqh=6faf89cb530cf2fdd2a96485230c6a0ee6824951&amp;tsid=4534536458</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22 14:23</t>
+        </is>
+      </c>
+      <c r="B213" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C213" s="2" t="inlineStr"/>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E213" s="2" t="inlineStr">
+        <is>
+          <t>4534443</t>
+        </is>
+      </c>
+      <c r="F213" s="2" t="inlineStr">
+        <is>
+          <t>Выбор поставщика на право поставкиблоков вентиляционных, бетонных, керамзитобетонных на объект Группы «Эталон» в г. Омск</t>
+        </is>
+      </c>
+      <c r="G213" s="2" t="inlineStr">
+        <is>
+          <t>АО "ГК "ЭТАЛОН"</t>
+        </is>
+      </c>
+      <c r="H213" s="2" t="inlineStr">
+        <is>
+          <t>АО "ГК "ЭТАЛОН"</t>
+        </is>
+      </c>
+      <c r="I213" s="2" t="inlineStr">
+        <is>
+          <t>7814116230</t>
+        </is>
+      </c>
+      <c r="J213" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K213" s="2" t="inlineStr">
+        <is>
+          <t>Бородин Юрий Алексеевич</t>
+        </is>
+      </c>
+      <c r="L213" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M213" s="2" t="inlineStr">
+        <is>
+          <t>70.10</t>
+        </is>
+      </c>
+      <c r="N213" s="2" t="inlineStr"/>
+      <c r="O213" s="2" t="inlineStr">
+        <is>
+          <t>22.07.2026 15:17 — 27.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P213" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Новоалексеевская, д 16 стр 5</t>
+        </is>
+      </c>
+      <c r="Q213" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/vybor-postavshchika-na-pravo-postavki-blokov-ventiliatsionnykh-betonnykh/tender-4534443/#btid=2&amp;sqh=3f47b23be4502797f48b5cfb5ea17fdac0b81785&amp;tsid=4534443458</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q210"/>
+  <autoFilter ref="A1:Q213"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -17991,6 +18224,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q208" r:id="rId207"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q209" r:id="rId208"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q210" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q211" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q212" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q213" r:id="rId212"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-23 03:44 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$213</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$214</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q213"/>
+  <dimension ref="A1:Q214"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -18012,8 +18012,93 @@
         </is>
       </c>
     </row>
+    <row r="214">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-23 03:44</t>
+        </is>
+      </c>
+      <c r="B214" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C214" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D214" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E214" s="2" t="inlineStr">
+        <is>
+          <t>32616229221</t>
+        </is>
+      </c>
+      <c r="F214" s="2" t="inlineStr">
+        <is>
+          <t>Поставка металлического пешеходного ограждения на железобетоннойплите марки ПБ для филиала «Иркутский» АО «ДСИО»</t>
+        </is>
+      </c>
+      <c r="G214" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ДОРОЖНАЯ СЛУЖБА ИРКУТСКОЙ ОБЛАСТИ"</t>
+        </is>
+      </c>
+      <c r="H214" s="2" t="inlineStr">
+        <is>
+          <t>АО "ДСИО"</t>
+        </is>
+      </c>
+      <c r="I214" s="2" t="inlineStr">
+        <is>
+          <t>3808166080</t>
+        </is>
+      </c>
+      <c r="J214" s="2" t="inlineStr">
+        <is>
+          <t>Иркутская обл</t>
+        </is>
+      </c>
+      <c r="K214" s="2" t="inlineStr">
+        <is>
+          <t>Аксаментов Владимир Сергеевич</t>
+        </is>
+      </c>
+      <c r="L214" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M214" s="2" t="inlineStr">
+        <is>
+          <t>52.21.22</t>
+        </is>
+      </c>
+      <c r="N214" s="2" t="inlineStr">
+        <is>
+          <t>2 627 118,00 ₽</t>
+        </is>
+      </c>
+      <c r="O214" s="2" t="inlineStr">
+        <is>
+          <t>23.07.2026 | 23.07.2026 | 04.08.2026</t>
+        </is>
+      </c>
+      <c r="P214" s="2" t="inlineStr">
+        <is>
+          <t>г Иркутск, ул Декабрьских Событий, д 88</t>
+        </is>
+      </c>
+      <c r="Q214" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/223/purchase/public/purchase/info/common-info.html?regNumber=32616229221</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q213"/>
+  <autoFilter ref="A1:Q214"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -18227,6 +18312,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q211" r:id="rId210"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q212" r:id="rId211"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q213" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q214" r:id="rId213"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-23 08:51 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$214</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$216</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q214"/>
+  <dimension ref="A1:Q216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -18097,8 +18097,166 @@
         </is>
       </c>
     </row>
+    <row r="215">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-23 08:51</t>
+        </is>
+      </c>
+      <c r="B215" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C215" s="2" t="inlineStr"/>
+      <c r="D215" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E215" s="2" t="inlineStr">
+        <is>
+          <t>4535447</t>
+        </is>
+      </c>
+      <c r="F215" s="2" t="inlineStr">
+        <is>
+          <t>Автоматика и телемеханика движения поездов, ВСП и тоннельные материалы...  (ВхШхГ) не более 99х35х186 мм, массаизделияне более 0,45 кг Модуль ... -3 36131-113-00-02 Полушпалажелезобетоннаявибро-шумопоглощающая типа LVT-НА-М ...  2 Вт, номинал 12 кОм Полушпалажелезобетоннаявибро-шумопоглощающая типа LVT-НА-М ...</t>
+        </is>
+      </c>
+      <c r="G215" s="2" t="inlineStr">
+        <is>
+          <t>АО "Мосинжпроект"</t>
+        </is>
+      </c>
+      <c r="H215" s="2" t="inlineStr">
+        <is>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
+        </is>
+      </c>
+      <c r="I215" s="2" t="inlineStr">
+        <is>
+          <t>7701885820</t>
+        </is>
+      </c>
+      <c r="J215" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K215" s="2" t="inlineStr">
+        <is>
+          <t>Сорокин Антон Павлович</t>
+        </is>
+      </c>
+      <c r="L215" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M215" s="2" t="inlineStr">
+        <is>
+          <t>71.12.2</t>
+        </is>
+      </c>
+      <c r="N215" s="2" t="inlineStr"/>
+      <c r="O215" s="2" t="inlineStr">
+        <is>
+          <t>23.07.2026 11:34 — 26.08.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P215" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+        </is>
+      </c>
+      <c r="Q215" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/avtomatika-i-telemekhanika-dvizheniia-poezdov-vsp-i-tonnelnye-materialy/tender-4535447/#btid=2&amp;sqh=dc8d114942fae1aa5116483b9a0fe1dcbecc09e8&amp;tsid=4535447003</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-23 08:51</t>
+        </is>
+      </c>
+      <c r="B216" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C216" s="2" t="inlineStr"/>
+      <c r="D216" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E216" s="2" t="inlineStr">
+        <is>
+          <t>4535271</t>
+        </is>
+      </c>
+      <c r="F216" s="2" t="inlineStr">
+        <is>
+          <t>Источники электропитания (ИБП, аккумуляторные батареи, блоки питания)...  х 1248 А·ч, включая соединительныеперемычки. Вид положительного электрода - трубчатая пластина ...  с коммутирующей арматурой, межэлементными и межряднымиперемычками, крепежами, комплектом для обслуживания АБ. Тип ...</t>
+        </is>
+      </c>
+      <c r="G216" s="2" t="inlineStr">
+        <is>
+          <t>АО "Мосинжпроект"</t>
+        </is>
+      </c>
+      <c r="H216" s="2" t="inlineStr">
+        <is>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
+        </is>
+      </c>
+      <c r="I216" s="2" t="inlineStr">
+        <is>
+          <t>7701885820</t>
+        </is>
+      </c>
+      <c r="J216" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K216" s="2" t="inlineStr">
+        <is>
+          <t>Сорокин Антон Павлович</t>
+        </is>
+      </c>
+      <c r="L216" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M216" s="2" t="inlineStr">
+        <is>
+          <t>71.12.2</t>
+        </is>
+      </c>
+      <c r="N216" s="2" t="inlineStr"/>
+      <c r="O216" s="2" t="inlineStr">
+        <is>
+          <t>23.07.2026 10:31 — 19.08.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P216" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+        </is>
+      </c>
+      <c r="Q216" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/istochniki-elektropitaniia-ibp-akkumuliatornye-batarei-bloki-pitaniia/tender-4535271/#btid=2&amp;sqh=5cb09f36f3aec0d006b9259ad7822207dfda37ac&amp;tsid=4535271003</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q214"/>
+  <autoFilter ref="A1:Q216"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -18313,6 +18471,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q212" r:id="rId211"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q213" r:id="rId212"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q214" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q215" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q216" r:id="rId215"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-23 14:31 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$216</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$221</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q216"/>
+  <dimension ref="A1:Q221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -18255,8 +18255,399 @@
         </is>
       </c>
     </row>
+    <row r="217">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-23 14:31</t>
+        </is>
+      </c>
+      <c r="B217" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C217" s="2" t="inlineStr"/>
+      <c r="D217" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E217" s="2" t="inlineStr">
+        <is>
+          <t>4536011</t>
+        </is>
+      </c>
+      <c r="F217" s="2" t="inlineStr">
+        <is>
+          <t>ЖБИизделия Для СЗРК Кольцо опорное с днищем Балки фундаментные Ступени</t>
+        </is>
+      </c>
+      <c r="G217" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+        </is>
+      </c>
+      <c r="H217" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+        </is>
+      </c>
+      <c r="I217" s="2" t="inlineStr">
+        <is>
+          <t>7805368914</t>
+        </is>
+      </c>
+      <c r="J217" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="K217" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
+        </is>
+      </c>
+      <c r="L217" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M217" s="2" t="inlineStr">
+        <is>
+          <t>46.90</t>
+        </is>
+      </c>
+      <c r="N217" s="2" t="inlineStr"/>
+      <c r="O217" s="2" t="inlineStr">
+        <is>
+          <t>23.07.2026 14:54 — 28.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P217" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
+        </is>
+      </c>
+      <c r="Q217" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/zhbi-izdeliia-dlia-szrk/tender-4536011/#btid=2&amp;sqh=e5bf33c9a4013fa7e30596deab334c9f56ce2011&amp;tsid=4536011004</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-23 14:31</t>
+        </is>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C218" s="2" t="inlineStr"/>
+      <c r="D218" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E218" s="2" t="inlineStr">
+        <is>
+          <t>4536053</t>
+        </is>
+      </c>
+      <c r="F218" s="2" t="inlineStr">
+        <is>
+          <t>ТМЦ_брус ЖБ4536053 ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "АИМ МЕНЕДЖМЕНТ"Железобетонные изделия</t>
+        </is>
+      </c>
+      <c r="G218" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H218" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I218" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J218" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K218" s="2" t="inlineStr"/>
+      <c r="L218" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M218" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N218" s="2" t="inlineStr"/>
+      <c r="O218" s="2" t="inlineStr">
+        <is>
+          <t>23.07.2026 15:16 — 29.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P218" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ. ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q218" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/tmts-brus-zhb/tender-4536053/#btid=2&amp;sqh=b61f57502c2681d293d58353f8f81d98583131ae&amp;tsid=4536053458</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-23 14:31</t>
+        </is>
+      </c>
+      <c r="B219" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C219" s="2" t="inlineStr"/>
+      <c r="D219" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E219" s="2" t="inlineStr">
+        <is>
+          <t>4536322</t>
+        </is>
+      </c>
+      <c r="F219" s="2" t="inlineStr">
+        <is>
+          <t>Закупка бетонного укрытия для ФТС "Пятерочка"4536322 ПУБЛИЧНОЕ АКЦИОНЕРНОЕ ОБЩЕСТВО "КОРПОРАТИВНЫЙ ЦЕНТР ИКС 5"Железобетонные изделия</t>
+        </is>
+      </c>
+      <c r="G219" s="2" t="inlineStr">
+        <is>
+          <t>ПАО "КОРПОРАТИВНЫЙ ЦЕНТР ИКС 5"</t>
+        </is>
+      </c>
+      <c r="H219" s="2" t="inlineStr">
+        <is>
+          <t>ПАО "КОРПОРАТИВНЫЙ ЦЕНТР ИКС 5"</t>
+        </is>
+      </c>
+      <c r="I219" s="2" t="inlineStr">
+        <is>
+          <t>9722079341</t>
+        </is>
+      </c>
+      <c r="J219" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K219" s="2" t="inlineStr">
+        <is>
+          <t>Шехтерман Игорь Владимирович</t>
+        </is>
+      </c>
+      <c r="L219" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M219" s="2" t="inlineStr">
+        <is>
+          <t>70.10</t>
+        </is>
+      </c>
+      <c r="N219" s="2" t="inlineStr"/>
+      <c r="O219" s="2" t="inlineStr">
+        <is>
+          <t>23.07.2026 16:43 — 29.07.2026 16:00</t>
+        </is>
+      </c>
+      <c r="P219" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Средняя Калитниковская, д 28 стр 4</t>
+        </is>
+      </c>
+      <c r="Q219" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-betonnogo-ukrytiia-dlia-fts-piaterochka/tender-4536322/#btid=2&amp;sqh=b61f57502c2681d293d58353f8f81d98583131ae&amp;tsid=4536322458</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-23 14:31</t>
+        </is>
+      </c>
+      <c r="B220" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C220" s="2" t="inlineStr"/>
+      <c r="D220" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E220" s="2" t="inlineStr">
+        <is>
+          <t>4536134</t>
+        </is>
+      </c>
+      <c r="F220" s="2" t="inlineStr">
+        <is>
+          <t>Вентиляторы промышленные и оборудование общеобменной вентиляции...  5Ф РешёткавентиляционнаяАМР 600х300М РешёткавентиляционнаяАМР 150х150М РешёткавентиляционнаяАМР 300х200М  ... мм.; масса 0,65 кгБлокконтроля сопротивления БСК-3.1 Канальный ...  533Па, габаритные размеры 700х467х2230 мм,блоков/моноблоков 5/1, в составе: - ...</t>
+        </is>
+      </c>
+      <c r="G220" s="2" t="inlineStr">
+        <is>
+          <t>АО "Мосинжпроект"</t>
+        </is>
+      </c>
+      <c r="H220" s="2" t="inlineStr">
+        <is>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
+        </is>
+      </c>
+      <c r="I220" s="2" t="inlineStr">
+        <is>
+          <t>7701885820</t>
+        </is>
+      </c>
+      <c r="J220" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K220" s="2" t="inlineStr">
+        <is>
+          <t>Сорокин Антон Павлович</t>
+        </is>
+      </c>
+      <c r="L220" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M220" s="2" t="inlineStr">
+        <is>
+          <t>71.12.2</t>
+        </is>
+      </c>
+      <c r="N220" s="2" t="inlineStr"/>
+      <c r="O220" s="2" t="inlineStr">
+        <is>
+          <t>23.07.2026 15:26 — 26.08.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P220" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+        </is>
+      </c>
+      <c r="Q220" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/ventiliatory-promyshlennye-i-oborudovanie-obshcheobmennoi-ventiliatsii/tender-4536134/#btid=2&amp;sqh=9ea0563d13cd85c48f1bd4d3b680169fde2f975a&amp;tsid=4536134003</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-23 14:31</t>
+        </is>
+      </c>
+      <c r="B221" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C221" s="2" t="inlineStr"/>
+      <c r="D221" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E221" s="2" t="inlineStr">
+        <is>
+          <t>4536144</t>
+        </is>
+      </c>
+      <c r="F221" s="2" t="inlineStr">
+        <is>
+          <t>Коммуникационное оборудование, компьютеры, комплектующие к ним, серверное оборудование и ПО...  телефонный Телта-214-4Блокакустический встраиваемый в балюстраду эскалатора ... 2х2 Комбайнер специализированный OMU Side (блок1) OMUSC1 Комбайнер специализированный  ...  для мониторинга в FlexGain View,вентиляционнаяпанель с фильтрами, комплект кабелей ...</t>
+        </is>
+      </c>
+      <c r="G221" s="2" t="inlineStr">
+        <is>
+          <t>АО "Мосинжпроект"</t>
+        </is>
+      </c>
+      <c r="H221" s="2" t="inlineStr">
+        <is>
+          <t>АО "МОСИНЖПРОЕКТ"</t>
+        </is>
+      </c>
+      <c r="I221" s="2" t="inlineStr">
+        <is>
+          <t>7701885820</t>
+        </is>
+      </c>
+      <c r="J221" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K221" s="2" t="inlineStr">
+        <is>
+          <t>Сорокин Антон Павлович</t>
+        </is>
+      </c>
+      <c r="L221" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M221" s="2" t="inlineStr">
+        <is>
+          <t>71.12.2</t>
+        </is>
+      </c>
+      <c r="N221" s="2" t="inlineStr"/>
+      <c r="O221" s="2" t="inlineStr">
+        <is>
+          <t>23.07.2026 15:29 — 26.08.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P221" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Сверчков пер, д 4/1 стр 1</t>
+        </is>
+      </c>
+      <c r="Q221" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/kommunikatsionnoe-oborudovanie-kompiutery-komplektuiushchie-k-nim/tender-4536144/#btid=2&amp;sqh=9ea0563d13cd85c48f1bd4d3b680169fde2f975a&amp;tsid=4536144003</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q216"/>
+  <autoFilter ref="A1:Q221"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -18473,6 +18864,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q214" r:id="rId213"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q215" r:id="rId214"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q216" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q217" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q218" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q219" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q220" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q221" r:id="rId220"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-24 03:39 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$221</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$222</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q221"/>
+  <dimension ref="A1:Q222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -18646,8 +18646,87 @@
         </is>
       </c>
     </row>
+    <row r="222">
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 03:39</t>
+        </is>
+      </c>
+      <c r="B222" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C222" s="2" t="inlineStr"/>
+      <c r="D222" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E222" s="2" t="inlineStr">
+        <is>
+          <t>4536510</t>
+        </is>
+      </c>
+      <c r="F222" s="2" t="inlineStr">
+        <is>
+          <t>ПеревозкаЖБИизделий панелевозами и длинномерами. г. Новосибирск</t>
+        </is>
+      </c>
+      <c r="G222" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СМРСТРОЙ"</t>
+        </is>
+      </c>
+      <c r="H222" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СМР СТРОЙ"</t>
+        </is>
+      </c>
+      <c r="I222" s="2" t="inlineStr">
+        <is>
+          <t>7701615809</t>
+        </is>
+      </c>
+      <c r="J222" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K222" s="2" t="inlineStr">
+        <is>
+          <t>Жукова Мария Дмитриевна</t>
+        </is>
+      </c>
+      <c r="L222" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M222" s="2" t="inlineStr">
+        <is>
+          <t>41.2</t>
+        </is>
+      </c>
+      <c r="N222" s="2" t="inlineStr"/>
+      <c r="O222" s="2" t="inlineStr">
+        <is>
+          <t>24.07.2026 05:07 — 31.07.2026 09:00</t>
+        </is>
+      </c>
+      <c r="P222" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Молодогвардейская, д 15</t>
+        </is>
+      </c>
+      <c r="Q222" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/perevozka-zhbi-izdelii-panelevozami-i-dlinnomerami-g-novosibirsk/tender-4536510/#btid=2&amp;sqh=7851ce7d38bf51d31425fd51feb78b87139bcb50&amp;tsid=4536510458</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q221"/>
+  <autoFilter ref="A1:Q222"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -18869,6 +18948,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q219" r:id="rId218"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q220" r:id="rId219"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q221" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q222" r:id="rId221"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-24 08:46 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$222</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$223</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q222"/>
+  <dimension ref="A1:Q223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -18725,8 +18725,93 @@
         </is>
       </c>
     </row>
+    <row r="223">
+      <c r="A223" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 08:46</t>
+        </is>
+      </c>
+      <c r="B223" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C223" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D223" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E223" s="2" t="inlineStr">
+        <is>
+          <t>32616234605</t>
+        </is>
+      </c>
+      <c r="F223" s="2" t="inlineStr">
+        <is>
+          <t>Выполнение ПИР, СМР, ПНР полным иждивением подрядчика по титулу: Строительство ТП-250-6/0,4 кВ,ЛЭП-6 кВ от ВЛ-6 кВ ф.2 ПС №109 "Юсупово"ЛР-6 кВ,ЛЭП-0,4 кВ (по сущ.опорам), в т.ч. ПИР, МО, Раменский р-н, с/пЧулковское Ю8-26-302-294697(176007) для нужд филиала ПАО «Россети Московский регион» - Южные электрические сети</t>
+        </is>
+      </c>
+      <c r="G223" s="2" t="inlineStr">
+        <is>
+          <t>ПУБЛИЧНОЕ АКЦИОНЕРНОЕ ОБЩЕСТВО "РОССЕТИ МОСКОВСКИЙ РЕГИОН"</t>
+        </is>
+      </c>
+      <c r="H223" s="2" t="inlineStr">
+        <is>
+          <t>ПАО "РОССЕТИ МОСКОВСКИЙ РЕГИОН", ПАО "РОССЕТИ МР"</t>
+        </is>
+      </c>
+      <c r="I223" s="2" t="inlineStr">
+        <is>
+          <t>5036065113</t>
+        </is>
+      </c>
+      <c r="J223" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K223" s="2" t="inlineStr">
+        <is>
+          <t>Пятигор Александр Михайлович</t>
+        </is>
+      </c>
+      <c r="L223" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M223" s="2" t="inlineStr">
+        <is>
+          <t>35.12.1</t>
+        </is>
+      </c>
+      <c r="N223" s="2" t="inlineStr">
+        <is>
+          <t>2 530 458,22 ₽</t>
+        </is>
+      </c>
+      <c r="O223" s="2" t="inlineStr">
+        <is>
+          <t>24.07.2026 | 24.07.2026 | 28.07.2026</t>
+        </is>
+      </c>
+      <c r="P223" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, 2-й Павелецкий проезд, д 3 стр 2</t>
+        </is>
+      </c>
+      <c r="Q223" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/223/purchase/public/purchase/info/common-info.html?regNumber=32616234605</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q222"/>
+  <autoFilter ref="A1:Q223"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -18949,6 +19034,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q220" r:id="rId219"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q221" r:id="rId220"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q222" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q223" r:id="rId222"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-24 14:12 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$223</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$229</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q223"/>
+  <dimension ref="A1:Q229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -18810,8 +18810,497 @@
         </is>
       </c>
     </row>
+    <row r="224">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 14:12</t>
+        </is>
+      </c>
+      <c r="B224" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C224" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D224" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E224" s="2" t="inlineStr">
+        <is>
+          <t>32616236659</t>
+        </is>
+      </c>
+      <c r="F224" s="2" t="inlineStr">
+        <is>
+          <t>Выполнение полного комплекса строительно-монтажных работ по монтажудорожныхплити устройству ограждения по объекту:«Строительство нового источника в районе перспективной застройки кв. 7.1 в г. Ро-стов-на-Дону на 16 Гкал/час (резерв)»</t>
+        </is>
+      </c>
+      <c r="G224" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "КРАСНОДАРТЕПЛОСЕТЬ"</t>
+        </is>
+      </c>
+      <c r="H224" s="2" t="inlineStr">
+        <is>
+          <t>АО "КРАСНОДАРТЕПЛОСЕТЬ"</t>
+        </is>
+      </c>
+      <c r="I224" s="2" t="inlineStr">
+        <is>
+          <t>2312122495</t>
+        </is>
+      </c>
+      <c r="J224" s="2" t="inlineStr">
+        <is>
+          <t>Краснодарский край</t>
+        </is>
+      </c>
+      <c r="K224" s="2" t="inlineStr">
+        <is>
+          <t>Харченко Виталий Александрович</t>
+        </is>
+      </c>
+      <c r="L224" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M224" s="2" t="inlineStr">
+        <is>
+          <t>35.30.14</t>
+        </is>
+      </c>
+      <c r="N224" s="2" t="inlineStr">
+        <is>
+          <t>3 116 860,25 ₽</t>
+        </is>
+      </c>
+      <c r="O224" s="2" t="inlineStr">
+        <is>
+          <t>24.07.2026 | 24.07.2026 | 03.08.2026</t>
+        </is>
+      </c>
+      <c r="P224" s="2" t="inlineStr">
+        <is>
+          <t>г Краснодар, ул Ставропольская, д 2</t>
+        </is>
+      </c>
+      <c r="Q224" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/223/purchase/public/purchase/info/common-info.html?regNumber=32616236659</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 14:12</t>
+        </is>
+      </c>
+      <c r="B225" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C225" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E225" s="2" t="inlineStr">
+        <is>
+          <t>32616236653</t>
+        </is>
+      </c>
+      <c r="F225" s="2" t="inlineStr">
+        <is>
+          <t>Выполнение полного комплекса строительно-монтажных работ по монтажудорожныхплити устройству ограждения по объекту: «Строительство новой котельной №28 в г. Ростов-на-Дону», расположенной на ЗУ с кадастровым номером № 61:44:0082615:23439»</t>
+        </is>
+      </c>
+      <c r="G225" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "КРАСНОДАРТЕПЛОСЕТЬ"</t>
+        </is>
+      </c>
+      <c r="H225" s="2" t="inlineStr">
+        <is>
+          <t>АО "КРАСНОДАРТЕПЛОСЕТЬ"</t>
+        </is>
+      </c>
+      <c r="I225" s="2" t="inlineStr">
+        <is>
+          <t>2312122495</t>
+        </is>
+      </c>
+      <c r="J225" s="2" t="inlineStr">
+        <is>
+          <t>Краснодарский край</t>
+        </is>
+      </c>
+      <c r="K225" s="2" t="inlineStr">
+        <is>
+          <t>Харченко Виталий Александрович</t>
+        </is>
+      </c>
+      <c r="L225" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M225" s="2" t="inlineStr">
+        <is>
+          <t>35.30.14</t>
+        </is>
+      </c>
+      <c r="N225" s="2" t="inlineStr">
+        <is>
+          <t>3 711 610,45 ₽</t>
+        </is>
+      </c>
+      <c r="O225" s="2" t="inlineStr">
+        <is>
+          <t>24.07.2026 | 24.07.2026 | 03.08.2026</t>
+        </is>
+      </c>
+      <c r="P225" s="2" t="inlineStr">
+        <is>
+          <t>г Краснодар, ул Ставропольская, д 2</t>
+        </is>
+      </c>
+      <c r="Q225" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/223/purchase/public/purchase/info/common-info.html?regNumber=32616236653</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 14:12</t>
+        </is>
+      </c>
+      <c r="B226" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C226" s="2" t="inlineStr"/>
+      <c r="D226" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E226" s="2" t="inlineStr">
+        <is>
+          <t>4537384</t>
+        </is>
+      </c>
+      <c r="F226" s="2" t="inlineStr">
+        <is>
+          <t>Реализация невостребованных складских остатков. Новые оригинальные запасные части для горного оборудования и спецтехники лот 3
+Реализация невостребованных складских остатков. Новые оригинальные запасные части для горного оборудования и спецтехники... 77794226;ГИДРАВЛИЧЕСКИЙ ПЕРЕКЛЮЧАТЕЛЬ;VOE23307414;ВАКУУМНЫЙПЛИТАИНДИКАТОРА ОБЪЕМА S13-48437- ...  для интеркулера SCANIA 797741704ПЛИТА;003746-001;ГИДРОРАСПРЕДЕЛИТЕЛЯ ОСНОВАНИЕ  ... 0);118мм,ВИБРАЦИОННЫЙ ПРЕДЕЛЬНОГО УРОВНЯДорожныйнасос Датчик потока скорости  ...</t>
+        </is>
+      </c>
+      <c r="G226" s="2" t="inlineStr">
+        <is>
+          <t>АО "АЗОТ-ВЗРЫВ"</t>
+        </is>
+      </c>
+      <c r="H226" s="2" t="inlineStr">
+        <is>
+          <t>АО "АЗОТ-ВЗРЫВ"</t>
+        </is>
+      </c>
+      <c r="I226" s="2" t="inlineStr">
+        <is>
+          <t>7727218041</t>
+        </is>
+      </c>
+      <c r="J226" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K226" s="2" t="inlineStr">
+        <is>
+          <t>Черниловский Илья Александрович</t>
+        </is>
+      </c>
+      <c r="L226" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M226" s="2" t="inlineStr">
+        <is>
+          <t>46.75.2</t>
+        </is>
+      </c>
+      <c r="N226" s="2" t="inlineStr"/>
+      <c r="O226" s="2" t="inlineStr">
+        <is>
+          <t>24.07.2026 13:26 — 12.08.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P226" s="2" t="inlineStr">
+        <is>
+          <t>121151, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДОРОГОМИЛОВО, УЛ. МОЖАЙСКИЙ ВАЛ, Д. 8, ЭТАЖ 11, ПОМЕЩ. LХХХI, КОМ.7, ОФИС 15</t>
+        </is>
+      </c>
+      <c r="Q226" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannykh-skladskikh-ostatkov-novye-originalnye/tender-4537384/#btid=2&amp;sqh=5e096dc6731dd4ab17dad1ddc6406d5d0eaac485&amp;tsid=4537384003</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 14:12</t>
+        </is>
+      </c>
+      <c r="B227" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C227" s="2" t="inlineStr"/>
+      <c r="D227" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E227" s="2" t="inlineStr">
+        <is>
+          <t>4537366</t>
+        </is>
+      </c>
+      <c r="F227" s="2" t="inlineStr">
+        <is>
+          <t>Реализация невостребованных складских остатков. Новые оригинальные запасные части для горного оборудования и спецтехники лот 2
+Реализация невостребованных складских остатков. Новые оригинальные запасные части для горного оборудования и спецтехники... К НАСОСУ CROSS2 C00000477 Набор уплотнительныхколецсвечногоколодцадвигателя ЗМЗ-406 Лента ободная ... ЭЛЕВАТОРАКольцоочистителя 9370620 110х130х10КОЛЬЦО;51828198КОЛЬЦОУПЛОТНИТЕЛЬНОЕ;034562-051КОЛЬЦОУПЛОТНИТЕЛЬНОЕ;4430508КОЛЬЦО;VOE991044КОЛЬЦО...</t>
+        </is>
+      </c>
+      <c r="G227" s="2" t="inlineStr">
+        <is>
+          <t>АО "АЗОТ-ВЗРЫВ"</t>
+        </is>
+      </c>
+      <c r="H227" s="2" t="inlineStr">
+        <is>
+          <t>АО "АЗОТ-ВЗРЫВ"</t>
+        </is>
+      </c>
+      <c r="I227" s="2" t="inlineStr">
+        <is>
+          <t>7727218041</t>
+        </is>
+      </c>
+      <c r="J227" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K227" s="2" t="inlineStr">
+        <is>
+          <t>Черниловский Илья Александрович</t>
+        </is>
+      </c>
+      <c r="L227" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M227" s="2" t="inlineStr">
+        <is>
+          <t>46.75.2</t>
+        </is>
+      </c>
+      <c r="N227" s="2" t="inlineStr"/>
+      <c r="O227" s="2" t="inlineStr">
+        <is>
+          <t>24.07.2026 13:19 — 12.08.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P227" s="2" t="inlineStr">
+        <is>
+          <t>121151, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДОРОГОМИЛОВО, УЛ. МОЖАЙСКИЙ ВАЛ, Д. 8, ЭТАЖ 11, ПОМЕЩ. LХХХI, КОМ.7, ОФИС 15</t>
+        </is>
+      </c>
+      <c r="Q227" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannykh-skladskikh-ostatkov-novye-originalnye/tender-4537366/#btid=2&amp;sqh=97734d9f9b3b7f3df90741930bc0512fa113b773&amp;tsid=4537366003</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 14:12</t>
+        </is>
+      </c>
+      <c r="B228" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C228" s="2" t="inlineStr"/>
+      <c r="D228" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E228" s="2" t="inlineStr">
+        <is>
+          <t>4537230</t>
+        </is>
+      </c>
+      <c r="F228" s="2" t="inlineStr">
+        <is>
+          <t>(Заявка Капотня 17698/ Лзк 287) Лотки4537230 ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "АРТСТРОЙТЕХНОЛОГИЯ"Железобетонные изделия</t>
+        </is>
+      </c>
+      <c r="G228" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="H228" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="I228" s="2" t="inlineStr">
+        <is>
+          <t>7724498866</t>
+        </is>
+      </c>
+      <c r="J228" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K228" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
+      <c r="L228" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M228" s="2" t="inlineStr">
+        <is>
+          <t>46.73</t>
+        </is>
+      </c>
+      <c r="N228" s="2" t="inlineStr"/>
+      <c r="O228" s="2" t="inlineStr">
+        <is>
+          <t>24.07.2026 12:12 — 27.07.2026 15:00</t>
+        </is>
+      </c>
+      <c r="P228" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+        </is>
+      </c>
+      <c r="Q228" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zaiavka-kapotnia-17698-lzk-287-lotki/tender-4537230/#btid=2&amp;sqh=669a3cb65da156ccf4def11afdf47b35c75edafe&amp;tsid=4537230459</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 14:12</t>
+        </is>
+      </c>
+      <c r="B229" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C229" s="2" t="inlineStr"/>
+      <c r="D229" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E229" s="2" t="inlineStr">
+        <is>
+          <t>4537308</t>
+        </is>
+      </c>
+      <c r="F229" s="2" t="inlineStr">
+        <is>
+          <t>Реализация невостребованных складских остатков. Новые оригинальные запасные части для горного оборудования и спецтехники лот 1
+Реализация невостребованных складских остатков. Новые оригинальные запасные части для горного оборудования и спецтехники... ЦЕНТРОБЕЖНОГО ОЧИСТИТЕЛЯ МАСЛА,А/М SCANIAПЕРЕМЫЧКАСОЕДИНИТЕЛЬНАЯ;022552-009;ДЛЯ КЛЕММНИКОВ, ... " 7/8 (Г) РАЗЪЕМ;57435034;ПЕРЕМЫЧКАКОНТАКТНОЙ ГРУППЫ БОЛТ;3521225;ДЛЯ ТКР ... 07005-01012;07005-01012_BST УСТРОЙСТВО;KL1212KK;ПЕРЕМЫЧКААКБ,300мм,S=35мм,КЛЕММА- ...</t>
+        </is>
+      </c>
+      <c r="G229" s="2" t="inlineStr">
+        <is>
+          <t>АО "АЗОТ-ВЗРЫВ"</t>
+        </is>
+      </c>
+      <c r="H229" s="2" t="inlineStr">
+        <is>
+          <t>АО "АЗОТ-ВЗРЫВ"</t>
+        </is>
+      </c>
+      <c r="I229" s="2" t="inlineStr">
+        <is>
+          <t>7727218041</t>
+        </is>
+      </c>
+      <c r="J229" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K229" s="2" t="inlineStr">
+        <is>
+          <t>Черниловский Илья Александрович</t>
+        </is>
+      </c>
+      <c r="L229" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M229" s="2" t="inlineStr">
+        <is>
+          <t>46.75.2</t>
+        </is>
+      </c>
+      <c r="N229" s="2" t="inlineStr"/>
+      <c r="O229" s="2" t="inlineStr">
+        <is>
+          <t>24.07.2026 13:09 — 12.08.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P229" s="2" t="inlineStr">
+        <is>
+          <t>121151, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДОРОГОМИЛОВО, УЛ. МОЖАЙСКИЙ ВАЛ, Д. 8, ЭТАЖ 11, ПОМЕЩ. LХХХI, КОМ.7, ОФИС 15</t>
+        </is>
+      </c>
+      <c r="Q229" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/realizatsiia-nevostrebovannykh-skladskikh-ostatkov-novye-originalnye/tender-4537308/#btid=2&amp;sqh=4ba7390edde27d045a48cf0934aa2a9ba5fcbe22&amp;tsid=4537308003</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q223"/>
+  <autoFilter ref="A1:Q229"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -19035,6 +19524,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q221" r:id="rId220"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q222" r:id="rId221"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q223" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q224" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q225" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q226" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q227" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q228" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q229" r:id="rId228"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-27 03:58 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$229</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$231</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q229"/>
+  <dimension ref="A1:Q231"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -19299,8 +19299,172 @@
         </is>
       </c>
     </row>
+    <row r="230">
+      <c r="A230" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27 03:58</t>
+        </is>
+      </c>
+      <c r="B230" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C230" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D230" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E230" s="2" t="inlineStr">
+        <is>
+          <t>32616237350</t>
+        </is>
+      </c>
+      <c r="F230" s="2" t="inlineStr">
+        <is>
+          <t>ПоставкаопорЛЭПдля филиала АО "ИЭСК" ПО ЗЭС в 1 квартале 2027 г.</t>
+        </is>
+      </c>
+      <c r="G230" s="2" t="inlineStr">
+        <is>
+          <t>ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "ЭН+ ТОРГОВЫЙ ДОМ"</t>
+        </is>
+      </c>
+      <c r="H230" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ЭН+ ТОРГОВЫЙ ДОМ"</t>
+        </is>
+      </c>
+      <c r="I230" s="2" t="inlineStr">
+        <is>
+          <t>3808118560</t>
+        </is>
+      </c>
+      <c r="J230" s="2" t="inlineStr">
+        <is>
+          <t>Иркутская обл</t>
+        </is>
+      </c>
+      <c r="K230" s="2" t="inlineStr">
+        <is>
+          <t>Лазарева Мария Анатольевна</t>
+        </is>
+      </c>
+      <c r="L230" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M230" s="2" t="inlineStr">
+        <is>
+          <t>46.69.9</t>
+        </is>
+      </c>
+      <c r="N230" s="2" t="inlineStr">
+        <is>
+          <t>0,00 ₽</t>
+        </is>
+      </c>
+      <c r="O230" s="2" t="inlineStr">
+        <is>
+          <t>27.07.2026 | 27.07.2026 | 11.08.2026</t>
+        </is>
+      </c>
+      <c r="P230" s="2" t="inlineStr">
+        <is>
+          <t>г Иркутск, ул Рабочая, стр 22, офис 509</t>
+        </is>
+      </c>
+      <c r="Q230" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/223/purchase/public/purchase/info/common-info.html?regNumber=32616237350</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27 03:58</t>
+        </is>
+      </c>
+      <c r="B231" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C231" s="2" t="inlineStr"/>
+      <c r="D231" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E231" s="2" t="inlineStr">
+        <is>
+          <t>4538054</t>
+        </is>
+      </c>
+      <c r="F231" s="2" t="inlineStr">
+        <is>
+          <t>Поставка материалов в рамках выполнения работ по объекту Железнодорожная станция Восточная. Устройство железнодорожной автоматики и телемеханики (СЦБ) ООО "Карбо-Л"... -4 (на 15 двухконтактных клемм, безперемычек), 1 шт. ЩИТКИ ДЛЯ СВЕТОФОРОВ (гарнитура ... -1 (на 9 двухконтактных клемм, безперемычек) применительно (ПЯ.00.000), 3 шт ...</t>
+        </is>
+      </c>
+      <c r="G231" s="2" t="inlineStr">
+        <is>
+          <t>ООО "УК "СИБАНТРАЦИТ"</t>
+        </is>
+      </c>
+      <c r="H231" s="2" t="inlineStr">
+        <is>
+          <t>ООО "УК "СИБАНТРАЦИТ"</t>
+        </is>
+      </c>
+      <c r="I231" s="2" t="inlineStr">
+        <is>
+          <t>9703160290</t>
+        </is>
+      </c>
+      <c r="J231" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K231" s="2" t="inlineStr">
+        <is>
+          <t>Мельников Сергей Владимирович</t>
+        </is>
+      </c>
+      <c r="L231" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M231" s="2" t="inlineStr">
+        <is>
+          <t>70.22</t>
+        </is>
+      </c>
+      <c r="N231" s="2" t="inlineStr"/>
+      <c r="O231" s="2" t="inlineStr">
+        <is>
+          <t>27.07.2026 06:00 — 30.07.2026 10:00</t>
+        </is>
+      </c>
+      <c r="P231" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Усачёва, д 2 стр 1, помещ 2/1</t>
+        </is>
+      </c>
+      <c r="Q231" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/postavka-materialov-v-ramkakh-vypolneniia-rabot-po-ob-ektu/tender-4538054/#btid=2&amp;sqh=20e0bd41fe902b1a21adeb42600732af02fafc2d&amp;tsid=4538054458</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q229"/>
+  <autoFilter ref="A1:Q231"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -19530,6 +19694,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q227" r:id="rId226"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q228" r:id="rId227"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q229" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q230" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q231" r:id="rId230"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-27 10:13 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$231</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$234</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q231"/>
+  <dimension ref="A1:Q234"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -19463,8 +19463,257 @@
         </is>
       </c>
     </row>
+    <row r="232">
+      <c r="A232" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27 10:13</t>
+        </is>
+      </c>
+      <c r="B232" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C232" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D232" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E232" s="2" t="inlineStr">
+        <is>
+          <t>32616237996</t>
+        </is>
+      </c>
+      <c r="F232" s="2" t="inlineStr">
+        <is>
+          <t>26Т0110050.0016. Проведение работ по компенсационному лесовосстановлению по объектам: «СтроительствоЛЭП-10 кВ от новой ячейки 10 кВ ПС 110/10 кВ № 48 до ТП-10/0,4 кВ Заявителя и установкой наопореЛЭП-10 кВ разъединителя, Мурманская обл., Кандалакшское лесничество (Договор ТП №43-0033742/19 от 29.08.2019 с ООО «Нордкап-Марикультура») ИП № 002-42-2-01.32-0888; «Строительство ВЛ-10 кВ отопоры(N) Л-3 ПС 150/10 кВ № 83 до границы участка Заявителя с установкой разъединителя на первой отпаечнойопоре и присоединением фидера 10 кВ Заявителя: Мурманская область, Р-21 «Кола» км 1230 (съезд на г. Апатиты) ЗУ 51:11:0030401:466 (ФКУ Упрдор «Кола», Дог.: № СПБ80-0371042/20 от 03.07.2020 года)» ИП №002-42-2-01.32-0893. для нужд Мурманского филиала ПАО "Россети Северо-Запад".</t>
+        </is>
+      </c>
+      <c r="G232" s="2" t="inlineStr">
+        <is>
+          <t>ПУБЛИЧНОЕ АКЦИОНЕРНОЕ ОБЩЕСТВО "РОССЕТИ СЕВЕРО-ЗАПАД"</t>
+        </is>
+      </c>
+      <c r="H232" s="2" t="inlineStr">
+        <is>
+          <t>ПАО "РОССЕТИ СЕВЕРО-ЗАПАД"</t>
+        </is>
+      </c>
+      <c r="I232" s="2" t="inlineStr">
+        <is>
+          <t>7802312751</t>
+        </is>
+      </c>
+      <c r="J232" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="K232" s="2" t="inlineStr">
+        <is>
+          <t>Торсунов Вячеслав Юрьевич</t>
+        </is>
+      </c>
+      <c r="L232" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M232" s="2" t="inlineStr">
+        <is>
+          <t>35.12.1</t>
+        </is>
+      </c>
+      <c r="N232" s="2" t="inlineStr">
+        <is>
+          <t>3 007 300,00 ₽</t>
+        </is>
+      </c>
+      <c r="O232" s="2" t="inlineStr">
+        <is>
+          <t>27.07.2026 | 27.07.2026 | 06.08.2026</t>
+        </is>
+      </c>
+      <c r="P232" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург, пл Конституции, д 3 литера а, помещ 16Н</t>
+        </is>
+      </c>
+      <c r="Q232" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/223/purchase/public/purchase/info/common-info.html?regNumber=32616237996</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27 10:13</t>
+        </is>
+      </c>
+      <c r="B233" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C233" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D233" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E233" s="2" t="inlineStr">
+        <is>
+          <t>32616238252</t>
+        </is>
+      </c>
+      <c r="F233" s="2" t="inlineStr">
+        <is>
+          <t>Поставкажелезобетонныхизделий для строительства трубопровода водоснабжения по ул. Проезжая</t>
+        </is>
+      </c>
+      <c r="G233" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПРОИЗВОДСТВЕННОЕ УПРАВЛЕНИЕ ВОДОСНАБЖЕНИЯ И ВОДООТВЕДЕНИЯ ГОРОДА ЧИТЫ"</t>
+        </is>
+      </c>
+      <c r="H233" s="2" t="inlineStr">
+        <is>
+          <t>АО "ВОДОКАНАЛ-ЧИТА"</t>
+        </is>
+      </c>
+      <c r="I233" s="2" t="inlineStr">
+        <is>
+          <t>7536064538</t>
+        </is>
+      </c>
+      <c r="J233" s="2" t="inlineStr">
+        <is>
+          <t>Забайкальский край</t>
+        </is>
+      </c>
+      <c r="K233" s="2" t="inlineStr">
+        <is>
+          <t>Филиппова Наталья Николаевна</t>
+        </is>
+      </c>
+      <c r="L233" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M233" s="2" t="inlineStr">
+        <is>
+          <t>36.00.1</t>
+        </is>
+      </c>
+      <c r="N233" s="2" t="inlineStr">
+        <is>
+          <t>140 627,30 ₽</t>
+        </is>
+      </c>
+      <c r="O233" s="2" t="inlineStr">
+        <is>
+          <t>27.07.2026 | 27.07.2026 | 04.08.2026</t>
+        </is>
+      </c>
+      <c r="P233" s="2" t="inlineStr">
+        <is>
+          <t>г Чита, ул Забайкальского Рабочего, д 63</t>
+        </is>
+      </c>
+      <c r="Q233" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/223/purchase/public/purchase/info/common-info.html?regNumber=32616238252</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27 10:13</t>
+        </is>
+      </c>
+      <c r="B234" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C234" s="2" t="inlineStr"/>
+      <c r="D234" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E234" s="2" t="inlineStr">
+        <is>
+          <t>4538849</t>
+        </is>
+      </c>
+      <c r="F234" s="2" t="inlineStr">
+        <is>
+          <t>Ж/б сваи Чер25А (железобетон) Бетон В30 W6 F1504538849 ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "АРТСТРОЙТЕХНОЛОГИЯ"Железобетонные изделия</t>
+        </is>
+      </c>
+      <c r="G234" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="H234" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="I234" s="2" t="inlineStr">
+        <is>
+          <t>7724498866</t>
+        </is>
+      </c>
+      <c r="J234" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K234" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
+      <c r="L234" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M234" s="2" t="inlineStr">
+        <is>
+          <t>46.73</t>
+        </is>
+      </c>
+      <c r="N234" s="2" t="inlineStr"/>
+      <c r="O234" s="2" t="inlineStr">
+        <is>
+          <t>27.07.2026 12:11 — 28.07.2026 13:06</t>
+        </is>
+      </c>
+      <c r="P234" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+        </is>
+      </c>
+      <c r="Q234" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zh-b-svai-cher25a-zhelezobeton-beton-v30-w6-f150/tender-4538849/#btid=2&amp;sqh=739e9e585fc26ce3294471c47fde58a154f1e1fd&amp;tsid=4538849459</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q231"/>
+  <autoFilter ref="A1:Q234"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -19696,6 +19945,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q229" r:id="rId228"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q230" r:id="rId229"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q231" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q232" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q233" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q234" r:id="rId233"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-27 15:01 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$234</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$238</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q234"/>
+  <dimension ref="A1:Q238"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -19712,8 +19712,321 @@
         </is>
       </c>
     </row>
+    <row r="235">
+      <c r="A235" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27 15:01</t>
+        </is>
+      </c>
+      <c r="B235" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C235" s="2" t="inlineStr"/>
+      <c r="D235" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E235" s="2" t="inlineStr">
+        <is>
+          <t>4539463</t>
+        </is>
+      </c>
+      <c r="F235" s="2" t="inlineStr">
+        <is>
+          <t>ЛЗК № 213 ЩОС
+ЖБИ изделия и комплектующие... -10 - 2 шт Рабочая камераколодцаК-15-10 - 1 шт ...  Рабочая камераколодцаК-15-5 - 1 шт ...  Рабочая камераколодцаК-10-10 - 4 штКольцогорловины К-7 ...</t>
+        </is>
+      </c>
+      <c r="G235" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="H235" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="I235" s="2" t="inlineStr">
+        <is>
+          <t>7724498866</t>
+        </is>
+      </c>
+      <c r="J235" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K235" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
+      <c r="L235" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M235" s="2" t="inlineStr">
+        <is>
+          <t>46.73</t>
+        </is>
+      </c>
+      <c r="N235" s="2" t="inlineStr"/>
+      <c r="O235" s="2" t="inlineStr">
+        <is>
+          <t>27.07.2026 16:04 — 29.07.2026 15:00</t>
+        </is>
+      </c>
+      <c r="P235" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+        </is>
+      </c>
+      <c r="Q235" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/lzk-213-shchos-zhbi-izdeliia-i-komplektuiushchie/tender-4539463/#btid=2&amp;sqh=7bf998fec6adb71382bc5cb2b72884a19f02a9d8&amp;tsid=4539463459</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27 15:01</t>
+        </is>
+      </c>
+      <c r="B236" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C236" s="2" t="inlineStr"/>
+      <c r="D236" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E236" s="2" t="inlineStr">
+        <is>
+          <t>4539139</t>
+        </is>
+      </c>
+      <c r="F236" s="2" t="inlineStr">
+        <is>
+          <t>ЗакупкаЖБИ</t>
+        </is>
+      </c>
+      <c r="G236" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H236" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I236" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J236" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K236" s="2" t="inlineStr"/>
+      <c r="L236" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M236" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N236" s="2" t="inlineStr"/>
+      <c r="O236" s="2" t="inlineStr">
+        <is>
+          <t>27.07.2026 14:08 — 28.07.2026 14:00</t>
+        </is>
+      </c>
+      <c r="P236" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ. ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q236" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi/tender-4539139/#btid=2&amp;sqh=bbe8186f49bfeaf81c187e3e15d53aabc275dd28&amp;tsid=4539139458</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27 15:01</t>
+        </is>
+      </c>
+      <c r="B237" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C237" s="2" t="inlineStr"/>
+      <c r="D237" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E237" s="2" t="inlineStr">
+        <is>
+          <t>4539603</t>
+        </is>
+      </c>
+      <c r="F237" s="2" t="inlineStr">
+        <is>
+          <t>ЛЗК 218 ЩОСЖБИ</t>
+        </is>
+      </c>
+      <c r="G237" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="H237" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="I237" s="2" t="inlineStr">
+        <is>
+          <t>7724498866</t>
+        </is>
+      </c>
+      <c r="J237" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K237" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
+      <c r="L237" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M237" s="2" t="inlineStr">
+        <is>
+          <t>46.73</t>
+        </is>
+      </c>
+      <c r="N237" s="2" t="inlineStr"/>
+      <c r="O237" s="2" t="inlineStr">
+        <is>
+          <t>27.07.2026 17:13 — 30.07.2026 15:00</t>
+        </is>
+      </c>
+      <c r="P237" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+        </is>
+      </c>
+      <c r="Q237" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/lzk-218-shchos-zhbi/tender-4539603/#btid=2&amp;sqh=bbe8186f49bfeaf81c187e3e15d53aabc275dd28&amp;tsid=4539603459</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27 15:01</t>
+        </is>
+      </c>
+      <c r="B238" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C238" s="2" t="inlineStr"/>
+      <c r="D238" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E238" s="2" t="inlineStr">
+        <is>
+          <t>4539029</t>
+        </is>
+      </c>
+      <c r="F238" s="2" t="inlineStr">
+        <is>
+          <t>Поставка ТМЦ (Фундамент под весы) для АО Разрез Колыванский... Добавка сухая гидрофобизирующая для бетонных ижелезобетонныхконструкций, повышение водонепроницаемости до W14 ... однокомпонентный полиуретановый карбонизированный антикоррозионный для металлическихизделийи конструкций, гидрофобный, температура эксплуатации ...</t>
+        </is>
+      </c>
+      <c r="G238" s="2" t="inlineStr">
+        <is>
+          <t>ООО "УК "СИБАНТРАЦИТ"</t>
+        </is>
+      </c>
+      <c r="H238" s="2" t="inlineStr">
+        <is>
+          <t>ООО "УК "СИБАНТРАЦИТ"</t>
+        </is>
+      </c>
+      <c r="I238" s="2" t="inlineStr">
+        <is>
+          <t>9703160290</t>
+        </is>
+      </c>
+      <c r="J238" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K238" s="2" t="inlineStr">
+        <is>
+          <t>Мельников Сергей Владимирович</t>
+        </is>
+      </c>
+      <c r="L238" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M238" s="2" t="inlineStr">
+        <is>
+          <t>70.22</t>
+        </is>
+      </c>
+      <c r="N238" s="2" t="inlineStr"/>
+      <c r="O238" s="2" t="inlineStr">
+        <is>
+          <t>27.07.2026 13:33 — 30.07.2026 10:00</t>
+        </is>
+      </c>
+      <c r="P238" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Усачёва, д 2 стр 1, помещ 2/1</t>
+        </is>
+      </c>
+      <c r="Q238" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/postavka-tmts-fundament-pod-vesy-dlia-ao-razrez-kolyvanskii/tender-4539029/#btid=2&amp;sqh=7904acabc543cfe7b7a3e9098340203df183d787&amp;tsid=4539029458</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q234"/>
+  <autoFilter ref="A1:Q238"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -19948,6 +20261,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q232" r:id="rId231"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q233" r:id="rId232"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q234" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q235" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q236" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q237" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q238" r:id="rId237"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-28 03:31 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$238</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$239</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q238"/>
+  <dimension ref="A1:Q239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -20025,8 +20025,83 @@
         </is>
       </c>
     </row>
+    <row r="239">
+      <c r="A239" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28 03:31</t>
+        </is>
+      </c>
+      <c r="B239" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C239" s="2" t="inlineStr"/>
+      <c r="D239" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E239" s="2" t="inlineStr">
+        <is>
+          <t>4539836</t>
+        </is>
+      </c>
+      <c r="F239" s="2" t="inlineStr">
+        <is>
+          <t>ТМЦЖБИСрочная поставка для нужд филиала "Канская теплосеть"</t>
+        </is>
+      </c>
+      <c r="G239" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H239" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I239" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J239" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K239" s="2" t="inlineStr"/>
+      <c r="L239" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M239" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N239" s="2" t="inlineStr"/>
+      <c r="O239" s="2" t="inlineStr">
+        <is>
+          <t>28.07.2026 06:13 — 30.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P239" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ. ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q239" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/tmts-zhbi-srochnaia-postavka-dlia-nuzhd-filiala-kanskaia-teploset/tender-4539836/#btid=2&amp;sqh=bdb3ebcacd3f34ae6232263adc82b2d0fb918c68&amp;tsid=4539836458</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q238"/>
+  <autoFilter ref="A1:Q239"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -20265,6 +20340,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q236" r:id="rId235"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q237" r:id="rId236"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q238" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q239" r:id="rId238"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-28 14:37 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$239</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$247</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q239"/>
+  <dimension ref="A1:Q247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -20100,8 +20100,661 @@
         </is>
       </c>
     </row>
+    <row r="240">
+      <c r="A240" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28 14:37</t>
+        </is>
+      </c>
+      <c r="B240" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C240" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D240" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E240" s="2" t="inlineStr">
+        <is>
+          <t>32616243300</t>
+        </is>
+      </c>
+      <c r="F240" s="2" t="inlineStr">
+        <is>
+          <t>Выполнение ПИР, СМР, ПНР полным иждивением Подрядчика по титулу: Реконструкция ТП-6/0,4 кВ №2158 с заменой тр-ра 160 кВА на тр-р 250 кВА, строительствоЛЭП-0,4 кВ (по сущ.опорам) от РУ-0,4 кВ ТП-2158, ПС №23 "Кварц", АВ, в т.ч. ПИР, МО, Раменский р-н, с/п Чулковское Ю8-26-303-304286(284932) для нужд филиала ПАО «Россети Московский регион» - Южные электрические сети</t>
+        </is>
+      </c>
+      <c r="G240" s="2" t="inlineStr">
+        <is>
+          <t>ПУБЛИЧНОЕ АКЦИОНЕРНОЕ ОБЩЕСТВО "РОССЕТИ МОСКОВСКИЙ РЕГИОН"</t>
+        </is>
+      </c>
+      <c r="H240" s="2" t="inlineStr">
+        <is>
+          <t>ПАО "РОССЕТИ МОСКОВСКИЙ РЕГИОН", ПАО "РОССЕТИ МР"</t>
+        </is>
+      </c>
+      <c r="I240" s="2" t="inlineStr">
+        <is>
+          <t>5036065113</t>
+        </is>
+      </c>
+      <c r="J240" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K240" s="2" t="inlineStr">
+        <is>
+          <t>Пятигор Александр Михайлович</t>
+        </is>
+      </c>
+      <c r="L240" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M240" s="2" t="inlineStr">
+        <is>
+          <t>35.12.1</t>
+        </is>
+      </c>
+      <c r="N240" s="2" t="inlineStr">
+        <is>
+          <t>803 743,26 ₽</t>
+        </is>
+      </c>
+      <c r="O240" s="2" t="inlineStr">
+        <is>
+          <t>28.07.2026 | 28.07.2026 | 31.07.2026</t>
+        </is>
+      </c>
+      <c r="P240" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, 2-й Павелецкий проезд, д 3 стр 2</t>
+        </is>
+      </c>
+      <c r="Q240" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/223/purchase/public/purchase/info/common-info.html?regNumber=32616243300</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28 14:37</t>
+        </is>
+      </c>
+      <c r="B241" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C241" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D241" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E241" s="2" t="inlineStr">
+        <is>
+          <t>32616243290</t>
+        </is>
+      </c>
+      <c r="F241" s="2" t="inlineStr">
+        <is>
+          <t>Выполнение СМР, ПНР полным иждивением Подрядчика по титулу: Реконструкция ТП-10/0,4 кВ №1727 с заменой тр-ра 160 кВА на тр-р 250 кВ и установкой АВ в РУ-0,4 кВ, строительствоЛЭП-0,4 кВ (по сущ.опорам) от РУ-0,4 кВ ТП-1727, ПС №478 "Талеж", в т.ч. ПИР, МО, г.о.Чехов, с. Новый Быт, территория общественно-деловая зона Новобытовская, стр 5 Ю8-25-303-278401(532230) для нужд филиала ПАО «Россети Московский регион» - Южные электрические сети</t>
+        </is>
+      </c>
+      <c r="G241" s="2" t="inlineStr">
+        <is>
+          <t>ПУБЛИЧНОЕ АКЦИОНЕРНОЕ ОБЩЕСТВО "РОССЕТИ МОСКОВСКИЙ РЕГИОН"</t>
+        </is>
+      </c>
+      <c r="H241" s="2" t="inlineStr">
+        <is>
+          <t>ПАО "РОССЕТИ МОСКОВСКИЙ РЕГИОН", ПАО "РОССЕТИ МР"</t>
+        </is>
+      </c>
+      <c r="I241" s="2" t="inlineStr">
+        <is>
+          <t>5036065113</t>
+        </is>
+      </c>
+      <c r="J241" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K241" s="2" t="inlineStr">
+        <is>
+          <t>Пятигор Александр Михайлович</t>
+        </is>
+      </c>
+      <c r="L241" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M241" s="2" t="inlineStr">
+        <is>
+          <t>35.12.1</t>
+        </is>
+      </c>
+      <c r="N241" s="2" t="inlineStr">
+        <is>
+          <t>1 541 671,84 ₽</t>
+        </is>
+      </c>
+      <c r="O241" s="2" t="inlineStr">
+        <is>
+          <t>28.07.2026 | 28.07.2026 | 31.07.2026</t>
+        </is>
+      </c>
+      <c r="P241" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, 2-й Павелецкий проезд, д 3 стр 2</t>
+        </is>
+      </c>
+      <c r="Q241" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/223/purchase/public/purchase/info/common-info.html?regNumber=32616243290</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28 14:37</t>
+        </is>
+      </c>
+      <c r="B242" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C242" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D242" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E242" s="2" t="inlineStr">
+        <is>
+          <t>32616242830</t>
+        </is>
+      </c>
+      <c r="F242" s="2" t="inlineStr">
+        <is>
+          <t>Выполнение СМР, ПНР полным иждивением Подрядчика по титулу: Реконструкция ТП-250-6/0,4 кВ №207 с заменой на КТП-400-6/0,4 кВ, строительствоЛЭП-0,4 (по сущ.опорам) кВ от РУ-0,4 кВ ТП-207, ПС №382 "Венюково", в т.ч. ПИР, МО, городской округ Чехов, деревня Скурыгино, улица Парковая, строение 3/1 Ю8-24-303-238178(633596) для нужд филиала ПАО «Россети Московский регион» - Южные электрические сети</t>
+        </is>
+      </c>
+      <c r="G242" s="2" t="inlineStr">
+        <is>
+          <t>ПУБЛИЧНОЕ АКЦИОНЕРНОЕ ОБЩЕСТВО "РОССЕТИ МОСКОВСКИЙ РЕГИОН"</t>
+        </is>
+      </c>
+      <c r="H242" s="2" t="inlineStr">
+        <is>
+          <t>ПАО "РОССЕТИ МОСКОВСКИЙ РЕГИОН", ПАО "РОССЕТИ МР"</t>
+        </is>
+      </c>
+      <c r="I242" s="2" t="inlineStr">
+        <is>
+          <t>5036065113</t>
+        </is>
+      </c>
+      <c r="J242" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K242" s="2" t="inlineStr">
+        <is>
+          <t>Пятигор Александр Михайлович</t>
+        </is>
+      </c>
+      <c r="L242" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M242" s="2" t="inlineStr">
+        <is>
+          <t>35.12.1</t>
+        </is>
+      </c>
+      <c r="N242" s="2" t="inlineStr">
+        <is>
+          <t>3 692 132,01 ₽</t>
+        </is>
+      </c>
+      <c r="O242" s="2" t="inlineStr">
+        <is>
+          <t>28.07.2026 | 28.07.2026 | 31.07.2026</t>
+        </is>
+      </c>
+      <c r="P242" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, 2-й Павелецкий проезд, д 3 стр 2</t>
+        </is>
+      </c>
+      <c r="Q242" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/223/purchase/public/purchase/info/common-info.html?regNumber=32616242830</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28 14:37</t>
+        </is>
+      </c>
+      <c r="B243" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D243" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E243" s="2" t="inlineStr">
+        <is>
+          <t>32616244300</t>
+        </is>
+      </c>
+      <c r="F243" s="2" t="inlineStr">
+        <is>
+          <t>Аукцион в электронной форме, участниками которого могут быть только субъекты малого и среднего предпринимательства на право заключения договора на поставку общестроительныхжелезобетонныхизделий для нужд АО "МосводоканалСтройТрест" в 2026 году</t>
+        </is>
+      </c>
+      <c r="G243" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "МОСВОДОКАНАЛСТРОЙТРЕСТ"</t>
+        </is>
+      </c>
+      <c r="H243" s="2" t="inlineStr">
+        <is>
+          <t>АО "МОСВОДОКАНАЛСТРОЙТРЕСТ"</t>
+        </is>
+      </c>
+      <c r="I243" s="2" t="inlineStr">
+        <is>
+          <t>7701867771</t>
+        </is>
+      </c>
+      <c r="J243" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K243" s="2" t="inlineStr">
+        <is>
+          <t>Авакян Григорий Григорьевич</t>
+        </is>
+      </c>
+      <c r="L243" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M243" s="2" t="inlineStr">
+        <is>
+          <t>43.99.9</t>
+        </is>
+      </c>
+      <c r="N243" s="2" t="inlineStr">
+        <is>
+          <t>47 000 000,00 ₽</t>
+        </is>
+      </c>
+      <c r="O243" s="2" t="inlineStr">
+        <is>
+          <t>28.07.2026 | 28.07.2026 | 13.08.2026</t>
+        </is>
+      </c>
+      <c r="P243" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Плетешковский пер, д 22</t>
+        </is>
+      </c>
+      <c r="Q243" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/223/purchase/public/purchase/info/common-info.html?regNumber=32616244300</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28 14:37</t>
+        </is>
+      </c>
+      <c r="B244" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C244" s="2" t="inlineStr"/>
+      <c r="D244" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E244" s="2" t="inlineStr">
+        <is>
+          <t>4540849</t>
+        </is>
+      </c>
+      <c r="F244" s="2" t="inlineStr">
+        <is>
+          <t>Свая забивнаяС80.30-13.1у серия 1.011.1-10 выпуск 1 Для СЗРКСвая забивнаяС80.30-13.1у серия 1.011.1-10 выпуск 1</t>
+        </is>
+      </c>
+      <c r="G244" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+        </is>
+      </c>
+      <c r="H244" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+        </is>
+      </c>
+      <c r="I244" s="2" t="inlineStr">
+        <is>
+          <t>7805368914</t>
+        </is>
+      </c>
+      <c r="J244" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="K244" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
+        </is>
+      </c>
+      <c r="L244" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M244" s="2" t="inlineStr">
+        <is>
+          <t>46.90</t>
+        </is>
+      </c>
+      <c r="N244" s="2" t="inlineStr"/>
+      <c r="O244" s="2" t="inlineStr">
+        <is>
+          <t>28.07.2026 13:15 — 30.07.2026 14:00</t>
+        </is>
+      </c>
+      <c r="P244" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1Н офис 1089</t>
+        </is>
+      </c>
+      <c r="Q244" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/svaia-zabivnaia-s80-30-13-1u-seriia-1-011-1-10-vypusk-1-dlia-szrk/tender-4540849/#btid=2&amp;sqh=38c1765cf9779a06c0bf1ead64bdcd7f0ef55da3&amp;tsid=4540849004</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28 14:37</t>
+        </is>
+      </c>
+      <c r="B245" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C245" s="2" t="inlineStr"/>
+      <c r="D245" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E245" s="2" t="inlineStr">
+        <is>
+          <t>4541374</t>
+        </is>
+      </c>
+      <c r="F245" s="2" t="inlineStr">
+        <is>
+          <t>Услуги по переработке ломажелезобетонных изделийдля получения вторичного щебня</t>
+        </is>
+      </c>
+      <c r="G245" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H245" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I245" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J245" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K245" s="2" t="inlineStr"/>
+      <c r="L245" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M245" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N245" s="2" t="inlineStr"/>
+      <c r="O245" s="2" t="inlineStr">
+        <is>
+          <t>28.07.2026 16:10 — 05.08.2026 16:00</t>
+        </is>
+      </c>
+      <c r="P245" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ. ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q245" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/uslugi-po-pererabotke-loma-zhelezobetonnykh-izdelii-dlia-polucheniia/tender-4541374/#btid=2&amp;sqh=7e4be0292755f4be32a501289d0a45069ed1762c&amp;tsid=4541374458</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28 14:37</t>
+        </is>
+      </c>
+      <c r="B246" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C246" s="2" t="inlineStr"/>
+      <c r="D246" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E246" s="2" t="inlineStr">
+        <is>
+          <t>4536594</t>
+        </is>
+      </c>
+      <c r="F246" s="2" t="inlineStr">
+        <is>
+          <t>Выполнение комплекса общестроительных работ при строительстве здания свободного назначения по адресу: г. Москва, ул.5-я Магистральная, вл.4
+Выполнение комплекса общестроительных работ при строительстве здания свободного назначения по адресу: г. Москва, ул.5-я Магистральная, вл.4... . Без материала . Устройство кирпичных стен безперемычек, с заделкой мест примыкания к плитам ...</t>
+        </is>
+      </c>
+      <c r="G246" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ГК ФСК"</t>
+        </is>
+      </c>
+      <c r="H246" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ГК ФСК"</t>
+        </is>
+      </c>
+      <c r="I246" s="2" t="inlineStr">
+        <is>
+          <t>7708332091</t>
+        </is>
+      </c>
+      <c r="J246" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K246" s="2" t="inlineStr">
+        <is>
+          <t>Трубников Дмитрий Александрович</t>
+        </is>
+      </c>
+      <c r="L246" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M246" s="2" t="inlineStr">
+        <is>
+          <t>64.99</t>
+        </is>
+      </c>
+      <c r="N246" s="2" t="inlineStr"/>
+      <c r="O246" s="2" t="inlineStr">
+        <is>
+          <t>28.07.2026 12:47 — 11.08.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P246" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Каланчевская, д 32, помещ 4/2П</t>
+        </is>
+      </c>
+      <c r="Q246" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/vypolnenie-kompleksa-obshchestroitelnykh-rabot-pri-stroitelstve-zdaniia/tender-4536594/#btid=2&amp;sqh=61d62a1cd903dc7557299fa937bfdeb7b63d5115&amp;tsid=4536594004</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28 14:37</t>
+        </is>
+      </c>
+      <c r="B247" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C247" s="2" t="inlineStr"/>
+      <c r="D247" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E247" s="2" t="inlineStr">
+        <is>
+          <t>4505847</t>
+        </is>
+      </c>
+      <c r="F247" s="2" t="inlineStr">
+        <is>
+          <t>Техническое обслуживание, ремонт холодильных систем ивентиляционногооборудования на заводе</t>
+        </is>
+      </c>
+      <c r="G247" s="2" t="inlineStr">
+        <is>
+          <t>ООО "Рекитт Бенкизер"</t>
+        </is>
+      </c>
+      <c r="H247" s="2" t="inlineStr">
+        <is>
+          <t>ООО "РЕКИТТ БЕНКИЗЕР"</t>
+        </is>
+      </c>
+      <c r="I247" s="2" t="inlineStr">
+        <is>
+          <t>7705495411</t>
+        </is>
+      </c>
+      <c r="J247" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K247" s="2" t="inlineStr">
+        <is>
+          <t>Захряпа Екатерина Владимировна</t>
+        </is>
+      </c>
+      <c r="L247" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M247" s="2" t="inlineStr">
+        <is>
+          <t>20.41.3</t>
+        </is>
+      </c>
+      <c r="N247" s="2" t="inlineStr"/>
+      <c r="O247" s="2" t="inlineStr">
+        <is>
+          <t>29.06.2026 13:28 — 29.07.2026 13:00</t>
+        </is>
+      </c>
+      <c r="P247" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Шлюзовая наб, д 4</t>
+        </is>
+      </c>
+      <c r="Q247" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/tekhnicheskoe-obsluzhivanie-remont-kholodilnykh-sistem-i-ventiliatsionnogo/tender-4505847/#btid=2&amp;sqh=5c1940fb4c06d01512dc87c102b0960c1f29924b&amp;tsid=4505847458</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q239"/>
+  <autoFilter ref="A1:Q247"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -20341,6 +20994,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q237" r:id="rId236"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q238" r:id="rId237"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q239" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q240" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q241" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q242" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q243" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q244" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q245" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q246" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q247" r:id="rId246"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-29 09:04 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$247</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$250</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q247"/>
+  <dimension ref="A1:Q250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -20753,8 +20753,241 @@
         </is>
       </c>
     </row>
+    <row r="248">
+      <c r="A248" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 09:04</t>
+        </is>
+      </c>
+      <c r="B248" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C248" s="2" t="inlineStr"/>
+      <c r="D248" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E248" s="2" t="inlineStr">
+        <is>
+          <t>4541823</t>
+        </is>
+      </c>
+      <c r="F248" s="2" t="inlineStr">
+        <is>
+          <t>Устройство площадки с укладкойплит ПАГУстройство площадки с укладкойплит ПАГ</t>
+        </is>
+      </c>
+      <c r="G248" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+        </is>
+      </c>
+      <c r="H248" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ТД ПОЛИМЕТАЛЛ"</t>
+        </is>
+      </c>
+      <c r="I248" s="2" t="inlineStr">
+        <is>
+          <t>7805368914</t>
+        </is>
+      </c>
+      <c r="J248" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="K248" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "ПОЛИМЕТАЛЛ УПРАВЛЯЮЩАЯ КОМПАНИЯ"</t>
+        </is>
+      </c>
+      <c r="L248" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M248" s="2" t="inlineStr">
+        <is>
+          <t>46.69.2</t>
+        </is>
+      </c>
+      <c r="N248" s="2" t="inlineStr"/>
+      <c r="O248" s="2" t="inlineStr">
+        <is>
+          <t>29.07.2026 07:57 — 05.08.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P248" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург, пр-кт Народного Ополчения, д 2 литера а, помещ 1-Н офис 1089</t>
+        </is>
+      </c>
+      <c r="Q248" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/ustroistvo-ploshchadki-s-ukladkoi-plit-pag/tender-4541823/#btid=2&amp;sqh=3dbbc0abe356f404e72e801ba760787a3f4f6d04&amp;tsid=4541823004</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 09:04</t>
+        </is>
+      </c>
+      <c r="B249" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C249" s="2" t="inlineStr"/>
+      <c r="D249" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E249" s="2" t="inlineStr">
+        <is>
+          <t>4542319</t>
+        </is>
+      </c>
+      <c r="F249" s="2" t="inlineStr">
+        <is>
+          <t>Комплекс услуг по благоустройствуУслуги по благоустройствуЖБИ</t>
+        </is>
+      </c>
+      <c r="G249" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СВЕЗА-ЛЕС"</t>
+        </is>
+      </c>
+      <c r="H249" s="2" t="inlineStr">
+        <is>
+          <t>ООО "СВЕЗА-ЛЕС"</t>
+        </is>
+      </c>
+      <c r="I249" s="2" t="inlineStr">
+        <is>
+          <t>7706207296</t>
+        </is>
+      </c>
+      <c r="J249" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="K249" s="2" t="inlineStr">
+        <is>
+          <t>Колчин Дмитрий Владимирович</t>
+        </is>
+      </c>
+      <c r="L249" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M249" s="2" t="inlineStr">
+        <is>
+          <t>70.10</t>
+        </is>
+      </c>
+      <c r="N249" s="2" t="inlineStr"/>
+      <c r="O249" s="2" t="inlineStr">
+        <is>
+          <t>29.07.2026 10:52 — 09.08.2026 00:00</t>
+        </is>
+      </c>
+      <c r="P249" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург, поселок Понтонный, ул Фанерная, д 5 литера а, офис 203</t>
+        </is>
+      </c>
+      <c r="Q249" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/kompleks-uslug-po-blagoustroistvu/tender-4542319/#btid=2&amp;sqh=09fa6c2cbe6305c5f783cac8eb926b11f878ed19&amp;tsid=4542319458</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 09:04</t>
+        </is>
+      </c>
+      <c r="B250" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C250" s="2" t="inlineStr"/>
+      <c r="D250" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E250" s="2" t="inlineStr">
+        <is>
+          <t>4542115</t>
+        </is>
+      </c>
+      <c r="F250" s="2" t="inlineStr">
+        <is>
+          <t>ЗакупкаЖБИ</t>
+        </is>
+      </c>
+      <c r="G250" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H250" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I250" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J250" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K250" s="2" t="inlineStr"/>
+      <c r="L250" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M250" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N250" s="2" t="inlineStr"/>
+      <c r="O250" s="2" t="inlineStr">
+        <is>
+          <t>29.07.2026 09:49 — 31.07.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P250" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ. ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q250" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi/tender-4542115/#btid=2&amp;sqh=09fa6c2cbe6305c5f783cac8eb926b11f878ed19&amp;tsid=4542115458</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q247"/>
+  <autoFilter ref="A1:Q250"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -21002,6 +21235,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q245" r:id="rId244"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q246" r:id="rId245"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q247" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q248" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q249" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q250" r:id="rId249"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-29 14:36 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$250</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$254</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q250"/>
+  <dimension ref="A1:Q254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -20986,8 +20986,331 @@
         </is>
       </c>
     </row>
+    <row r="251">
+      <c r="A251" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 14:36</t>
+        </is>
+      </c>
+      <c r="B251" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C251" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D251" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E251" s="2" t="inlineStr">
+        <is>
+          <t>32616247049</t>
+        </is>
+      </c>
+      <c r="F251" s="2" t="inlineStr">
+        <is>
+          <t>Право заключения договора на поставкудорожныхплитна ВТРК «Ведучи»</t>
+        </is>
+      </c>
+      <c r="G251" s="2" t="inlineStr">
+        <is>
+          <t>АКЦИОНЕРНОЕ ОБЩЕСТВО "КАВКАЗ.РФ"</t>
+        </is>
+      </c>
+      <c r="H251" s="2" t="inlineStr">
+        <is>
+          <t>АО "КАВКАЗ.РФ"</t>
+        </is>
+      </c>
+      <c r="I251" s="2" t="inlineStr">
+        <is>
+          <t>2632100740</t>
+        </is>
+      </c>
+      <c r="J251" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K251" s="2" t="inlineStr">
+        <is>
+          <t>Юмшанов Андрей Александрович</t>
+        </is>
+      </c>
+      <c r="L251" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M251" s="2" t="inlineStr">
+        <is>
+          <t>49.39.2</t>
+        </is>
+      </c>
+      <c r="N251" s="2" t="inlineStr">
+        <is>
+          <t>3 424 477,10 ₽</t>
+        </is>
+      </c>
+      <c r="O251" s="2" t="inlineStr">
+        <is>
+          <t>29.07.2026 | 29.07.2026 | 06.08.2026</t>
+        </is>
+      </c>
+      <c r="P251" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Тестовская, д 10, помещ I</t>
+        </is>
+      </c>
+      <c r="Q251" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/223/purchase/public/purchase/info/common-info.html?regNumber=32616247049</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 14:36</t>
+        </is>
+      </c>
+      <c r="B252" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C252" s="2" t="inlineStr"/>
+      <c r="D252" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E252" s="2" t="inlineStr">
+        <is>
+          <t>4539524</t>
+        </is>
+      </c>
+      <c r="F252" s="2" t="inlineStr">
+        <is>
+          <t>13-Х-1. Заключение договора на поставкудорожных плитна объект: «Дальневосточный детский центр отдыха и оздоровления в Хабаровском крае» (1 лот)</t>
+        </is>
+      </c>
+      <c r="G252" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ПРОМСТРОЙ"</t>
+        </is>
+      </c>
+      <c r="H252" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ПРОМСТРОЙ"</t>
+        </is>
+      </c>
+      <c r="I252" s="2" t="inlineStr">
+        <is>
+          <t>9723169975</t>
+        </is>
+      </c>
+      <c r="J252" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K252" s="2" t="inlineStr">
+        <is>
+          <t>Султанов Владислав Назипович</t>
+        </is>
+      </c>
+      <c r="L252" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M252" s="2" t="inlineStr">
+        <is>
+          <t>71.12.2</t>
+        </is>
+      </c>
+      <c r="N252" s="2" t="inlineStr"/>
+      <c r="O252" s="2" t="inlineStr">
+        <is>
+          <t>29.07.2026 14:57 — 05.08.2026 11:00</t>
+        </is>
+      </c>
+      <c r="P252" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Волгоградский пр-кт, д 42 к 5, ком 9</t>
+        </is>
+      </c>
+      <c r="Q252" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/13-kh-1-zakliuchenie-dogovora-na-postavku-dorozhnykh-plit-na-ob-ekt/tender-4539524/#btid=2&amp;sqh=5bd48cf93a28eba58c8875c251bc232cdf46600a&amp;tsid=4539524004</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 14:36</t>
+        </is>
+      </c>
+      <c r="B253" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C253" s="2" t="inlineStr"/>
+      <c r="D253" s="2" t="inlineStr">
+        <is>
+          <t>Поставка</t>
+        </is>
+      </c>
+      <c r="E253" s="2" t="inlineStr">
+        <is>
+          <t>4539526</t>
+        </is>
+      </c>
+      <c r="F253" s="2" t="inlineStr">
+        <is>
+          <t>13-Х-2. Заключение договора на поставкудорожных плитна объект: «Дальневосточный детский центр отдыха и оздоровления в Хабаровском крае» (2 лот)</t>
+        </is>
+      </c>
+      <c r="G253" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ПРОМСТРОЙ"</t>
+        </is>
+      </c>
+      <c r="H253" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ПРОМСТРОЙ"</t>
+        </is>
+      </c>
+      <c r="I253" s="2" t="inlineStr">
+        <is>
+          <t>9723169975</t>
+        </is>
+      </c>
+      <c r="J253" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K253" s="2" t="inlineStr">
+        <is>
+          <t>Султанов Владислав Назипович</t>
+        </is>
+      </c>
+      <c r="L253" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M253" s="2" t="inlineStr">
+        <is>
+          <t>71.12.2</t>
+        </is>
+      </c>
+      <c r="N253" s="2" t="inlineStr"/>
+      <c r="O253" s="2" t="inlineStr">
+        <is>
+          <t>29.07.2026 14:57 — 05.08.2026 11:00</t>
+        </is>
+      </c>
+      <c r="P253" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Волгоградский пр-кт, д 42 к 5, ком 9</t>
+        </is>
+      </c>
+      <c r="Q253" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/13-kh-2-zakliuchenie-dogovora-na-postavku-dorozhnykh-plit-na-ob-ekt/tender-4539526/#btid=2&amp;sqh=5bd48cf93a28eba58c8875c251bc232cdf46600a&amp;tsid=4539526004</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 14:36</t>
+        </is>
+      </c>
+      <c r="B254" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C254" s="2" t="inlineStr"/>
+      <c r="D254" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E254" s="2" t="inlineStr">
+        <is>
+          <t>4542825</t>
+        </is>
+      </c>
+      <c r="F254" s="2" t="inlineStr">
+        <is>
+          <t>Шпала ЖБ Ш1 (в сборе с комплектом креплений КБ-65)
+Шпала ЖБ Ш1 (в сборе с комплектом креплений КБ-65)4542825 АКЦИОНЕРНОЕ ОБЩЕСТВО "ХОЛДИНГ ЭРСО"Железобетонные изделия</t>
+        </is>
+      </c>
+      <c r="G254" s="2" t="inlineStr">
+        <is>
+          <t>АО "ХОЛДИНГ ЭРСО"</t>
+        </is>
+      </c>
+      <c r="H254" s="2" t="inlineStr">
+        <is>
+          <t>АО "ХОЛДИНГ ЭРСО"</t>
+        </is>
+      </c>
+      <c r="I254" s="2" t="inlineStr">
+        <is>
+          <t>7718013390</t>
+        </is>
+      </c>
+      <c r="J254" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K254" s="2" t="inlineStr">
+        <is>
+          <t>Гурин Сергей Владимирович</t>
+        </is>
+      </c>
+      <c r="L254" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M254" s="2" t="inlineStr">
+        <is>
+          <t>27.11.13</t>
+        </is>
+      </c>
+      <c r="N254" s="2" t="inlineStr"/>
+      <c r="O254" s="2" t="inlineStr">
+        <is>
+          <t>29.07.2026 13:48 — 05.08.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P254" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Электрозаводская, д 21</t>
+        </is>
+      </c>
+      <c r="Q254" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/market/shpala-zhb-sh1-v-sbore-s-komplektom-kreplenii-kb-65/tender-4542825/#btid=2&amp;sqh=8c52196a5c00836a52117c003586012ec70ea2d7&amp;tsid=4542825004</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q250"/>
+  <autoFilter ref="A1:Q254"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -21238,6 +21561,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q248" r:id="rId247"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q249" r:id="rId248"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q250" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q251" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q252" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q253" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q254" r:id="rId253"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-30 08:50 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$254</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$255</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q254"/>
+  <dimension ref="A1:Q255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -21309,8 +21309,87 @@
         </is>
       </c>
     </row>
+    <row r="255">
+      <c r="A255" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30 08:50</t>
+        </is>
+      </c>
+      <c r="B255" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C255" s="2" t="inlineStr"/>
+      <c r="D255" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E255" s="2" t="inlineStr">
+        <is>
+          <t>4542654</t>
+        </is>
+      </c>
+      <c r="F255" s="2" t="inlineStr">
+        <is>
+          <t>Закупка свай для ИП "Реализация мер по защите подстанции от БПЛА"4542654 АКЦИОНЕРНОЕ ОБЩЕСТВО "ЦЕМРОС"Железобетонные изделия</t>
+        </is>
+      </c>
+      <c r="G255" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЦЕМРОС"</t>
+        </is>
+      </c>
+      <c r="H255" s="2" t="inlineStr">
+        <is>
+          <t>АО "ЦЕМРОС"</t>
+        </is>
+      </c>
+      <c r="I255" s="2" t="inlineStr">
+        <is>
+          <t>7708117908</t>
+        </is>
+      </c>
+      <c r="J255" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K255" s="2" t="inlineStr">
+        <is>
+          <t>Шматов Вячеслав Вячеславович</t>
+        </is>
+      </c>
+      <c r="L255" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M255" s="2" t="inlineStr">
+        <is>
+          <t>23.51</t>
+        </is>
+      </c>
+      <c r="N255" s="2" t="inlineStr"/>
+      <c r="O255" s="2" t="inlineStr">
+        <is>
+          <t>30.07.2026 08:54 — 10.08.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P255" s="2" t="inlineStr">
+        <is>
+          <t>121357, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ МОЖАЙСКИЙ, УЛ. ВЕРЕЙСКАЯ, Д. 29, СТР. 34, ЭТАЖ 5, ПОМЕЩ./КОМ. I/4</t>
+        </is>
+      </c>
+      <c r="Q255" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-svai-dlia-ip-realizatsiia-mer-po-zashchite-podstantsii-ot-bpla/tender-4542654/#btid=2&amp;sqh=3f00e500ba956a8e7b4c130521cd2ca5ab8ee1ac&amp;tsid=4542654458</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q254"/>
+  <autoFilter ref="A1:Q255"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -21565,6 +21644,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q252" r:id="rId251"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q253" r:id="rId252"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q254" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q255" r:id="rId254"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-30 14:31 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$255</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$259</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q255"/>
+  <dimension ref="A1:Q259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -21388,8 +21388,330 @@
         </is>
       </c>
     </row>
+    <row r="256">
+      <c r="A256" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30 14:31</t>
+        </is>
+      </c>
+      <c r="B256" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C256" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D256" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E256" s="2" t="inlineStr">
+        <is>
+          <t>32616253024</t>
+        </is>
+      </c>
+      <c r="F256" s="2" t="inlineStr">
+        <is>
+          <t>Организация и проведение общественных обсуждений по объекту «Реконструкция газопровода-отвода и ГРС №6 г. Краснодара». Этап 1. Реконструкция узла редуцирования газа на действующем газопроводе-перемычке «Россия-Турция» - ГРС ВНИИриса» для нужд ООО "Газпром проектирование" (для субъектов малого и среднего предпринимательства) (26/2.3/00082947/ГППроект)</t>
+        </is>
+      </c>
+      <c r="G256" s="2" t="inlineStr">
+        <is>
+          <t>ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "ГАЗПРОМ ПРОЕКТИРОВАНИЕ"</t>
+        </is>
+      </c>
+      <c r="H256" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ГАЗПРОМ ПРОЕКТИРОВАНИЕ"</t>
+        </is>
+      </c>
+      <c r="I256" s="2" t="inlineStr">
+        <is>
+          <t>0560022871</t>
+        </is>
+      </c>
+      <c r="J256" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="K256" s="2" t="inlineStr">
+        <is>
+          <t>Вагарин Владимир Анатольевич</t>
+        </is>
+      </c>
+      <c r="L256" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M256" s="2" t="inlineStr">
+        <is>
+          <t>71.12.12</t>
+        </is>
+      </c>
+      <c r="N256" s="2" t="inlineStr">
+        <is>
+          <t>1 453 853,00 ₽</t>
+        </is>
+      </c>
+      <c r="O256" s="2" t="inlineStr">
+        <is>
+          <t>30.07.2026 | 30.07.2026 | 11.08.2026</t>
+        </is>
+      </c>
+      <c r="P256" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург, Суворовский пр-кт, д 16/13 литера а, помещ 19Н</t>
+        </is>
+      </c>
+      <c r="Q256" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/223/purchase/public/purchase/info/common-info.html?regNumber=32616253024</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30 14:31</t>
+        </is>
+      </c>
+      <c r="B257" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C257" s="2" t="inlineStr"/>
+      <c r="D257" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E257" s="2" t="inlineStr">
+        <is>
+          <t>4544175</t>
+        </is>
+      </c>
+      <c r="F257" s="2" t="inlineStr">
+        <is>
+          <t>ДорожнаяЛЗК 288 (Заявка № 17840, 17853) ЖБИ</t>
+        </is>
+      </c>
+      <c r="G257" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="H257" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АРТСТРОЙТЕХНОЛОГИЯ"</t>
+        </is>
+      </c>
+      <c r="I257" s="2" t="inlineStr">
+        <is>
+          <t>7724498866</t>
+        </is>
+      </c>
+      <c r="J257" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K257" s="2" t="inlineStr">
+        <is>
+          <t>Городний Анатолий Валерьевич</t>
+        </is>
+      </c>
+      <c r="L257" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M257" s="2" t="inlineStr">
+        <is>
+          <t>46.73</t>
+        </is>
+      </c>
+      <c r="N257" s="2" t="inlineStr"/>
+      <c r="O257" s="2" t="inlineStr">
+        <is>
+          <t>30.07.2026 12:10 — 31.07.2026 17:00</t>
+        </is>
+      </c>
+      <c r="P257" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, Каширское шоссе, д 8 к 2, помещ 2П</t>
+        </is>
+      </c>
+      <c r="Q257" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/dorozhnaia-lzk-288-zaiavka-17840-17853-zhbi/tender-4544175/#btid=2&amp;sqh=9b6960e6981e51e4e067c152b692d15a2de3f05d&amp;tsid=4544175459</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30 14:31</t>
+        </is>
+      </c>
+      <c r="B258" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C258" s="2" t="inlineStr"/>
+      <c r="D258" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E258" s="2" t="inlineStr">
+        <is>
+          <t>4544461</t>
+        </is>
+      </c>
+      <c r="F258" s="2" t="inlineStr">
+        <is>
+          <t>Выбор генерального подрядчика на строительство детской академии в КП Папушево Парк...  временных дорог и площадок издорожных плит(с последующей разборкой) Срезка  ...  наплавляемой гидроизоляции под ж/бплитой(верхний слой) Устройство монолитной ...  опалубки колонн подвала Установка опалубкиплитыперекрытия (криволинейная геометрия) Установка ...</t>
+        </is>
+      </c>
+      <c r="G258" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ДСК ГРУПП"</t>
+        </is>
+      </c>
+      <c r="H258" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ДСК ГРУПП"</t>
+        </is>
+      </c>
+      <c r="I258" s="2" t="inlineStr">
+        <is>
+          <t>7727416195</t>
+        </is>
+      </c>
+      <c r="J258" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K258" s="2" t="inlineStr">
+        <is>
+          <t>Архипов Александр Альбертович</t>
+        </is>
+      </c>
+      <c r="L258" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M258" s="2" t="inlineStr">
+        <is>
+          <t>41.20</t>
+        </is>
+      </c>
+      <c r="N258" s="2" t="inlineStr"/>
+      <c r="O258" s="2" t="inlineStr">
+        <is>
+          <t>30.07.2026 16:32 — 07.08.2026 14:00</t>
+        </is>
+      </c>
+      <c r="P258" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Шверника, д 4 стр 2, помещ I, ком 6</t>
+        </is>
+      </c>
+      <c r="Q258" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/vybor-generalnogo-podriadchika-na-stroitelstvo-detskoi-akademii-v-kp/tender-4544461/#btid=2&amp;sqh=9b6960e6981e51e4e067c152b692d15a2de3f05d&amp;tsid=4544461458</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30 14:31</t>
+        </is>
+      </c>
+      <c r="B259" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C259" s="2" t="inlineStr"/>
+      <c r="D259" s="2" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="E259" s="2" t="inlineStr">
+        <is>
+          <t>4544326</t>
+        </is>
+      </c>
+      <c r="F259" s="2" t="inlineStr">
+        <is>
+          <t>Закупка карнизных плит для объекта строительства г. Пермь "Пермский строительный колледж"4544326 ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "КИНЕТИКА"Железобетонные изделия</t>
+        </is>
+      </c>
+      <c r="G259" s="2" t="inlineStr">
+        <is>
+          <t>ООО "КИНЕТИКА"</t>
+        </is>
+      </c>
+      <c r="H259" s="2" t="inlineStr">
+        <is>
+          <t>ООО "КИНЕТИКА"</t>
+        </is>
+      </c>
+      <c r="I259" s="2" t="inlineStr">
+        <is>
+          <t>9703136308</t>
+        </is>
+      </c>
+      <c r="J259" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K259" s="2" t="inlineStr">
+        <is>
+          <t>Широкова Анастасия Вячеславовна</t>
+        </is>
+      </c>
+      <c r="L259" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M259" s="2" t="inlineStr">
+        <is>
+          <t>62.01</t>
+        </is>
+      </c>
+      <c r="N259" s="2" t="inlineStr"/>
+      <c r="O259" s="2" t="inlineStr">
+        <is>
+          <t>30.07.2026 13:12 — 05.08.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P259" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ЗАМОСКВОРЕЧЬЕ, УЛ. ДУБИНИНСКАЯ, Д. 11/17, СТР. 3, ПОМЕЩ. 66А/Ч</t>
+        </is>
+      </c>
+      <c r="Q259" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-karniznykh-plit-dlia-ob-ekta-stroitelstva-g-perm-permskii/tender-4544326/#btid=2&amp;sqh=99eb551c3736f0002f29c0db17a5fd45f0dcf907&amp;tsid=4544326458</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q255"/>
+  <autoFilter ref="A1:Q259"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -21645,6 +21967,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q253" r:id="rId252"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q254" r:id="rId253"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q255" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q256" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q257" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q258" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q259" r:id="rId258"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-31 09:20 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$259</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$261</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q259"/>
+  <dimension ref="A1:Q261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -21710,8 +21710,158 @@
         </is>
       </c>
     </row>
+    <row r="260">
+      <c r="A260" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-31 09:20</t>
+        </is>
+      </c>
+      <c r="B260" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C260" s="2" t="inlineStr"/>
+      <c r="D260" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E260" s="2" t="inlineStr">
+        <is>
+          <t>4545806</t>
+        </is>
+      </c>
+      <c r="F260" s="2" t="inlineStr">
+        <is>
+          <t>ЗакупкаЖБИ</t>
+        </is>
+      </c>
+      <c r="G260" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H260" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I260" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J260" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K260" s="2" t="inlineStr"/>
+      <c r="L260" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M260" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N260" s="2" t="inlineStr"/>
+      <c r="O260" s="2" t="inlineStr">
+        <is>
+          <t>31.07.2026 11:52 — 03.08.2026 12:00</t>
+        </is>
+      </c>
+      <c r="P260" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ. ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q260" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zakupka-zhbi/tender-4545806/#btid=2&amp;sqh=68925aa23cf047b220893075532d4cfece9c81a5&amp;tsid=4545806458</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-31 09:20</t>
+        </is>
+      </c>
+      <c r="B261" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C261" s="2" t="inlineStr"/>
+      <c r="D261" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E261" s="2" t="inlineStr">
+        <is>
+          <t>4545669</t>
+        </is>
+      </c>
+      <c r="F261" s="2" t="inlineStr">
+        <is>
+          <t>Перемычки4545669 ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "АИМ МЕНЕДЖМЕНТ"Железобетонные изделия</t>
+        </is>
+      </c>
+      <c r="G261" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H261" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I261" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J261" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K261" s="2" t="inlineStr"/>
+      <c r="L261" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M261" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N261" s="2" t="inlineStr"/>
+      <c r="O261" s="2" t="inlineStr">
+        <is>
+          <t>31.07.2026 10:57 — 10.08.2026 08:00</t>
+        </is>
+      </c>
+      <c r="P261" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ. ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q261" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/peremychki/tender-4545669/#btid=2&amp;sqh=be19cc57cff445a6d782374bf690724a646e2661&amp;tsid=4545669458</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q259"/>
+  <autoFilter ref="A1:Q261"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -21971,6 +22121,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q257" r:id="rId256"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q258" r:id="rId257"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q259" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q260" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q261" r:id="rId260"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
leads: обновление 2026-07-31 14:34 UTC
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лиды" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$261</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лиды'!$A$1:$Q$263</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q261"/>
+  <dimension ref="A1:Q263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -21860,8 +21860,168 @@
         </is>
       </c>
     </row>
+    <row r="262">
+      <c r="A262" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-31 14:34</t>
+        </is>
+      </c>
+      <c r="B262" s="2" t="inlineStr">
+        <is>
+          <t>ЕИС</t>
+        </is>
+      </c>
+      <c r="C262" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D262" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E262" s="2" t="inlineStr">
+        <is>
+          <t>32616256678</t>
+        </is>
+      </c>
+      <c r="F262" s="2" t="inlineStr">
+        <is>
+          <t>Железобетонныеизделия</t>
+        </is>
+      </c>
+      <c r="G262" s="2" t="inlineStr">
+        <is>
+          <t>ГОСУДАРСТВЕННОЕ УНИТАРНОЕ ПРЕДПРИЯТИЕ КРАСНОДАРСКОГО КРАЯ "КУБАНЬВОДКОМПЛЕКС"</t>
+        </is>
+      </c>
+      <c r="H262" s="2" t="inlineStr">
+        <is>
+          <t>ГУП КК "КУБАНЬВОДКОМПЛЕКС"</t>
+        </is>
+      </c>
+      <c r="I262" s="2" t="inlineStr">
+        <is>
+          <t>2310010637</t>
+        </is>
+      </c>
+      <c r="J262" s="2" t="inlineStr">
+        <is>
+          <t>Краснодарский край</t>
+        </is>
+      </c>
+      <c r="K262" s="2" t="inlineStr">
+        <is>
+          <t>Лазарев Александр Александрович</t>
+        </is>
+      </c>
+      <c r="L262" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M262" s="2" t="inlineStr">
+        <is>
+          <t>36.00.1</t>
+        </is>
+      </c>
+      <c r="N262" s="2" t="inlineStr">
+        <is>
+          <t>191 603,57 ₽</t>
+        </is>
+      </c>
+      <c r="O262" s="2" t="inlineStr">
+        <is>
+          <t>31.07.2026 | 31.07.2026 | 07.08.2026</t>
+        </is>
+      </c>
+      <c r="P262" s="2" t="inlineStr">
+        <is>
+          <t>г Краснодар, ул им. Каляева, д 196</t>
+        </is>
+      </c>
+      <c r="Q262" s="3" t="inlineStr">
+        <is>
+          <t>https://zakupki.gov.ru/223/purchase/public/purchase/info/common-info.html?regNumber=32616256678</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-31 14:34</t>
+        </is>
+      </c>
+      <c r="B263" s="2" t="inlineStr">
+        <is>
+          <t>b2b-center</t>
+        </is>
+      </c>
+      <c r="C263" s="2" t="inlineStr"/>
+      <c r="D263" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="E263" s="2" t="inlineStr">
+        <is>
+          <t>4546139</t>
+        </is>
+      </c>
+      <c r="F263" s="2" t="inlineStr">
+        <is>
+          <t>ЖБИПЛИТА ПАГ14А800 6000*2000*140ММ ГОСТ25912-2015ПЛИТАЖБ П10.5 СЕРИЯ 3.407. ...  3.407.1-157 выпуск 1ПлитаПТ-10,5 995*495*60ММ ...</t>
+        </is>
+      </c>
+      <c r="G263" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="H263" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АИМ МЕНЕДЖМЕНТ"</t>
+        </is>
+      </c>
+      <c r="I263" s="2" t="inlineStr">
+        <is>
+          <t>9725042029</t>
+        </is>
+      </c>
+      <c r="J263" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="K263" s="2" t="inlineStr"/>
+      <c r="L263" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M263" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N263" s="2" t="inlineStr"/>
+      <c r="O263" s="2" t="inlineStr">
+        <is>
+          <t>31.07.2026 14:02 — 06.08.2026 20:00</t>
+        </is>
+      </c>
+      <c r="P263" s="2" t="inlineStr">
+        <is>
+          <t>115054, Г.МОСКВА, ВН.ТЕР.Г. МУНИЦИПАЛЬНЫЙ ОКРУГ ДАНИЛОВСКИЙ, УЛ. ДУБИНИНСКАЯ, Д. 53, СТР. 6, ЭТАЖ 7,8, ПОМЕЩ. VIII, IX</t>
+        </is>
+      </c>
+      <c r="Q263" s="3" t="inlineStr">
+        <is>
+          <t>https://www.b2b-center.ru/app/market-next/zhbi/tender-4546139/#btid=2&amp;sqh=e61456ce604356a76b139feeea6d4ab4ceaac56f&amp;tsid=4546139458</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q261"/>
+  <autoFilter ref="A1:Q263"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -22123,6 +22283,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q259" r:id="rId258"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q260" r:id="rId259"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q261" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q262" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q263" r:id="rId262"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>